<commit_message>
Scan 07.09.2026 18:41 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V22"/>
+  <dimension ref="A1:V21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>157.44</v>
+        <v>158.78</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,22 +614,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>85.40000000000001</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>60.1</v>
+        <v>61</v>
       </c>
       <c r="K2" t="n">
         <v>6</v>
       </c>
       <c r="L2" t="n">
-        <v>4.26</v>
+        <v>4.22</v>
       </c>
       <c r="M2" t="n">
-        <v>55</v>
+        <v>55.2</v>
       </c>
       <c r="N2" t="n">
-        <v>17.5</v>
+        <v>17.7</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>48.7</v>
+        <v>49.1</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -673,30 +673,30 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>NXPI</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>227.57</v>
+        <v>573.01</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -710,34 +710,34 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>83</v>
+        <v>83.5</v>
       </c>
       <c r="J3" t="n">
-        <v>43.6</v>
+        <v>52.1</v>
       </c>
       <c r="K3" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="L3" t="n">
-        <v>2.59</v>
+        <v>2.11</v>
       </c>
       <c r="M3" t="n">
-        <v>41.2</v>
+        <v>21.6</v>
       </c>
       <c r="N3" t="n">
-        <v>21.2</v>
+        <v>23.7</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>43.2</v>
+        <v>49.9</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -752,10 +752,14 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V3" t="inlineStr">
         <is>
           <t>No</t>
@@ -765,30 +769,30 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>NXPI</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>567.64</v>
+        <v>227.84</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -802,34 +806,34 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>82.5</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>49</v>
+        <v>43.9</v>
       </c>
       <c r="K4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L4" t="n">
-        <v>2.13</v>
+        <v>2.59</v>
       </c>
       <c r="M4" t="n">
-        <v>21.9</v>
+        <v>41.2</v>
       </c>
       <c r="N4" t="n">
-        <v>24.8</v>
+        <v>21.3</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>48.8</v>
+        <v>43.3</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -844,17 +848,13 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -865,7 +865,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>230.49</v>
+        <v>230.36</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -901,16 +901,19 @@
         <v>81.40000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>60.5</v>
+        <v>60.4</v>
       </c>
       <c r="K5" t="n">
         <v>7</v>
       </c>
       <c r="L5" t="n">
-        <v>3.28</v>
+        <v>3.29</v>
       </c>
       <c r="M5" t="n">
-        <v>33.6</v>
+        <v>45.4</v>
+      </c>
+      <c r="N5" t="n">
+        <v>89.90000000000001</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -958,7 +961,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>87.06</v>
+        <v>87.76000000000001</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -991,22 +994,22 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>80.8</v>
+        <v>81.2</v>
       </c>
       <c r="J6" t="n">
-        <v>55.2</v>
+        <v>58.1</v>
       </c>
       <c r="K6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L6" t="n">
-        <v>2.38</v>
+        <v>2.4</v>
       </c>
       <c r="M6" t="n">
         <v>28.7</v>
       </c>
       <c r="N6" t="n">
-        <v>25.7</v>
+        <v>25.9</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1014,7 +1017,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>60.7</v>
+        <v>61.7</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1038,7 +1041,7 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>TTM Squeeze</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
@@ -1054,7 +1057,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>769.59</v>
+        <v>770.1900000000001</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1087,19 +1090,22 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>78.59999999999999</v>
+        <v>78.5</v>
       </c>
       <c r="J7" t="n">
-        <v>55</v>
+        <v>55.6</v>
       </c>
       <c r="K7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L7" t="n">
         <v>0.75</v>
       </c>
       <c r="M7" t="n">
-        <v>10.9</v>
+        <v>11.7</v>
+      </c>
+      <c r="N7" t="n">
+        <v>35.9</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1107,7 +1113,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>64.5</v>
+        <v>64.7</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1139,30 +1145,30 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>UPS</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>102.64</v>
+        <v>217.72</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1179,19 +1185,19 @@
         <v>78.3</v>
       </c>
       <c r="J8" t="n">
-        <v>43.8</v>
+        <v>55</v>
       </c>
       <c r="K8" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="L8" t="n">
-        <v>1.79</v>
+        <v>2.16</v>
       </c>
       <c r="M8" t="n">
-        <v>28.5</v>
+        <v>26.4</v>
       </c>
       <c r="N8" t="n">
-        <v>44.1</v>
+        <v>34.5</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1199,31 +1205,31 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>49</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>Squeeze Expanding</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
@@ -1235,30 +1241,30 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>UPS</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>217.07</v>
+        <v>102.29</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1272,51 +1278,54 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>78.09999999999999</v>
+        <v>77.8</v>
       </c>
       <c r="J9" t="n">
-        <v>54.1</v>
+        <v>42.8</v>
       </c>
       <c r="K9" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="L9" t="n">
-        <v>2.15</v>
+        <v>1.85</v>
       </c>
       <c r="M9" t="n">
-        <v>28.4</v>
+        <v>28.5</v>
+      </c>
+      <c r="N9" t="n">
+        <v>44.4</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>64.09999999999999</v>
+        <v>48.6</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>Squeeze Expanding</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
@@ -1328,11 +1337,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>JPM</t>
+          <t>CHTR</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>358.43</v>
+        <v>151.99</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1365,34 +1374,34 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>74.59999999999999</v>
+        <v>74.8</v>
       </c>
       <c r="J10" t="n">
-        <v>54.7</v>
+        <v>52.2</v>
       </c>
       <c r="K10" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L10" t="n">
-        <v>1.65</v>
+        <v>5.06</v>
       </c>
       <c r="M10" t="n">
-        <v>17.3</v>
+        <v>60.7</v>
       </c>
       <c r="N10" t="n">
-        <v>5.2</v>
+        <v>56.4</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>67.09999999999999</v>
+        <v>44.2</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -1410,7 +1419,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr"/>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V10" t="inlineStr">
         <is>
           <t>No</t>
@@ -1420,11 +1433,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CHTR</t>
+          <t>JPM</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>150.97</v>
+        <v>358.64</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1457,34 +1470,34 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>73.3</v>
+        <v>74.7</v>
       </c>
       <c r="J11" t="n">
-        <v>51.4</v>
+        <v>55</v>
       </c>
       <c r="K11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L11" t="n">
-        <v>5.09</v>
+        <v>1.65</v>
       </c>
       <c r="M11" t="n">
-        <v>60.8</v>
+        <v>17.3</v>
       </c>
       <c r="N11" t="n">
-        <v>56.5</v>
+        <v>4.9</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>43.8</v>
+        <v>67.2</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1502,11 +1515,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr">
         <is>
           <t>No</t>
@@ -1516,11 +1525,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AMP</t>
+          <t>BAC</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>563.76</v>
+        <v>62.68</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1553,22 +1562,22 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>70.7</v>
+        <v>70.2</v>
       </c>
       <c r="J12" t="n">
-        <v>58.5</v>
+        <v>55.3</v>
       </c>
       <c r="K12" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="L12" t="n">
-        <v>2.11</v>
+        <v>1.7</v>
       </c>
       <c r="M12" t="n">
-        <v>18.7</v>
+        <v>16.6</v>
       </c>
       <c r="N12" t="n">
-        <v>8.9</v>
+        <v>17.1</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1576,7 +1585,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>69.7</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1585,12 +1594,12 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -1608,30 +1617,30 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>KHC</t>
+          <t>AMP</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>24.86</v>
+        <v>560.5599999999999</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1645,22 +1654,22 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>69.2</v>
+        <v>67.2</v>
       </c>
       <c r="J13" t="n">
-        <v>44.9</v>
+        <v>56.3</v>
       </c>
       <c r="K13" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L13" t="n">
-        <v>2.7</v>
+        <v>2.22</v>
       </c>
       <c r="M13" t="n">
-        <v>35.3</v>
+        <v>18.9</v>
       </c>
       <c r="N13" t="n">
-        <v>92</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1668,11 +1677,11 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>52.9</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -1682,7 +1691,7 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -1692,23 +1701,23 @@
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>Divergence, Squeeze Expanding</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BAC</t>
+          <t>XLF</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>62.67</v>
+        <v>58.1</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1741,22 +1750,19 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>67.8</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="J14" t="n">
-        <v>52.9</v>
+        <v>55.5</v>
       </c>
       <c r="K14" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L14" t="n">
-        <v>1.73</v>
+        <v>1.18</v>
       </c>
       <c r="M14" t="n">
-        <v>16.7</v>
-      </c>
-      <c r="N14" t="n">
-        <v>17.8</v>
+        <v>25.4</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1764,11 +1770,11 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>66</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -1788,7 +1794,7 @@
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>Squeeze Expanding</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
@@ -1800,78 +1806,81 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>XLF</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>58.18</v>
+        <v>33.72</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>65.7</v>
+        <v>63.1</v>
       </c>
       <c r="J15" t="n">
-        <v>56.3</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="K15" t="n">
-        <v>20</v>
+        <v>89</v>
       </c>
       <c r="L15" t="n">
-        <v>1.18</v>
+        <v>3.15</v>
       </c>
       <c r="M15" t="n">
-        <v>14.9</v>
+        <v>43.6</v>
+      </c>
+      <c r="N15" t="n">
+        <v>91.7</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>70.40000000000001</v>
+        <v>53.3</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -1879,11 +1888,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+      <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr">
         <is>
           <t>No</t>
@@ -1893,11 +1898,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>33.74</v>
+        <v>151</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1930,30 +1935,30 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>63.1</v>
+        <v>63</v>
       </c>
       <c r="J16" t="n">
-        <v>64.2</v>
+        <v>67.7</v>
       </c>
       <c r="K16" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="L16" t="n">
-        <v>3.15</v>
+        <v>2.27</v>
       </c>
       <c r="M16" t="n">
-        <v>43.6</v>
+        <v>25.9</v>
       </c>
       <c r="N16" t="n">
-        <v>91.7</v>
+        <v>42.6</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>53.3</v>
+        <v>68.2</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1985,11 +1990,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>MRK</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>150.45</v>
+        <v>150.33</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -2022,22 +2027,22 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>62.1</v>
+        <v>61.2</v>
       </c>
       <c r="J17" t="n">
-        <v>66.2</v>
+        <v>62.3</v>
       </c>
       <c r="K17" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="L17" t="n">
-        <v>2.28</v>
+        <v>2.57</v>
       </c>
       <c r="M17" t="n">
-        <v>26</v>
+        <v>42.9</v>
       </c>
       <c r="N17" t="n">
-        <v>43.2</v>
+        <v>96.7</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2045,7 +2050,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>67.8</v>
+        <v>71.2</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2054,17 +2059,17 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
@@ -2077,11 +2082,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>MRK</t>
+          <t>EL</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>150.23</v>
+        <v>103.86</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2114,19 +2119,22 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>60.9</v>
+        <v>58.1</v>
       </c>
       <c r="J18" t="n">
-        <v>62.1</v>
+        <v>67.3</v>
       </c>
       <c r="K18" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="L18" t="n">
-        <v>2.57</v>
+        <v>3.34</v>
       </c>
       <c r="M18" t="n">
-        <v>28</v>
+        <v>55.9</v>
+      </c>
+      <c r="N18" t="n">
+        <v>62</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -2134,7 +2142,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>71.09999999999999</v>
+        <v>63</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2143,17 +2151,17 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
@@ -2166,11 +2174,11 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>EL</t>
+          <t>TGT</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>103.38</v>
+        <v>164.44</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2199,23 +2207,26 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>57.3</v>
+        <v>46.7</v>
       </c>
       <c r="J19" t="n">
-        <v>66.7</v>
+        <v>63.6</v>
       </c>
       <c r="K19" t="n">
-        <v>93</v>
+        <v>65</v>
       </c>
       <c r="L19" t="n">
-        <v>3.32</v>
+        <v>2.48</v>
       </c>
       <c r="M19" t="n">
-        <v>33.1</v>
+        <v>29.9</v>
+      </c>
+      <c r="N19" t="n">
+        <v>48</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -2223,7 +2234,7 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>62.7</v>
+        <v>73.5</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2232,17 +2243,17 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U19" t="inlineStr"/>
@@ -2255,30 +2266,30 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TGT</t>
+          <t>HON</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>164.33</v>
+        <v>209.61</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2288,34 +2299,34 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>46.2</v>
+        <v>43.5</v>
       </c>
       <c r="J20" t="n">
-        <v>63.5</v>
+        <v>34.8</v>
       </c>
       <c r="K20" t="n">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="L20" t="n">
-        <v>2.46</v>
+        <v>2.3</v>
       </c>
       <c r="M20" t="n">
-        <v>29.9</v>
+        <v>27.4</v>
       </c>
       <c r="N20" t="n">
-        <v>48</v>
+        <v>46.8</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>73.5</v>
+        <v>40.3</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2329,12 +2340,12 @@
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U20" t="inlineStr"/>
@@ -2351,7 +2362,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>132.55</v>
+        <v>132.08</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2384,22 +2395,22 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>42.6</v>
+        <v>42.4</v>
       </c>
       <c r="J21" t="n">
-        <v>24.2</v>
+        <v>22.8</v>
       </c>
       <c r="K21" t="n">
         <v>96</v>
       </c>
       <c r="L21" t="n">
-        <v>1.89</v>
+        <v>1.9</v>
       </c>
       <c r="M21" t="n">
-        <v>23.1</v>
+        <v>23</v>
       </c>
       <c r="N21" t="n">
-        <v>54.3</v>
+        <v>53.8</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2407,7 +2418,7 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>33.8</v>
+        <v>33.6</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2431,98 +2442,6 @@
       </c>
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>HON</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>207.79</v>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>41.5</v>
-      </c>
-      <c r="J22" t="n">
-        <v>32</v>
-      </c>
-      <c r="K22" t="n">
-        <v>92</v>
-      </c>
-      <c r="L22" t="n">
-        <v>2.25</v>
-      </c>
-      <c r="M22" t="n">
-        <v>27.1</v>
-      </c>
-      <c r="N22" t="n">
-        <v>45.8</v>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P22" t="n">
-        <v>39.6</v>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T22" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr"/>
-      <c r="V22" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 08.09.2026 17:51 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V21"/>
+  <dimension ref="A1:V25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>158.78</v>
+        <v>162.32</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,22 +614,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>85.90000000000001</v>
+        <v>84.8</v>
       </c>
       <c r="J2" t="n">
-        <v>61</v>
+        <v>63.3</v>
       </c>
       <c r="K2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L2" t="n">
-        <v>4.22</v>
+        <v>4.56</v>
       </c>
       <c r="M2" t="n">
-        <v>55.2</v>
+        <v>54.5</v>
       </c>
       <c r="N2" t="n">
-        <v>17.7</v>
+        <v>16.8</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>49.1</v>
+        <v>50.3</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -673,11 +673,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>573.01</v>
+        <v>218.35</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -710,30 +710,30 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>83.5</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>52.1</v>
+        <v>55.9</v>
       </c>
       <c r="K3" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="L3" t="n">
-        <v>2.11</v>
+        <v>2.07</v>
       </c>
       <c r="M3" t="n">
-        <v>21.6</v>
+        <v>26.4</v>
       </c>
       <c r="N3" t="n">
-        <v>23.7</v>
+        <v>34.6</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>49.9</v>
+        <v>64.8</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -747,7 +747,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -769,11 +769,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NXPI</t>
+          <t>CI</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>227.84</v>
+        <v>277.69</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -806,22 +806,22 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>83.09999999999999</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>43.9</v>
+        <v>46.7</v>
       </c>
       <c r="K4" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="L4" t="n">
-        <v>2.59</v>
+        <v>2.09</v>
       </c>
       <c r="M4" t="n">
-        <v>41.2</v>
+        <v>27.7</v>
       </c>
       <c r="N4" t="n">
-        <v>21.3</v>
+        <v>20.1</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -829,62 +829,66 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>43.3</v>
+        <v>47.8</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>NXPI</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>230.36</v>
+        <v>224.13</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -898,30 +902,30 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>81.40000000000001</v>
+        <v>81.7</v>
       </c>
       <c r="J5" t="n">
-        <v>60.4</v>
+        <v>40.9</v>
       </c>
       <c r="K5" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="L5" t="n">
-        <v>3.29</v>
+        <v>2.71</v>
       </c>
       <c r="M5" t="n">
-        <v>45.4</v>
+        <v>41.4</v>
       </c>
       <c r="N5" t="n">
-        <v>89.90000000000001</v>
+        <v>21.5</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>61.8</v>
+        <v>42.3</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -935,7 +939,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -945,71 +949,71 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>Squeeze Expanding</t>
+          <t>Divergence</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GM</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>87.76000000000001</v>
+        <v>248.25</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>81.2</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="J6" t="n">
-        <v>58.1</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="K6" t="n">
-        <v>4</v>
+        <v>99</v>
       </c>
       <c r="L6" t="n">
-        <v>2.4</v>
+        <v>4.53</v>
       </c>
       <c r="M6" t="n">
-        <v>28.7</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="N6" t="n">
-        <v>25.9</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1017,21 +1021,21 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>61.7</v>
+        <v>65.8</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1041,23 +1045,23 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>Divergence</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>ANET</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>770.1900000000001</v>
+        <v>198.76</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1090,22 +1094,22 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>78.5</v>
+        <v>81.3</v>
       </c>
       <c r="J7" t="n">
-        <v>55.6</v>
+        <v>56.8</v>
       </c>
       <c r="K7" t="n">
         <v>4</v>
       </c>
       <c r="L7" t="n">
-        <v>0.75</v>
+        <v>3.78</v>
       </c>
       <c r="M7" t="n">
-        <v>11.7</v>
+        <v>56.1</v>
       </c>
       <c r="N7" t="n">
-        <v>35.9</v>
+        <v>58.3</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1113,7 +1117,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>64.7</v>
+        <v>63.3</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1122,12 +1126,12 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -1135,7 +1139,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr"/>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V7" t="inlineStr">
         <is>
           <t>No</t>
@@ -1145,30 +1153,30 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>217.72</v>
+        <v>232.13</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1182,30 +1190,30 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>78.3</v>
+        <v>81</v>
       </c>
       <c r="J8" t="n">
-        <v>55</v>
+        <v>47.6</v>
       </c>
       <c r="K8" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="L8" t="n">
-        <v>2.16</v>
+        <v>2.32</v>
       </c>
       <c r="M8" t="n">
-        <v>26.4</v>
+        <v>29.5</v>
       </c>
       <c r="N8" t="n">
-        <v>34.5</v>
+        <v>17</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>64.40000000000001</v>
+        <v>45.4</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1214,12 +1222,12 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -1229,42 +1237,42 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>UPS</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>102.29</v>
+        <v>767.61</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1278,30 +1286,27 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>77.8</v>
+        <v>79.8</v>
       </c>
       <c r="J9" t="n">
-        <v>42.8</v>
+        <v>53</v>
       </c>
       <c r="K9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L9" t="n">
-        <v>1.85</v>
+        <v>0.73</v>
       </c>
       <c r="M9" t="n">
-        <v>28.5</v>
-      </c>
-      <c r="N9" t="n">
-        <v>44.4</v>
+        <v>12.3</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>48.6</v>
+        <v>63.4</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1315,7 +1320,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1323,11 +1328,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
           <t>No</t>
@@ -1337,11 +1338,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CHTR</t>
+          <t>GM</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>151.99</v>
+        <v>85.81999999999999</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1374,30 +1375,30 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>74.8</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="J10" t="n">
-        <v>52.2</v>
+        <v>50.8</v>
       </c>
       <c r="K10" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L10" t="n">
-        <v>5.06</v>
+        <v>2.52</v>
       </c>
       <c r="M10" t="n">
-        <v>60.7</v>
+        <v>25.1</v>
       </c>
       <c r="N10" t="n">
-        <v>56.4</v>
+        <v>14</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>44.2</v>
+        <v>58</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1421,23 +1422,23 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>TTM Squeeze</t>
+          <t>TTM Squeeze, Divergence</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>JPM</t>
+          <t>BAC</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>358.64</v>
+        <v>62.76</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1470,22 +1471,19 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>74.7</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>55</v>
+        <v>55.8</v>
       </c>
       <c r="K11" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="L11" t="n">
-        <v>1.65</v>
+        <v>1.62</v>
       </c>
       <c r="M11" t="n">
-        <v>17.3</v>
-      </c>
-      <c r="N11" t="n">
-        <v>4.9</v>
+        <v>22.8</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1493,7 +1491,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>67.2</v>
+        <v>66.8</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1502,12 +1500,12 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1525,30 +1523,30 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BAC</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>62.68</v>
+        <v>552.01</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1562,85 +1560,89 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>70.2</v>
+        <v>74.3</v>
       </c>
       <c r="J12" t="n">
-        <v>55.3</v>
+        <v>41</v>
       </c>
       <c r="K12" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="L12" t="n">
-        <v>1.7</v>
+        <v>2.4</v>
       </c>
       <c r="M12" t="n">
-        <v>16.6</v>
+        <v>21.7</v>
       </c>
       <c r="N12" t="n">
-        <v>17.1</v>
+        <v>24</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>66.59999999999999</v>
+        <v>45.9</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AMP</t>
+          <t>UPS</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>560.5599999999999</v>
+        <v>100.85</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1654,34 +1656,34 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>67.2</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="J13" t="n">
-        <v>56.3</v>
+        <v>38.7</v>
       </c>
       <c r="K13" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L13" t="n">
-        <v>2.22</v>
+        <v>1.83</v>
       </c>
       <c r="M13" t="n">
-        <v>18.9</v>
+        <v>28.5</v>
       </c>
       <c r="N13" t="n">
-        <v>9.800000000000001</v>
+        <v>44.1</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>69.09999999999999</v>
+        <v>46.8</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -1691,7 +1693,7 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -1701,23 +1703,23 @@
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>TTM Squeeze</t>
+          <t>Divergence, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>XLF</t>
+          <t>JPM</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>58.1</v>
+        <v>355.65</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1750,19 +1752,22 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>65.59999999999999</v>
+        <v>73.3</v>
       </c>
       <c r="J14" t="n">
-        <v>55.5</v>
+        <v>50.8</v>
       </c>
       <c r="K14" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="L14" t="n">
-        <v>1.18</v>
+        <v>1.61</v>
       </c>
       <c r="M14" t="n">
-        <v>25.4</v>
+        <v>17.3</v>
+      </c>
+      <c r="N14" t="n">
+        <v>5.1</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1770,11 +1775,11 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>70.09999999999999</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -1794,7 +1799,7 @@
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>TTM Squeeze</t>
+          <t>Squeeze Expanding</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
@@ -1806,81 +1811,81 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>AMP</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>33.72</v>
+        <v>559.71</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>63.1</v>
+        <v>72.3</v>
       </c>
       <c r="J15" t="n">
-        <v>64.09999999999999</v>
+        <v>55.7</v>
       </c>
       <c r="K15" t="n">
-        <v>89</v>
+        <v>7</v>
       </c>
       <c r="L15" t="n">
-        <v>3.15</v>
+        <v>2.09</v>
       </c>
       <c r="M15" t="n">
-        <v>43.6</v>
+        <v>18.4</v>
       </c>
       <c r="N15" t="n">
-        <v>91.7</v>
+        <v>7.5</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>53.3</v>
+        <v>68.7</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>FIRED</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -1888,7 +1893,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr"/>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>Squeeze Fired</t>
+        </is>
+      </c>
       <c r="V15" t="inlineStr">
         <is>
           <t>No</t>
@@ -1898,15 +1907,15 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>CHTR</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>151</v>
+        <v>145.33</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -1921,128 +1930,129 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>63</v>
+        <v>67.2</v>
       </c>
       <c r="J16" t="n">
-        <v>67.7</v>
+        <v>46.9</v>
       </c>
       <c r="K16" t="n">
-        <v>90</v>
+        <v>8</v>
       </c>
       <c r="L16" t="n">
-        <v>2.27</v>
+        <v>5.22</v>
       </c>
       <c r="M16" t="n">
-        <v>25.9</v>
+        <v>59.7</v>
       </c>
       <c r="N16" t="n">
-        <v>42.6</v>
+        <v>55</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>68.2</v>
+        <v>41.7</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>MRK</t>
+          <t>XLF</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>150.33</v>
+        <v>57.55</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>61.2</v>
+        <v>62.3</v>
       </c>
       <c r="J17" t="n">
-        <v>62.3</v>
+        <v>50.2</v>
       </c>
       <c r="K17" t="n">
-        <v>91</v>
+        <v>21</v>
       </c>
       <c r="L17" t="n">
-        <v>2.57</v>
+        <v>1.19</v>
       </c>
       <c r="M17" t="n">
-        <v>42.9</v>
-      </c>
-      <c r="N17" t="n">
-        <v>96.7</v>
+        <v>15.6</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2050,11 +2060,11 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>71.2</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -2069,24 +2079,28 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>EL</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>103.86</v>
+        <v>32.44</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2119,30 +2133,30 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>58.1</v>
+        <v>60.8</v>
       </c>
       <c r="J18" t="n">
-        <v>67.3</v>
+        <v>53.8</v>
       </c>
       <c r="K18" t="n">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="L18" t="n">
-        <v>3.34</v>
+        <v>3.38</v>
       </c>
       <c r="M18" t="n">
-        <v>55.9</v>
+        <v>41.7</v>
       </c>
       <c r="N18" t="n">
-        <v>62</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>63</v>
+        <v>48.6</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2151,34 +2165,38 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U18" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TGT</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>164.44</v>
+        <v>146.93</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2207,26 +2225,26 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>46.7</v>
+        <v>60.4</v>
       </c>
       <c r="J19" t="n">
-        <v>63.6</v>
+        <v>57.5</v>
       </c>
       <c r="K19" t="n">
-        <v>65</v>
+        <v>87</v>
       </c>
       <c r="L19" t="n">
-        <v>2.48</v>
+        <v>2.53</v>
       </c>
       <c r="M19" t="n">
-        <v>29.9</v>
+        <v>27.5</v>
       </c>
       <c r="N19" t="n">
-        <v>48</v>
+        <v>52.6</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -2234,7 +2252,7 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>73.5</v>
+        <v>62.6</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2256,40 +2274,44 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr"/>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>HON</t>
+          <t>MRK</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>209.61</v>
+        <v>148.96</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2303,30 +2325,30 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>43.5</v>
+        <v>57.8</v>
       </c>
       <c r="J20" t="n">
-        <v>34.8</v>
+        <v>59.6</v>
       </c>
       <c r="K20" t="n">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="L20" t="n">
-        <v>2.3</v>
+        <v>2.61</v>
       </c>
       <c r="M20" t="n">
-        <v>27.4</v>
+        <v>43</v>
       </c>
       <c r="N20" t="n">
-        <v>46.8</v>
+        <v>97.3</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>40.3</v>
+        <v>69.5</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2340,12 +2362,12 @@
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U20" t="inlineStr"/>
@@ -2358,90 +2380,467 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>EL</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>101.19</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>55.4</v>
+      </c>
+      <c r="J21" t="n">
+        <v>60.6</v>
+      </c>
+      <c r="K21" t="n">
+        <v>92</v>
+      </c>
+      <c r="L21" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="M21" t="n">
+        <v>56.1</v>
+      </c>
+      <c r="N21" t="n">
+        <v>62.6</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P21" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>DLTR</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>124.27</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="J22" t="n">
+        <v>42.4</v>
+      </c>
+      <c r="K22" t="n">
+        <v>13</v>
+      </c>
+      <c r="L22" t="n">
+        <v>4.14</v>
+      </c>
+      <c r="M22" t="n">
+        <v>31.7</v>
+      </c>
+      <c r="N22" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P22" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>TTWO</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>214.63</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>51</v>
+      </c>
+      <c r="J23" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="K23" t="n">
+        <v>89</v>
+      </c>
+      <c r="L23" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="M23" t="n">
+        <v>42</v>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P23" t="n">
+        <v>43</v>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>TJX</t>
         </is>
       </c>
-      <c r="B21" t="n">
-        <v>132.08</v>
-      </c>
-      <c r="C21" t="inlineStr">
+      <c r="B24" t="n">
+        <v>129.31</v>
+      </c>
+      <c r="C24" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>Credit Put</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>7-21 DTE</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>EXPANSION</t>
         </is>
       </c>
-      <c r="I21" t="n">
-        <v>42.4</v>
-      </c>
-      <c r="J21" t="n">
-        <v>22.8</v>
-      </c>
-      <c r="K21" t="n">
-        <v>96</v>
-      </c>
-      <c r="L21" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="M21" t="n">
-        <v>23</v>
-      </c>
-      <c r="N21" t="n">
-        <v>53.8</v>
-      </c>
-      <c r="O21" t="inlineStr">
+      <c r="I24" t="n">
+        <v>42.8</v>
+      </c>
+      <c r="J24" t="n">
+        <v>20</v>
+      </c>
+      <c r="K24" t="n">
+        <v>94</v>
+      </c>
+      <c r="L24" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="M24" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="N24" t="n">
+        <v>52.3</v>
+      </c>
+      <c r="O24" t="inlineStr">
         <is>
           <t>Bearish</t>
         </is>
       </c>
-      <c r="P21" t="n">
-        <v>33.6</v>
-      </c>
-      <c r="Q21" t="inlineStr">
+      <c r="P24" t="n">
+        <v>32</v>
+      </c>
+      <c r="Q24" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="R21" t="inlineStr">
+      <c r="R24" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="S21" t="inlineStr">
+      <c r="S24" t="inlineStr">
         <is>
           <t>red</t>
         </is>
       </c>
-      <c r="T21" t="inlineStr">
+      <c r="T24" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="U21" t="inlineStr"/>
-      <c r="V21" t="inlineStr">
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>HON</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>208.22</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>38.6</v>
+      </c>
+      <c r="J25" t="n">
+        <v>33.7</v>
+      </c>
+      <c r="K25" t="n">
+        <v>81</v>
+      </c>
+      <c r="L25" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="M25" t="n">
+        <v>27</v>
+      </c>
+      <c r="N25" t="n">
+        <v>45.4</v>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P25" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 09.09.2026 17:45 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V25"/>
+  <dimension ref="A1:V16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>162.32</v>
+        <v>238.69</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,22 +614,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>84.8</v>
+        <v>80.7</v>
       </c>
       <c r="J2" t="n">
-        <v>63.3</v>
+        <v>54.2</v>
       </c>
       <c r="K2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L2" t="n">
-        <v>4.56</v>
+        <v>2.43</v>
       </c>
       <c r="M2" t="n">
-        <v>54.5</v>
+        <v>26.7</v>
       </c>
       <c r="N2" t="n">
-        <v>16.8</v>
+        <v>13.1</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,11 +637,11 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>50.3</v>
+        <v>47.4</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -656,12 +656,12 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Squeeze Expanding</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -673,30 +673,30 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>CI</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>218.35</v>
+        <v>276.05</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -710,30 +710,30 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>84.09999999999999</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="J3" t="n">
-        <v>55.9</v>
+        <v>46.7</v>
       </c>
       <c r="K3" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="L3" t="n">
-        <v>2.07</v>
+        <v>2.23</v>
       </c>
       <c r="M3" t="n">
-        <v>26.4</v>
+        <v>25.6</v>
       </c>
       <c r="N3" t="n">
-        <v>34.6</v>
+        <v>15.4</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>64.8</v>
+        <v>47.7</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -742,12 +742,12 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -757,27 +757,27 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>TTM Squeeze, Divergence</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>277.69</v>
+        <v>247.68</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -792,48 +792,48 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>81.90000000000001</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>46.7</v>
+        <v>66.3</v>
       </c>
       <c r="K4" t="n">
-        <v>8</v>
+        <v>97</v>
       </c>
       <c r="L4" t="n">
-        <v>2.09</v>
+        <v>4.42</v>
       </c>
       <c r="M4" t="n">
-        <v>27.7</v>
+        <v>75</v>
       </c>
       <c r="N4" t="n">
-        <v>20.1</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>47.8</v>
+        <v>65.5</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -843,7 +843,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -851,44 +851,40 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>NXPI</t>
+          <t>XOM</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>224.13</v>
+        <v>164.77</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -902,30 +898,30 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>81.7</v>
+        <v>74</v>
       </c>
       <c r="J5" t="n">
-        <v>40.9</v>
+        <v>60.1</v>
       </c>
       <c r="K5" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="L5" t="n">
-        <v>2.71</v>
+        <v>2.16</v>
       </c>
       <c r="M5" t="n">
-        <v>41.4</v>
+        <v>25.7</v>
       </c>
       <c r="N5" t="n">
-        <v>21.5</v>
+        <v>54.7</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>42.3</v>
+        <v>61.8</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -939,7 +935,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -949,27 +945,27 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>Squeeze Expanding</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>248.25</v>
+        <v>554.5</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -984,48 +980,48 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>81.59999999999999</v>
+        <v>71.5</v>
       </c>
       <c r="J6" t="n">
-        <v>66.90000000000001</v>
+        <v>42.7</v>
       </c>
       <c r="K6" t="n">
-        <v>99</v>
+        <v>13</v>
       </c>
       <c r="L6" t="n">
-        <v>4.53</v>
+        <v>2.34</v>
       </c>
       <c r="M6" t="n">
-        <v>75.59999999999999</v>
+        <v>21.4</v>
       </c>
       <c r="N6" t="n">
-        <v>93.90000000000001</v>
+        <v>23.2</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>65.8</v>
+        <v>46.3</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1035,7 +1031,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1045,42 +1041,42 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ANET</t>
+          <t>UPS</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>198.76</v>
+        <v>99.39</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1094,30 +1090,30 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>81.3</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="J7" t="n">
-        <v>56.8</v>
+        <v>35.2</v>
       </c>
       <c r="K7" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="L7" t="n">
-        <v>3.78</v>
+        <v>1.8</v>
       </c>
       <c r="M7" t="n">
-        <v>56.1</v>
+        <v>21.8</v>
       </c>
       <c r="N7" t="n">
-        <v>58.3</v>
+        <v>17.9</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>63.3</v>
+        <v>45.2</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1126,12 +1122,12 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -1141,23 +1137,23 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>Squeeze Expanding</t>
+          <t>Divergence, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>PG</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>232.13</v>
+        <v>142.57</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1190,22 +1186,22 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>81</v>
+        <v>66.5</v>
       </c>
       <c r="J8" t="n">
-        <v>47.6</v>
+        <v>41.4</v>
       </c>
       <c r="K8" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="L8" t="n">
-        <v>2.32</v>
+        <v>1.64</v>
       </c>
       <c r="M8" t="n">
-        <v>29.5</v>
+        <v>15.6</v>
       </c>
       <c r="N8" t="n">
-        <v>17</v>
+        <v>12.6</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1213,7 +1209,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>45.4</v>
+        <v>44.3</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1249,30 +1245,30 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>CHTR</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>767.61</v>
+        <v>136.04</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1286,31 +1282,34 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>79.8</v>
+        <v>54.6</v>
       </c>
       <c r="J9" t="n">
-        <v>53</v>
+        <v>40.7</v>
       </c>
       <c r="K9" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="L9" t="n">
-        <v>0.73</v>
+        <v>5.95</v>
       </c>
       <c r="M9" t="n">
-        <v>12.3</v>
+        <v>60.2</v>
+      </c>
+      <c r="N9" t="n">
+        <v>55.7</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>63.4</v>
+        <v>38.6</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1325,84 +1324,88 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>GM</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>85.81999999999999</v>
+        <v>32.13</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>78.90000000000001</v>
+        <v>51.6</v>
       </c>
       <c r="J10" t="n">
-        <v>50.8</v>
+        <v>51.6</v>
       </c>
       <c r="K10" t="n">
-        <v>1</v>
+        <v>81</v>
       </c>
       <c r="L10" t="n">
-        <v>2.52</v>
+        <v>3.32</v>
       </c>
       <c r="M10" t="n">
-        <v>25.1</v>
+        <v>40.7</v>
       </c>
       <c r="N10" t="n">
-        <v>14</v>
+        <v>82.7</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>58</v>
+        <v>47.6</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -1417,73 +1420,72 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr">
+        <is>
           <t>No</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence</t>
-        </is>
-      </c>
-      <c r="V10" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>BAC</t>
+          <t>EL</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>62.76</v>
+        <v>98.69</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>77.90000000000001</v>
+        <v>51.4</v>
       </c>
       <c r="J11" t="n">
-        <v>55.8</v>
+        <v>55.1</v>
       </c>
       <c r="K11" t="n">
-        <v>12</v>
+        <v>90</v>
       </c>
       <c r="L11" t="n">
-        <v>1.62</v>
+        <v>3.64</v>
       </c>
       <c r="M11" t="n">
-        <v>22.8</v>
+        <v>56.8</v>
+      </c>
+      <c r="N11" t="n">
+        <v>64</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1491,7 +1493,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>66.8</v>
+        <v>57.7</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1500,82 +1502,86 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>TJX</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>552.01</v>
+        <v>126.1</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>74.3</v>
+        <v>49.1</v>
       </c>
       <c r="J12" t="n">
-        <v>41</v>
+        <v>17.4</v>
       </c>
       <c r="K12" t="n">
-        <v>10</v>
+        <v>95</v>
       </c>
       <c r="L12" t="n">
-        <v>2.4</v>
+        <v>2.15</v>
       </c>
       <c r="M12" t="n">
-        <v>21.7</v>
+        <v>20.9</v>
       </c>
       <c r="N12" t="n">
-        <v>24</v>
+        <v>41.9</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1583,11 +1589,11 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>45.9</v>
+        <v>30.4</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -1602,12 +1608,12 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+          <t>Divergence</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
@@ -1619,15 +1625,15 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>UPS</t>
+          <t>MRK</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>100.85</v>
+        <v>147.85</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -1642,44 +1648,44 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>74.09999999999999</v>
+        <v>47.6</v>
       </c>
       <c r="J13" t="n">
-        <v>38.7</v>
+        <v>57.5</v>
       </c>
       <c r="K13" t="n">
-        <v>4</v>
+        <v>88</v>
       </c>
       <c r="L13" t="n">
-        <v>1.83</v>
+        <v>2.48</v>
       </c>
       <c r="M13" t="n">
-        <v>28.5</v>
+        <v>43.2</v>
       </c>
       <c r="N13" t="n">
-        <v>44.1</v>
+        <v>98</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>46.8</v>
+        <v>68.3</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1693,81 +1699,77 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="inlineStr">
+        <is>
           <t>No</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V13" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>JPM</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>355.65</v>
+        <v>145.71</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>73.3</v>
+        <v>44.8</v>
       </c>
       <c r="J14" t="n">
-        <v>50.8</v>
+        <v>54.8</v>
       </c>
       <c r="K14" t="n">
-        <v>10</v>
+        <v>71</v>
       </c>
       <c r="L14" t="n">
-        <v>1.61</v>
+        <v>2.45</v>
       </c>
       <c r="M14" t="n">
-        <v>17.3</v>
+        <v>26.7</v>
       </c>
       <c r="N14" t="n">
-        <v>5.1</v>
+        <v>48.2</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1775,7 +1777,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>64.90000000000001</v>
+        <v>61.1</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1794,14 +1796,10 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr">
         <is>
           <t>No</t>
@@ -1811,30 +1809,30 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>AMP</t>
+          <t>DLTR</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>559.71</v>
+        <v>121</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1844,26 +1842,26 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>72.3</v>
+        <v>41.9</v>
       </c>
       <c r="J15" t="n">
-        <v>55.7</v>
+        <v>38.3</v>
       </c>
       <c r="K15" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="L15" t="n">
-        <v>2.09</v>
+        <v>4.18</v>
       </c>
       <c r="M15" t="n">
-        <v>18.4</v>
+        <v>32.6</v>
       </c>
       <c r="N15" t="n">
-        <v>7.5</v>
+        <v>13</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1871,7 +1869,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>68.7</v>
+        <v>51.2</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1890,76 +1888,76 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>Squeeze Fired</t>
+          <t>Squeeze Fired, Divergence</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CHTR</t>
+          <t>HON</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>145.33</v>
+        <v>206.38</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>67.2</v>
+        <v>38.1</v>
       </c>
       <c r="J16" t="n">
-        <v>46.9</v>
+        <v>32.2</v>
       </c>
       <c r="K16" t="n">
-        <v>8</v>
+        <v>83</v>
       </c>
       <c r="L16" t="n">
-        <v>5.22</v>
+        <v>2.07</v>
       </c>
       <c r="M16" t="n">
-        <v>59.7</v>
+        <v>26.9</v>
       </c>
       <c r="N16" t="n">
-        <v>55</v>
+        <v>44.8</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1967,11 +1965,11 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>41.7</v>
+        <v>39</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -1981,866 +1979,16 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>XLF</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>57.55</v>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Debit Call</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>62.3</v>
-      </c>
-      <c r="J17" t="n">
-        <v>50.2</v>
-      </c>
-      <c r="K17" t="n">
-        <v>21</v>
-      </c>
-      <c r="L17" t="n">
-        <v>1.19</v>
-      </c>
-      <c r="M17" t="n">
-        <v>15.6</v>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P17" t="n">
-        <v>65.90000000000001</v>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T17" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence</t>
-        </is>
-      </c>
-      <c r="V17" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>CPRT</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>32.44</v>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>60.8</v>
-      </c>
-      <c r="J18" t="n">
-        <v>53.8</v>
-      </c>
-      <c r="K18" t="n">
-        <v>87</v>
-      </c>
-      <c r="L18" t="n">
-        <v>3.38</v>
-      </c>
-      <c r="M18" t="n">
-        <v>41.7</v>
-      </c>
-      <c r="N18" t="n">
-        <v>85.59999999999999</v>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P18" t="n">
-        <v>48.6</v>
-      </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S18" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T18" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U18" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
-      <c r="V18" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>GILD</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>146.93</v>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>60.4</v>
-      </c>
-      <c r="J19" t="n">
-        <v>57.5</v>
-      </c>
-      <c r="K19" t="n">
-        <v>87</v>
-      </c>
-      <c r="L19" t="n">
-        <v>2.53</v>
-      </c>
-      <c r="M19" t="n">
-        <v>27.5</v>
-      </c>
-      <c r="N19" t="n">
-        <v>52.6</v>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P19" t="n">
-        <v>62.6</v>
-      </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T19" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>MRK</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>148.96</v>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>57.8</v>
-      </c>
-      <c r="J20" t="n">
-        <v>59.6</v>
-      </c>
-      <c r="K20" t="n">
-        <v>89</v>
-      </c>
-      <c r="L20" t="n">
-        <v>2.61</v>
-      </c>
-      <c r="M20" t="n">
-        <v>43</v>
-      </c>
-      <c r="N20" t="n">
-        <v>97.3</v>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P20" t="n">
-        <v>69.5</v>
-      </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S20" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T20" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U20" t="inlineStr"/>
-      <c r="V20" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>EL</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>101.19</v>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>55.4</v>
-      </c>
-      <c r="J21" t="n">
-        <v>60.6</v>
-      </c>
-      <c r="K21" t="n">
-        <v>92</v>
-      </c>
-      <c r="L21" t="n">
-        <v>3.47</v>
-      </c>
-      <c r="M21" t="n">
-        <v>56.1</v>
-      </c>
-      <c r="N21" t="n">
-        <v>62.6</v>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P21" t="n">
-        <v>60.1</v>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
-      <c r="V21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>DLTR</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>124.27</v>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>SQUEEZE</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>53.6</v>
-      </c>
-      <c r="J22" t="n">
-        <v>42.4</v>
-      </c>
-      <c r="K22" t="n">
-        <v>13</v>
-      </c>
-      <c r="L22" t="n">
-        <v>4.14</v>
-      </c>
-      <c r="M22" t="n">
-        <v>31.7</v>
-      </c>
-      <c r="N22" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P22" t="n">
-        <v>53.7</v>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T22" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V22" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>TTWO</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>214.63</v>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>51</v>
-      </c>
-      <c r="J23" t="n">
-        <v>31.2</v>
-      </c>
-      <c r="K23" t="n">
-        <v>89</v>
-      </c>
-      <c r="L23" t="n">
-        <v>3.72</v>
-      </c>
-      <c r="M23" t="n">
-        <v>42</v>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P23" t="n">
-        <v>43</v>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>TJX</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>129.31</v>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>42.8</v>
-      </c>
-      <c r="J24" t="n">
-        <v>20</v>
-      </c>
-      <c r="K24" t="n">
-        <v>94</v>
-      </c>
-      <c r="L24" t="n">
-        <v>1.98</v>
-      </c>
-      <c r="M24" t="n">
-        <v>22.7</v>
-      </c>
-      <c r="N24" t="n">
-        <v>52.3</v>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P24" t="n">
-        <v>32</v>
-      </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S24" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T24" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
-      <c r="V24" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>HON</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>208.22</v>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>38.6</v>
-      </c>
-      <c r="J25" t="n">
-        <v>33.7</v>
-      </c>
-      <c r="K25" t="n">
-        <v>81</v>
-      </c>
-      <c r="L25" t="n">
-        <v>2.18</v>
-      </c>
-      <c r="M25" t="n">
-        <v>27</v>
-      </c>
-      <c r="N25" t="n">
-        <v>45.4</v>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P25" t="n">
-        <v>39.7</v>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S25" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T25" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U25" t="inlineStr"/>
-      <c r="V25" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 10.09.2026 17:37 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -31,10 +31,10 @@
       <sz val="11"/>
     </font>
     <font>
-      <color rgb="0022c55e"/>
+      <color rgb="00ef4444"/>
     </font>
     <font>
-      <color rgb="00ef4444"/>
+      <color rgb="0022c55e"/>
     </font>
   </fonts>
   <fills count="3">
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>CI</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>238.69</v>
+        <v>279.52</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -590,17 +590,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -614,30 +614,30 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>80.7</v>
+        <v>78.7</v>
       </c>
       <c r="J2" t="n">
-        <v>54.2</v>
+        <v>50.4</v>
       </c>
       <c r="K2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="L2" t="n">
-        <v>2.43</v>
+        <v>2.26</v>
       </c>
       <c r="M2" t="n">
-        <v>26.7</v>
+        <v>25.6</v>
       </c>
       <c r="N2" t="n">
-        <v>13.1</v>
+        <v>15.4</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>47.4</v>
+        <v>49.7</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -651,40 +651,40 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>276.05</v>
+        <v>300.76</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -710,34 +710,34 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>78.40000000000001</v>
+        <v>78.5</v>
       </c>
       <c r="J3" t="n">
-        <v>46.7</v>
+        <v>46</v>
       </c>
       <c r="K3" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="L3" t="n">
-        <v>2.23</v>
+        <v>4.62</v>
       </c>
       <c r="M3" t="n">
-        <v>25.6</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="N3" t="n">
-        <v>15.4</v>
+        <v>49.9</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>47.7</v>
+        <v>52</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -752,12 +752,12 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Divergence</t>
+          <t>Divergence, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -769,81 +769,81 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>247.68</v>
+        <v>236.24</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>75.90000000000001</v>
+        <v>78.2</v>
       </c>
       <c r="J4" t="n">
-        <v>66.3</v>
+        <v>51.4</v>
       </c>
       <c r="K4" t="n">
-        <v>97</v>
+        <v>8</v>
       </c>
       <c r="L4" t="n">
-        <v>4.42</v>
+        <v>2.65</v>
       </c>
       <c r="M4" t="n">
-        <v>75</v>
+        <v>27.6</v>
       </c>
       <c r="N4" t="n">
-        <v>92.59999999999999</v>
+        <v>14.4</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>65.5</v>
+        <v>46.6</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -851,10 +851,14 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr"/>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -865,14 +869,14 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>164.77</v>
+        <v>165.6</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -898,22 +902,22 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>74</v>
+        <v>72.3</v>
       </c>
       <c r="J5" t="n">
-        <v>60.1</v>
+        <v>61.4</v>
       </c>
       <c r="K5" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="L5" t="n">
-        <v>2.16</v>
+        <v>2.21</v>
       </c>
       <c r="M5" t="n">
-        <v>25.7</v>
+        <v>24.7</v>
       </c>
       <c r="N5" t="n">
-        <v>54.7</v>
+        <v>48.8</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -921,7 +925,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>61.8</v>
+        <v>62.2</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -957,18 +961,18 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>554.5</v>
+        <v>244.02</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -980,48 +984,48 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>71.5</v>
+        <v>69.8</v>
       </c>
       <c r="J6" t="n">
-        <v>42.7</v>
+        <v>63.5</v>
       </c>
       <c r="K6" t="n">
-        <v>13</v>
+        <v>95</v>
       </c>
       <c r="L6" t="n">
-        <v>2.34</v>
+        <v>4.35</v>
       </c>
       <c r="M6" t="n">
-        <v>21.4</v>
+        <v>75</v>
       </c>
       <c r="N6" t="n">
-        <v>23.2</v>
+        <v>92.7</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>46.3</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1031,7 +1035,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1039,11 +1043,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr">
         <is>
           <t>No</t>
@@ -1053,18 +1053,18 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>UPS</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>99.39</v>
+        <v>548.45</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -1090,22 +1090,22 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>68.59999999999999</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="J7" t="n">
-        <v>35.2</v>
+        <v>40</v>
       </c>
       <c r="K7" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="L7" t="n">
-        <v>1.8</v>
+        <v>2.3</v>
       </c>
       <c r="M7" t="n">
-        <v>21.8</v>
+        <v>21.5</v>
       </c>
       <c r="N7" t="n">
-        <v>17.9</v>
+        <v>23.4</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1113,11 +1113,11 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>45.2</v>
+        <v>45.3</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1132,12 +1132,12 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>Divergence, Squeeze Expanding</t>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
@@ -1153,14 +1153,14 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>142.57</v>
+        <v>142.93</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -1186,22 +1186,22 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>66.5</v>
+        <v>62.6</v>
       </c>
       <c r="J8" t="n">
-        <v>41.4</v>
+        <v>42.6</v>
       </c>
       <c r="K8" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="L8" t="n">
-        <v>1.64</v>
+        <v>1.55</v>
       </c>
       <c r="M8" t="n">
-        <v>15.6</v>
+        <v>14.7</v>
       </c>
       <c r="N8" t="n">
-        <v>12.6</v>
+        <v>5.9</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1209,7 +1209,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>44.3</v>
+        <v>44.8</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1233,30 +1233,30 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CHTR</t>
+          <t>TMUS</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>136.04</v>
+        <v>175.9</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -1282,22 +1282,22 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>54.6</v>
+        <v>62.2</v>
       </c>
       <c r="J9" t="n">
-        <v>40.7</v>
+        <v>43.2</v>
       </c>
       <c r="K9" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="L9" t="n">
-        <v>5.95</v>
+        <v>2.58</v>
       </c>
       <c r="M9" t="n">
-        <v>60.2</v>
+        <v>30.1</v>
       </c>
       <c r="N9" t="n">
-        <v>55.7</v>
+        <v>39.5</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1305,7 +1305,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>38.6</v>
+        <v>41.8</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1341,11 +1341,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>TTWO</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>32.13</v>
+        <v>218.01</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1354,17 +1354,17 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1378,22 +1378,22 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>51.6</v>
+        <v>55.2</v>
       </c>
       <c r="J10" t="n">
-        <v>51.6</v>
+        <v>38.7</v>
       </c>
       <c r="K10" t="n">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="L10" t="n">
-        <v>3.32</v>
+        <v>3.64</v>
       </c>
       <c r="M10" t="n">
-        <v>40.7</v>
+        <v>35.9</v>
       </c>
       <c r="N10" t="n">
-        <v>82.7</v>
+        <v>58.3</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1401,7 +1401,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>47.6</v>
+        <v>44.7</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1410,12 +1410,12 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1433,18 +1433,18 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>EL</t>
+          <t>CHTR</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>98.69</v>
+        <v>139.95</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -1456,44 +1456,44 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>51.4</v>
+        <v>50.7</v>
       </c>
       <c r="J11" t="n">
-        <v>55.1</v>
+        <v>44.5</v>
       </c>
       <c r="K11" t="n">
-        <v>90</v>
+        <v>21</v>
       </c>
       <c r="L11" t="n">
-        <v>3.64</v>
+        <v>5.85</v>
       </c>
       <c r="M11" t="n">
-        <v>56.8</v>
+        <v>62.2</v>
       </c>
       <c r="N11" t="n">
-        <v>64</v>
+        <v>58.5</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>57.7</v>
+        <v>39.8</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1512,84 +1512,80 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TJX</t>
+          <t>BKR</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>126.1</v>
+        <v>59.45</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>49.1</v>
+        <v>44.2</v>
       </c>
       <c r="J12" t="n">
-        <v>17.4</v>
+        <v>37.2</v>
       </c>
       <c r="K12" t="n">
-        <v>95</v>
+        <v>17</v>
       </c>
       <c r="L12" t="n">
-        <v>2.15</v>
+        <v>3.45</v>
       </c>
       <c r="M12" t="n">
-        <v>20.9</v>
+        <v>29.3</v>
       </c>
       <c r="N12" t="n">
         <v>41.9</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>30.4</v>
+        <v>49.7</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1603,7 +1599,7 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -1613,7 +1609,7 @@
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>Divergence, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
@@ -1625,11 +1621,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MRK</t>
+          <t>TJX</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>147.85</v>
+        <v>126.49</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1638,17 +1634,17 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1662,30 +1658,30 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>47.6</v>
+        <v>43.3</v>
       </c>
       <c r="J13" t="n">
-        <v>57.5</v>
+        <v>18.8</v>
       </c>
       <c r="K13" t="n">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="L13" t="n">
-        <v>2.48</v>
+        <v>2.03</v>
       </c>
       <c r="M13" t="n">
-        <v>43.2</v>
+        <v>20.8</v>
       </c>
       <c r="N13" t="n">
-        <v>98</v>
+        <v>41.2</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>68.3</v>
+        <v>30.6</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1699,12 +1695,12 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U13" t="inlineStr"/>
@@ -1717,18 +1713,18 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>EL</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>145.71</v>
+        <v>97.84</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -1750,26 +1746,26 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>44.8</v>
+        <v>41.4</v>
       </c>
       <c r="J14" t="n">
-        <v>54.8</v>
+        <v>53.3</v>
       </c>
       <c r="K14" t="n">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="L14" t="n">
-        <v>2.45</v>
+        <v>3.42</v>
       </c>
       <c r="M14" t="n">
-        <v>26.7</v>
+        <v>56.8</v>
       </c>
       <c r="N14" t="n">
-        <v>48.2</v>
+        <v>64</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1777,7 +1773,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>61.1</v>
+        <v>56.9</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1809,71 +1805,71 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>DLTR</t>
+          <t>HON</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>121</v>
+        <v>202.27</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>41.9</v>
+        <v>35.8</v>
       </c>
       <c r="J15" t="n">
-        <v>38.3</v>
+        <v>29.1</v>
       </c>
       <c r="K15" t="n">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="L15" t="n">
-        <v>4.18</v>
+        <v>2.14</v>
       </c>
       <c r="M15" t="n">
-        <v>32.6</v>
+        <v>26.6</v>
       </c>
       <c r="N15" t="n">
-        <v>13</v>
+        <v>43.7</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>51.2</v>
+        <v>37.5</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>FIRED</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -1883,89 +1879,82 @@
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>Squeeze Fired, Divergence</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>HON</t>
+          <t>DLTR</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>206.38</v>
+        <v>119.05</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>38.1</v>
+        <v>34.1</v>
       </c>
       <c r="J16" t="n">
-        <v>32.2</v>
+        <v>36.8</v>
       </c>
       <c r="K16" t="n">
-        <v>83</v>
+        <v>47</v>
       </c>
       <c r="L16" t="n">
-        <v>2.07</v>
+        <v>4.14</v>
       </c>
       <c r="M16" t="n">
-        <v>26.9</v>
-      </c>
-      <c r="N16" t="n">
-        <v>44.8</v>
+        <v>37.3</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>39</v>
+        <v>49.9</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Scan 11.09.2026 17:42 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -31,10 +31,10 @@
       <sz val="11"/>
     </font>
     <font>
-      <color rgb="00ef4444"/>
+      <color rgb="0022c55e"/>
     </font>
     <font>
-      <color rgb="0022c55e"/>
+      <color rgb="00ef4444"/>
     </font>
   </fonts>
   <fills count="3">
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V16"/>
+  <dimension ref="A1:V20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>279.52</v>
+        <v>83.61</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -590,17 +590,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -614,34 +614,34 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>78.7</v>
+        <v>87.8</v>
       </c>
       <c r="J2" t="n">
-        <v>50.4</v>
+        <v>56.8</v>
       </c>
       <c r="K2" t="n">
         <v>2</v>
       </c>
       <c r="L2" t="n">
-        <v>2.26</v>
+        <v>3.12</v>
       </c>
       <c r="M2" t="n">
-        <v>25.6</v>
+        <v>36.8</v>
       </c>
       <c r="N2" t="n">
-        <v>15.4</v>
+        <v>19</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>49.7</v>
+        <v>59.7</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -651,7 +651,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -661,23 +661,23 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Divergence</t>
+          <t>Squeeze Expanding</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>300.76</v>
+        <v>39.18</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -686,17 +686,17 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -710,22 +710,22 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>78.5</v>
+        <v>83.2</v>
       </c>
       <c r="J3" t="n">
-        <v>46</v>
+        <v>58.5</v>
       </c>
       <c r="K3" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="L3" t="n">
-        <v>4.62</v>
+        <v>5.74</v>
       </c>
       <c r="M3" t="n">
-        <v>73.59999999999999</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="N3" t="n">
-        <v>49.9</v>
+        <v>40.7</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -733,11 +733,11 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>52</v>
+        <v>56.7</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -747,7 +747,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -757,30 +757,30 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Divergence, Squeeze Expanding</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>NXPI</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>236.24</v>
+        <v>237.91</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -806,22 +806,22 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>78.2</v>
+        <v>82.2</v>
       </c>
       <c r="J4" t="n">
-        <v>51.4</v>
+        <v>54.9</v>
       </c>
       <c r="K4" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L4" t="n">
-        <v>2.65</v>
+        <v>3</v>
       </c>
       <c r="M4" t="n">
-        <v>27.6</v>
+        <v>38.6</v>
       </c>
       <c r="N4" t="n">
-        <v>14.4</v>
+        <v>17</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -833,7 +833,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>FIRED</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -843,7 +843,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -853,23 +853,23 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+          <t>Squeeze Fired, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>XOM</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>165.6</v>
+        <v>301.84</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -878,17 +878,17 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -902,22 +902,22 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>72.3</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>61.4</v>
+        <v>46.7</v>
       </c>
       <c r="K5" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="L5" t="n">
-        <v>2.21</v>
+        <v>4.47</v>
       </c>
       <c r="M5" t="n">
-        <v>24.7</v>
+        <v>53.2</v>
       </c>
       <c r="N5" t="n">
-        <v>48.8</v>
+        <v>13.6</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -925,7 +925,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>62.2</v>
+        <v>52.3</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -934,12 +934,12 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -947,11 +947,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
           <t>No</t>
@@ -961,18 +957,18 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>AEP</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>244.02</v>
+        <v>123.91</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -984,44 +980,44 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>69.8</v>
+        <v>79.8</v>
       </c>
       <c r="J6" t="n">
-        <v>63.5</v>
+        <v>45.7</v>
       </c>
       <c r="K6" t="n">
-        <v>95</v>
+        <v>9</v>
       </c>
       <c r="L6" t="n">
-        <v>4.35</v>
+        <v>1.64</v>
       </c>
       <c r="M6" t="n">
-        <v>75</v>
+        <v>15.4</v>
       </c>
       <c r="N6" t="n">
-        <v>92.7</v>
+        <v>19</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>64.09999999999999</v>
+        <v>46.8</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1030,17 +1026,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
@@ -1053,11 +1049,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>XOM</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>548.45</v>
+        <v>165.57</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1066,17 +1062,17 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1090,70 +1086,66 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>67.59999999999999</v>
+        <v>79.8</v>
       </c>
       <c r="J7" t="n">
-        <v>40</v>
+        <v>61.3</v>
       </c>
       <c r="K7" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="L7" t="n">
-        <v>2.3</v>
+        <v>2.15</v>
       </c>
       <c r="M7" t="n">
-        <v>21.5</v>
+        <v>24.7</v>
       </c>
       <c r="N7" t="n">
-        <v>23.4</v>
+        <v>48.6</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>45.3</v>
+        <v>62.2</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>142.93</v>
+        <v>239.79</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1162,17 +1154,17 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1186,54 +1178,54 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>62.6</v>
+        <v>79.5</v>
       </c>
       <c r="J8" t="n">
-        <v>42.6</v>
+        <v>56.8</v>
       </c>
       <c r="K8" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="L8" t="n">
-        <v>1.55</v>
+        <v>5.61</v>
       </c>
       <c r="M8" t="n">
-        <v>14.7</v>
+        <v>79.8</v>
       </c>
       <c r="N8" t="n">
-        <v>5.9</v>
+        <v>40.5</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>44.8</v>
+        <v>60.9</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>Squeeze Expanding</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
@@ -1245,11 +1237,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TMUS</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>175.9</v>
+        <v>380.1</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1258,17 +1250,17 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1282,77 +1274,77 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>62.2</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="J9" t="n">
-        <v>43.2</v>
+        <v>57.4</v>
       </c>
       <c r="K9" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="L9" t="n">
-        <v>2.58</v>
+        <v>2.78</v>
       </c>
       <c r="M9" t="n">
-        <v>30.1</v>
+        <v>30.8</v>
       </c>
       <c r="N9" t="n">
-        <v>39.5</v>
+        <v>19.1</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>41.8</v>
+        <v>54</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+          <t>Squeeze Expanding</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TTWO</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>218.01</v>
+        <v>240.77</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -1364,36 +1356,36 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I10" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="J10" t="n">
         <v>55.2</v>
       </c>
-      <c r="J10" t="n">
-        <v>38.7</v>
-      </c>
       <c r="K10" t="n">
-        <v>90</v>
+        <v>9</v>
       </c>
       <c r="L10" t="n">
-        <v>3.64</v>
+        <v>2.87</v>
       </c>
       <c r="M10" t="n">
-        <v>35.9</v>
+        <v>28.5</v>
       </c>
       <c r="N10" t="n">
-        <v>58.3</v>
+        <v>15.6</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1401,11 +1393,11 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>44.7</v>
+        <v>48</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -1415,7 +1407,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1423,7 +1415,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr"/>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V10" t="inlineStr">
         <is>
           <t>No</t>
@@ -1433,11 +1429,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CHTR</t>
+          <t>MET</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>139.95</v>
+        <v>97.03</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1446,17 +1442,17 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1466,56 +1462,60 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>50.7</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>44.5</v>
+        <v>54.3</v>
       </c>
       <c r="K11" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="L11" t="n">
-        <v>5.85</v>
+        <v>1.9</v>
       </c>
       <c r="M11" t="n">
-        <v>62.2</v>
+        <v>22.6</v>
       </c>
       <c r="N11" t="n">
-        <v>58.5</v>
+        <v>41.9</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>39.8</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V11" t="inlineStr">
         <is>
           <t>No</t>
@@ -1525,11 +1525,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BKR</t>
+          <t>TMUS</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>59.45</v>
+        <v>183.48</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1538,17 +1538,17 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1562,118 +1562,118 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>44.2</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="J12" t="n">
-        <v>37.2</v>
+        <v>53.6</v>
       </c>
       <c r="K12" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="L12" t="n">
-        <v>3.45</v>
+        <v>2.63</v>
       </c>
       <c r="M12" t="n">
-        <v>29.3</v>
+        <v>28.6</v>
       </c>
       <c r="N12" t="n">
-        <v>41.9</v>
+        <v>33</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>49.7</v>
+        <v>46.9</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>Divergence, Squeeze Expanding</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TJX</t>
+          <t>PG</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>126.49</v>
+        <v>145.37</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>43.3</v>
+        <v>65</v>
       </c>
       <c r="J13" t="n">
-        <v>18.8</v>
+        <v>50.4</v>
       </c>
       <c r="K13" t="n">
-        <v>95</v>
+        <v>16</v>
       </c>
       <c r="L13" t="n">
-        <v>2.03</v>
+        <v>1.58</v>
       </c>
       <c r="M13" t="n">
-        <v>20.8</v>
+        <v>14.9</v>
       </c>
       <c r="N13" t="n">
-        <v>41.2</v>
+        <v>7.6</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1681,21 +1681,21 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>30.6</v>
+        <v>48.4</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -1703,7 +1703,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr"/>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V13" t="inlineStr">
         <is>
           <t>No</t>
@@ -1713,18 +1717,18 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>EL</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>97.84</v>
+        <v>681.58</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -1750,22 +1754,22 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>41.4</v>
+        <v>63.4</v>
       </c>
       <c r="J14" t="n">
-        <v>53.3</v>
+        <v>62.8</v>
       </c>
       <c r="K14" t="n">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="L14" t="n">
-        <v>3.42</v>
+        <v>2.55</v>
       </c>
       <c r="M14" t="n">
-        <v>56.8</v>
+        <v>35</v>
       </c>
       <c r="N14" t="n">
-        <v>64</v>
+        <v>63.8</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1773,7 +1777,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>56.9</v>
+        <v>63.3</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1782,17 +1786,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
@@ -1805,11 +1809,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>HON</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>202.27</v>
+        <v>248.47</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1818,17 +1822,17 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1842,30 +1846,30 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>35.8</v>
+        <v>63</v>
       </c>
       <c r="J15" t="n">
-        <v>29.1</v>
+        <v>65.2</v>
       </c>
       <c r="K15" t="n">
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="L15" t="n">
-        <v>2.14</v>
+        <v>4.14</v>
       </c>
       <c r="M15" t="n">
-        <v>26.6</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="N15" t="n">
-        <v>43.7</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>37.5</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1879,12 +1883,12 @@
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U15" t="inlineStr"/>
@@ -1897,18 +1901,18 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>DLTR</t>
+          <t>CVS</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>119.05</v>
+        <v>94.38</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -1930,56 +1934,435 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>62.9</v>
+      </c>
+      <c r="J16" t="n">
+        <v>42.3</v>
+      </c>
+      <c r="K16" t="n">
+        <v>5</v>
+      </c>
+      <c r="L16" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="M16" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="N16" t="n">
+        <v>33.2</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P16" t="n">
+        <v>52.3</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>NOC</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>521.4</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>43.6</v>
+      </c>
+      <c r="J17" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="K17" t="n">
+        <v>81</v>
+      </c>
+      <c r="L17" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="M17" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="N17" t="n">
+        <v>46.6</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P17" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr"/>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>TJX</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>126.32</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>42.6</v>
+      </c>
+      <c r="J18" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="K18" t="n">
+        <v>91</v>
+      </c>
+      <c r="L18" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="M18" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="N18" t="n">
+        <v>41.1</v>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P18" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr"/>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>HON</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>202.7</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
           <t>NEUTRAL</t>
         </is>
       </c>
-      <c r="I16" t="n">
-        <v>34.1</v>
-      </c>
-      <c r="J16" t="n">
-        <v>36.8</v>
-      </c>
-      <c r="K16" t="n">
-        <v>47</v>
-      </c>
-      <c r="L16" t="n">
-        <v>4.14</v>
-      </c>
-      <c r="M16" t="n">
-        <v>37.3</v>
-      </c>
-      <c r="O16" t="inlineStr">
+      <c r="I19" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="J19" t="n">
+        <v>30</v>
+      </c>
+      <c r="K19" t="n">
+        <v>71</v>
+      </c>
+      <c r="L19" t="n">
+        <v>2</v>
+      </c>
+      <c r="M19" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="N19" t="n">
+        <v>43.7</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P19" t="n">
+        <v>37.6</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr"/>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>BKR</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>58.31</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="J20" t="n">
+        <v>33.8</v>
+      </c>
+      <c r="K20" t="n">
+        <v>34</v>
+      </c>
+      <c r="L20" t="n">
+        <v>3.73</v>
+      </c>
+      <c r="M20" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="N20" t="n">
+        <v>42.3</v>
+      </c>
+      <c r="O20" t="inlineStr">
         <is>
           <t>Bullish</t>
         </is>
       </c>
-      <c r="P16" t="n">
-        <v>49.9</v>
-      </c>
-      <c r="Q16" t="inlineStr">
+      <c r="P20" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="Q20" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="R16" t="inlineStr">
+      <c r="R20" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T16" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr"/>
-      <c r="V16" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan 14.09.2026 19:12 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V20"/>
+  <dimension ref="A1:V30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>MET</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>83.61</v>
+        <v>97.36</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,22 +614,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>87.8</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>56.8</v>
+        <v>55.4</v>
       </c>
       <c r="K2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L2" t="n">
-        <v>3.12</v>
+        <v>1.79</v>
       </c>
       <c r="M2" t="n">
-        <v>36.8</v>
+        <v>22.4</v>
       </c>
       <c r="N2" t="n">
-        <v>19</v>
+        <v>40.7</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,11 +637,11 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>59.7</v>
+        <v>68.5</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>FIRED</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -656,12 +656,12 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Squeeze Expanding</t>
+          <t>Squeeze Fired</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -673,11 +673,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>39.18</v>
+        <v>79.31999999999999</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -710,22 +710,22 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>83.2</v>
+        <v>78.7</v>
       </c>
       <c r="J3" t="n">
-        <v>58.5</v>
+        <v>46.8</v>
       </c>
       <c r="K3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L3" t="n">
-        <v>5.74</v>
+        <v>3.84</v>
       </c>
       <c r="M3" t="n">
-        <v>82.09999999999999</v>
+        <v>40.6</v>
       </c>
       <c r="N3" t="n">
-        <v>40.7</v>
+        <v>28.1</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -733,11 +733,11 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>56.7</v>
+        <v>53.7</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -757,23 +757,23 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>Divergence</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NXPI</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>237.91</v>
+        <v>343.7</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -806,34 +806,34 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>82.2</v>
+        <v>77.8</v>
       </c>
       <c r="J4" t="n">
-        <v>54.9</v>
+        <v>53.4</v>
       </c>
       <c r="K4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L4" t="n">
-        <v>3</v>
+        <v>2.27</v>
       </c>
       <c r="M4" t="n">
-        <v>38.6</v>
+        <v>26.7</v>
       </c>
       <c r="N4" t="n">
-        <v>17</v>
+        <v>33.7</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>46.6</v>
+        <v>51.8</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>FIRED</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -853,7 +853,7 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>Squeeze Fired, Squeeze Expanding</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -865,30 +865,30 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>301.84</v>
+        <v>249.21</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -902,52 +902,56 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>79.90000000000001</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>46.7</v>
+        <v>61.1</v>
       </c>
       <c r="K5" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="L5" t="n">
-        <v>4.47</v>
+        <v>2.91</v>
       </c>
       <c r="M5" t="n">
-        <v>53.2</v>
+        <v>30.1</v>
       </c>
       <c r="N5" t="n">
-        <v>13.6</v>
+        <v>17.8</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>52.3</v>
+        <v>50.6</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>FIRED</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Squeeze Fired, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V5" t="inlineStr">
         <is>
           <t>No</t>
@@ -957,11 +961,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>123.91</v>
+        <v>928.22</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -994,66 +998,70 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>79.8</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>45.7</v>
+        <v>46.9</v>
       </c>
       <c r="K6" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="L6" t="n">
-        <v>1.64</v>
+        <v>5.28</v>
       </c>
       <c r="M6" t="n">
-        <v>15.4</v>
+        <v>54.7</v>
       </c>
       <c r="N6" t="n">
-        <v>19</v>
+        <v>2.1</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>46.8</v>
+        <v>57.4</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>XOM</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>165.57</v>
+        <v>347.23</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1086,22 +1094,19 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>79.8</v>
+        <v>77</v>
       </c>
       <c r="J7" t="n">
-        <v>61.3</v>
+        <v>53.8</v>
       </c>
       <c r="K7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L7" t="n">
-        <v>2.15</v>
+        <v>2.36</v>
       </c>
       <c r="M7" t="n">
-        <v>24.7</v>
-      </c>
-      <c r="N7" t="n">
-        <v>48.6</v>
+        <v>30</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1109,11 +1114,11 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>62.2</v>
+        <v>52.3</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1123,15 +1128,19 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V7" t="inlineStr">
         <is>
           <t>No</t>
@@ -1141,30 +1150,30 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>CVS</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>239.79</v>
+        <v>95.91</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1178,22 +1187,22 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>79.5</v>
+        <v>76.8</v>
       </c>
       <c r="J8" t="n">
-        <v>56.8</v>
+        <v>48.2</v>
       </c>
       <c r="K8" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="L8" t="n">
-        <v>5.61</v>
+        <v>2.36</v>
       </c>
       <c r="M8" t="n">
-        <v>79.8</v>
+        <v>27.5</v>
       </c>
       <c r="N8" t="n">
-        <v>40.5</v>
+        <v>34.1</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1201,7 +1210,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>60.9</v>
+        <v>54.1</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1215,7 +1224,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -1223,11 +1232,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
           <t>No</t>
@@ -1237,11 +1242,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>380.1</v>
+        <v>37.36</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1274,22 +1279,19 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>77.59999999999999</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="J9" t="n">
-        <v>57.4</v>
+        <v>52.3</v>
       </c>
       <c r="K9" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="L9" t="n">
-        <v>2.78</v>
+        <v>6.54</v>
       </c>
       <c r="M9" t="n">
-        <v>30.8</v>
-      </c>
-      <c r="N9" t="n">
-        <v>19.1</v>
+        <v>68.8</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1297,21 +1299,21 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>54</v>
+        <v>54.2</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1321,23 +1323,23 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>Squeeze Expanding</t>
+          <t>TTM Squeeze, Divergence</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>ACN</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>240.77</v>
+        <v>193.98</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1370,22 +1372,22 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>76.90000000000001</v>
+        <v>76.3</v>
       </c>
       <c r="J10" t="n">
-        <v>55.2</v>
+        <v>62.9</v>
       </c>
       <c r="K10" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="L10" t="n">
-        <v>2.87</v>
+        <v>3.55</v>
       </c>
       <c r="M10" t="n">
-        <v>28.5</v>
+        <v>39</v>
       </c>
       <c r="N10" t="n">
-        <v>15.6</v>
+        <v>25.9</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1393,11 +1395,11 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>48</v>
+        <v>55.7</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -1412,12 +1414,12 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>Squeeze Expanding</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
@@ -1429,30 +1431,30 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MET</t>
+          <t>CCI</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>97.03</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1466,30 +1468,30 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>76.40000000000001</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>54.3</v>
+        <v>45.4</v>
       </c>
       <c r="K11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L11" t="n">
-        <v>1.9</v>
+        <v>2.71</v>
       </c>
       <c r="M11" t="n">
-        <v>22.6</v>
+        <v>25.4</v>
       </c>
       <c r="N11" t="n">
-        <v>41.9</v>
+        <v>36.8</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>67.90000000000001</v>
+        <v>38.5</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1498,12 +1500,12 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1513,23 +1515,23 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>TTM Squeeze</t>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TMUS</t>
+          <t>GM</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>183.48</v>
+        <v>86.95999999999999</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1562,30 +1564,30 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>66.40000000000001</v>
+        <v>74.5</v>
       </c>
       <c r="J12" t="n">
-        <v>53.6</v>
+        <v>54.2</v>
       </c>
       <c r="K12" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="L12" t="n">
-        <v>2.63</v>
+        <v>2.61</v>
       </c>
       <c r="M12" t="n">
-        <v>28.6</v>
+        <v>25.1</v>
       </c>
       <c r="N12" t="n">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>46.9</v>
+        <v>59.5</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1621,11 +1623,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>AEP</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>145.37</v>
+        <v>122.54</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1658,44 +1660,44 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="J13" t="n">
-        <v>50.4</v>
+        <v>40.3</v>
       </c>
       <c r="K13" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="L13" t="n">
-        <v>1.58</v>
+        <v>1.68</v>
       </c>
       <c r="M13" t="n">
-        <v>14.9</v>
+        <v>15.4</v>
       </c>
       <c r="N13" t="n">
-        <v>7.6</v>
+        <v>19.1</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>48.4</v>
+        <v>45.3</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -1705,71 +1707,68 @@
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>Divergence</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>681.58</v>
+        <v>222.05</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>63.4</v>
+        <v>72.7</v>
       </c>
       <c r="J14" t="n">
-        <v>62.8</v>
+        <v>49.4</v>
       </c>
       <c r="K14" t="n">
-        <v>99</v>
+        <v>6</v>
       </c>
       <c r="L14" t="n">
-        <v>2.55</v>
+        <v>6.6</v>
       </c>
       <c r="M14" t="n">
-        <v>35</v>
-      </c>
-      <c r="N14" t="n">
-        <v>63.8</v>
+        <v>64.7</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1777,7 +1776,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>63.3</v>
+        <v>56.3</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1786,12 +1785,12 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -1799,91 +1798,95 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr"/>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>TMUS</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>248.47</v>
+        <v>183.13</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>63</v>
+        <v>70.3</v>
       </c>
       <c r="J15" t="n">
-        <v>65.2</v>
+        <v>53.3</v>
       </c>
       <c r="K15" t="n">
-        <v>94</v>
+        <v>13</v>
       </c>
       <c r="L15" t="n">
-        <v>4.14</v>
+        <v>2.52</v>
       </c>
       <c r="M15" t="n">
-        <v>73.59999999999999</v>
+        <v>28</v>
       </c>
       <c r="N15" t="n">
-        <v>89.90000000000001</v>
+        <v>31.1</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>65.90000000000001</v>
+        <v>46.6</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -1891,7 +1894,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr"/>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V15" t="inlineStr">
         <is>
           <t>No</t>
@@ -1901,67 +1908,64 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CVS</t>
+          <t>TSN</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>94.38</v>
+        <v>52.99</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>62.9</v>
+        <v>63</v>
       </c>
       <c r="J16" t="n">
-        <v>42.3</v>
+        <v>39.7</v>
       </c>
       <c r="K16" t="n">
-        <v>5</v>
+        <v>85</v>
       </c>
       <c r="L16" t="n">
-        <v>2.54</v>
+        <v>2.73</v>
       </c>
       <c r="M16" t="n">
-        <v>27.2</v>
-      </c>
-      <c r="N16" t="n">
-        <v>33.2</v>
+        <v>25.5</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>52.3</v>
+        <v>37.8</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1980,47 +1984,43 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>NOC</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>521.4</v>
+        <v>259.18</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2034,30 +2034,30 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>43.6</v>
+        <v>62.3</v>
       </c>
       <c r="J17" t="n">
-        <v>39.9</v>
+        <v>69.7</v>
       </c>
       <c r="K17" t="n">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="L17" t="n">
-        <v>2.1</v>
+        <v>4.09</v>
       </c>
       <c r="M17" t="n">
-        <v>24.1</v>
+        <v>74.2</v>
       </c>
       <c r="N17" t="n">
-        <v>46.6</v>
+        <v>91.2</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>41.6</v>
+        <v>68</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2066,12 +2066,12 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
@@ -2089,30 +2089,30 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TJX</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>126.32</v>
+        <v>678.63</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2126,30 +2126,30 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>42.6</v>
+        <v>61.1</v>
       </c>
       <c r="J18" t="n">
-        <v>18.4</v>
+        <v>61.7</v>
       </c>
       <c r="K18" t="n">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="L18" t="n">
-        <v>2.03</v>
+        <v>2.65</v>
       </c>
       <c r="M18" t="n">
-        <v>20.7</v>
+        <v>34.7</v>
       </c>
       <c r="N18" t="n">
-        <v>41.1</v>
+        <v>62.9</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>30.5</v>
+        <v>62.5</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2158,12 +2158,12 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
@@ -2181,67 +2181,67 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>HON</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>202.7</v>
+        <v>276.94</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>31.5</v>
+        <v>61</v>
       </c>
       <c r="J19" t="n">
-        <v>30</v>
+        <v>38.2</v>
       </c>
       <c r="K19" t="n">
-        <v>71</v>
+        <v>18</v>
       </c>
       <c r="L19" t="n">
-        <v>2</v>
+        <v>5.42</v>
       </c>
       <c r="M19" t="n">
-        <v>26.5</v>
+        <v>56.8</v>
       </c>
       <c r="N19" t="n">
-        <v>43.7</v>
+        <v>20.1</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>37.6</v>
+        <v>46.6</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2263,104 +2263,1045 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr"/>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>GS</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>989.27</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>58.4</v>
+      </c>
+      <c r="J20" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="K20" t="n">
+        <v>19</v>
+      </c>
+      <c r="L20" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="M20" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="N20" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P20" t="n">
+        <v>50.7</v>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>MDT</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>93.70999999999999</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Debit Call</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>56.3</v>
+      </c>
+      <c r="J21" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="K21" t="n">
+        <v>3</v>
+      </c>
+      <c r="L21" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="M21" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="N21" t="n">
+        <v>30.1</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P21" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>207.39</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>56</v>
+      </c>
+      <c r="J22" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="K22" t="n">
+        <v>19</v>
+      </c>
+      <c r="L22" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="M22" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="N22" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P22" t="n">
+        <v>54.1</v>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>143.35</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="J23" t="n">
+        <v>45.3</v>
+      </c>
+      <c r="K23" t="n">
+        <v>10</v>
+      </c>
+      <c r="L23" t="n">
+        <v>6</v>
+      </c>
+      <c r="M23" t="n">
+        <v>55.1</v>
+      </c>
+      <c r="N23" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P23" t="n">
+        <v>44.2</v>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>NOC</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>527.8</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="J24" t="n">
+        <v>44.3</v>
+      </c>
+      <c r="K24" t="n">
+        <v>69</v>
+      </c>
+      <c r="L24" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="M24" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="N24" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P24" t="n">
+        <v>43.1</v>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>59.15</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="J25" t="n">
+        <v>33.6</v>
+      </c>
+      <c r="K25" t="n">
+        <v>13</v>
+      </c>
+      <c r="L25" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="M25" t="n">
+        <v>22</v>
+      </c>
+      <c r="N25" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P25" t="n">
+        <v>54.4</v>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>TJX</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>126.27</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>41.7</v>
+      </c>
+      <c r="J26" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="K26" t="n">
+        <v>89</v>
+      </c>
+      <c r="L26" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="M26" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="N26" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P26" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr"/>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>199.45</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="J27" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="K27" t="n">
+        <v>92</v>
+      </c>
+      <c r="L27" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="M27" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P27" t="n">
+        <v>37.4</v>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr"/>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>GD</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>357.3</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>38.1</v>
+      </c>
+      <c r="J28" t="n">
+        <v>34</v>
+      </c>
+      <c r="K28" t="n">
+        <v>86</v>
+      </c>
+      <c r="L28" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="M28" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="N28" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P28" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>HON</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>200.47</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="J29" t="n">
+        <v>28</v>
+      </c>
+      <c r="K29" t="n">
+        <v>57</v>
+      </c>
+      <c r="L29" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="M29" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="N29" t="n">
+        <v>43</v>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P29" t="n">
+        <v>36.8</v>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr"/>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>BKR</t>
         </is>
       </c>
-      <c r="B20" t="n">
-        <v>58.31</v>
-      </c>
-      <c r="C20" t="inlineStr">
+      <c r="B30" t="n">
+        <v>56.58</v>
+      </c>
+      <c r="C30" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="D30" s="3" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>SELL</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>Debit Put</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>30-60 DTE</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="H30" t="inlineStr">
         <is>
           <t>NEUTRAL</t>
         </is>
       </c>
-      <c r="I20" t="n">
-        <v>28.1</v>
-      </c>
-      <c r="J20" t="n">
-        <v>33.8</v>
-      </c>
-      <c r="K20" t="n">
-        <v>34</v>
-      </c>
-      <c r="L20" t="n">
-        <v>3.73</v>
-      </c>
-      <c r="M20" t="n">
-        <v>29.4</v>
-      </c>
-      <c r="N20" t="n">
-        <v>42.3</v>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P20" t="n">
-        <v>48.1</v>
-      </c>
-      <c r="Q20" t="inlineStr">
+      <c r="I30" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="J30" t="n">
+        <v>29.3</v>
+      </c>
+      <c r="K30" t="n">
+        <v>49</v>
+      </c>
+      <c r="L30" t="n">
+        <v>4</v>
+      </c>
+      <c r="M30" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="N30" t="n">
+        <v>52</v>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="P30" t="n">
+        <v>45.7</v>
+      </c>
+      <c r="Q30" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="R20" t="inlineStr">
+      <c r="R30" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="S20" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T20" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U20" t="inlineStr">
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
         <is>
           <t>Divergence</t>
         </is>
       </c>
-      <c r="V20" t="inlineStr">
+      <c r="V30" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>

</xml_diff>

<commit_message>
Scan 15.09.2026 18:05 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V30"/>
+  <dimension ref="A1:V25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MET</t>
+          <t>ACN</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>97.36</v>
+        <v>197.15</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,34 +614,34 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>85.90000000000001</v>
+        <v>84</v>
       </c>
       <c r="J2" t="n">
-        <v>55.4</v>
+        <v>64.8</v>
       </c>
       <c r="K2" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="L2" t="n">
-        <v>1.79</v>
+        <v>3.54</v>
       </c>
       <c r="M2" t="n">
-        <v>22.4</v>
+        <v>39.6</v>
       </c>
       <c r="N2" t="n">
-        <v>40.7</v>
+        <v>27</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>68.5</v>
+        <v>56.9</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>FIRED</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -656,14 +656,10 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>Squeeze Fired</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
         <is>
           <t>No</t>
@@ -673,11 +669,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>79.31999999999999</v>
+        <v>340.04</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -710,22 +706,22 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>78.7</v>
+        <v>80.2</v>
       </c>
       <c r="J3" t="n">
-        <v>46.8</v>
+        <v>50.1</v>
       </c>
       <c r="K3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L3" t="n">
-        <v>3.84</v>
+        <v>2.24</v>
       </c>
       <c r="M3" t="n">
-        <v>40.6</v>
+        <v>24</v>
       </c>
       <c r="N3" t="n">
-        <v>28.1</v>
+        <v>24.2</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -733,47 +729,47 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>53.7</v>
+        <v>50.6</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>343.7</v>
+        <v>250.86</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -806,34 +802,34 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>77.8</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>53.4</v>
+        <v>62.2</v>
       </c>
       <c r="K4" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="L4" t="n">
-        <v>2.27</v>
+        <v>2.8</v>
       </c>
       <c r="M4" t="n">
-        <v>26.7</v>
+        <v>30</v>
       </c>
       <c r="N4" t="n">
-        <v>33.7</v>
+        <v>17.7</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>51.8</v>
+        <v>51.1</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -843,17 +839,17 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>Squeeze Expanding</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -865,11 +861,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>249.21</v>
+        <v>343.54</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -902,34 +898,34 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>77.40000000000001</v>
+        <v>79.5</v>
       </c>
       <c r="J5" t="n">
-        <v>61.1</v>
+        <v>50.7</v>
       </c>
       <c r="K5" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="L5" t="n">
-        <v>2.91</v>
+        <v>2.32</v>
       </c>
       <c r="M5" t="n">
-        <v>30.1</v>
+        <v>25.6</v>
       </c>
       <c r="N5" t="n">
-        <v>17.8</v>
+        <v>30.9</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>50.6</v>
+        <v>51.1</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>FIRED</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -939,7 +935,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -949,7 +945,7 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>Squeeze Fired, Squeeze Expanding</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
@@ -961,11 +957,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>AIG</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>928.22</v>
+        <v>75.55</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -998,30 +994,30 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>77.40000000000001</v>
+        <v>79.2</v>
       </c>
       <c r="J6" t="n">
-        <v>46.9</v>
+        <v>44.9</v>
       </c>
       <c r="K6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L6" t="n">
-        <v>5.28</v>
+        <v>1.68</v>
       </c>
       <c r="M6" t="n">
-        <v>54.7</v>
+        <v>14.9</v>
       </c>
       <c r="N6" t="n">
-        <v>2.1</v>
+        <v>3.5</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>57.4</v>
+        <v>46.3</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1030,57 +1026,57 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>CVS</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>347.23</v>
+        <v>94.79000000000001</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1094,19 +1090,22 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>77</v>
+        <v>76.7</v>
       </c>
       <c r="J7" t="n">
-        <v>53.8</v>
+        <v>44.2</v>
       </c>
       <c r="K7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L7" t="n">
-        <v>2.36</v>
+        <v>2.31</v>
       </c>
       <c r="M7" t="n">
-        <v>30</v>
+        <v>27.2</v>
+      </c>
+      <c r="N7" t="n">
+        <v>33.1</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1114,11 +1113,11 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>52.3</v>
+        <v>52.8</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1133,14 +1132,10 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr">
         <is>
           <t>No</t>
@@ -1150,11 +1145,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CVS</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>95.91</v>
+        <v>924.11</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1187,22 +1182,22 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>76.8</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="J8" t="n">
-        <v>48.2</v>
+        <v>46.4</v>
       </c>
       <c r="K8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L8" t="n">
-        <v>2.36</v>
+        <v>4.94</v>
       </c>
       <c r="M8" t="n">
-        <v>27.5</v>
+        <v>55.1</v>
       </c>
       <c r="N8" t="n">
-        <v>34.1</v>
+        <v>2.6</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1210,29 +1205,33 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>54.1</v>
+        <v>57.1</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V8" t="inlineStr">
         <is>
           <t>No</t>
@@ -1242,11 +1241,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>37.36</v>
+        <v>77.75</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1279,19 +1278,22 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>76.59999999999999</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="J9" t="n">
-        <v>52.3</v>
+        <v>44</v>
       </c>
       <c r="K9" t="n">
         <v>1</v>
       </c>
       <c r="L9" t="n">
-        <v>6.54</v>
+        <v>3.75</v>
       </c>
       <c r="M9" t="n">
-        <v>68.8</v>
+        <v>41.5</v>
+      </c>
+      <c r="N9" t="n">
+        <v>30.2</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1299,11 +1301,11 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>54.2</v>
+        <v>51.9</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1313,7 +1315,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1321,25 +1323,21 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence</t>
-        </is>
-      </c>
+      <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ACN</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>193.98</v>
+        <v>36.26</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1372,44 +1370,44 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>76.3</v>
+        <v>73.7</v>
       </c>
       <c r="J10" t="n">
-        <v>62.9</v>
+        <v>49.5</v>
       </c>
       <c r="K10" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="L10" t="n">
-        <v>3.55</v>
+        <v>6.44</v>
       </c>
       <c r="M10" t="n">
-        <v>39</v>
+        <v>88.2</v>
       </c>
       <c r="N10" t="n">
-        <v>25.9</v>
+        <v>46.7</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>55.7</v>
+        <v>52.8</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1419,7 +1417,7 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>Squeeze Expanding</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
@@ -1431,30 +1429,30 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CCI</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>74.59999999999999</v>
+        <v>222.53</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1468,34 +1466,34 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>74.90000000000001</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>45.4</v>
+        <v>49.7</v>
       </c>
       <c r="K11" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L11" t="n">
-        <v>2.71</v>
+        <v>6.24</v>
       </c>
       <c r="M11" t="n">
-        <v>25.4</v>
+        <v>82.3</v>
       </c>
       <c r="N11" t="n">
-        <v>36.8</v>
+        <v>42.6</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>38.5</v>
+        <v>56.4</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1505,33 +1503,29 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>GM</t>
+          <t>TMUS</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>86.95999999999999</v>
+        <v>181.34</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1564,30 +1558,30 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>74.5</v>
+        <v>72.3</v>
       </c>
       <c r="J12" t="n">
-        <v>54.2</v>
+        <v>50.6</v>
       </c>
       <c r="K12" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="L12" t="n">
-        <v>2.61</v>
+        <v>2.49</v>
       </c>
       <c r="M12" t="n">
-        <v>25.1</v>
+        <v>27.3</v>
       </c>
       <c r="N12" t="n">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>59.5</v>
+        <v>45.2</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1596,22 +1590,22 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
@@ -1623,30 +1617,30 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>GM</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>122.54</v>
+        <v>85.66</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1660,34 +1654,31 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>74</v>
+        <v>72.2</v>
       </c>
       <c r="J13" t="n">
-        <v>40.3</v>
+        <v>50.1</v>
       </c>
       <c r="K13" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="L13" t="n">
-        <v>1.68</v>
+        <v>2.77</v>
       </c>
       <c r="M13" t="n">
-        <v>15.4</v>
-      </c>
-      <c r="N13" t="n">
-        <v>19.1</v>
+        <v>32.8</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>45.3</v>
+        <v>57.7</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -1697,7 +1688,7 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -1707,7 +1698,7 @@
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>TTM Squeeze, Divergence</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
@@ -1719,30 +1710,30 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>CCI</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>222.05</v>
+        <v>72.42</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1756,31 +1747,34 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>72.7</v>
+        <v>62.7</v>
       </c>
       <c r="J14" t="n">
-        <v>49.4</v>
+        <v>38.7</v>
       </c>
       <c r="K14" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="L14" t="n">
-        <v>6.6</v>
+        <v>2.94</v>
       </c>
       <c r="M14" t="n">
-        <v>64.7</v>
+        <v>26.5</v>
+      </c>
+      <c r="N14" t="n">
+        <v>40.5</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>56.3</v>
+        <v>35.8</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -1790,17 +1784,17 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
@@ -1812,11 +1806,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TMUS</t>
+          <t>MDT</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>183.13</v>
+        <v>94.06999999999999</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1849,30 +1843,30 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>70.3</v>
+        <v>61.7</v>
       </c>
       <c r="J15" t="n">
-        <v>53.3</v>
+        <v>61.1</v>
       </c>
       <c r="K15" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="L15" t="n">
-        <v>2.52</v>
+        <v>2.54</v>
       </c>
       <c r="M15" t="n">
-        <v>28</v>
+        <v>21.6</v>
       </c>
       <c r="N15" t="n">
-        <v>31.1</v>
+        <v>29.4</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>46.6</v>
+        <v>60.9</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1908,30 +1902,30 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TSN</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>52.99</v>
+        <v>259.02</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1945,27 +1939,30 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>63</v>
+        <v>58.7</v>
       </c>
       <c r="J16" t="n">
-        <v>39.7</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="K16" t="n">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="L16" t="n">
-        <v>2.73</v>
+        <v>3.91</v>
       </c>
       <c r="M16" t="n">
-        <v>25.5</v>
+        <v>74.40000000000001</v>
+      </c>
+      <c r="N16" t="n">
+        <v>91.5</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>37.8</v>
+        <v>68</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1979,12 +1976,12 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
@@ -1997,11 +1994,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>259.18</v>
+        <v>686.5700000000001</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -2034,22 +2031,22 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>62.3</v>
+        <v>57.5</v>
       </c>
       <c r="J17" t="n">
-        <v>69.7</v>
+        <v>64</v>
       </c>
       <c r="K17" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="L17" t="n">
-        <v>4.09</v>
+        <v>2.44</v>
       </c>
       <c r="M17" t="n">
-        <v>74.2</v>
+        <v>34.4</v>
       </c>
       <c r="N17" t="n">
-        <v>91.2</v>
+        <v>61.8</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2057,7 +2054,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>68</v>
+        <v>63.4</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2089,15 +2086,15 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>678.63</v>
+        <v>142.41</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -2112,44 +2109,44 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>61.1</v>
+        <v>55.1</v>
       </c>
       <c r="J18" t="n">
-        <v>61.7</v>
+        <v>44.5</v>
       </c>
       <c r="K18" t="n">
-        <v>96</v>
+        <v>13</v>
       </c>
       <c r="L18" t="n">
-        <v>2.65</v>
+        <v>5.65</v>
       </c>
       <c r="M18" t="n">
-        <v>34.7</v>
+        <v>47.9</v>
       </c>
       <c r="N18" t="n">
-        <v>62.9</v>
+        <v>19.2</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>62.5</v>
+        <v>43.9</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2158,12 +2155,12 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
@@ -2171,7 +2168,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U18" t="inlineStr"/>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V18" t="inlineStr">
         <is>
           <t>No</t>
@@ -2181,67 +2182,67 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>NOC</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>276.94</v>
+        <v>533.95</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>61</v>
+        <v>45.3</v>
       </c>
       <c r="J19" t="n">
-        <v>38.2</v>
+        <v>48.2</v>
       </c>
       <c r="K19" t="n">
-        <v>18</v>
+        <v>62</v>
       </c>
       <c r="L19" t="n">
-        <v>5.42</v>
+        <v>2.14</v>
       </c>
       <c r="M19" t="n">
-        <v>56.8</v>
+        <v>24.2</v>
       </c>
       <c r="N19" t="n">
-        <v>20.1</v>
+        <v>47.2</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>46.6</v>
+        <v>44.5</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2250,98 +2251,94 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>GS</t>
+          <t>PSA</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>989.27</v>
+        <v>297.49</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>58.4</v>
+        <v>44.8</v>
       </c>
       <c r="J20" t="n">
-        <v>39.7</v>
+        <v>34.5</v>
       </c>
       <c r="K20" t="n">
-        <v>19</v>
+        <v>94</v>
       </c>
       <c r="L20" t="n">
-        <v>2.69</v>
+        <v>2.05</v>
       </c>
       <c r="M20" t="n">
-        <v>26.2</v>
+        <v>15.5</v>
       </c>
       <c r="N20" t="n">
-        <v>18.9</v>
+        <v>0.7</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>50.7</v>
+        <v>44.5</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -2356,47 +2353,43 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U20" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MDT</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>93.70999999999999</v>
+        <v>202.58</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2406,26 +2399,26 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>56.3</v>
+        <v>44.6</v>
       </c>
       <c r="J21" t="n">
-        <v>60.2</v>
+        <v>34.9</v>
       </c>
       <c r="K21" t="n">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="L21" t="n">
-        <v>2.58</v>
+        <v>2.76</v>
       </c>
       <c r="M21" t="n">
-        <v>21.8</v>
+        <v>24.6</v>
       </c>
       <c r="N21" t="n">
-        <v>30.1</v>
+        <v>26.5</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2433,11 +2426,11 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>60.5</v>
+        <v>50.3</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>FIRED</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -2447,93 +2440,93 @@
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>Squeeze Fired, Divergence</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>TJX</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>207.39</v>
+        <v>124.29</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>56</v>
+        <v>43.4</v>
       </c>
       <c r="J22" t="n">
-        <v>39.9</v>
+        <v>16.7</v>
       </c>
       <c r="K22" t="n">
-        <v>19</v>
+        <v>87</v>
       </c>
       <c r="L22" t="n">
-        <v>2.6</v>
+        <v>2.05</v>
       </c>
       <c r="M22" t="n">
-        <v>23.5</v>
+        <v>20.7</v>
       </c>
       <c r="N22" t="n">
-        <v>21.9</v>
+        <v>40.7</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P22" t="n">
-        <v>54.1</v>
+        <v>29.5</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -2548,12 +2541,12 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+          <t>Divergence</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
@@ -2565,59 +2558,59 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>143.35</v>
+        <v>195.91</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>54.9</v>
+        <v>40.1</v>
       </c>
       <c r="J23" t="n">
-        <v>45.3</v>
+        <v>34.2</v>
       </c>
       <c r="K23" t="n">
-        <v>10</v>
+        <v>94</v>
       </c>
       <c r="L23" t="n">
-        <v>6</v>
+        <v>2.11</v>
       </c>
       <c r="M23" t="n">
-        <v>55.1</v>
+        <v>22.5</v>
       </c>
       <c r="N23" t="n">
-        <v>40.9</v>
+        <v>35.8</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2625,7 +2618,7 @@
         </is>
       </c>
       <c r="P23" t="n">
-        <v>44.2</v>
+        <v>34.9</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -2639,7 +2632,7 @@
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
@@ -2647,25 +2640,21 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U23" t="inlineStr"/>
       <c r="V23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>NOC</t>
+          <t>GD</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>527.8</v>
+        <v>358.01</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -2698,30 +2687,30 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>43.9</v>
+        <v>37.6</v>
       </c>
       <c r="J24" t="n">
-        <v>44.3</v>
+        <v>35.2</v>
       </c>
       <c r="K24" t="n">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="L24" t="n">
-        <v>2.18</v>
+        <v>1.73</v>
       </c>
       <c r="M24" t="n">
-        <v>24.2</v>
+        <v>15.6</v>
       </c>
       <c r="N24" t="n">
-        <v>47.1</v>
+        <v>0.8</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P24" t="n">
-        <v>43.1</v>
+        <v>48.8</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -2757,7 +2746,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>59.15</v>
+        <v>59.58</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -2786,26 +2775,26 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>43.5</v>
+        <v>35.8</v>
       </c>
       <c r="J25" t="n">
-        <v>33.6</v>
+        <v>35.6</v>
       </c>
       <c r="K25" t="n">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="L25" t="n">
-        <v>2.49</v>
+        <v>2.4</v>
       </c>
       <c r="M25" t="n">
-        <v>22</v>
+        <v>20.8</v>
       </c>
       <c r="N25" t="n">
-        <v>51.2</v>
+        <v>43.1</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2813,11 +2802,11 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>54.4</v>
+        <v>55.6</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>FIRED</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -2832,478 +2821,17 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>Divergence, Squeeze Expanding</t>
+          <t>Squeeze Fired</t>
         </is>
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>TJX</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>126.27</v>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>41.7</v>
-      </c>
-      <c r="J26" t="n">
-        <v>19.2</v>
-      </c>
-      <c r="K26" t="n">
-        <v>89</v>
-      </c>
-      <c r="L26" t="n">
-        <v>1.95</v>
-      </c>
-      <c r="M26" t="n">
-        <v>20.8</v>
-      </c>
-      <c r="N26" t="n">
-        <v>41.5</v>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P26" t="n">
-        <v>30.6</v>
-      </c>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R26" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S26" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T26" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U26" t="inlineStr"/>
-      <c r="V26" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>199.45</v>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>40.2</v>
-      </c>
-      <c r="J27" t="n">
-        <v>38.9</v>
-      </c>
-      <c r="K27" t="n">
-        <v>92</v>
-      </c>
-      <c r="L27" t="n">
-        <v>2.08</v>
-      </c>
-      <c r="M27" t="n">
-        <v>28.5</v>
-      </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P27" t="n">
-        <v>37.4</v>
-      </c>
-      <c r="Q27" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R27" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S27" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T27" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U27" t="inlineStr"/>
-      <c r="V27" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>GD</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>357.3</v>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>38.1</v>
-      </c>
-      <c r="J28" t="n">
-        <v>34</v>
-      </c>
-      <c r="K28" t="n">
-        <v>86</v>
-      </c>
-      <c r="L28" t="n">
-        <v>1.73</v>
-      </c>
-      <c r="M28" t="n">
-        <v>15.5</v>
-      </c>
-      <c r="N28" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P28" t="n">
-        <v>48.4</v>
-      </c>
-      <c r="Q28" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S28" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T28" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U28" t="inlineStr"/>
-      <c r="V28" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>HON</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>200.47</v>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>27.8</v>
-      </c>
-      <c r="J29" t="n">
-        <v>28</v>
-      </c>
-      <c r="K29" t="n">
-        <v>57</v>
-      </c>
-      <c r="L29" t="n">
-        <v>2.13</v>
-      </c>
-      <c r="M29" t="n">
-        <v>26.3</v>
-      </c>
-      <c r="N29" t="n">
-        <v>43</v>
-      </c>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P29" t="n">
-        <v>36.8</v>
-      </c>
-      <c r="Q29" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R29" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S29" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T29" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U29" t="inlineStr"/>
-      <c r="V29" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>BKR</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>56.58</v>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I30" t="n">
-        <v>20.4</v>
-      </c>
-      <c r="J30" t="n">
-        <v>29.3</v>
-      </c>
-      <c r="K30" t="n">
-        <v>49</v>
-      </c>
-      <c r="L30" t="n">
-        <v>4</v>
-      </c>
-      <c r="M30" t="n">
-        <v>31.2</v>
-      </c>
-      <c r="N30" t="n">
-        <v>52</v>
-      </c>
-      <c r="O30" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="P30" t="n">
-        <v>45.7</v>
-      </c>
-      <c r="Q30" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R30" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S30" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U30" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
-      <c r="V30" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan 16.09.2026 18:05 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V25"/>
+  <dimension ref="A1:V23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>197.15</v>
+        <v>190.38</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,22 +614,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>84</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>64.8</v>
+        <v>58.4</v>
       </c>
       <c r="K2" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="L2" t="n">
-        <v>3.54</v>
+        <v>3.57</v>
       </c>
       <c r="M2" t="n">
         <v>39.6</v>
       </c>
       <c r="N2" t="n">
-        <v>27</v>
+        <v>27.1</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>56.9</v>
+        <v>54.3</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -646,12 +646,12 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>340.04</v>
+        <v>342.91</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -706,22 +706,22 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>80.2</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>50.1</v>
+        <v>52.4</v>
       </c>
       <c r="K3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L3" t="n">
-        <v>2.24</v>
+        <v>2.1</v>
       </c>
       <c r="M3" t="n">
-        <v>24</v>
+        <v>23.7</v>
       </c>
       <c r="N3" t="n">
-        <v>24.2</v>
+        <v>23.2</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -729,7 +729,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>50.6</v>
+        <v>51.5</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -753,7 +753,7 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>TTM Squeeze</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -765,11 +765,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>250.86</v>
+        <v>346.16</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -802,34 +802,34 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>79.59999999999999</v>
+        <v>84.2</v>
       </c>
       <c r="J4" t="n">
-        <v>62.2</v>
+        <v>52.6</v>
       </c>
       <c r="K4" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="L4" t="n">
-        <v>2.8</v>
+        <v>2.18</v>
       </c>
       <c r="M4" t="n">
-        <v>30</v>
+        <v>25.2</v>
       </c>
       <c r="N4" t="n">
-        <v>17.7</v>
+        <v>29.5</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>51.1</v>
+        <v>52</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -839,17 +839,17 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>Squeeze Expanding</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -861,30 +861,30 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>CCI</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>343.54</v>
+        <v>74.39</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -898,30 +898,30 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>79.5</v>
+        <v>78.2</v>
       </c>
       <c r="J5" t="n">
-        <v>50.7</v>
+        <v>49.4</v>
       </c>
       <c r="K5" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L5" t="n">
-        <v>2.32</v>
+        <v>2.71</v>
       </c>
       <c r="M5" t="n">
-        <v>25.6</v>
+        <v>25.9</v>
       </c>
       <c r="N5" t="n">
-        <v>30.9</v>
+        <v>35.5</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>51.1</v>
+        <v>39.7</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -940,7 +940,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -957,11 +957,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AIG</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>75.55</v>
+        <v>936.8</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -994,30 +994,30 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>79.2</v>
+        <v>77</v>
       </c>
       <c r="J6" t="n">
-        <v>44.9</v>
+        <v>48.2</v>
       </c>
       <c r="K6" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="L6" t="n">
-        <v>1.68</v>
+        <v>4.47</v>
       </c>
       <c r="M6" t="n">
-        <v>14.9</v>
+        <v>50.8</v>
       </c>
       <c r="N6" t="n">
-        <v>3.5</v>
+        <v>0</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>46.3</v>
+        <v>58</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1026,17 +1026,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1053,11 +1053,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CVS</t>
+          <t>NXPI</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>94.79000000000001</v>
+        <v>222.4</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1090,34 +1090,34 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>76.7</v>
+        <v>74.8</v>
       </c>
       <c r="J7" t="n">
-        <v>44.2</v>
+        <v>42.7</v>
       </c>
       <c r="K7" t="n">
         <v>2</v>
       </c>
       <c r="L7" t="n">
-        <v>2.31</v>
+        <v>3.31</v>
       </c>
       <c r="M7" t="n">
-        <v>27.2</v>
+        <v>31.4</v>
       </c>
       <c r="N7" t="n">
-        <v>33.1</v>
+        <v>5.3</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>52.8</v>
+        <v>42.4</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1135,7 +1135,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr"/>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V7" t="inlineStr">
         <is>
           <t>No</t>
@@ -1145,30 +1149,30 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>GM</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>924.11</v>
+        <v>84.65000000000001</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1182,22 +1186,19 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>76.59999999999999</v>
+        <v>73</v>
       </c>
       <c r="J8" t="n">
-        <v>46.4</v>
+        <v>47.2</v>
       </c>
       <c r="K8" t="n">
         <v>1</v>
       </c>
       <c r="L8" t="n">
-        <v>4.94</v>
+        <v>2.61</v>
       </c>
       <c r="M8" t="n">
-        <v>55.1</v>
-      </c>
-      <c r="N8" t="n">
-        <v>2.6</v>
+        <v>32.6</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1205,7 +1206,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>57.1</v>
+        <v>55.9</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1224,7 +1225,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1241,11 +1242,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>MDT</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>77.75</v>
+        <v>93.36</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1278,22 +1279,22 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>75.90000000000001</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="J9" t="n">
-        <v>44</v>
+        <v>58.5</v>
       </c>
       <c r="K9" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L9" t="n">
-        <v>3.75</v>
+        <v>2.4</v>
       </c>
       <c r="M9" t="n">
-        <v>41.5</v>
+        <v>21.6</v>
       </c>
       <c r="N9" t="n">
-        <v>30.2</v>
+        <v>29.3</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1301,11 +1302,11 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>51.9</v>
+        <v>60</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1315,7 +1316,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1323,7 +1324,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr"/>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V9" t="inlineStr">
         <is>
           <t>No</t>
@@ -1333,30 +1338,30 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>AMP</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>36.26</v>
+        <v>545.42</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1370,22 +1375,22 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>73.7</v>
+        <v>68.2</v>
       </c>
       <c r="J10" t="n">
-        <v>49.5</v>
+        <v>45.1</v>
       </c>
       <c r="K10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L10" t="n">
-        <v>6.44</v>
+        <v>2.05</v>
       </c>
       <c r="M10" t="n">
-        <v>88.2</v>
+        <v>18.8</v>
       </c>
       <c r="N10" t="n">
-        <v>46.7</v>
+        <v>9.4</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1393,7 +1398,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>52.8</v>
+        <v>62.2</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1412,32 +1417,32 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>TSN</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>222.53</v>
+        <v>52.66</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1452,44 +1457,44 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>73.59999999999999</v>
+        <v>57.9</v>
       </c>
       <c r="J11" t="n">
-        <v>49.7</v>
+        <v>39</v>
       </c>
       <c r="K11" t="n">
-        <v>7</v>
+        <v>81</v>
       </c>
       <c r="L11" t="n">
-        <v>6.24</v>
+        <v>2.45</v>
       </c>
       <c r="M11" t="n">
-        <v>82.3</v>
+        <v>28</v>
       </c>
       <c r="N11" t="n">
-        <v>42.6</v>
+        <v>53.4</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>56.4</v>
+        <v>37.2</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1503,7 +1508,7 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1521,30 +1526,30 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TMUS</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>181.34</v>
+        <v>143.95</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1558,22 +1563,22 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>72.3</v>
+        <v>55.7</v>
       </c>
       <c r="J12" t="n">
-        <v>50.6</v>
+        <v>46.4</v>
       </c>
       <c r="K12" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="L12" t="n">
-        <v>2.49</v>
+        <v>5.57</v>
       </c>
       <c r="M12" t="n">
-        <v>27.3</v>
+        <v>48.4</v>
       </c>
       <c r="N12" t="n">
-        <v>29</v>
+        <v>20.8</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1581,11 +1586,11 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>45.2</v>
+        <v>44.4</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -1603,11 +1608,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+      <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr">
         <is>
           <t>No</t>
@@ -1617,56 +1618,59 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>GM</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>85.66</v>
+        <v>251.33</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>72.2</v>
+        <v>53.6</v>
       </c>
       <c r="J13" t="n">
-        <v>50.1</v>
+        <v>63</v>
       </c>
       <c r="K13" t="n">
-        <v>1</v>
+        <v>85</v>
       </c>
       <c r="L13" t="n">
-        <v>2.77</v>
+        <v>3.89</v>
       </c>
       <c r="M13" t="n">
-        <v>32.8</v>
+        <v>75</v>
+      </c>
+      <c r="N13" t="n">
+        <v>92.59999999999999</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1674,11 +1678,11 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>57.7</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -1693,76 +1697,72 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CCI</t>
+          <t>TTWO</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>72.42</v>
+        <v>213.29</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>62.7</v>
+        <v>53.5</v>
       </c>
       <c r="J14" t="n">
-        <v>38.7</v>
+        <v>38.5</v>
       </c>
       <c r="K14" t="n">
-        <v>10</v>
+        <v>75</v>
       </c>
       <c r="L14" t="n">
-        <v>2.94</v>
+        <v>3.57</v>
       </c>
       <c r="M14" t="n">
-        <v>26.5</v>
+        <v>38.9</v>
       </c>
       <c r="N14" t="n">
-        <v>40.5</v>
+        <v>68.2</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1770,11 +1770,11 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>35.8</v>
+        <v>42.6</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -1789,76 +1789,72 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>MDT</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>94.06999999999999</v>
+        <v>671.4299999999999</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>61.7</v>
+        <v>52.8</v>
       </c>
       <c r="J15" t="n">
-        <v>61.1</v>
+        <v>57.2</v>
       </c>
       <c r="K15" t="n">
-        <v>5</v>
+        <v>92</v>
       </c>
       <c r="L15" t="n">
-        <v>2.54</v>
+        <v>2.45</v>
       </c>
       <c r="M15" t="n">
-        <v>21.6</v>
+        <v>34.7</v>
       </c>
       <c r="N15" t="n">
-        <v>29.4</v>
+        <v>62.7</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1866,21 +1862,21 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>60.9</v>
+        <v>61.3</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -1888,11 +1884,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr">
         <is>
           <t>No</t>
@@ -1902,15 +1894,15 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>259.02</v>
+        <v>207.07</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -1925,36 +1917,36 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>58.7</v>
+        <v>52.2</v>
       </c>
       <c r="J16" t="n">
-        <v>69.40000000000001</v>
+        <v>40.2</v>
       </c>
       <c r="K16" t="n">
-        <v>89</v>
+        <v>24</v>
       </c>
       <c r="L16" t="n">
-        <v>3.91</v>
+        <v>2.51</v>
       </c>
       <c r="M16" t="n">
-        <v>74.40000000000001</v>
+        <v>22.5</v>
       </c>
       <c r="N16" t="n">
-        <v>91.5</v>
+        <v>17.3</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1962,29 +1954,33 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>68</v>
+        <v>53.8</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V16" t="inlineStr">
         <is>
           <t>No</t>
@@ -1994,15 +1990,15 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>FANG</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>686.5700000000001</v>
+        <v>196.08</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -2017,36 +2013,36 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>57.5</v>
+        <v>49.4</v>
       </c>
       <c r="J17" t="n">
-        <v>64</v>
+        <v>43.9</v>
       </c>
       <c r="K17" t="n">
-        <v>94</v>
+        <v>8</v>
       </c>
       <c r="L17" t="n">
-        <v>2.44</v>
+        <v>3.95</v>
       </c>
       <c r="M17" t="n">
-        <v>34.4</v>
+        <v>35.9</v>
       </c>
       <c r="N17" t="n">
-        <v>61.8</v>
+        <v>69.7</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2054,99 +2050,103 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>63.4</v>
+        <v>53</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U17" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>PSA</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>142.41</v>
+        <v>297.67</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>55.1</v>
+        <v>48</v>
       </c>
       <c r="J18" t="n">
-        <v>44.5</v>
+        <v>39.5</v>
       </c>
       <c r="K18" t="n">
-        <v>13</v>
+        <v>92</v>
       </c>
       <c r="L18" t="n">
-        <v>5.65</v>
+        <v>1.97</v>
       </c>
       <c r="M18" t="n">
-        <v>47.9</v>
+        <v>16.1</v>
       </c>
       <c r="N18" t="n">
-        <v>19.2</v>
+        <v>5.3</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>43.9</v>
+        <v>46.4</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2155,24 +2155,20 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U18" t="inlineStr">
-        <is>
-          <t>Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr">
         <is>
           <t>No</t>
@@ -2182,11 +2178,11 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>NOC</t>
+          <t>TJX</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>533.95</v>
+        <v>124.97</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2215,26 +2211,26 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>45.3</v>
+        <v>42.2</v>
       </c>
       <c r="J19" t="n">
-        <v>48.2</v>
+        <v>18.5</v>
       </c>
       <c r="K19" t="n">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="L19" t="n">
-        <v>2.14</v>
+        <v>2</v>
       </c>
       <c r="M19" t="n">
-        <v>24.2</v>
+        <v>20.7</v>
       </c>
       <c r="N19" t="n">
-        <v>47.2</v>
+        <v>41</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -2242,7 +2238,7 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>44.5</v>
+        <v>29.8</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2251,17 +2247,17 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U19" t="inlineStr"/>
@@ -2274,11 +2270,11 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PSA</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>297.49</v>
+        <v>195.8</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2311,22 +2307,22 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>44.8</v>
+        <v>40.7</v>
       </c>
       <c r="J20" t="n">
-        <v>34.5</v>
+        <v>35.3</v>
       </c>
       <c r="K20" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="L20" t="n">
-        <v>2.05</v>
+        <v>2.01</v>
       </c>
       <c r="M20" t="n">
-        <v>15.5</v>
+        <v>21</v>
       </c>
       <c r="N20" t="n">
-        <v>0.7</v>
+        <v>27.8</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2334,7 +2330,7 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>44.5</v>
+        <v>34.9</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2366,71 +2362,68 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>XEL</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>202.58</v>
+        <v>73.06</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>44.6</v>
+        <v>38.7</v>
       </c>
       <c r="J21" t="n">
-        <v>34.9</v>
+        <v>35.1</v>
       </c>
       <c r="K21" t="n">
-        <v>24</v>
+        <v>91</v>
       </c>
       <c r="L21" t="n">
-        <v>2.76</v>
+        <v>1.88</v>
       </c>
       <c r="M21" t="n">
-        <v>24.6</v>
-      </c>
-      <c r="N21" t="n">
-        <v>26.5</v>
+        <v>26.1</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>50.3</v>
+        <v>39.9</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>FIRED</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -2445,28 +2438,24 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t>Squeeze Fired, Divergence</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr"/>
       <c r="V21" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>TJX</t>
+          <t>GD</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>124.29</v>
+        <v>360.41</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -2495,34 +2484,31 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>43.4</v>
+        <v>37.8</v>
       </c>
       <c r="J22" t="n">
-        <v>16.7</v>
+        <v>38.8</v>
       </c>
       <c r="K22" t="n">
-        <v>87</v>
+        <v>67</v>
       </c>
       <c r="L22" t="n">
-        <v>2.05</v>
+        <v>1.74</v>
       </c>
       <c r="M22" t="n">
-        <v>20.7</v>
-      </c>
-      <c r="N22" t="n">
-        <v>40.7</v>
+        <v>23</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P22" t="n">
-        <v>29.5</v>
+        <v>49.8</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
@@ -2544,81 +2530,77 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U22" t="inlineStr"/>
       <c r="V22" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>BAC</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>195.91</v>
+        <v>58.26</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>40.1</v>
+        <v>24.4</v>
       </c>
       <c r="J23" t="n">
-        <v>34.2</v>
+        <v>30.2</v>
       </c>
       <c r="K23" t="n">
-        <v>94</v>
+        <v>42</v>
       </c>
       <c r="L23" t="n">
-        <v>2.11</v>
+        <v>2.45</v>
       </c>
       <c r="M23" t="n">
-        <v>22.5</v>
+        <v>21.4</v>
       </c>
       <c r="N23" t="n">
-        <v>35.8</v>
+        <v>47</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>34.9</v>
+        <v>52</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -2640,198 +2622,14 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U23" t="inlineStr"/>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>GD</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>358.01</v>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>37.6</v>
-      </c>
-      <c r="J24" t="n">
-        <v>35.2</v>
-      </c>
-      <c r="K24" t="n">
-        <v>78</v>
-      </c>
-      <c r="L24" t="n">
-        <v>1.73</v>
-      </c>
-      <c r="M24" t="n">
-        <v>15.6</v>
-      </c>
-      <c r="N24" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P24" t="n">
-        <v>48.8</v>
-      </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S24" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T24" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U24" t="inlineStr"/>
-      <c r="V24" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>BAC</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>59.58</v>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>35.8</v>
-      </c>
-      <c r="J25" t="n">
-        <v>35.6</v>
-      </c>
-      <c r="K25" t="n">
-        <v>27</v>
-      </c>
-      <c r="L25" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="M25" t="n">
-        <v>20.8</v>
-      </c>
-      <c r="N25" t="n">
-        <v>43.1</v>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P25" t="n">
-        <v>55.6</v>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>FIRED</t>
-        </is>
-      </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S25" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T25" t="inlineStr">
-        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="U25" t="inlineStr">
-        <is>
-          <t>Squeeze Fired</t>
-        </is>
-      </c>
-      <c r="V25" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan 17.09.2026 18:05 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V23"/>
+  <dimension ref="A1:V26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ACN</t>
+          <t>TSLA</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>190.38</v>
+        <v>368.33</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,22 +614,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>87.09999999999999</v>
+        <v>81.5</v>
       </c>
       <c r="J2" t="n">
-        <v>58.4</v>
+        <v>55.7</v>
       </c>
       <c r="K2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L2" t="n">
-        <v>3.57</v>
+        <v>3.51</v>
       </c>
       <c r="M2" t="n">
-        <v>39.6</v>
+        <v>44.6</v>
       </c>
       <c r="N2" t="n">
-        <v>27.1</v>
+        <v>36.9</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,29 +637,33 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>54.3</v>
+        <v>48.6</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V2" t="inlineStr">
         <is>
           <t>No</t>
@@ -669,11 +673,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>XLK</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>342.91</v>
+        <v>188.08</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -706,22 +710,19 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>85.09999999999999</v>
+        <v>80.5</v>
       </c>
       <c r="J3" t="n">
-        <v>52.4</v>
+        <v>55.8</v>
       </c>
       <c r="K3" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L3" t="n">
-        <v>2.1</v>
+        <v>1.77</v>
       </c>
       <c r="M3" t="n">
-        <v>23.7</v>
-      </c>
-      <c r="N3" t="n">
-        <v>23.2</v>
+        <v>21.9</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -729,11 +730,11 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>51.5</v>
+        <v>62.6</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>FIRED</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -743,7 +744,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -753,7 +754,7 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>Squeeze Fired, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -765,11 +766,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>346.16</v>
+        <v>261.75</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -802,22 +803,22 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>84.2</v>
+        <v>80</v>
       </c>
       <c r="J4" t="n">
-        <v>52.6</v>
+        <v>52.9</v>
       </c>
       <c r="K4" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="L4" t="n">
-        <v>2.18</v>
+        <v>6.19</v>
       </c>
       <c r="M4" t="n">
-        <v>25.2</v>
+        <v>60.2</v>
       </c>
       <c r="N4" t="n">
-        <v>29.5</v>
+        <v>29.1</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -825,7 +826,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>52</v>
+        <v>51.9</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -861,30 +862,30 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CCI</t>
+          <t>DHR</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>74.39</v>
+        <v>212.18</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -898,34 +899,34 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>78.2</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>49.4</v>
+        <v>57.3</v>
       </c>
       <c r="K5" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="L5" t="n">
-        <v>2.71</v>
+        <v>2.61</v>
       </c>
       <c r="M5" t="n">
-        <v>25.9</v>
+        <v>28.9</v>
       </c>
       <c r="N5" t="n">
-        <v>35.5</v>
+        <v>36.1</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>39.7</v>
+        <v>56.6</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -935,7 +936,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -945,7 +946,7 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>TTM Squeeze</t>
+          <t>Squeeze Expanding</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
@@ -957,30 +958,30 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>936.8</v>
+        <v>716.7</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -994,22 +995,19 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>77</v>
+        <v>76.5</v>
       </c>
       <c r="J6" t="n">
-        <v>48.2</v>
+        <v>52.9</v>
       </c>
       <c r="K6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L6" t="n">
-        <v>4.47</v>
+        <v>1.28</v>
       </c>
       <c r="M6" t="n">
-        <v>50.8</v>
-      </c>
-      <c r="N6" t="n">
-        <v>0</v>
+        <v>16.7</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1017,7 +1015,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>58</v>
+        <v>57.9</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1026,12 +1024,12 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1053,30 +1051,30 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>NXPI</t>
+          <t>AZN</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>222.4</v>
+        <v>165.66</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1090,22 +1088,22 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>74.8</v>
+        <v>76.3</v>
       </c>
       <c r="J7" t="n">
-        <v>42.7</v>
+        <v>54.2</v>
       </c>
       <c r="K7" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="L7" t="n">
-        <v>3.31</v>
+        <v>2.14</v>
       </c>
       <c r="M7" t="n">
-        <v>31.4</v>
+        <v>21.6</v>
       </c>
       <c r="N7" t="n">
-        <v>5.3</v>
+        <v>14.8</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1113,11 +1111,11 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>42.4</v>
+        <v>44</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1137,7 +1135,7 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>Squeeze Expanding</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
@@ -1149,11 +1147,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GM</t>
+          <t>WDAY</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>84.65000000000001</v>
+        <v>198.62</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1186,19 +1184,19 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>73</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="J8" t="n">
-        <v>47.2</v>
+        <v>57.6</v>
       </c>
       <c r="K8" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="L8" t="n">
-        <v>2.61</v>
+        <v>4.42</v>
       </c>
       <c r="M8" t="n">
-        <v>32.6</v>
+        <v>48.9</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1206,21 +1204,21 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>55.9</v>
+        <v>62.2</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -1230,7 +1228,7 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>TTM Squeeze</t>
+          <t>Squeeze Expanding</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
@@ -1242,11 +1240,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MDT</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>93.36</v>
+        <v>40.54</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1279,22 +1277,22 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>68.90000000000001</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="J9" t="n">
-        <v>58.5</v>
+        <v>59.2</v>
       </c>
       <c r="K9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L9" t="n">
-        <v>2.4</v>
+        <v>6.28</v>
       </c>
       <c r="M9" t="n">
-        <v>21.6</v>
+        <v>87</v>
       </c>
       <c r="N9" t="n">
-        <v>29.3</v>
+        <v>45.5</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1302,7 +1300,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>60</v>
+        <v>58.2</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1311,17 +1309,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1338,11 +1336,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AMP</t>
+          <t>NXPI</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>545.42</v>
+        <v>225.62</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1375,30 +1373,27 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>68.2</v>
+        <v>74.3</v>
       </c>
       <c r="J10" t="n">
-        <v>45.1</v>
+        <v>47</v>
       </c>
       <c r="K10" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L10" t="n">
-        <v>2.05</v>
+        <v>3.51</v>
       </c>
       <c r="M10" t="n">
-        <v>18.8</v>
-      </c>
-      <c r="N10" t="n">
-        <v>9.4</v>
+        <v>43.6</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>62.2</v>
+        <v>43.5</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1407,108 +1402,108 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TSN</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>52.66</v>
+        <v>110.07</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>57.9</v>
+        <v>71.5</v>
       </c>
       <c r="J11" t="n">
-        <v>39</v>
+        <v>47.4</v>
       </c>
       <c r="K11" t="n">
-        <v>81</v>
+        <v>2</v>
       </c>
       <c r="L11" t="n">
-        <v>2.45</v>
+        <v>2.49</v>
       </c>
       <c r="M11" t="n">
-        <v>28</v>
+        <v>33.9</v>
       </c>
       <c r="N11" t="n">
-        <v>53.4</v>
+        <v>47</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>37.2</v>
+        <v>55.1</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1516,7 +1511,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr"/>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V11" t="inlineStr">
         <is>
           <t>No</t>
@@ -1526,59 +1525,59 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>SYK</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>143.95</v>
+        <v>282.43</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>55.7</v>
+        <v>68.5</v>
       </c>
       <c r="J12" t="n">
-        <v>46.4</v>
+        <v>34.4</v>
       </c>
       <c r="K12" t="n">
-        <v>13</v>
+        <v>98</v>
       </c>
       <c r="L12" t="n">
-        <v>5.57</v>
+        <v>3.49</v>
       </c>
       <c r="M12" t="n">
-        <v>48.4</v>
+        <v>35.5</v>
       </c>
       <c r="N12" t="n">
-        <v>20.8</v>
+        <v>64</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1586,7 +1585,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>44.4</v>
+        <v>36.2</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1600,7 +1599,7 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -1618,15 +1617,15 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>251.33</v>
+        <v>68.20999999999999</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -1641,66 +1640,70 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>53.6</v>
+        <v>64.2</v>
       </c>
       <c r="J13" t="n">
-        <v>63</v>
+        <v>39.3</v>
       </c>
       <c r="K13" t="n">
-        <v>85</v>
+        <v>3</v>
       </c>
       <c r="L13" t="n">
-        <v>3.89</v>
+        <v>5.85</v>
       </c>
       <c r="M13" t="n">
-        <v>75</v>
+        <v>53.7</v>
       </c>
       <c r="N13" t="n">
-        <v>92.59999999999999</v>
+        <v>24.4</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>66.40000000000001</v>
+        <v>38.5</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V13" t="inlineStr">
         <is>
           <t>No</t>
@@ -1710,71 +1713,71 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TTWO</t>
+          <t>AMP</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>213.29</v>
+        <v>547.14</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>53.5</v>
+        <v>57.8</v>
       </c>
       <c r="J14" t="n">
-        <v>38.5</v>
+        <v>47</v>
       </c>
       <c r="K14" t="n">
-        <v>75</v>
+        <v>8</v>
       </c>
       <c r="L14" t="n">
-        <v>3.57</v>
+        <v>2.34</v>
       </c>
       <c r="M14" t="n">
-        <v>38.9</v>
+        <v>19.8</v>
       </c>
       <c r="N14" t="n">
-        <v>68.2</v>
+        <v>13.4</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>42.6</v>
+        <v>63</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -1784,15 +1787,19 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V14" t="inlineStr">
         <is>
           <t>No</t>
@@ -1802,30 +1809,30 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>TSN</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>671.4299999999999</v>
+        <v>52.63</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1835,34 +1842,34 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>52.8</v>
+        <v>54.1</v>
       </c>
       <c r="J15" t="n">
-        <v>57.2</v>
+        <v>40</v>
       </c>
       <c r="K15" t="n">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="L15" t="n">
-        <v>2.45</v>
+        <v>2.37</v>
       </c>
       <c r="M15" t="n">
-        <v>34.7</v>
+        <v>28.2</v>
       </c>
       <c r="N15" t="n">
-        <v>62.7</v>
+        <v>50.6</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>61.3</v>
+        <v>37.1</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1871,12 +1878,12 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -1894,81 +1901,81 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>PSA</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>207.07</v>
+        <v>299.35</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>52.2</v>
+        <v>51.7</v>
       </c>
       <c r="J16" t="n">
-        <v>40.2</v>
+        <v>43.1</v>
       </c>
       <c r="K16" t="n">
-        <v>24</v>
+        <v>90</v>
       </c>
       <c r="L16" t="n">
-        <v>2.51</v>
+        <v>1.98</v>
       </c>
       <c r="M16" t="n">
-        <v>22.5</v>
+        <v>16.9</v>
       </c>
       <c r="N16" t="n">
-        <v>17.3</v>
+        <v>11.2</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>53.8</v>
+        <v>47.3</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
@@ -1976,11 +1983,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+      <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr">
         <is>
           <t>No</t>
@@ -1990,81 +1993,81 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>FANG</t>
+          <t>TJX</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>196.08</v>
+        <v>125.88</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>49.4</v>
+        <v>51.4</v>
       </c>
       <c r="J17" t="n">
-        <v>43.9</v>
+        <v>27.1</v>
       </c>
       <c r="K17" t="n">
-        <v>8</v>
+        <v>83</v>
       </c>
       <c r="L17" t="n">
-        <v>3.95</v>
+        <v>2.15</v>
       </c>
       <c r="M17" t="n">
-        <v>35.9</v>
+        <v>21.7</v>
       </c>
       <c r="N17" t="n">
-        <v>69.7</v>
+        <v>46.4</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>53</v>
+        <v>30.3</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
@@ -2072,25 +2075,21 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PSA</t>
+          <t>TTWO</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>297.67</v>
+        <v>210.08</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2119,34 +2118,31 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>48</v>
+        <v>49.7</v>
       </c>
       <c r="J18" t="n">
-        <v>39.5</v>
+        <v>35.7</v>
       </c>
       <c r="K18" t="n">
-        <v>92</v>
+        <v>74</v>
       </c>
       <c r="L18" t="n">
-        <v>1.97</v>
+        <v>3.55</v>
       </c>
       <c r="M18" t="n">
-        <v>16.1</v>
-      </c>
-      <c r="N18" t="n">
-        <v>5.3</v>
+        <v>37.5</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>46.4</v>
+        <v>41.3</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2155,17 +2151,17 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
@@ -2178,71 +2174,71 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TJX</t>
+          <t>FANG</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>124.97</v>
+        <v>196.06</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>42.2</v>
+        <v>47.6</v>
       </c>
       <c r="J19" t="n">
-        <v>18.5</v>
+        <v>44.4</v>
       </c>
       <c r="K19" t="n">
-        <v>85</v>
+        <v>9</v>
       </c>
       <c r="L19" t="n">
-        <v>2</v>
+        <v>3.78</v>
       </c>
       <c r="M19" t="n">
-        <v>20.7</v>
+        <v>36.1</v>
       </c>
       <c r="N19" t="n">
-        <v>41</v>
+        <v>71</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>29.8</v>
+        <v>53</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>FIRED</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -2252,15 +2248,19 @@
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U19" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>Squeeze Fired, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V19" t="inlineStr">
         <is>
           <t>No</t>
@@ -2270,30 +2270,30 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>195.8</v>
+        <v>244.75</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2303,34 +2303,34 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>40.7</v>
+        <v>46.6</v>
       </c>
       <c r="J20" t="n">
-        <v>35.3</v>
+        <v>57.9</v>
       </c>
       <c r="K20" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="L20" t="n">
-        <v>2.01</v>
+        <v>3.96</v>
       </c>
       <c r="M20" t="n">
-        <v>21</v>
+        <v>75.7</v>
       </c>
       <c r="N20" t="n">
-        <v>27.8</v>
+        <v>94</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>34.9</v>
+        <v>64.3</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2344,12 +2344,12 @@
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U20" t="inlineStr"/>
@@ -2362,30 +2362,30 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>XEL</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>73.06</v>
+        <v>683.99</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2395,31 +2395,34 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>38.7</v>
+        <v>46.1</v>
       </c>
       <c r="J21" t="n">
+        <v>60.9</v>
+      </c>
+      <c r="K21" t="n">
+        <v>71</v>
+      </c>
+      <c r="L21" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="M21" t="n">
         <v>35.1</v>
       </c>
-      <c r="K21" t="n">
-        <v>91</v>
-      </c>
-      <c r="L21" t="n">
-        <v>1.88</v>
-      </c>
-      <c r="M21" t="n">
-        <v>26.1</v>
+      <c r="N21" t="n">
+        <v>64.09999999999999</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>39.9</v>
+        <v>63.2</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2428,12 +2431,12 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
@@ -2451,11 +2454,11 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>GD</t>
+          <t>IDXX</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>360.41</v>
+        <v>512.11</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -2484,31 +2487,34 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>37.8</v>
+        <v>45.9</v>
       </c>
       <c r="J22" t="n">
-        <v>38.8</v>
+        <v>36.7</v>
       </c>
       <c r="K22" t="n">
-        <v>67</v>
+        <v>99</v>
       </c>
       <c r="L22" t="n">
-        <v>1.74</v>
+        <v>2.6</v>
       </c>
       <c r="M22" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="N22" t="n">
+        <v>15.5</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P22" t="n">
-        <v>49.8</v>
+        <v>37.3</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
@@ -2517,17 +2523,17 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U22" t="inlineStr"/>
@@ -2540,67 +2546,67 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>BAC</t>
+          <t>XEL</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>58.26</v>
+        <v>73.56</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>24.4</v>
+        <v>40.4</v>
       </c>
       <c r="J23" t="n">
-        <v>30.2</v>
+        <v>38.6</v>
       </c>
       <c r="K23" t="n">
-        <v>42</v>
+        <v>88</v>
       </c>
       <c r="L23" t="n">
-        <v>2.45</v>
+        <v>1.79</v>
       </c>
       <c r="M23" t="n">
-        <v>21.4</v>
+        <v>17.4</v>
       </c>
       <c r="N23" t="n">
-        <v>47</v>
+        <v>36.2</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>52</v>
+        <v>40.9</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -2622,12 +2628,288 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U23" t="inlineStr">
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>194.65</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>39</v>
+      </c>
+      <c r="J24" t="n">
+        <v>33.6</v>
+      </c>
+      <c r="K24" t="n">
+        <v>89</v>
+      </c>
+      <c r="L24" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="M24" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="N24" t="n">
+        <v>23</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P24" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>HSY</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>170.01</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>35.1</v>
+      </c>
+      <c r="J25" t="n">
+        <v>35.9</v>
+      </c>
+      <c r="K25" t="n">
+        <v>84</v>
+      </c>
+      <c r="L25" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="M25" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="N25" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P25" t="n">
+        <v>40.8</v>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>303.39</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>34</v>
+      </c>
+      <c r="J26" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="K26" t="n">
+        <v>81</v>
+      </c>
+      <c r="L26" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="M26" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="N26" t="n">
+        <v>38</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P26" t="n">
+        <v>38.8</v>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
         <is>
           <t>Divergence</t>
         </is>
       </c>
-      <c r="V23" t="inlineStr">
+      <c r="V26" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>

</xml_diff>

<commit_message>
Scan 18.09.2026 17:37 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V26"/>
+  <dimension ref="A1:V27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>AZN</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>368.33</v>
+        <v>166.21</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,22 +614,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>81.5</v>
+        <v>85</v>
       </c>
       <c r="J2" t="n">
-        <v>55.7</v>
+        <v>55.1</v>
       </c>
       <c r="K2" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="L2" t="n">
-        <v>3.51</v>
+        <v>2.03</v>
       </c>
       <c r="M2" t="n">
-        <v>44.6</v>
+        <v>21.8</v>
       </c>
       <c r="N2" t="n">
-        <v>36.9</v>
+        <v>15.5</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,11 +637,11 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>48.6</v>
+        <v>44.5</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -651,17 +651,17 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>Squeeze Expanding</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -677,7 +677,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>188.08</v>
+        <v>188.29</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -710,16 +710,16 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>80.5</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="J3" t="n">
-        <v>55.8</v>
+        <v>56.1</v>
       </c>
       <c r="K3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L3" t="n">
-        <v>1.77</v>
+        <v>1.67</v>
       </c>
       <c r="M3" t="n">
         <v>21.9</v>
@@ -730,11 +730,11 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>62.6</v>
+        <v>62.7</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>FIRED</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -749,12 +749,12 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Squeeze Fired, Squeeze Expanding</t>
+          <t>Squeeze Expanding</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>261.75</v>
+        <v>268.12</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -803,34 +803,34 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>80</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="J4" t="n">
+        <v>55.2</v>
+      </c>
+      <c r="K4" t="n">
+        <v>5</v>
+      </c>
+      <c r="L4" t="n">
+        <v>5.65</v>
+      </c>
+      <c r="M4" t="n">
+        <v>60.3</v>
+      </c>
+      <c r="N4" t="n">
+        <v>29.3</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P4" t="n">
         <v>52.9</v>
       </c>
-      <c r="K4" t="n">
-        <v>3</v>
-      </c>
-      <c r="L4" t="n">
-        <v>6.19</v>
-      </c>
-      <c r="M4" t="n">
-        <v>60.2</v>
-      </c>
-      <c r="N4" t="n">
-        <v>29.1</v>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P4" t="n">
-        <v>51.9</v>
-      </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -845,12 +845,12 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>Squeeze Expanding</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -862,11 +862,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DHR</t>
+          <t>TSLA</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>212.18</v>
+        <v>362.62</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -899,44 +899,44 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>78.90000000000001</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>57.3</v>
+        <v>52.9</v>
       </c>
       <c r="K5" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="L5" t="n">
-        <v>2.61</v>
+        <v>3.46</v>
       </c>
       <c r="M5" t="n">
-        <v>28.9</v>
+        <v>44.4</v>
       </c>
       <c r="N5" t="n">
-        <v>36.1</v>
+        <v>36.5</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>56.6</v>
+        <v>47.3</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>Squeeze Expanding</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>716.7</v>
+        <v>717.34</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -995,19 +995,19 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>76.5</v>
+        <v>82.8</v>
       </c>
       <c r="J6" t="n">
-        <v>52.9</v>
+        <v>53.3</v>
       </c>
       <c r="K6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L6" t="n">
-        <v>1.28</v>
+        <v>1.21</v>
       </c>
       <c r="M6" t="n">
-        <v>16.7</v>
+        <v>16.6</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1015,7 +1015,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>57.9</v>
+        <v>58</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1029,7 +1029,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1051,11 +1051,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AZN</t>
+          <t>DHR</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>165.66</v>
+        <v>210.67</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1088,30 +1088,30 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>76.3</v>
+        <v>81.2</v>
       </c>
       <c r="J7" t="n">
-        <v>54.2</v>
+        <v>55</v>
       </c>
       <c r="K7" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="L7" t="n">
-        <v>2.14</v>
+        <v>2.6</v>
       </c>
       <c r="M7" t="n">
-        <v>21.6</v>
+        <v>29.2</v>
       </c>
       <c r="N7" t="n">
-        <v>14.8</v>
+        <v>36.9</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1125,7 +1125,7 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -1133,11 +1133,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr">
         <is>
           <t>No</t>
@@ -1151,7 +1147,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>198.62</v>
+        <v>195.01</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1184,19 +1180,22 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>76.09999999999999</v>
+        <v>77.8</v>
       </c>
       <c r="J8" t="n">
-        <v>57.6</v>
+        <v>54.6</v>
       </c>
       <c r="K8" t="n">
         <v>7</v>
       </c>
       <c r="L8" t="n">
-        <v>4.42</v>
+        <v>4.31</v>
       </c>
       <c r="M8" t="n">
-        <v>48.9</v>
+        <v>71.90000000000001</v>
+      </c>
+      <c r="N8" t="n">
+        <v>83.3</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1204,7 +1203,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>62.2</v>
+        <v>61.2</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1213,12 +1212,12 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -1226,11 +1225,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
           <t>No</t>
@@ -1244,7 +1239,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>40.54</v>
+        <v>38.88</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1277,22 +1272,22 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>75.09999999999999</v>
+        <v>76.7</v>
       </c>
       <c r="J9" t="n">
-        <v>59.2</v>
+        <v>54.9</v>
       </c>
       <c r="K9" t="n">
         <v>7</v>
       </c>
       <c r="L9" t="n">
-        <v>6.28</v>
+        <v>6.39</v>
       </c>
       <c r="M9" t="n">
-        <v>87</v>
+        <v>86.8</v>
       </c>
       <c r="N9" t="n">
-        <v>45.5</v>
+        <v>45.3</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1300,7 +1295,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>58.2</v>
+        <v>56.1</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1309,22 +1304,22 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
@@ -1336,15 +1331,15 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>NXPI</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>225.62</v>
+        <v>670.65</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -1359,45 +1354,48 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>74.3</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="J10" t="n">
-        <v>47</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="K10" t="n">
-        <v>3</v>
+        <v>94</v>
       </c>
       <c r="L10" t="n">
-        <v>3.51</v>
+        <v>3.06</v>
       </c>
       <c r="M10" t="n">
-        <v>43.6</v>
+        <v>34.2</v>
+      </c>
+      <c r="N10" t="n">
+        <v>39.3</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>43.5</v>
+        <v>57.1</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -1407,7 +1405,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1417,23 +1415,23 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>Divergence</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>NXPI</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>110.07</v>
+        <v>226.41</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1466,30 +1464,27 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>71.5</v>
+        <v>75.5</v>
       </c>
       <c r="J11" t="n">
-        <v>47.4</v>
+        <v>47.6</v>
       </c>
       <c r="K11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L11" t="n">
-        <v>2.49</v>
+        <v>3.52</v>
       </c>
       <c r="M11" t="n">
-        <v>33.9</v>
-      </c>
-      <c r="N11" t="n">
-        <v>47</v>
+        <v>44.1</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>55.1</v>
+        <v>43.7</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1525,81 +1520,81 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SYK</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>282.43</v>
+        <v>108.89</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>68.5</v>
+        <v>69.7</v>
       </c>
       <c r="J12" t="n">
-        <v>34.4</v>
+        <v>44.8</v>
       </c>
       <c r="K12" t="n">
-        <v>98</v>
+        <v>4</v>
       </c>
       <c r="L12" t="n">
-        <v>3.49</v>
+        <v>2.51</v>
       </c>
       <c r="M12" t="n">
-        <v>35.5</v>
+        <v>34.1</v>
       </c>
       <c r="N12" t="n">
-        <v>64</v>
+        <v>47.5</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>36.2</v>
+        <v>53.7</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -1607,10 +1602,14 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr"/>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1621,7 +1620,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>68.20999999999999</v>
+        <v>68.93000000000001</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1654,22 +1653,22 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>64.2</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="J13" t="n">
-        <v>39.3</v>
+        <v>40.7</v>
       </c>
       <c r="K13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L13" t="n">
-        <v>5.85</v>
+        <v>5.51</v>
       </c>
       <c r="M13" t="n">
-        <v>53.7</v>
+        <v>53.5</v>
       </c>
       <c r="N13" t="n">
-        <v>24.4</v>
+        <v>24.1</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1677,7 +1676,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>38.5</v>
+        <v>39</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1713,71 +1712,71 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AMP</t>
+          <t>SYK</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>547.14</v>
+        <v>277.26</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>57.8</v>
+        <v>65</v>
       </c>
       <c r="J14" t="n">
-        <v>47</v>
+        <v>32.1</v>
       </c>
       <c r="K14" t="n">
-        <v>8</v>
+        <v>99</v>
       </c>
       <c r="L14" t="n">
-        <v>2.34</v>
+        <v>3.28</v>
       </c>
       <c r="M14" t="n">
-        <v>19.8</v>
+        <v>35.6</v>
       </c>
       <c r="N14" t="n">
-        <v>13.4</v>
+        <v>64.3</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>63</v>
+        <v>34</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -1787,19 +1786,15 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr">
         <is>
           <t>No</t>
@@ -1809,59 +1804,59 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TSN</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>52.63</v>
+        <v>230.3</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>54.1</v>
+        <v>59.6</v>
       </c>
       <c r="J15" t="n">
-        <v>40</v>
+        <v>44.6</v>
       </c>
       <c r="K15" t="n">
-        <v>79</v>
+        <v>19</v>
       </c>
       <c r="L15" t="n">
-        <v>2.37</v>
+        <v>3.35</v>
       </c>
       <c r="M15" t="n">
-        <v>28.2</v>
+        <v>32.3</v>
       </c>
       <c r="N15" t="n">
-        <v>50.6</v>
+        <v>20.9</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1869,7 +1864,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>37.1</v>
+        <v>45.1</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1878,104 +1873,108 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="U15" t="inlineStr"/>
-      <c r="V15" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PSA</t>
+          <t>AMP</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>299.35</v>
+        <v>545.67</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>51.7</v>
+        <v>56.9</v>
       </c>
       <c r="J16" t="n">
-        <v>43.1</v>
+        <v>46</v>
       </c>
       <c r="K16" t="n">
-        <v>90</v>
+        <v>11</v>
       </c>
       <c r="L16" t="n">
-        <v>1.98</v>
+        <v>2.24</v>
       </c>
       <c r="M16" t="n">
-        <v>16.9</v>
+        <v>19.6</v>
       </c>
       <c r="N16" t="n">
-        <v>11.2</v>
+        <v>12.9</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>47.3</v>
+        <v>62.3</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
@@ -1983,7 +1982,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr"/>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V16" t="inlineStr">
         <is>
           <t>No</t>
@@ -1993,11 +1996,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TJX</t>
+          <t>TSN</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>125.88</v>
+        <v>53.06</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -2026,26 +2029,26 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>51.4</v>
+        <v>56.4</v>
       </c>
       <c r="J17" t="n">
-        <v>27.1</v>
+        <v>42.8</v>
       </c>
       <c r="K17" t="n">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="L17" t="n">
-        <v>2.15</v>
+        <v>2.4</v>
       </c>
       <c r="M17" t="n">
-        <v>21.7</v>
+        <v>28.4</v>
       </c>
       <c r="N17" t="n">
-        <v>46.4</v>
+        <v>50.3</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2053,7 +2056,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>30.3</v>
+        <v>38.1</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2085,11 +2088,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TTWO</t>
+          <t>TJX</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>210.08</v>
+        <v>128.76</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2122,19 +2125,22 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>49.7</v>
+        <v>56.3</v>
       </c>
       <c r="J18" t="n">
-        <v>35.7</v>
+        <v>35.9</v>
       </c>
       <c r="K18" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="L18" t="n">
-        <v>3.55</v>
+        <v>2.17</v>
       </c>
       <c r="M18" t="n">
-        <v>37.5</v>
+        <v>22.8</v>
+      </c>
+      <c r="N18" t="n">
+        <v>52.6</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -2142,7 +2148,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>41.3</v>
+        <v>33.5</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2151,17 +2157,17 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
@@ -2174,81 +2180,81 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>FANG</t>
+          <t>PSA</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>196.06</v>
+        <v>299.16</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>47.6</v>
+        <v>54.2</v>
       </c>
       <c r="J19" t="n">
-        <v>44.4</v>
+        <v>43.2</v>
       </c>
       <c r="K19" t="n">
-        <v>9</v>
+        <v>85</v>
       </c>
       <c r="L19" t="n">
-        <v>3.78</v>
+        <v>1.95</v>
       </c>
       <c r="M19" t="n">
-        <v>36.1</v>
+        <v>17.4</v>
       </c>
       <c r="N19" t="n">
-        <v>71</v>
+        <v>15.2</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>53</v>
+        <v>47.2</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>FIRED</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
@@ -2256,11 +2262,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>Squeeze Fired, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr">
         <is>
           <t>No</t>
@@ -2270,15 +2272,15 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>GM</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>244.75</v>
+        <v>82.03</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -2293,36 +2295,36 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>46.6</v>
+        <v>45.1</v>
       </c>
       <c r="J20" t="n">
-        <v>57.9</v>
+        <v>41.8</v>
       </c>
       <c r="K20" t="n">
-        <v>80</v>
+        <v>13</v>
       </c>
       <c r="L20" t="n">
-        <v>3.96</v>
+        <v>3.46</v>
       </c>
       <c r="M20" t="n">
-        <v>75.7</v>
+        <v>30.2</v>
       </c>
       <c r="N20" t="n">
-        <v>94</v>
+        <v>30.8</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2330,11 +2332,11 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>64.3</v>
+        <v>51.5</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -2344,7 +2346,7 @@
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
@@ -2352,40 +2354,44 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U20" t="inlineStr"/>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>MMM</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>683.99</v>
+        <v>165.01</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2395,26 +2401,26 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>46.1</v>
+        <v>45</v>
       </c>
       <c r="J21" t="n">
-        <v>60.9</v>
+        <v>40.2</v>
       </c>
       <c r="K21" t="n">
-        <v>71</v>
+        <v>82</v>
       </c>
       <c r="L21" t="n">
-        <v>2.46</v>
+        <v>2.08</v>
       </c>
       <c r="M21" t="n">
-        <v>35.1</v>
+        <v>16.3</v>
       </c>
       <c r="N21" t="n">
-        <v>64.09999999999999</v>
+        <v>3.6</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2422,7 +2428,7 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>63.2</v>
+        <v>51.6</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2431,12 +2437,12 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
@@ -2454,81 +2460,81 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>IDXX</t>
+          <t>FANG</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>512.11</v>
+        <v>193.38</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>45.9</v>
+        <v>44.3</v>
       </c>
       <c r="J22" t="n">
-        <v>36.7</v>
+        <v>42.1</v>
       </c>
       <c r="K22" t="n">
-        <v>99</v>
+        <v>10</v>
       </c>
       <c r="L22" t="n">
-        <v>2.6</v>
+        <v>3.65</v>
       </c>
       <c r="M22" t="n">
-        <v>24</v>
+        <v>36.3</v>
       </c>
       <c r="N22" t="n">
-        <v>15.5</v>
+        <v>72.2</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P22" t="n">
-        <v>37.3</v>
+        <v>51.7</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>FIRED</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
@@ -2536,7 +2542,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U22" t="inlineStr"/>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>Squeeze Fired, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V22" t="inlineStr">
         <is>
           <t>No</t>
@@ -2550,7 +2560,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>73.56</v>
+        <v>72.53</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -2583,22 +2593,22 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>40.4</v>
+        <v>38.9</v>
       </c>
       <c r="J23" t="n">
-        <v>38.6</v>
+        <v>34.8</v>
       </c>
       <c r="K23" t="n">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="L23" t="n">
-        <v>1.79</v>
+        <v>1.82</v>
       </c>
       <c r="M23" t="n">
-        <v>17.4</v>
+        <v>17.9</v>
       </c>
       <c r="N23" t="n">
-        <v>36.2</v>
+        <v>39.8</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2606,7 +2616,7 @@
         </is>
       </c>
       <c r="P23" t="n">
-        <v>40.9</v>
+        <v>39</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -2638,30 +2648,30 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>194.65</v>
+        <v>238.66</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2671,34 +2681,34 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I24" t="n">
-        <v>39</v>
+        <v>37.1</v>
       </c>
       <c r="J24" t="n">
-        <v>33.6</v>
+        <v>54</v>
       </c>
       <c r="K24" t="n">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="L24" t="n">
-        <v>2.22</v>
+        <v>3.86</v>
       </c>
       <c r="M24" t="n">
-        <v>20.5</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="N24" t="n">
-        <v>23</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P24" t="n">
-        <v>34.4</v>
+        <v>62</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -2712,12 +2722,12 @@
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U24" t="inlineStr"/>
@@ -2730,11 +2740,11 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>HSY</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>170.01</v>
+        <v>192.42</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -2767,22 +2777,22 @@
         </is>
       </c>
       <c r="I25" t="n">
-        <v>35.1</v>
+        <v>36.2</v>
       </c>
       <c r="J25" t="n">
-        <v>35.9</v>
+        <v>30.7</v>
       </c>
       <c r="K25" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="L25" t="n">
         <v>2.12</v>
       </c>
       <c r="M25" t="n">
-        <v>19.8</v>
+        <v>20.5</v>
       </c>
       <c r="N25" t="n">
-        <v>9.9</v>
+        <v>22.9</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2790,7 +2800,7 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>40.8</v>
+        <v>33.5</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
@@ -2826,7 +2836,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>303.39</v>
+        <v>300.32</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -2859,22 +2869,22 @@
         </is>
       </c>
       <c r="I26" t="n">
-        <v>34</v>
+        <v>34.4</v>
       </c>
       <c r="J26" t="n">
-        <v>32.5</v>
+        <v>29.9</v>
       </c>
       <c r="K26" t="n">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="L26" t="n">
-        <v>2.15</v>
+        <v>2.07</v>
       </c>
       <c r="M26" t="n">
-        <v>20.9</v>
+        <v>20.8</v>
       </c>
       <c r="N26" t="n">
-        <v>38</v>
+        <v>37.2</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -2882,7 +2892,7 @@
         </is>
       </c>
       <c r="P26" t="n">
-        <v>38.8</v>
+        <v>37.9</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
@@ -2904,14 +2914,102 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U26" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U26" t="inlineStr"/>
       <c r="V26" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>HSY</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>168.21</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>32.9</v>
+      </c>
+      <c r="J27" t="n">
+        <v>33.4</v>
+      </c>
+      <c r="K27" t="n">
+        <v>84</v>
+      </c>
+      <c r="L27" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="M27" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="N27" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P27" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr"/>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan 21.09.2026 19:13 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -31,10 +31,10 @@
       <sz val="11"/>
     </font>
     <font>
-      <color rgb="0022c55e"/>
+      <color rgb="00ef4444"/>
     </font>
     <font>
-      <color rgb="00ef4444"/>
+      <color rgb="0022c55e"/>
     </font>
   </fonts>
   <fills count="3">
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V27"/>
+  <dimension ref="A1:V30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -448,7 +448,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
     <col width="6" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
@@ -577,67 +577,67 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AZN</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>166.21</v>
+        <v>744.36</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>85</v>
+        <v>95.2</v>
       </c>
       <c r="J2" t="n">
-        <v>55.1</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="K2" t="n">
-        <v>13</v>
+        <v>100</v>
       </c>
       <c r="L2" t="n">
-        <v>2.03</v>
+        <v>4.01</v>
       </c>
       <c r="M2" t="n">
-        <v>21.8</v>
+        <v>47.8</v>
       </c>
       <c r="N2" t="n">
-        <v>15.5</v>
+        <v>77.5</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>44.5</v>
+        <v>63.7</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -651,7 +651,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -659,11 +659,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
         <is>
           <t>No</t>
@@ -673,18 +669,18 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>XLK</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>188.29</v>
+        <v>381.89</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -710,19 +706,22 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>84.90000000000001</v>
+        <v>89.5</v>
       </c>
       <c r="J3" t="n">
-        <v>56.1</v>
+        <v>58.6</v>
       </c>
       <c r="K3" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L3" t="n">
-        <v>1.67</v>
+        <v>2.97</v>
       </c>
       <c r="M3" t="n">
-        <v>21.9</v>
+        <v>30.1</v>
+      </c>
+      <c r="N3" t="n">
+        <v>17</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -730,11 +729,11 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>62.7</v>
+        <v>54.5</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>FIRED</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -744,17 +743,17 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Squeeze Expanding</t>
+          <t>Squeeze Fired, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -766,18 +765,18 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>DHR</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>268.12</v>
+        <v>214.84</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -803,22 +802,22 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>83.59999999999999</v>
+        <v>88.59999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>55.2</v>
+        <v>60.1</v>
       </c>
       <c r="K4" t="n">
         <v>5</v>
       </c>
       <c r="L4" t="n">
-        <v>5.65</v>
+        <v>2.5</v>
       </c>
       <c r="M4" t="n">
-        <v>60.3</v>
+        <v>28.6</v>
       </c>
       <c r="N4" t="n">
-        <v>29.3</v>
+        <v>34.8</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -826,7 +825,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>52.9</v>
+        <v>57.8</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -840,7 +839,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -848,11 +847,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
         <is>
           <t>No</t>
@@ -862,18 +857,18 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>XLK</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>362.62</v>
+        <v>194.64</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -899,44 +894,41 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>82.90000000000001</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>52.9</v>
+        <v>65</v>
       </c>
       <c r="K5" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="L5" t="n">
-        <v>3.46</v>
+        <v>1.78</v>
       </c>
       <c r="M5" t="n">
-        <v>44.4</v>
-      </c>
-      <c r="N5" t="n">
-        <v>36.5</v>
+        <v>24.7</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>47.3</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -946,7 +938,7 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>TTM Squeeze</t>
+          <t>Squeeze Expanding</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
@@ -958,18 +950,18 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>AZN</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>717.34</v>
+        <v>168.64</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -991,35 +983,38 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>82.8</v>
+        <v>86.3</v>
       </c>
       <c r="J6" t="n">
-        <v>53.3</v>
+        <v>58.9</v>
       </c>
       <c r="K6" t="n">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="L6" t="n">
-        <v>1.21</v>
+        <v>1.97</v>
       </c>
       <c r="M6" t="n">
-        <v>16.6</v>
+        <v>22.2</v>
+      </c>
+      <c r="N6" t="n">
+        <v>17</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>58</v>
+        <v>46.4</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1029,19 +1024,15 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr">
         <is>
           <t>No</t>
@@ -1051,18 +1042,18 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DHR</t>
+          <t>TSLA</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>210.67</v>
+        <v>375.61</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -1088,34 +1079,34 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>81.2</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>55</v>
+        <v>58.7</v>
       </c>
       <c r="K7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L7" t="n">
-        <v>2.6</v>
+        <v>3.4</v>
       </c>
       <c r="M7" t="n">
-        <v>29.2</v>
+        <v>44.4</v>
       </c>
       <c r="N7" t="n">
-        <v>36.9</v>
+        <v>36.6</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>56</v>
+        <v>50.3</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1130,10 +1121,14 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V7" t="inlineStr">
         <is>
           <t>No</t>
@@ -1143,18 +1138,18 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>WDAY</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>195.01</v>
+        <v>41.14</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -1180,22 +1175,22 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>77.8</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="J8" t="n">
-        <v>54.6</v>
+        <v>59.5</v>
       </c>
       <c r="K8" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="L8" t="n">
-        <v>4.31</v>
+        <v>6.09</v>
       </c>
       <c r="M8" t="n">
-        <v>71.90000000000001</v>
+        <v>86.2</v>
       </c>
       <c r="N8" t="n">
-        <v>83.3</v>
+        <v>44.7</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1203,29 +1198,33 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>61.2</v>
+        <v>58.5</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V8" t="inlineStr">
         <is>
           <t>No</t>
@@ -1235,18 +1234,18 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>38.88</v>
+        <v>741.55</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -1272,22 +1271,19 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>76.7</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="J9" t="n">
-        <v>54.9</v>
+        <v>65.7</v>
       </c>
       <c r="K9" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="L9" t="n">
-        <v>6.39</v>
+        <v>1.41</v>
       </c>
       <c r="M9" t="n">
-        <v>86.8</v>
-      </c>
-      <c r="N9" t="n">
-        <v>45.3</v>
+        <v>17.8</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1295,31 +1291,31 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>56.1</v>
+        <v>63.2</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>FIRED</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>TTM Squeeze</t>
+          <t>Squeeze Fired, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
@@ -1331,59 +1327,59 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>BIIB</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>670.65</v>
+        <v>221.25</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>76.09999999999999</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="J10" t="n">
-        <v>68.09999999999999</v>
+        <v>57.2</v>
       </c>
       <c r="K10" t="n">
-        <v>94</v>
+        <v>6</v>
       </c>
       <c r="L10" t="n">
-        <v>3.06</v>
+        <v>2.51</v>
       </c>
       <c r="M10" t="n">
-        <v>34.2</v>
+        <v>28</v>
       </c>
       <c r="N10" t="n">
-        <v>39.3</v>
+        <v>15.6</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1391,11 +1387,11 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>57.1</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -1410,28 +1406,28 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>NXPI</t>
+          <t>WDAY</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>226.41</v>
+        <v>192.64</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1440,17 +1436,17 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1464,41 +1460,41 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>75.5</v>
+        <v>79.3</v>
       </c>
       <c r="J11" t="n">
-        <v>47.6</v>
+        <v>52.9</v>
       </c>
       <c r="K11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L11" t="n">
-        <v>3.52</v>
+        <v>4.1</v>
       </c>
       <c r="M11" t="n">
-        <v>44.1</v>
+        <v>54</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>43.7</v>
+        <v>60.3</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1506,11 +1502,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+      <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr">
         <is>
           <t>No</t>
@@ -1520,18 +1512,18 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>108.89</v>
+        <v>338.46</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -1557,22 +1549,22 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>69.7</v>
+        <v>79</v>
       </c>
       <c r="J12" t="n">
-        <v>44.8</v>
+        <v>45.6</v>
       </c>
       <c r="K12" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L12" t="n">
-        <v>2.51</v>
+        <v>1.4</v>
       </c>
       <c r="M12" t="n">
-        <v>34.1</v>
+        <v>15.1</v>
       </c>
       <c r="N12" t="n">
-        <v>47.5</v>
+        <v>8.1</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1580,7 +1572,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>53.7</v>
+        <v>53</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1589,45 +1581,45 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>VLO</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>68.93000000000001</v>
+        <v>398.12</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -1639,91 +1631,88 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>67.59999999999999</v>
+        <v>78.8</v>
       </c>
       <c r="J13" t="n">
-        <v>40.7</v>
+        <v>66.8</v>
       </c>
       <c r="K13" t="n">
-        <v>4</v>
+        <v>86</v>
       </c>
       <c r="L13" t="n">
-        <v>5.51</v>
+        <v>3.78</v>
       </c>
       <c r="M13" t="n">
-        <v>53.5</v>
-      </c>
-      <c r="N13" t="n">
-        <v>24.1</v>
+        <v>53.4</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>39</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>Divergence</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SYK</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>277.26</v>
+        <v>259.27</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -1735,44 +1724,44 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>65</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="J14" t="n">
-        <v>32.1</v>
+        <v>53.4</v>
       </c>
       <c r="K14" t="n">
-        <v>99</v>
+        <v>16</v>
       </c>
       <c r="L14" t="n">
-        <v>3.28</v>
+        <v>2.17</v>
       </c>
       <c r="M14" t="n">
-        <v>35.6</v>
+        <v>26.1</v>
       </c>
       <c r="N14" t="n">
-        <v>64.3</v>
+        <v>16.2</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>34</v>
+        <v>54.1</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1781,12 +1770,12 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -1794,7 +1783,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr"/>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V14" t="inlineStr">
         <is>
           <t>No</t>
@@ -1804,18 +1797,18 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>APP</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>230.3</v>
+        <v>333.01</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -1841,22 +1834,19 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>59.6</v>
+        <v>76.8</v>
       </c>
       <c r="J15" t="n">
-        <v>44.6</v>
+        <v>51.3</v>
       </c>
       <c r="K15" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="L15" t="n">
-        <v>3.35</v>
+        <v>5.13</v>
       </c>
       <c r="M15" t="n">
-        <v>32.3</v>
-      </c>
-      <c r="N15" t="n">
-        <v>20.9</v>
+        <v>55.2</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1864,7 +1854,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>45.1</v>
+        <v>40.2</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1873,12 +1863,12 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -1888,23 +1878,23 @@
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>Divergence, Squeeze Expanding</t>
+          <t>Squeeze Expanding</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AMP</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>545.67</v>
+        <v>184.73</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1913,17 +1903,17 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1937,22 +1927,22 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>56.9</v>
+        <v>76.7</v>
       </c>
       <c r="J16" t="n">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="K16" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="L16" t="n">
-        <v>2.24</v>
+        <v>4.2</v>
       </c>
       <c r="M16" t="n">
-        <v>19.6</v>
+        <v>49.9</v>
       </c>
       <c r="N16" t="n">
-        <v>12.9</v>
+        <v>22.9</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1960,31 +1950,31 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>62.3</v>
+        <v>49.3</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>Squeeze Expanding</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
@@ -1996,18 +1986,18 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TSN</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>53.06</v>
+        <v>322.43</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -2019,12 +2009,12 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2033,30 +2023,30 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>56.4</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="J17" t="n">
-        <v>42.8</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="K17" t="n">
-        <v>77</v>
+        <v>35</v>
       </c>
       <c r="L17" t="n">
-        <v>2.4</v>
+        <v>6.22</v>
       </c>
       <c r="M17" t="n">
-        <v>28.4</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="N17" t="n">
-        <v>50.3</v>
+        <v>48.9</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>38.1</v>
+        <v>60.3</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2070,12 +2060,12 @@
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
@@ -2088,71 +2078,71 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TJX</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>128.76</v>
+        <v>110.82</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>56.3</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="J18" t="n">
-        <v>35.9</v>
+        <v>49.4</v>
       </c>
       <c r="K18" t="n">
-        <v>78</v>
+        <v>2</v>
       </c>
       <c r="L18" t="n">
-        <v>2.17</v>
+        <v>2.42</v>
       </c>
       <c r="M18" t="n">
-        <v>22.8</v>
+        <v>34.2</v>
       </c>
       <c r="N18" t="n">
-        <v>52.6</v>
+        <v>47.8</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>33.5</v>
+        <v>55.7</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -2167,10 +2157,14 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U18" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V18" t="inlineStr">
         <is>
           <t>No</t>
@@ -2180,18 +2174,18 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PSA</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>299.16</v>
+        <v>774.38</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -2203,44 +2197,41 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>54.2</v>
+        <v>73.5</v>
       </c>
       <c r="J19" t="n">
-        <v>43.2</v>
+        <v>60.3</v>
       </c>
       <c r="K19" t="n">
-        <v>85</v>
+        <v>18</v>
       </c>
       <c r="L19" t="n">
-        <v>1.95</v>
+        <v>0.97</v>
       </c>
       <c r="M19" t="n">
-        <v>17.4</v>
-      </c>
-      <c r="N19" t="n">
-        <v>15.2</v>
+        <v>12.3</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>47.2</v>
+        <v>65.3</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2254,15 +2245,19 @@
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U19" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V19" t="inlineStr">
         <is>
           <t>No</t>
@@ -2272,81 +2267,81 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>GM</t>
+          <t>TJX</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>82.03</v>
+        <v>130.93</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>45.1</v>
+        <v>65.8</v>
       </c>
       <c r="J20" t="n">
-        <v>41.8</v>
+        <v>42</v>
       </c>
       <c r="K20" t="n">
-        <v>13</v>
+        <v>72</v>
       </c>
       <c r="L20" t="n">
-        <v>3.46</v>
+        <v>2.3</v>
       </c>
       <c r="M20" t="n">
-        <v>30.2</v>
+        <v>24.4</v>
       </c>
       <c r="N20" t="n">
-        <v>30.8</v>
+        <v>61.4</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>51.5</v>
+        <v>36</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
@@ -2354,32 +2349,28 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U20" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MMM</t>
+          <t>SYK</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>165.01</v>
+        <v>274.28</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -2405,30 +2396,30 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>45</v>
+        <v>62.8</v>
       </c>
       <c r="J21" t="n">
-        <v>40.2</v>
+        <v>30.9</v>
       </c>
       <c r="K21" t="n">
-        <v>82</v>
+        <v>100</v>
       </c>
       <c r="L21" t="n">
-        <v>2.08</v>
+        <v>3.18</v>
       </c>
       <c r="M21" t="n">
-        <v>16.3</v>
+        <v>35.6</v>
       </c>
       <c r="N21" t="n">
-        <v>3.6</v>
+        <v>64.3</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>51.6</v>
+        <v>32.9</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2460,18 +2451,18 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>FANG</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>193.38</v>
+        <v>230.46</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -2493,38 +2484,38 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>44.3</v>
+        <v>58.4</v>
       </c>
       <c r="J22" t="n">
-        <v>42.1</v>
+        <v>44.9</v>
       </c>
       <c r="K22" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="L22" t="n">
-        <v>3.65</v>
+        <v>3.27</v>
       </c>
       <c r="M22" t="n">
-        <v>36.3</v>
+        <v>32.2</v>
       </c>
       <c r="N22" t="n">
-        <v>72.2</v>
+        <v>20.8</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P22" t="n">
-        <v>51.7</v>
+        <v>45.2</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>FIRED</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -2534,19 +2525,15 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t>Squeeze Fired, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr"/>
       <c r="V22" t="inlineStr">
         <is>
           <t>No</t>
@@ -2556,71 +2543,71 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>XEL</t>
+          <t>GM</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>72.53</v>
+        <v>84.69</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>38.9</v>
+        <v>53.3</v>
       </c>
       <c r="J23" t="n">
-        <v>34.8</v>
+        <v>48.5</v>
       </c>
       <c r="K23" t="n">
-        <v>85</v>
+        <v>9</v>
       </c>
       <c r="L23" t="n">
-        <v>1.82</v>
+        <v>3.33</v>
       </c>
       <c r="M23" t="n">
-        <v>17.9</v>
+        <v>31.2</v>
       </c>
       <c r="N23" t="n">
-        <v>39.8</v>
+        <v>34.2</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>39</v>
+        <v>55.4</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
@@ -2635,10 +2622,14 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V23" t="inlineStr">
         <is>
           <t>No</t>
@@ -2648,18 +2639,18 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>XLE</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>238.66</v>
+        <v>62.79</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -2671,36 +2662,36 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I24" t="n">
-        <v>37.1</v>
+        <v>52.7</v>
       </c>
       <c r="J24" t="n">
-        <v>54</v>
+        <v>47.3</v>
       </c>
       <c r="K24" t="n">
-        <v>78</v>
+        <v>9</v>
       </c>
       <c r="L24" t="n">
-        <v>3.86</v>
+        <v>2.18</v>
       </c>
       <c r="M24" t="n">
-        <v>75.40000000000001</v>
+        <v>23</v>
       </c>
       <c r="N24" t="n">
-        <v>93.40000000000001</v>
+        <v>58.8</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2708,7 +2699,7 @@
         </is>
       </c>
       <c r="P24" t="n">
-        <v>62</v>
+        <v>60.1</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -2727,80 +2718,84 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="U24" t="inlineStr"/>
-      <c r="V24" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>XOM</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>192.42</v>
+        <v>159.44</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>36.2</v>
+        <v>49.9</v>
       </c>
       <c r="J25" t="n">
-        <v>30.7</v>
+        <v>46.6</v>
       </c>
       <c r="K25" t="n">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="L25" t="n">
-        <v>2.12</v>
+        <v>2.49</v>
       </c>
       <c r="M25" t="n">
-        <v>20.5</v>
+        <v>27.5</v>
       </c>
       <c r="N25" t="n">
-        <v>22.9</v>
+        <v>65</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P25" t="n">
-        <v>33.5</v>
+        <v>56.7</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
@@ -2814,7 +2809,7 @@
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
@@ -2822,28 +2817,32 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U25" t="inlineStr"/>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>HD</t>
+          <t>MMM</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>300.32</v>
+        <v>165</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -2865,34 +2864,34 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>34.4</v>
+        <v>45.6</v>
       </c>
       <c r="J26" t="n">
-        <v>29.9</v>
+        <v>40.8</v>
       </c>
       <c r="K26" t="n">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="L26" t="n">
-        <v>2.07</v>
+        <v>2.01</v>
       </c>
       <c r="M26" t="n">
-        <v>20.8</v>
+        <v>15.9</v>
       </c>
       <c r="N26" t="n">
-        <v>37.2</v>
+        <v>1.8</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P26" t="n">
-        <v>37.9</v>
+        <v>51.5</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
@@ -2924,18 +2923,18 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>HSY</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>168.21</v>
+        <v>192.58</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D27" s="3" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -2961,22 +2960,22 @@
         </is>
       </c>
       <c r="I27" t="n">
-        <v>32.9</v>
+        <v>37.5</v>
       </c>
       <c r="J27" t="n">
-        <v>33.4</v>
+        <v>31</v>
       </c>
       <c r="K27" t="n">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="L27" t="n">
-        <v>2.06</v>
+        <v>2.19</v>
       </c>
       <c r="M27" t="n">
-        <v>19.2</v>
+        <v>18.9</v>
       </c>
       <c r="N27" t="n">
-        <v>6.5</v>
+        <v>14.3</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -2984,7 +2983,7 @@
         </is>
       </c>
       <c r="P27" t="n">
-        <v>39.7</v>
+        <v>33.6</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
@@ -3008,6 +3007,286 @@
       </c>
       <c r="U27" t="inlineStr"/>
       <c r="V27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>XEL</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>71.87</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>37.2</v>
+      </c>
+      <c r="J28" t="n">
+        <v>32.6</v>
+      </c>
+      <c r="K28" t="n">
+        <v>93</v>
+      </c>
+      <c r="L28" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="M28" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="N28" t="n">
+        <v>37</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P28" t="n">
+        <v>37.8</v>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>299.08</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>36.3</v>
+      </c>
+      <c r="J29" t="n">
+        <v>29.1</v>
+      </c>
+      <c r="K29" t="n">
+        <v>86</v>
+      </c>
+      <c r="L29" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="M29" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="N29" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P29" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr"/>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>HSY</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>167.35</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>33.9</v>
+      </c>
+      <c r="J30" t="n">
+        <v>33.9</v>
+      </c>
+      <c r="K30" t="n">
+        <v>79</v>
+      </c>
+      <c r="L30" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="M30" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="N30" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P30" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr"/>
+      <c r="V30" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 22.09.2026 18:01 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V30"/>
+  <dimension ref="A1:V20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>744.36</v>
+        <v>740.88</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -617,19 +617,19 @@
         <v>95.2</v>
       </c>
       <c r="J2" t="n">
-        <v>78.09999999999999</v>
+        <v>77.7</v>
       </c>
       <c r="K2" t="n">
         <v>100</v>
       </c>
       <c r="L2" t="n">
-        <v>4.01</v>
+        <v>4.04</v>
       </c>
       <c r="M2" t="n">
-        <v>47.8</v>
+        <v>47.1</v>
       </c>
       <c r="N2" t="n">
-        <v>77.5</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>63.7</v>
+        <v>63.5</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>381.89</v>
+        <v>386.02</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -706,22 +706,22 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>89.5</v>
+        <v>90.8</v>
       </c>
       <c r="J3" t="n">
-        <v>58.6</v>
+        <v>60.8</v>
       </c>
       <c r="K3" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="L3" t="n">
-        <v>2.97</v>
+        <v>2.85</v>
       </c>
       <c r="M3" t="n">
-        <v>30.1</v>
+        <v>30</v>
       </c>
       <c r="N3" t="n">
-        <v>17</v>
+        <v>16.7</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -729,11 +729,11 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>54.5</v>
+        <v>55.6</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>FIRED</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -748,12 +748,12 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Squeeze Fired, Squeeze Expanding</t>
+          <t>Squeeze Expanding</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -765,11 +765,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DHR</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>214.84</v>
+        <v>773.79</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -802,22 +802,22 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>88.59999999999999</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>60.1</v>
+        <v>60</v>
       </c>
       <c r="K4" t="n">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="L4" t="n">
-        <v>2.5</v>
+        <v>0.89</v>
       </c>
       <c r="M4" t="n">
-        <v>28.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="N4" t="n">
-        <v>34.8</v>
+        <v>16.5</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -825,7 +825,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>57.8</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -847,7 +847,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr"/>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V4" t="inlineStr">
         <is>
           <t>No</t>
@@ -857,30 +861,30 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>XLK</t>
+          <t>APP</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>194.64</v>
+        <v>327.34</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -894,31 +898,34 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>86.40000000000001</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="K5" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="L5" t="n">
-        <v>1.78</v>
+        <v>5.06</v>
       </c>
       <c r="M5" t="n">
-        <v>24.7</v>
+        <v>45</v>
+      </c>
+      <c r="N5" t="n">
+        <v>4.6</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>66.59999999999999</v>
+        <v>39.4</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -928,7 +935,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -938,7 +945,7 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>Squeeze Expanding</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
@@ -950,30 +957,30 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AZN</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>168.64</v>
+        <v>336.23</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -983,56 +990,60 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>86.3</v>
+        <v>77.3</v>
       </c>
       <c r="J6" t="n">
-        <v>58.9</v>
+        <v>42.6</v>
       </c>
       <c r="K6" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="L6" t="n">
-        <v>1.97</v>
+        <v>1.42</v>
       </c>
       <c r="M6" t="n">
-        <v>22.2</v>
+        <v>15.2</v>
       </c>
       <c r="N6" t="n">
-        <v>17</v>
+        <v>8.6</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>46.4</v>
+        <v>51.5</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V6" t="inlineStr">
         <is>
           <t>No</t>
@@ -1042,81 +1053,81 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>VLO</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>375.61</v>
+        <v>385.95</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>85.90000000000001</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>58.7</v>
+        <v>58.6</v>
       </c>
       <c r="K7" t="n">
-        <v>4</v>
+        <v>79</v>
       </c>
       <c r="L7" t="n">
-        <v>3.4</v>
+        <v>4.31</v>
       </c>
       <c r="M7" t="n">
-        <v>44.4</v>
+        <v>30.8</v>
       </c>
       <c r="N7" t="n">
-        <v>36.6</v>
+        <v>29.9</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>50.3</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -1126,42 +1137,42 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>Divergence</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>41.14</v>
+        <v>105.45</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1175,22 +1186,22 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>81.90000000000001</v>
+        <v>63.2</v>
       </c>
       <c r="J8" t="n">
-        <v>59.5</v>
+        <v>39.3</v>
       </c>
       <c r="K8" t="n">
         <v>9</v>
       </c>
       <c r="L8" t="n">
-        <v>6.09</v>
+        <v>3.12</v>
       </c>
       <c r="M8" t="n">
-        <v>86.2</v>
+        <v>37.3</v>
       </c>
       <c r="N8" t="n">
-        <v>44.7</v>
+        <v>55.6</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1198,7 +1209,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>58.5</v>
+        <v>49.8</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1207,12 +1218,12 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -1222,27 +1233,27 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>BKNG</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>741.55</v>
+        <v>162.46</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -1257,100 +1268,103 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>81.90000000000001</v>
+        <v>62.1</v>
       </c>
       <c r="J9" t="n">
-        <v>65.7</v>
+        <v>24.8</v>
       </c>
       <c r="K9" t="n">
-        <v>16</v>
+        <v>99</v>
       </c>
       <c r="L9" t="n">
-        <v>1.41</v>
+        <v>4.07</v>
       </c>
       <c r="M9" t="n">
-        <v>17.8</v>
+        <v>32.9</v>
+      </c>
+      <c r="N9" t="n">
+        <v>39.3</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>63.2</v>
+        <v>39.8</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>FIRED</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>Squeeze Fired, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V9" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>221.25</v>
+        <v>231.23</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1360,60 +1374,56 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>79.59999999999999</v>
+        <v>58.5</v>
       </c>
       <c r="J10" t="n">
-        <v>57.2</v>
+        <v>45.7</v>
       </c>
       <c r="K10" t="n">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="L10" t="n">
-        <v>2.51</v>
+        <v>3.17</v>
       </c>
       <c r="M10" t="n">
-        <v>28</v>
+        <v>32.3</v>
       </c>
       <c r="N10" t="n">
-        <v>15.6</v>
+        <v>21</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>65.09999999999999</v>
+        <v>45.5</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr">
         <is>
           <t>No</t>
@@ -1423,15 +1433,15 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>WDAY</t>
+          <t>SYK</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>192.64</v>
+        <v>276.36</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -1446,41 +1456,44 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>79.3</v>
+        <v>58.2</v>
       </c>
       <c r="J11" t="n">
-        <v>52.9</v>
+        <v>33</v>
       </c>
       <c r="K11" t="n">
-        <v>5</v>
+        <v>97</v>
       </c>
       <c r="L11" t="n">
-        <v>4.1</v>
+        <v>2.97</v>
       </c>
       <c r="M11" t="n">
-        <v>54</v>
+        <v>35</v>
+      </c>
+      <c r="N11" t="n">
+        <v>62.3</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>60.3</v>
+        <v>33.7</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1494,7 +1507,7 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1512,71 +1525,71 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>AON</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>338.46</v>
+        <v>287.07</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>79</v>
+        <v>57.8</v>
       </c>
       <c r="J12" t="n">
-        <v>45.6</v>
+        <v>26.5</v>
       </c>
       <c r="K12" t="n">
-        <v>8</v>
+        <v>98</v>
       </c>
       <c r="L12" t="n">
-        <v>1.4</v>
+        <v>2.92</v>
       </c>
       <c r="M12" t="n">
-        <v>15.1</v>
+        <v>35.9</v>
       </c>
       <c r="N12" t="n">
-        <v>8.1</v>
+        <v>88.59999999999999</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>53</v>
+        <v>31.7</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -1591,14 +1604,10 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr">
         <is>
           <t>No</t>
@@ -1608,30 +1617,30 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>VLO</t>
+          <t>FICO</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>398.12</v>
+        <v>924</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1645,27 +1654,30 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>78.8</v>
+        <v>51.7</v>
       </c>
       <c r="J13" t="n">
-        <v>66.8</v>
+        <v>34.1</v>
       </c>
       <c r="K13" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="L13" t="n">
-        <v>3.78</v>
+        <v>4.67</v>
       </c>
       <c r="M13" t="n">
-        <v>53.4</v>
+        <v>64.8</v>
+      </c>
+      <c r="N13" t="n">
+        <v>65</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>76.59999999999999</v>
+        <v>37.7</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1679,52 +1691,48 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>GM</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>259.27</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1738,22 +1746,22 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>78.40000000000001</v>
+        <v>51.5</v>
       </c>
       <c r="J14" t="n">
-        <v>53.4</v>
+        <v>47.2</v>
       </c>
       <c r="K14" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="L14" t="n">
-        <v>2.17</v>
+        <v>3.26</v>
       </c>
       <c r="M14" t="n">
-        <v>26.1</v>
+        <v>30.5</v>
       </c>
       <c r="N14" t="n">
-        <v>16.2</v>
+        <v>31.8</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1761,31 +1769,31 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>54.1</v>
+        <v>54.6</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>Squeeze Expanding</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
@@ -1797,11 +1805,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>APP</t>
+          <t>XLE</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>333.01</v>
+        <v>62.02</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1834,27 +1842,27 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>76.8</v>
+        <v>50.4</v>
       </c>
       <c r="J15" t="n">
-        <v>51.3</v>
+        <v>45.3</v>
       </c>
       <c r="K15" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="L15" t="n">
-        <v>5.13</v>
+        <v>2.13</v>
       </c>
       <c r="M15" t="n">
-        <v>55.2</v>
+        <v>25.4</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>40.2</v>
+        <v>59</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1863,12 +1871,12 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -1878,27 +1886,27 @@
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>Squeeze Expanding</t>
+          <t>Divergence, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>NSC</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>184.73</v>
+        <v>314.29</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -1913,36 +1921,36 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>76.7</v>
+        <v>49.8</v>
       </c>
       <c r="J16" t="n">
-        <v>52</v>
+        <v>34.6</v>
       </c>
       <c r="K16" t="n">
-        <v>16</v>
+        <v>98</v>
       </c>
       <c r="L16" t="n">
-        <v>4.2</v>
+        <v>1.85</v>
       </c>
       <c r="M16" t="n">
-        <v>49.9</v>
+        <v>18.2</v>
       </c>
       <c r="N16" t="n">
-        <v>22.9</v>
+        <v>29.7</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1950,7 +1958,7 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>49.3</v>
+        <v>47.6</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1959,12 +1967,12 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
@@ -1972,11 +1980,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr">
         <is>
           <t>No</t>
@@ -1986,15 +1990,15 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>UNP</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>322.43</v>
+        <v>273.32</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -2009,36 +2013,36 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>76.59999999999999</v>
+        <v>46.9</v>
       </c>
       <c r="J17" t="n">
-        <v>69.40000000000001</v>
+        <v>31.4</v>
       </c>
       <c r="K17" t="n">
-        <v>35</v>
+        <v>92</v>
       </c>
       <c r="L17" t="n">
-        <v>6.22</v>
+        <v>2.11</v>
       </c>
       <c r="M17" t="n">
-        <v>78.59999999999999</v>
+        <v>19.9</v>
       </c>
       <c r="N17" t="n">
-        <v>48.9</v>
+        <v>27.4</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2046,7 +2050,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>60.3</v>
+        <v>48.8</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2055,12 +2059,12 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
@@ -2078,71 +2082,71 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>HD</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>110.82</v>
+        <v>304.62</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>76.40000000000001</v>
+        <v>39.7</v>
       </c>
       <c r="J18" t="n">
-        <v>49.4</v>
+        <v>38.1</v>
       </c>
       <c r="K18" t="n">
-        <v>2</v>
+        <v>81</v>
       </c>
       <c r="L18" t="n">
-        <v>2.42</v>
+        <v>2.12</v>
       </c>
       <c r="M18" t="n">
-        <v>34.2</v>
+        <v>21.5</v>
       </c>
       <c r="N18" t="n">
-        <v>47.8</v>
+        <v>41.1</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>55.7</v>
+        <v>40</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -2157,14 +2161,10 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U18" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr">
         <is>
           <t>No</t>
@@ -2174,15 +2174,15 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>774.38</v>
+        <v>130.84</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -2197,41 +2197,44 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>73.5</v>
+        <v>38.8</v>
       </c>
       <c r="J19" t="n">
-        <v>60.3</v>
+        <v>32.1</v>
       </c>
       <c r="K19" t="n">
-        <v>18</v>
+        <v>89</v>
       </c>
       <c r="L19" t="n">
-        <v>0.97</v>
+        <v>1.66</v>
       </c>
       <c r="M19" t="n">
-        <v>12.3</v>
+        <v>16.8</v>
+      </c>
+      <c r="N19" t="n">
+        <v>16.7</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>65.3</v>
+        <v>36.5</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2240,12 +2243,12 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
@@ -2253,11 +2256,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr">
         <is>
           <t>No</t>
@@ -2267,11 +2266,11 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TJX</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>130.93</v>
+        <v>195.6</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2304,22 +2303,22 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>65.8</v>
+        <v>33.7</v>
       </c>
       <c r="J20" t="n">
-        <v>42</v>
+        <v>39.3</v>
       </c>
       <c r="K20" t="n">
-        <v>72</v>
+        <v>56</v>
       </c>
       <c r="L20" t="n">
-        <v>2.3</v>
+        <v>2.2</v>
       </c>
       <c r="M20" t="n">
-        <v>24.4</v>
+        <v>20.2</v>
       </c>
       <c r="N20" t="n">
-        <v>61.4</v>
+        <v>21</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2327,7 +2326,7 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>36</v>
+        <v>36.1</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2351,942 +2350,6 @@
       </c>
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>SYK</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>274.28</v>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>62.8</v>
-      </c>
-      <c r="J21" t="n">
-        <v>30.9</v>
-      </c>
-      <c r="K21" t="n">
-        <v>100</v>
-      </c>
-      <c r="L21" t="n">
-        <v>3.18</v>
-      </c>
-      <c r="M21" t="n">
-        <v>35.6</v>
-      </c>
-      <c r="N21" t="n">
-        <v>64.3</v>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P21" t="n">
-        <v>32.9</v>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U21" t="inlineStr"/>
-      <c r="V21" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>IBM</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>230.46</v>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>58.4</v>
-      </c>
-      <c r="J22" t="n">
-        <v>44.9</v>
-      </c>
-      <c r="K22" t="n">
-        <v>21</v>
-      </c>
-      <c r="L22" t="n">
-        <v>3.27</v>
-      </c>
-      <c r="M22" t="n">
-        <v>32.2</v>
-      </c>
-      <c r="N22" t="n">
-        <v>20.8</v>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P22" t="n">
-        <v>45.2</v>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T22" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr"/>
-      <c r="V22" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>GM</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>84.69</v>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>SQUEEZE</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>53.3</v>
-      </c>
-      <c r="J23" t="n">
-        <v>48.5</v>
-      </c>
-      <c r="K23" t="n">
-        <v>9</v>
-      </c>
-      <c r="L23" t="n">
-        <v>3.33</v>
-      </c>
-      <c r="M23" t="n">
-        <v>31.2</v>
-      </c>
-      <c r="N23" t="n">
-        <v>34.2</v>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P23" t="n">
-        <v>55.4</v>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
-      <c r="V23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>XLE</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>62.79</v>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>SQUEEZE</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>52.7</v>
-      </c>
-      <c r="J24" t="n">
-        <v>47.3</v>
-      </c>
-      <c r="K24" t="n">
-        <v>9</v>
-      </c>
-      <c r="L24" t="n">
-        <v>2.18</v>
-      </c>
-      <c r="M24" t="n">
-        <v>23</v>
-      </c>
-      <c r="N24" t="n">
-        <v>58.8</v>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P24" t="n">
-        <v>60.1</v>
-      </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S24" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T24" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V24" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>XOM</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>159.44</v>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>SQUEEZE</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>49.9</v>
-      </c>
-      <c r="J25" t="n">
-        <v>46.6</v>
-      </c>
-      <c r="K25" t="n">
-        <v>18</v>
-      </c>
-      <c r="L25" t="n">
-        <v>2.49</v>
-      </c>
-      <c r="M25" t="n">
-        <v>27.5</v>
-      </c>
-      <c r="N25" t="n">
-        <v>65</v>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P25" t="n">
-        <v>56.7</v>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S25" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T25" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U25" t="inlineStr">
-        <is>
-          <t>Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V25" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>MMM</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>165</v>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>45.6</v>
-      </c>
-      <c r="J26" t="n">
-        <v>40.8</v>
-      </c>
-      <c r="K26" t="n">
-        <v>79</v>
-      </c>
-      <c r="L26" t="n">
-        <v>2.01</v>
-      </c>
-      <c r="M26" t="n">
-        <v>15.9</v>
-      </c>
-      <c r="N26" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P26" t="n">
-        <v>51.5</v>
-      </c>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R26" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S26" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T26" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U26" t="inlineStr"/>
-      <c r="V26" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>192.58</v>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="J27" t="n">
-        <v>31</v>
-      </c>
-      <c r="K27" t="n">
-        <v>81</v>
-      </c>
-      <c r="L27" t="n">
-        <v>2.19</v>
-      </c>
-      <c r="M27" t="n">
-        <v>18.9</v>
-      </c>
-      <c r="N27" t="n">
-        <v>14.3</v>
-      </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P27" t="n">
-        <v>33.6</v>
-      </c>
-      <c r="Q27" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R27" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S27" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T27" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U27" t="inlineStr"/>
-      <c r="V27" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>XEL</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>71.87</v>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>37.2</v>
-      </c>
-      <c r="J28" t="n">
-        <v>32.6</v>
-      </c>
-      <c r="K28" t="n">
-        <v>93</v>
-      </c>
-      <c r="L28" t="n">
-        <v>1.74</v>
-      </c>
-      <c r="M28" t="n">
-        <v>17.5</v>
-      </c>
-      <c r="N28" t="n">
-        <v>37</v>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P28" t="n">
-        <v>37.8</v>
-      </c>
-      <c r="Q28" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S28" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T28" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U28" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
-      <c r="V28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>HD</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>299.08</v>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>36.3</v>
-      </c>
-      <c r="J29" t="n">
-        <v>29.1</v>
-      </c>
-      <c r="K29" t="n">
-        <v>86</v>
-      </c>
-      <c r="L29" t="n">
-        <v>2.08</v>
-      </c>
-      <c r="M29" t="n">
-        <v>19.7</v>
-      </c>
-      <c r="N29" t="n">
-        <v>31.1</v>
-      </c>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P29" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="Q29" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R29" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S29" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T29" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U29" t="inlineStr"/>
-      <c r="V29" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>HSY</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>167.35</v>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I30" t="n">
-        <v>33.9</v>
-      </c>
-      <c r="J30" t="n">
-        <v>33.9</v>
-      </c>
-      <c r="K30" t="n">
-        <v>79</v>
-      </c>
-      <c r="L30" t="n">
-        <v>2.16</v>
-      </c>
-      <c r="M30" t="n">
-        <v>19.8</v>
-      </c>
-      <c r="N30" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="O30" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P30" t="n">
-        <v>39.2</v>
-      </c>
-      <c r="Q30" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R30" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S30" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U30" t="inlineStr"/>
-      <c r="V30" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 23.09.2026 18:21 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V20"/>
+  <dimension ref="A1:V18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>740.88</v>
+        <v>749</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,22 +614,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>95.2</v>
+        <v>94</v>
       </c>
       <c r="J2" t="n">
-        <v>77.7</v>
+        <v>78.7</v>
       </c>
       <c r="K2" t="n">
         <v>100</v>
       </c>
       <c r="L2" t="n">
-        <v>4.04</v>
+        <v>3.94</v>
       </c>
       <c r="M2" t="n">
         <v>47.1</v>
       </c>
       <c r="N2" t="n">
-        <v>75.59999999999999</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>63.5</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>386.02</v>
+        <v>383.51</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -706,22 +706,22 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>90.8</v>
+        <v>87.5</v>
       </c>
       <c r="J3" t="n">
-        <v>60.8</v>
+        <v>59.5</v>
       </c>
       <c r="K3" t="n">
         <v>14</v>
       </c>
       <c r="L3" t="n">
-        <v>2.85</v>
+        <v>2.99</v>
       </c>
       <c r="M3" t="n">
-        <v>30</v>
+        <v>29.9</v>
       </c>
       <c r="N3" t="n">
-        <v>16.7</v>
+        <v>16.4</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -729,7 +729,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>55.6</v>
+        <v>54.9</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -765,11 +765,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>MET</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>773.79</v>
+        <v>97.36</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -802,22 +802,22 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>80.40000000000001</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>60</v>
+        <v>54.2</v>
       </c>
       <c r="K4" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="L4" t="n">
-        <v>0.89</v>
+        <v>1.87</v>
       </c>
       <c r="M4" t="n">
-        <v>9.699999999999999</v>
+        <v>18.6</v>
       </c>
       <c r="N4" t="n">
-        <v>16.5</v>
+        <v>16.8</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -825,11 +825,11 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>65.09999999999999</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -844,12 +844,12 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>Squeeze Expanding</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -861,11 +861,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>APP</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>327.34</v>
+        <v>335.81</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -898,30 +898,30 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>78.90000000000001</v>
+        <v>76.5</v>
       </c>
       <c r="J5" t="n">
-        <v>49</v>
+        <v>42.1</v>
       </c>
       <c r="K5" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L5" t="n">
-        <v>5.06</v>
+        <v>1.46</v>
       </c>
       <c r="M5" t="n">
-        <v>45</v>
+        <v>15.2</v>
       </c>
       <c r="N5" t="n">
-        <v>4.6</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>39.4</v>
+        <v>51.2</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -930,57 +930,57 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>TTM Squeeze</t>
+          <t>TTM Squeeze, Divergence</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>336.23</v>
+        <v>768.5</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -994,22 +994,22 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>77.3</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>42.6</v>
+        <v>55.2</v>
       </c>
       <c r="K6" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="L6" t="n">
-        <v>1.42</v>
+        <v>0.97</v>
       </c>
       <c r="M6" t="n">
-        <v>15.2</v>
+        <v>9.9</v>
       </c>
       <c r="N6" t="n">
-        <v>8.6</v>
+        <v>18.4</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1017,31 +1017,31 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>51.5</v>
+        <v>63.6</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>TTM Squeeze</t>
+          <t>Squeeze Expanding</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
@@ -1053,15 +1053,15 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>VLO</t>
+          <t>APP</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>385.95</v>
+        <v>314.03</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -1076,68 +1076,68 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>68.90000000000001</v>
+        <v>71.3</v>
       </c>
       <c r="J7" t="n">
-        <v>58.6</v>
+        <v>44.2</v>
       </c>
       <c r="K7" t="n">
-        <v>79</v>
+        <v>7</v>
       </c>
       <c r="L7" t="n">
-        <v>4.31</v>
+        <v>5.93</v>
       </c>
       <c r="M7" t="n">
-        <v>30.8</v>
+        <v>47.1</v>
       </c>
       <c r="N7" t="n">
-        <v>29.9</v>
+        <v>7.1</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>72.09999999999999</v>
+        <v>37.4</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>TTM Squeeze, Divergence</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
@@ -1153,7 +1153,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>105.45</v>
+        <v>106.46</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1186,22 +1186,22 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>63.2</v>
+        <v>66.2</v>
       </c>
       <c r="J8" t="n">
-        <v>39.3</v>
+        <v>40.8</v>
       </c>
       <c r="K8" t="n">
         <v>9</v>
       </c>
       <c r="L8" t="n">
-        <v>3.12</v>
+        <v>2.92</v>
       </c>
       <c r="M8" t="n">
-        <v>37.3</v>
+        <v>36.3</v>
       </c>
       <c r="N8" t="n">
-        <v>55.6</v>
+        <v>53.2</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1209,7 +1209,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>49.8</v>
+        <v>50.9</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1245,30 +1245,30 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BKNG</t>
+          <t>VLO</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>162.46</v>
+        <v>372.7</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1278,34 +1278,34 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>62.1</v>
+        <v>63.7</v>
       </c>
       <c r="J9" t="n">
-        <v>24.8</v>
+        <v>51.5</v>
       </c>
       <c r="K9" t="n">
-        <v>99</v>
+        <v>79</v>
       </c>
       <c r="L9" t="n">
-        <v>4.07</v>
+        <v>4.72</v>
       </c>
       <c r="M9" t="n">
-        <v>32.9</v>
+        <v>34.5</v>
       </c>
       <c r="N9" t="n">
-        <v>39.3</v>
+        <v>46</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>39.8</v>
+        <v>67.8</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1319,12 +1319,12 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1345,7 +1345,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>231.23</v>
+        <v>235.04</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1374,26 +1374,26 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>58.5</v>
+        <v>60.8</v>
       </c>
       <c r="J10" t="n">
-        <v>45.7</v>
+        <v>49</v>
       </c>
       <c r="K10" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="L10" t="n">
-        <v>3.17</v>
+        <v>3.11</v>
       </c>
       <c r="M10" t="n">
-        <v>32.3</v>
+        <v>32.6</v>
       </c>
       <c r="N10" t="n">
-        <v>21</v>
+        <v>21.3</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1401,7 +1401,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>45.5</v>
+        <v>46.7</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>276.36</v>
+        <v>272.28</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1470,22 +1470,22 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>58.2</v>
+        <v>58.6</v>
       </c>
       <c r="J11" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="K11" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L11" t="n">
-        <v>2.97</v>
+        <v>3.05</v>
       </c>
       <c r="M11" t="n">
-        <v>35</v>
+        <v>34.7</v>
       </c>
       <c r="N11" t="n">
-        <v>62.3</v>
+        <v>61.4</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1493,7 +1493,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>33.7</v>
+        <v>32.5</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1525,11 +1525,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AON</t>
+          <t>NSC</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>287.07</v>
+        <v>316.4</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1562,30 +1562,30 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>57.8</v>
+        <v>55.6</v>
       </c>
       <c r="J12" t="n">
-        <v>26.5</v>
+        <v>37.6</v>
       </c>
       <c r="K12" t="n">
         <v>98</v>
       </c>
       <c r="L12" t="n">
-        <v>2.92</v>
+        <v>1.94</v>
       </c>
       <c r="M12" t="n">
-        <v>35.9</v>
+        <v>18.9</v>
       </c>
       <c r="N12" t="n">
-        <v>88.59999999999999</v>
+        <v>33.1</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>31.7</v>
+        <v>48.7</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1617,67 +1617,64 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>FICO</t>
+          <t>XLE</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>924</v>
+        <v>62.4</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>51.7</v>
+        <v>53.4</v>
       </c>
       <c r="J13" t="n">
-        <v>34.1</v>
+        <v>47.1</v>
       </c>
       <c r="K13" t="n">
-        <v>89</v>
+        <v>10</v>
       </c>
       <c r="L13" t="n">
-        <v>4.67</v>
+        <v>2.05</v>
       </c>
       <c r="M13" t="n">
-        <v>64.8</v>
-      </c>
-      <c r="N13" t="n">
-        <v>65</v>
+        <v>26.3</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>37.7</v>
+        <v>60</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1691,7 +1688,7 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -1699,7 +1696,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr"/>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V13" t="inlineStr">
         <is>
           <t>No</t>
@@ -1713,7 +1714,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>84.09999999999999</v>
+        <v>84.25</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1746,22 +1747,22 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>51.5</v>
+        <v>53.3</v>
       </c>
       <c r="J14" t="n">
-        <v>47.2</v>
+        <v>47.5</v>
       </c>
       <c r="K14" t="n">
         <v>14</v>
       </c>
       <c r="L14" t="n">
-        <v>3.26</v>
+        <v>3.19</v>
       </c>
       <c r="M14" t="n">
         <v>30.5</v>
       </c>
       <c r="N14" t="n">
-        <v>31.8</v>
+        <v>31.9</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1769,7 +1770,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>54.6</v>
+        <v>54.7</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1805,56 +1806,59 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>XLE</t>
+          <t>UNP</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>62.02</v>
+        <v>276.13</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>50.4</v>
+        <v>52.7</v>
       </c>
       <c r="J15" t="n">
-        <v>45.3</v>
+        <v>35.9</v>
       </c>
       <c r="K15" t="n">
-        <v>10</v>
+        <v>91</v>
       </c>
       <c r="L15" t="n">
-        <v>2.13</v>
+        <v>2.25</v>
       </c>
       <c r="M15" t="n">
-        <v>25.4</v>
+        <v>20.8</v>
+      </c>
+      <c r="N15" t="n">
+        <v>31.9</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1862,7 +1866,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>59</v>
+        <v>50.2</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1876,7 +1880,7 @@
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -1884,25 +1888,21 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>NSC</t>
+          <t>DLTR</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>314.29</v>
+        <v>113.29</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1935,30 +1935,30 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>49.8</v>
+        <v>40.3</v>
       </c>
       <c r="J16" t="n">
-        <v>34.6</v>
+        <v>35.1</v>
       </c>
       <c r="K16" t="n">
-        <v>98</v>
+        <v>85</v>
       </c>
       <c r="L16" t="n">
-        <v>1.85</v>
+        <v>3.6</v>
       </c>
       <c r="M16" t="n">
-        <v>18.2</v>
+        <v>37</v>
       </c>
       <c r="N16" t="n">
-        <v>29.7</v>
+        <v>24.1</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>47.6</v>
+        <v>46.2</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1990,11 +1990,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>UNP</t>
+          <t>HD</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>273.32</v>
+        <v>299.99</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -2027,30 +2027,27 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>46.9</v>
+        <v>37.3</v>
       </c>
       <c r="J17" t="n">
-        <v>31.4</v>
+        <v>32.2</v>
       </c>
       <c r="K17" t="n">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="L17" t="n">
         <v>2.11</v>
       </c>
       <c r="M17" t="n">
-        <v>19.9</v>
-      </c>
-      <c r="N17" t="n">
-        <v>27.4</v>
+        <v>25.5</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>48.8</v>
+        <v>37.8</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2082,11 +2079,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>HD</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>304.62</v>
+        <v>193.4</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2115,26 +2112,26 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>39.7</v>
+        <v>33.7</v>
       </c>
       <c r="J18" t="n">
-        <v>38.1</v>
+        <v>34.9</v>
       </c>
       <c r="K18" t="n">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="L18" t="n">
-        <v>2.12</v>
+        <v>2.2</v>
       </c>
       <c r="M18" t="n">
-        <v>21.5</v>
+        <v>19</v>
       </c>
       <c r="N18" t="n">
-        <v>41.1</v>
+        <v>13</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -2142,7 +2139,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>40</v>
+        <v>34.3</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2166,190 +2163,6 @@
       </c>
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>PEP</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>130.84</v>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>38.8</v>
-      </c>
-      <c r="J19" t="n">
-        <v>32.1</v>
-      </c>
-      <c r="K19" t="n">
-        <v>89</v>
-      </c>
-      <c r="L19" t="n">
-        <v>1.66</v>
-      </c>
-      <c r="M19" t="n">
-        <v>16.8</v>
-      </c>
-      <c r="N19" t="n">
-        <v>16.7</v>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P19" t="n">
-        <v>36.5</v>
-      </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T19" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U19" t="inlineStr"/>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>195.6</v>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>33.7</v>
-      </c>
-      <c r="J20" t="n">
-        <v>39.3</v>
-      </c>
-      <c r="K20" t="n">
-        <v>56</v>
-      </c>
-      <c r="L20" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="M20" t="n">
-        <v>20.2</v>
-      </c>
-      <c r="N20" t="n">
-        <v>21</v>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P20" t="n">
-        <v>36.1</v>
-      </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S20" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T20" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U20" t="inlineStr"/>
-      <c r="V20" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 24.09.2026 18:21 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V18"/>
+  <dimension ref="A1:V12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -448,7 +448,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
     <col width="6" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>749</v>
+        <v>261.9</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,22 +614,19 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>94</v>
+        <v>77.7</v>
       </c>
       <c r="J2" t="n">
-        <v>78.7</v>
+        <v>68.3</v>
       </c>
       <c r="K2" t="n">
-        <v>100</v>
+        <v>81</v>
       </c>
       <c r="L2" t="n">
-        <v>3.94</v>
+        <v>5.04</v>
       </c>
       <c r="M2" t="n">
-        <v>47.1</v>
-      </c>
-      <c r="N2" t="n">
-        <v>75.40000000000001</v>
+        <v>53.3</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,7 +634,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>64.09999999999999</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -669,30 +666,30 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>383.51</v>
+        <v>335.93</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -706,22 +703,22 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>87.5</v>
+        <v>73.5</v>
       </c>
       <c r="J3" t="n">
-        <v>59.5</v>
+        <v>42.7</v>
       </c>
       <c r="K3" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="L3" t="n">
-        <v>2.99</v>
+        <v>1.43</v>
       </c>
       <c r="M3" t="n">
-        <v>29.9</v>
+        <v>15.2</v>
       </c>
       <c r="N3" t="n">
-        <v>16.4</v>
+        <v>9</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -729,31 +726,31 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>54.9</v>
+        <v>51.3</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Squeeze Expanding</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -765,30 +762,30 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MET</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>97.36</v>
+        <v>105.99</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -802,22 +799,22 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>80.59999999999999</v>
+        <v>63.5</v>
       </c>
       <c r="J4" t="n">
-        <v>54.2</v>
+        <v>40</v>
       </c>
       <c r="K4" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="L4" t="n">
-        <v>1.87</v>
+        <v>2.63</v>
       </c>
       <c r="M4" t="n">
-        <v>18.6</v>
+        <v>34.8</v>
       </c>
       <c r="N4" t="n">
-        <v>16.8</v>
+        <v>49.4</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -825,7 +822,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>68.40000000000001</v>
+        <v>50.4</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -834,12 +831,12 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -861,71 +858,71 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>BKNG</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>335.81</v>
+        <v>156.81</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>76.5</v>
+        <v>61.6</v>
       </c>
       <c r="J5" t="n">
-        <v>42.1</v>
+        <v>23</v>
       </c>
       <c r="K5" t="n">
-        <v>4</v>
+        <v>96</v>
       </c>
       <c r="L5" t="n">
-        <v>1.46</v>
+        <v>4.16</v>
       </c>
       <c r="M5" t="n">
-        <v>15.2</v>
+        <v>34.7</v>
       </c>
       <c r="N5" t="n">
-        <v>8.699999999999999</v>
+        <v>44</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>51.2</v>
+        <v>37.9</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -940,76 +937,72 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>VLO</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>768.5</v>
+        <v>390.29</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>73.90000000000001</v>
+        <v>57.7</v>
       </c>
       <c r="J6" t="n">
-        <v>55.2</v>
+        <v>59</v>
       </c>
       <c r="K6" t="n">
-        <v>19</v>
+        <v>69</v>
       </c>
       <c r="L6" t="n">
-        <v>0.97</v>
+        <v>4.58</v>
       </c>
       <c r="M6" t="n">
-        <v>9.9</v>
+        <v>34.1</v>
       </c>
       <c r="N6" t="n">
-        <v>18.4</v>
+        <v>44.2</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1017,7 +1010,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>63.6</v>
+        <v>73.7</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1026,24 +1019,20 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr">
         <is>
           <t>No</t>
@@ -1053,59 +1042,56 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>APP</t>
+          <t>SYK</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>314.03</v>
+        <v>271.23</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>71.3</v>
+        <v>55.5</v>
       </c>
       <c r="J7" t="n">
-        <v>44.2</v>
+        <v>29.5</v>
       </c>
       <c r="K7" t="n">
-        <v>7</v>
+        <v>94</v>
       </c>
       <c r="L7" t="n">
-        <v>5.93</v>
+        <v>2.95</v>
       </c>
       <c r="M7" t="n">
-        <v>47.1</v>
-      </c>
-      <c r="N7" t="n">
-        <v>7.1</v>
+        <v>34</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1113,21 +1099,21 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>37.4</v>
+        <v>32.2</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -1135,73 +1121,69 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence</t>
-        </is>
-      </c>
+      <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>NSC</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>106.46</v>
+        <v>313.45</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>66.2</v>
+        <v>50.2</v>
       </c>
       <c r="J8" t="n">
-        <v>40.8</v>
+        <v>34.4</v>
       </c>
       <c r="K8" t="n">
-        <v>9</v>
+        <v>95</v>
       </c>
       <c r="L8" t="n">
-        <v>2.92</v>
+        <v>1.84</v>
       </c>
       <c r="M8" t="n">
-        <v>36.3</v>
+        <v>18.4</v>
       </c>
       <c r="N8" t="n">
-        <v>53.2</v>
+        <v>29.9</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1209,11 +1191,11 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>50.9</v>
+        <v>47.2</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -1228,47 +1210,43 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>VLO</t>
+          <t>UNP</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>372.7</v>
+        <v>273.02</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1278,26 +1256,26 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>63.7</v>
+        <v>49.7</v>
       </c>
       <c r="J9" t="n">
-        <v>51.5</v>
+        <v>32.9</v>
       </c>
       <c r="K9" t="n">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="L9" t="n">
-        <v>4.72</v>
+        <v>2.14</v>
       </c>
       <c r="M9" t="n">
-        <v>34.5</v>
+        <v>20.7</v>
       </c>
       <c r="N9" t="n">
-        <v>46</v>
+        <v>31.1</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1305,7 +1283,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>67.8</v>
+        <v>48.6</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1319,89 +1297,85 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>DLTR</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>235.04</v>
+        <v>114.86</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>60.8</v>
+        <v>40.7</v>
       </c>
       <c r="J10" t="n">
-        <v>49</v>
+        <v>38.6</v>
       </c>
       <c r="K10" t="n">
-        <v>19</v>
+        <v>82</v>
       </c>
       <c r="L10" t="n">
-        <v>3.11</v>
+        <v>3.42</v>
       </c>
       <c r="M10" t="n">
-        <v>32.6</v>
+        <v>37.3</v>
       </c>
       <c r="N10" t="n">
-        <v>21.3</v>
+        <v>25</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>46.7</v>
+        <v>47.4</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1433,11 +1407,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SYK</t>
+          <t>HD</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>272.28</v>
+        <v>292.76</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1470,22 +1444,22 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>58.6</v>
+        <v>36</v>
       </c>
       <c r="J11" t="n">
-        <v>30</v>
+        <v>25.4</v>
       </c>
       <c r="K11" t="n">
-        <v>98</v>
+        <v>83</v>
       </c>
       <c r="L11" t="n">
-        <v>3.05</v>
+        <v>2.26</v>
       </c>
       <c r="M11" t="n">
-        <v>34.7</v>
+        <v>19.2</v>
       </c>
       <c r="N11" t="n">
-        <v>61.4</v>
+        <v>19.8</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1493,7 +1467,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>32.5</v>
+        <v>35.8</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1515,21 +1489,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr"/>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>NSC</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>316.4</v>
+        <v>188.57</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1558,34 +1536,34 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>55.6</v>
+        <v>29.4</v>
       </c>
       <c r="J12" t="n">
-        <v>37.6</v>
+        <v>27.3</v>
       </c>
       <c r="K12" t="n">
-        <v>98</v>
+        <v>53</v>
       </c>
       <c r="L12" t="n">
-        <v>1.94</v>
+        <v>2.32</v>
       </c>
       <c r="M12" t="n">
-        <v>18.9</v>
+        <v>18.1</v>
       </c>
       <c r="N12" t="n">
-        <v>33.1</v>
+        <v>7.2</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>48.7</v>
+        <v>31.9</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1607,564 +1585,14 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr"/>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>XLE</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>62.4</v>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>SQUEEZE</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>53.4</v>
-      </c>
-      <c r="J13" t="n">
-        <v>47.1</v>
-      </c>
-      <c r="K13" t="n">
-        <v>10</v>
-      </c>
-      <c r="L13" t="n">
-        <v>2.05</v>
-      </c>
-      <c r="M13" t="n">
-        <v>26.3</v>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P13" t="n">
-        <v>60</v>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T13" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V13" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>GM</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>84.25</v>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>SQUEEZE</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>53.3</v>
-      </c>
-      <c r="J14" t="n">
-        <v>47.5</v>
-      </c>
-      <c r="K14" t="n">
-        <v>14</v>
-      </c>
-      <c r="L14" t="n">
-        <v>3.19</v>
-      </c>
-      <c r="M14" t="n">
-        <v>30.5</v>
-      </c>
-      <c r="N14" t="n">
-        <v>31.9</v>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P14" t="n">
-        <v>54.7</v>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S14" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T14" t="inlineStr">
-        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V14" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>UNP</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>276.13</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>52.7</v>
-      </c>
-      <c r="J15" t="n">
-        <v>35.9</v>
-      </c>
-      <c r="K15" t="n">
-        <v>91</v>
-      </c>
-      <c r="L15" t="n">
-        <v>2.25</v>
-      </c>
-      <c r="M15" t="n">
-        <v>20.8</v>
-      </c>
-      <c r="N15" t="n">
-        <v>31.9</v>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P15" t="n">
-        <v>50.2</v>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U15" t="inlineStr"/>
-      <c r="V15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>DLTR</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>113.29</v>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>40.3</v>
-      </c>
-      <c r="J16" t="n">
-        <v>35.1</v>
-      </c>
-      <c r="K16" t="n">
-        <v>85</v>
-      </c>
-      <c r="L16" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="M16" t="n">
-        <v>37</v>
-      </c>
-      <c r="N16" t="n">
-        <v>24.1</v>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="P16" t="n">
-        <v>46.2</v>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T16" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr"/>
-      <c r="V16" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>HD</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>299.99</v>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>37.3</v>
-      </c>
-      <c r="J17" t="n">
-        <v>32.2</v>
-      </c>
-      <c r="K17" t="n">
-        <v>83</v>
-      </c>
-      <c r="L17" t="n">
-        <v>2.11</v>
-      </c>
-      <c r="M17" t="n">
-        <v>25.5</v>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P17" t="n">
-        <v>37.8</v>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T17" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>193.4</v>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>33.7</v>
-      </c>
-      <c r="J18" t="n">
-        <v>34.9</v>
-      </c>
-      <c r="K18" t="n">
-        <v>63</v>
-      </c>
-      <c r="L18" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="M18" t="n">
-        <v>19</v>
-      </c>
-      <c r="N18" t="n">
-        <v>13</v>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P18" t="n">
-        <v>34.3</v>
-      </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S18" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T18" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan 25.09.2026 18:25 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V12"/>
+  <dimension ref="A1:V16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>261.9</v>
+        <v>751.54</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,19 +614,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>77.7</v>
+        <v>92</v>
       </c>
       <c r="J2" t="n">
-        <v>68.3</v>
+        <v>71.3</v>
       </c>
       <c r="K2" t="n">
-        <v>81</v>
+        <v>99</v>
       </c>
       <c r="L2" t="n">
-        <v>5.04</v>
+        <v>4.07</v>
       </c>
       <c r="M2" t="n">
-        <v>53.3</v>
+        <v>48.1</v>
+      </c>
+      <c r="N2" t="n">
+        <v>78.3</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -634,7 +637,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>72.09999999999999</v>
+        <v>64.3</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -656,25 +659,29 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr"/>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>335.93</v>
+        <v>325.85</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -689,70 +696,66 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>73.5</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>42.7</v>
+        <v>61.2</v>
       </c>
       <c r="K3" t="n">
-        <v>8</v>
+        <v>89</v>
       </c>
       <c r="L3" t="n">
-        <v>1.43</v>
+        <v>3.27</v>
       </c>
       <c r="M3" t="n">
-        <v>15.2</v>
+        <v>43.1</v>
       </c>
       <c r="N3" t="n">
-        <v>9</v>
+        <v>62.7</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>51.3</v>
+        <v>49.4</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr">
         <is>
           <t>No</t>
@@ -762,30 +765,30 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>JNJ</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>105.99</v>
+        <v>270.61</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -799,22 +802,22 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>63.5</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>40</v>
+        <v>56.1</v>
       </c>
       <c r="K4" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="L4" t="n">
-        <v>2.63</v>
+        <v>1.83</v>
       </c>
       <c r="M4" t="n">
-        <v>34.8</v>
+        <v>18.9</v>
       </c>
       <c r="N4" t="n">
-        <v>49.4</v>
+        <v>34.3</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -822,11 +825,11 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>50.4</v>
+        <v>63.4</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>FIRED</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -836,17 +839,17 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>Squeeze Fired</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -858,15 +861,15 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BKNG</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>156.81</v>
+        <v>518.5700000000001</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -881,66 +884,70 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>61.6</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>23</v>
+        <v>64.2</v>
       </c>
       <c r="K5" t="n">
-        <v>96</v>
+        <v>7</v>
       </c>
       <c r="L5" t="n">
-        <v>4.16</v>
+        <v>2.38</v>
       </c>
       <c r="M5" t="n">
-        <v>34.7</v>
+        <v>24.1</v>
       </c>
       <c r="N5" t="n">
-        <v>44</v>
+        <v>17.4</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>37.9</v>
+        <v>65</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V5" t="inlineStr">
         <is>
           <t>No</t>
@@ -950,30 +957,30 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>VLO</t>
+          <t>BKNG</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>390.29</v>
+        <v>162.31</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -983,34 +990,34 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>57.7</v>
+        <v>63.4</v>
       </c>
       <c r="J6" t="n">
-        <v>59</v>
+        <v>31.6</v>
       </c>
       <c r="K6" t="n">
-        <v>69</v>
+        <v>94</v>
       </c>
       <c r="L6" t="n">
-        <v>4.58</v>
+        <v>4.03</v>
       </c>
       <c r="M6" t="n">
-        <v>34.1</v>
+        <v>36.6</v>
       </c>
       <c r="N6" t="n">
-        <v>44.2</v>
+        <v>49.1</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>73.7</v>
+        <v>39.8</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1024,12 +1031,12 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
@@ -1042,11 +1049,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SYK</t>
+          <t>AON</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>271.23</v>
+        <v>278.79</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1079,19 +1086,22 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>55.5</v>
+        <v>53</v>
       </c>
       <c r="J7" t="n">
-        <v>29.5</v>
+        <v>25.7</v>
       </c>
       <c r="K7" t="n">
         <v>94</v>
       </c>
       <c r="L7" t="n">
-        <v>2.95</v>
+        <v>2.71</v>
       </c>
       <c r="M7" t="n">
-        <v>34</v>
+        <v>35.9</v>
+      </c>
+      <c r="N7" t="n">
+        <v>89</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1099,7 +1109,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>32.2</v>
+        <v>29.9</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1131,11 +1141,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>NSC</t>
+          <t>SYK</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>313.45</v>
+        <v>273.02</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1168,30 +1178,30 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>50.2</v>
+        <v>48.2</v>
       </c>
       <c r="J8" t="n">
-        <v>34.4</v>
+        <v>32.8</v>
       </c>
       <c r="K8" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="L8" t="n">
-        <v>1.84</v>
+        <v>2.76</v>
       </c>
       <c r="M8" t="n">
-        <v>18.4</v>
+        <v>35</v>
       </c>
       <c r="N8" t="n">
-        <v>29.9</v>
+        <v>62.2</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>47.2</v>
+        <v>32.6</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1223,11 +1233,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>UNP</t>
+          <t>FICO</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>273.02</v>
+        <v>862.01</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1260,30 +1270,30 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>49.7</v>
+        <v>47.2</v>
       </c>
       <c r="J9" t="n">
-        <v>32.9</v>
+        <v>29.4</v>
       </c>
       <c r="K9" t="n">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="L9" t="n">
-        <v>2.14</v>
+        <v>4.55</v>
       </c>
       <c r="M9" t="n">
-        <v>20.7</v>
+        <v>62.6</v>
       </c>
       <c r="N9" t="n">
-        <v>31.1</v>
+        <v>61.1</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>48.6</v>
+        <v>35.5</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1315,11 +1325,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>DLTR</t>
+          <t>DASH</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>114.86</v>
+        <v>191.82</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1352,30 +1362,30 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>40.7</v>
+        <v>46.5</v>
       </c>
       <c r="J10" t="n">
-        <v>38.6</v>
+        <v>37.8</v>
       </c>
       <c r="K10" t="n">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="L10" t="n">
-        <v>3.42</v>
+        <v>3.71</v>
       </c>
       <c r="M10" t="n">
-        <v>37.3</v>
+        <v>32.1</v>
       </c>
       <c r="N10" t="n">
-        <v>25</v>
+        <v>15.5</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>47.4</v>
+        <v>49.2</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1407,11 +1417,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>HD</t>
+          <t>AXP</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>292.76</v>
+        <v>309.51</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1444,22 +1454,22 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>36</v>
+        <v>45.7</v>
       </c>
       <c r="J11" t="n">
-        <v>25.4</v>
+        <v>37.6</v>
       </c>
       <c r="K11" t="n">
         <v>83</v>
       </c>
       <c r="L11" t="n">
-        <v>2.26</v>
+        <v>2.02</v>
       </c>
       <c r="M11" t="n">
-        <v>19.2</v>
+        <v>20.8</v>
       </c>
       <c r="N11" t="n">
-        <v>19.8</v>
+        <v>17.5</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1467,7 +1477,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>35.8</v>
+        <v>40.4</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1476,38 +1486,34 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>SBUX</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>188.57</v>
+        <v>94.31999999999999</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1536,63 +1542,427 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>43.6</v>
+      </c>
+      <c r="J12" t="n">
+        <v>29.1</v>
+      </c>
+      <c r="K12" t="n">
+        <v>98</v>
+      </c>
+      <c r="L12" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="M12" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="N12" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P12" t="n">
+        <v>41.7</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>NSC</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>313.2</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>42.3</v>
+      </c>
+      <c r="J13" t="n">
+        <v>34.2</v>
+      </c>
+      <c r="K13" t="n">
+        <v>86</v>
+      </c>
+      <c r="L13" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="M13" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="N13" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ADSK</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>211.62</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
           <t>NEUTRAL</t>
         </is>
       </c>
-      <c r="I12" t="n">
-        <v>29.4</v>
-      </c>
-      <c r="J12" t="n">
-        <v>27.3</v>
-      </c>
-      <c r="K12" t="n">
-        <v>53</v>
-      </c>
-      <c r="L12" t="n">
-        <v>2.32</v>
-      </c>
-      <c r="M12" t="n">
-        <v>18.1</v>
-      </c>
-      <c r="N12" t="n">
-        <v>7.2</v>
-      </c>
-      <c r="O12" t="inlineStr">
+      <c r="I14" t="n">
+        <v>41.9</v>
+      </c>
+      <c r="J14" t="n">
+        <v>38.1</v>
+      </c>
+      <c r="K14" t="n">
+        <v>74</v>
+      </c>
+      <c r="L14" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="M14" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="N14" t="n">
+        <v>86.5</v>
+      </c>
+      <c r="O14" t="inlineStr">
         <is>
           <t>Bearish</t>
         </is>
       </c>
-      <c r="P12" t="n">
-        <v>31.9</v>
-      </c>
-      <c r="Q12" t="inlineStr">
+      <c r="P14" t="n">
+        <v>42.2</v>
+      </c>
+      <c r="Q14" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr">
+      <c r="R14" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr">
+      <c r="S14" t="inlineStr">
         <is>
           <t>red</t>
         </is>
       </c>
-      <c r="T12" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
-      <c r="V12" t="inlineStr">
-        <is>
-          <t>Yes</t>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>DLTR</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>114.08</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>41.1</v>
+      </c>
+      <c r="J15" t="n">
+        <v>38.4</v>
+      </c>
+      <c r="K15" t="n">
+        <v>81</v>
+      </c>
+      <c r="L15" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="M15" t="n">
+        <v>37.8</v>
+      </c>
+      <c r="N15" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="P15" t="n">
+        <v>46.8</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>UNP</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>273.11</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="J16" t="n">
+        <v>32.9</v>
+      </c>
+      <c r="K16" t="n">
+        <v>74</v>
+      </c>
+      <c r="L16" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="M16" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="N16" t="n">
+        <v>26.1</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P16" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan 28.09.2026 20:28 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V16"/>
+  <dimension ref="A1:V23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>751.54</v>
+        <v>715.62</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,22 +614,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>92</v>
+        <v>87.5</v>
       </c>
       <c r="J2" t="n">
-        <v>71.3</v>
+        <v>61</v>
       </c>
       <c r="K2" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="L2" t="n">
-        <v>4.07</v>
+        <v>4.42</v>
       </c>
       <c r="M2" t="n">
-        <v>48.1</v>
+        <v>50.6</v>
       </c>
       <c r="N2" t="n">
-        <v>78.3</v>
+        <v>85.3</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>64.3</v>
+        <v>59.5</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -646,17 +646,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -673,67 +673,67 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>JNJ</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>325.85</v>
+        <v>271.95</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>76.59999999999999</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>61.2</v>
+        <v>58.5</v>
       </c>
       <c r="K3" t="n">
-        <v>89</v>
+        <v>2</v>
       </c>
       <c r="L3" t="n">
-        <v>3.27</v>
+        <v>1.8</v>
       </c>
       <c r="M3" t="n">
-        <v>43.1</v>
+        <v>18.8</v>
       </c>
       <c r="N3" t="n">
-        <v>62.7</v>
+        <v>33.5</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>49.4</v>
+        <v>64</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -747,7 +747,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -755,7 +755,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr"/>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V3" t="inlineStr">
         <is>
           <t>No</t>
@@ -765,81 +769,81 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>JNJ</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>270.61</v>
+        <v>326.7</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>76.09999999999999</v>
+        <v>75.5</v>
       </c>
       <c r="J4" t="n">
-        <v>56.1</v>
+        <v>61.5</v>
       </c>
       <c r="K4" t="n">
-        <v>1</v>
+        <v>82</v>
       </c>
       <c r="L4" t="n">
-        <v>1.83</v>
+        <v>3.29</v>
       </c>
       <c r="M4" t="n">
-        <v>18.9</v>
+        <v>43.1</v>
       </c>
       <c r="N4" t="n">
-        <v>34.3</v>
+        <v>62.7</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>63.4</v>
+        <v>49.6</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>FIRED</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -847,11 +851,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>Squeeze Fired</t>
-        </is>
-      </c>
+      <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
         <is>
           <t>No</t>
@@ -865,7 +865,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>518.5700000000001</v>
+        <v>509.22</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -898,22 +898,22 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>74.40000000000001</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="J5" t="n">
-        <v>64.2</v>
+        <v>58.6</v>
       </c>
       <c r="K5" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L5" t="n">
-        <v>2.38</v>
+        <v>2.47</v>
       </c>
       <c r="M5" t="n">
-        <v>24.1</v>
+        <v>23.8</v>
       </c>
       <c r="N5" t="n">
-        <v>17.4</v>
+        <v>16.6</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -921,7 +921,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>65</v>
+        <v>62.7</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -945,7 +945,7 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
@@ -957,71 +957,71 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BKNG</t>
+          <t>MET</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>162.31</v>
+        <v>95.81999999999999</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>63.4</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>31.6</v>
+        <v>47</v>
       </c>
       <c r="K6" t="n">
-        <v>94</v>
+        <v>6</v>
       </c>
       <c r="L6" t="n">
-        <v>4.03</v>
+        <v>2.02</v>
       </c>
       <c r="M6" t="n">
-        <v>36.6</v>
+        <v>19.7</v>
       </c>
       <c r="N6" t="n">
-        <v>49.1</v>
+        <v>23.8</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>39.8</v>
+        <v>63.5</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1031,48 +1031,52 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AON</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>278.79</v>
+        <v>607.87</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1086,30 +1090,30 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>53</v>
+        <v>67.7</v>
       </c>
       <c r="J7" t="n">
-        <v>25.7</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="K7" t="n">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="L7" t="n">
-        <v>2.71</v>
+        <v>4.26</v>
       </c>
       <c r="M7" t="n">
-        <v>35.9</v>
+        <v>55.5</v>
       </c>
       <c r="N7" t="n">
-        <v>89</v>
+        <v>30.6</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>29.9</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1118,12 +1122,12 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -1131,21 +1135,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr"/>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SYK</t>
+          <t>BKNG</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>273.02</v>
+        <v>163.87</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1178,22 +1186,22 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>48.2</v>
+        <v>63.7</v>
       </c>
       <c r="J8" t="n">
-        <v>32.8</v>
+        <v>33.8</v>
       </c>
       <c r="K8" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="L8" t="n">
-        <v>2.76</v>
+        <v>3.94</v>
       </c>
       <c r="M8" t="n">
-        <v>35</v>
+        <v>37.7</v>
       </c>
       <c r="N8" t="n">
-        <v>62.2</v>
+        <v>52.2</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1201,7 +1209,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>32.6</v>
+        <v>40.4</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1210,17 +1218,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
@@ -1233,15 +1241,15 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>FICO</t>
+          <t>KDP</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>862.01</v>
+        <v>31.46</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -1256,44 +1264,44 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>47.2</v>
+        <v>59.6</v>
       </c>
       <c r="J9" t="n">
-        <v>29.4</v>
+        <v>49.6</v>
       </c>
       <c r="K9" t="n">
-        <v>94</v>
+        <v>16</v>
       </c>
       <c r="L9" t="n">
-        <v>4.55</v>
+        <v>2.64</v>
       </c>
       <c r="M9" t="n">
-        <v>62.6</v>
+        <v>26.8</v>
       </c>
       <c r="N9" t="n">
-        <v>61.1</v>
+        <v>56.1</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>35.5</v>
+        <v>54</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1315,21 +1323,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr"/>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>DASH</t>
+          <t>ABNB</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>191.82</v>
+        <v>156.08</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1362,30 +1374,30 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>46.5</v>
+        <v>56</v>
       </c>
       <c r="J10" t="n">
-        <v>37.8</v>
+        <v>37.2</v>
       </c>
       <c r="K10" t="n">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="L10" t="n">
-        <v>3.71</v>
+        <v>3.7</v>
       </c>
       <c r="M10" t="n">
-        <v>32.1</v>
+        <v>36.7</v>
       </c>
       <c r="N10" t="n">
-        <v>15.5</v>
+        <v>42.6</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>49.2</v>
+        <v>50.9</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1417,11 +1429,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AXP</t>
+          <t>AON</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>309.51</v>
+        <v>272.1</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1454,22 +1466,22 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>45.7</v>
+        <v>52.6</v>
       </c>
       <c r="J11" t="n">
-        <v>37.6</v>
+        <v>22.8</v>
       </c>
       <c r="K11" t="n">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="L11" t="n">
-        <v>2.02</v>
+        <v>2.82</v>
       </c>
       <c r="M11" t="n">
-        <v>20.8</v>
+        <v>36</v>
       </c>
       <c r="N11" t="n">
-        <v>17.5</v>
+        <v>89.2</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1477,7 +1489,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>40.4</v>
+        <v>28.4</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1486,17 +1498,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
@@ -1509,11 +1521,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SBUX</t>
+          <t>DASH</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>94.31999999999999</v>
+        <v>178.39</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1542,26 +1554,26 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>43.6</v>
+        <v>51.3</v>
       </c>
       <c r="J12" t="n">
-        <v>29.1</v>
+        <v>29.8</v>
       </c>
       <c r="K12" t="n">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="L12" t="n">
-        <v>2.14</v>
+        <v>4.67</v>
       </c>
       <c r="M12" t="n">
-        <v>19.8</v>
+        <v>39</v>
       </c>
       <c r="N12" t="n">
-        <v>1.1</v>
+        <v>30.7</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1569,7 +1581,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>41.7</v>
+        <v>44.6</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1591,21 +1603,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr"/>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>NSC</t>
+          <t>FDX</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>313.2</v>
+        <v>289.65</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1638,22 +1654,22 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>42.3</v>
+        <v>50.2</v>
       </c>
       <c r="J13" t="n">
-        <v>34.2</v>
+        <v>35.9</v>
       </c>
       <c r="K13" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="L13" t="n">
-        <v>1.62</v>
+        <v>2.55</v>
       </c>
       <c r="M13" t="n">
-        <v>17.9</v>
+        <v>25.1</v>
       </c>
       <c r="N13" t="n">
-        <v>27.5</v>
+        <v>29.1</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1661,7 +1677,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>47.1</v>
+        <v>43.7</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1693,11 +1709,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ADSK</t>
+          <t>SBUX</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>211.62</v>
+        <v>95.27</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1726,26 +1742,26 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>41.9</v>
+        <v>47.6</v>
       </c>
       <c r="J14" t="n">
-        <v>38.1</v>
+        <v>33.8</v>
       </c>
       <c r="K14" t="n">
-        <v>74</v>
+        <v>93</v>
       </c>
       <c r="L14" t="n">
-        <v>3.42</v>
+        <v>2.21</v>
       </c>
       <c r="M14" t="n">
-        <v>48.4</v>
+        <v>20.3</v>
       </c>
       <c r="N14" t="n">
-        <v>86.5</v>
+        <v>3.3</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1753,7 +1769,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>42.2</v>
+        <v>43</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1785,11 +1801,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>DLTR</t>
+          <t>SYK</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>114.08</v>
+        <v>275.31</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1822,30 +1838,30 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>41.1</v>
+        <v>46.5</v>
       </c>
       <c r="J15" t="n">
-        <v>38.4</v>
+        <v>35.4</v>
       </c>
       <c r="K15" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="L15" t="n">
-        <v>3.3</v>
+        <v>2.66</v>
       </c>
       <c r="M15" t="n">
-        <v>37.8</v>
+        <v>35.2</v>
       </c>
       <c r="N15" t="n">
-        <v>26.2</v>
+        <v>63.1</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>46.8</v>
+        <v>34</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1854,17 +1870,17 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U15" t="inlineStr"/>
@@ -1877,11 +1893,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>UNP</t>
+          <t>FICO</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>273.11</v>
+        <v>840.89</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1910,34 +1926,34 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>35.5</v>
+        <v>45.7</v>
       </c>
       <c r="J16" t="n">
-        <v>32.9</v>
+        <v>27.8</v>
       </c>
       <c r="K16" t="n">
-        <v>74</v>
+        <v>90</v>
       </c>
       <c r="L16" t="n">
-        <v>1.81</v>
+        <v>4.55</v>
       </c>
       <c r="M16" t="n">
-        <v>19.7</v>
+        <v>62.7</v>
       </c>
       <c r="N16" t="n">
-        <v>26.1</v>
+        <v>61.3</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>48.7</v>
+        <v>34.7</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1961,6 +1977,654 @@
       </c>
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>AXP</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>306.33</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>45</v>
+      </c>
+      <c r="J17" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="K17" t="n">
+        <v>82</v>
+      </c>
+      <c r="L17" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="M17" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="N17" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P17" t="n">
+        <v>39.1</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr"/>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>DLTR</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>116.02</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>44.7</v>
+      </c>
+      <c r="J18" t="n">
+        <v>42.8</v>
+      </c>
+      <c r="K18" t="n">
+        <v>79</v>
+      </c>
+      <c r="L18" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="M18" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="N18" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P18" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr"/>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>ROP</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>354</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>42.1</v>
+      </c>
+      <c r="J19" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="K19" t="n">
+        <v>98</v>
+      </c>
+      <c r="L19" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="M19" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="N19" t="n">
+        <v>37.9</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P19" t="n">
+        <v>42.7</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>ADSK</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>207.19</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="J20" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="K20" t="n">
+        <v>65</v>
+      </c>
+      <c r="L20" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="M20" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="N20" t="n">
+        <v>85.59999999999999</v>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P20" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>NSC</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>313.05</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>37.4</v>
+      </c>
+      <c r="J21" t="n">
+        <v>34.1</v>
+      </c>
+      <c r="K21" t="n">
+        <v>70</v>
+      </c>
+      <c r="L21" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="M21" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="N21" t="n">
+        <v>26.1</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P21" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>APD</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>278.75</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>34.8</v>
+      </c>
+      <c r="J22" t="n">
+        <v>34.1</v>
+      </c>
+      <c r="K22" t="n">
+        <v>83</v>
+      </c>
+      <c r="L22" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="M22" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="N22" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P22" t="n">
+        <v>43.3</v>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>UNP</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>274.1</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>32.7</v>
+      </c>
+      <c r="J23" t="n">
+        <v>34.1</v>
+      </c>
+      <c r="K23" t="n">
+        <v>64</v>
+      </c>
+      <c r="L23" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="M23" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="N23" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P23" t="n">
+        <v>49.2</v>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 29.09.2026 19:15 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V23"/>
+  <dimension ref="A1:V24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -448,8 +448,8 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="6" customWidth="1" min="11" max="11"/>
-    <col width="6" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>715.62</v>
+        <v>732.72</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,22 +614,19 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>87.5</v>
+        <v>81.5</v>
       </c>
       <c r="J2" t="n">
-        <v>61</v>
+        <v>63.7</v>
       </c>
       <c r="K2" t="n">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="L2" t="n">
-        <v>4.42</v>
+        <v>4.11</v>
       </c>
       <c r="M2" t="n">
-        <v>50.6</v>
-      </c>
-      <c r="N2" t="n">
-        <v>85.3</v>
+        <v>45.8</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,7 +634,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>59.5</v>
+        <v>61.7</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -646,86 +643,82 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>JNJ</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>271.95</v>
+        <v>422.36</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>79.59999999999999</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="J3" t="n">
-        <v>58.5</v>
+        <v>60.3</v>
       </c>
       <c r="K3" t="n">
-        <v>2</v>
+        <v>90</v>
       </c>
       <c r="L3" t="n">
-        <v>1.8</v>
+        <v>2.36</v>
       </c>
       <c r="M3" t="n">
-        <v>18.8</v>
+        <v>39.7</v>
       </c>
       <c r="N3" t="n">
-        <v>33.5</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -733,7 +726,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>64</v>
+        <v>61.3</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -747,7 +740,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -755,11 +748,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr">
         <is>
           <t>No</t>
@@ -769,71 +758,71 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>326.7</v>
+        <v>510.67</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>75.5</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>61.5</v>
+        <v>59.3</v>
       </c>
       <c r="K4" t="n">
-        <v>82</v>
+        <v>7</v>
       </c>
       <c r="L4" t="n">
-        <v>3.29</v>
+        <v>2.43</v>
       </c>
       <c r="M4" t="n">
-        <v>43.1</v>
+        <v>21.9</v>
       </c>
       <c r="N4" t="n">
-        <v>62.7</v>
+        <v>11.7</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>49.6</v>
+        <v>63.1</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -843,15 +832,19 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V4" t="inlineStr">
         <is>
           <t>No</t>
@@ -861,71 +854,71 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>509.22</v>
+        <v>322.21</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>74.59999999999999</v>
+        <v>70</v>
       </c>
       <c r="J5" t="n">
-        <v>58.6</v>
+        <v>58.2</v>
       </c>
       <c r="K5" t="n">
-        <v>5</v>
+        <v>68</v>
       </c>
       <c r="L5" t="n">
-        <v>2.47</v>
+        <v>3.42</v>
       </c>
       <c r="M5" t="n">
-        <v>23.8</v>
+        <v>43.3</v>
       </c>
       <c r="N5" t="n">
-        <v>16.6</v>
+        <v>63.2</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>62.7</v>
+        <v>48.6</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -935,19 +928,15 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
           <t>No</t>
@@ -961,7 +950,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>95.81999999999999</v>
+        <v>95.42</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -994,22 +983,22 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>69.40000000000001</v>
+        <v>65</v>
       </c>
       <c r="J6" t="n">
-        <v>47</v>
+        <v>45.4</v>
       </c>
       <c r="K6" t="n">
         <v>6</v>
       </c>
       <c r="L6" t="n">
-        <v>2.02</v>
+        <v>2.03</v>
       </c>
       <c r="M6" t="n">
-        <v>19.7</v>
+        <v>19.6</v>
       </c>
       <c r="N6" t="n">
-        <v>23.8</v>
+        <v>22.7</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1017,7 +1006,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>63.5</v>
+        <v>62.4</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1041,71 +1030,71 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>KDP</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>607.87</v>
+        <v>31.05</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>67.7</v>
+        <v>64</v>
       </c>
       <c r="J7" t="n">
-        <v>65.59999999999999</v>
+        <v>48</v>
       </c>
       <c r="K7" t="n">
-        <v>85</v>
+        <v>19</v>
       </c>
       <c r="L7" t="n">
-        <v>4.26</v>
+        <v>2.52</v>
       </c>
       <c r="M7" t="n">
-        <v>55.5</v>
+        <v>24.4</v>
       </c>
       <c r="N7" t="n">
-        <v>30.6</v>
+        <v>45.3</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1113,7 +1102,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>67.40000000000001</v>
+        <v>53.1</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1122,12 +1111,12 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -1137,42 +1126,42 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>Squeeze Expanding</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BKNG</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>163.87</v>
+        <v>609.1799999999999</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1186,30 +1175,30 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>63.7</v>
+        <v>62.8</v>
       </c>
       <c r="J8" t="n">
-        <v>33.8</v>
+        <v>65.8</v>
       </c>
       <c r="K8" t="n">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="L8" t="n">
-        <v>3.94</v>
+        <v>4.04</v>
       </c>
       <c r="M8" t="n">
-        <v>37.7</v>
+        <v>55.1</v>
       </c>
       <c r="N8" t="n">
-        <v>52.2</v>
+        <v>30</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>40.4</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1223,12 +1212,12 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
@@ -1241,15 +1230,15 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>FICO</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>31.46</v>
+        <v>614.55</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -1264,44 +1253,44 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>59.6</v>
+        <v>60</v>
       </c>
       <c r="J9" t="n">
-        <v>49.6</v>
+        <v>16.4</v>
       </c>
       <c r="K9" t="n">
-        <v>16</v>
+        <v>100</v>
       </c>
       <c r="L9" t="n">
-        <v>2.64</v>
+        <v>10.73</v>
       </c>
       <c r="M9" t="n">
-        <v>26.8</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="N9" t="n">
-        <v>56.1</v>
+        <v>100</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>54</v>
+        <v>28.2</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1337,11 +1326,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ABNB</t>
+          <t>BKNG</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>156.08</v>
+        <v>163.31</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1374,30 +1363,30 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>56</v>
+        <v>59.8</v>
       </c>
       <c r="J10" t="n">
-        <v>37.2</v>
+        <v>33.4</v>
       </c>
       <c r="K10" t="n">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="L10" t="n">
-        <v>3.7</v>
+        <v>3.68</v>
       </c>
       <c r="M10" t="n">
-        <v>36.7</v>
+        <v>36.9</v>
       </c>
       <c r="N10" t="n">
-        <v>42.6</v>
+        <v>50</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>50.9</v>
+        <v>40.1</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1406,17 +1395,17 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U10" t="inlineStr"/>
@@ -1429,11 +1418,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AON</t>
+          <t>ABNB</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>272.1</v>
+        <v>157.73</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1466,30 +1455,27 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>52.6</v>
+        <v>57.8</v>
       </c>
       <c r="J11" t="n">
-        <v>22.8</v>
+        <v>39.5</v>
       </c>
       <c r="K11" t="n">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="L11" t="n">
-        <v>2.82</v>
+        <v>3.57</v>
       </c>
       <c r="M11" t="n">
-        <v>36</v>
-      </c>
-      <c r="N11" t="n">
-        <v>89.2</v>
+        <v>41.1</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>28.4</v>
+        <v>52</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1521,11 +1507,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DASH</t>
+          <t>CMG</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>178.39</v>
+        <v>32.12</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1554,26 +1540,26 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>51.3</v>
+        <v>56.8</v>
       </c>
       <c r="J12" t="n">
-        <v>29.8</v>
+        <v>36.5</v>
       </c>
       <c r="K12" t="n">
-        <v>80</v>
+        <v>97</v>
       </c>
       <c r="L12" t="n">
-        <v>4.67</v>
+        <v>3.92</v>
       </c>
       <c r="M12" t="n">
-        <v>39</v>
+        <v>35.9</v>
       </c>
       <c r="N12" t="n">
-        <v>30.7</v>
+        <v>33.4</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1581,7 +1567,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>44.6</v>
+        <v>44.7</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1603,25 +1589,21 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>FDX</t>
+          <t>AON</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>289.65</v>
+        <v>274.93</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1654,30 +1636,30 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>50.2</v>
+        <v>54.2</v>
       </c>
       <c r="J13" t="n">
-        <v>35.9</v>
+        <v>25.9</v>
       </c>
       <c r="K13" t="n">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="L13" t="n">
-        <v>2.55</v>
+        <v>2.71</v>
       </c>
       <c r="M13" t="n">
-        <v>25.1</v>
+        <v>36.1</v>
       </c>
       <c r="N13" t="n">
-        <v>29.1</v>
+        <v>89.7</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>43.7</v>
+        <v>29</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1709,11 +1691,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SBUX</t>
+          <t>DASH</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>95.27</v>
+        <v>186.19</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1742,26 +1724,26 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>47.6</v>
+        <v>51.8</v>
       </c>
       <c r="J14" t="n">
-        <v>33.8</v>
+        <v>38.5</v>
       </c>
       <c r="K14" t="n">
-        <v>93</v>
+        <v>74</v>
       </c>
       <c r="L14" t="n">
-        <v>2.21</v>
+        <v>4.52</v>
       </c>
       <c r="M14" t="n">
-        <v>20.3</v>
+        <v>41.4</v>
       </c>
       <c r="N14" t="n">
-        <v>3.3</v>
+        <v>35.8</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1769,7 +1751,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>43</v>
+        <v>47.2</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1801,11 +1783,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SYK</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>275.31</v>
+        <v>49.53</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1838,30 +1820,30 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>46.5</v>
+        <v>50.3</v>
       </c>
       <c r="J15" t="n">
-        <v>35.4</v>
+        <v>34.5</v>
       </c>
       <c r="K15" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="L15" t="n">
-        <v>2.66</v>
+        <v>3.4</v>
       </c>
       <c r="M15" t="n">
-        <v>35.2</v>
+        <v>35.5</v>
       </c>
       <c r="N15" t="n">
-        <v>63.1</v>
+        <v>40.6</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>34</v>
+        <v>47.5</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1870,34 +1852,38 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="U15" t="inlineStr"/>
-      <c r="V15" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>FICO</t>
+          <t>FDX</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>840.89</v>
+        <v>287.91</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1930,30 +1916,30 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>45.7</v>
+        <v>49.1</v>
       </c>
       <c r="J16" t="n">
-        <v>27.8</v>
+        <v>34.9</v>
       </c>
       <c r="K16" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="L16" t="n">
-        <v>4.55</v>
+        <v>2.45</v>
       </c>
       <c r="M16" t="n">
-        <v>62.7</v>
+        <v>25.1</v>
       </c>
       <c r="N16" t="n">
-        <v>61.3</v>
+        <v>29</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>34.7</v>
+        <v>42.9</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1985,11 +1971,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>AXP</t>
+          <t>SYK</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>306.33</v>
+        <v>276.93</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -2018,26 +2004,23 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>45</v>
+        <v>48.3</v>
       </c>
       <c r="J17" t="n">
-        <v>34.9</v>
+        <v>37.2</v>
       </c>
       <c r="K17" t="n">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="L17" t="n">
-        <v>1.98</v>
+        <v>2.57</v>
       </c>
       <c r="M17" t="n">
-        <v>20.7</v>
-      </c>
-      <c r="N17" t="n">
-        <v>17.2</v>
+        <v>34.8</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2045,7 +2028,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>39.1</v>
+        <v>34.8</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2054,17 +2037,17 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
@@ -2077,11 +2060,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>DLTR</t>
+          <t>SBUX</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>116.02</v>
+        <v>95.22</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2110,34 +2093,34 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>44.7</v>
+        <v>48.2</v>
       </c>
       <c r="J18" t="n">
-        <v>42.8</v>
+        <v>33.7</v>
       </c>
       <c r="K18" t="n">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="L18" t="n">
-        <v>3.35</v>
+        <v>2.14</v>
       </c>
       <c r="M18" t="n">
-        <v>38.3</v>
+        <v>20.3</v>
       </c>
       <c r="N18" t="n">
-        <v>27.4</v>
+        <v>3.1</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>48.3</v>
+        <v>42.9</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2169,11 +2152,11 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ROP</t>
+          <t>BKR</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>354</v>
+        <v>55.98</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2206,30 +2189,30 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>42.1</v>
+        <v>46</v>
       </c>
       <c r="J19" t="n">
-        <v>27.5</v>
+        <v>34.1</v>
       </c>
       <c r="K19" t="n">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="L19" t="n">
-        <v>2.7</v>
+        <v>2.64</v>
       </c>
       <c r="M19" t="n">
-        <v>25.2</v>
+        <v>27</v>
       </c>
       <c r="N19" t="n">
-        <v>37.9</v>
+        <v>29.8</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>42.7</v>
+        <v>44.8</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2251,25 +2234,21 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ADSK</t>
+          <t>AXP</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>207.19</v>
+        <v>305.5</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2298,26 +2277,26 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>38.9</v>
+        <v>41.7</v>
       </c>
       <c r="J20" t="n">
-        <v>35.5</v>
+        <v>34.3</v>
       </c>
       <c r="K20" t="n">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="L20" t="n">
-        <v>3.56</v>
+        <v>1.86</v>
       </c>
       <c r="M20" t="n">
-        <v>48.1</v>
+        <v>20.3</v>
       </c>
       <c r="N20" t="n">
-        <v>85.59999999999999</v>
+        <v>15.1</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2325,7 +2304,7 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>40.9</v>
+        <v>38.8</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2357,11 +2336,11 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>NSC</t>
+          <t>ROP</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>313.05</v>
+        <v>348.98</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2390,34 +2369,31 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>37.4</v>
+        <v>38.8</v>
       </c>
       <c r="J21" t="n">
-        <v>34.1</v>
+        <v>25.5</v>
       </c>
       <c r="K21" t="n">
-        <v>70</v>
+        <v>95</v>
       </c>
       <c r="L21" t="n">
-        <v>1.53</v>
+        <v>2.62</v>
       </c>
       <c r="M21" t="n">
-        <v>17.7</v>
-      </c>
-      <c r="N21" t="n">
-        <v>26.1</v>
+        <v>34.9</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>47.1</v>
+        <v>41.4</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2449,11 +2425,11 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>APD</t>
+          <t>VRSK</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>278.75</v>
+        <v>164.99</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -2486,22 +2462,19 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>34.8</v>
+        <v>37</v>
       </c>
       <c r="J22" t="n">
-        <v>34.1</v>
+        <v>32.9</v>
       </c>
       <c r="K22" t="n">
         <v>83</v>
       </c>
       <c r="L22" t="n">
-        <v>1.84</v>
+        <v>3.06</v>
       </c>
       <c r="M22" t="n">
-        <v>18.9</v>
-      </c>
-      <c r="N22" t="n">
-        <v>12.4</v>
+        <v>41.9</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -2509,7 +2482,7 @@
         </is>
       </c>
       <c r="P22" t="n">
-        <v>43.3</v>
+        <v>37.5</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
@@ -2541,11 +2514,11 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>UNP</t>
+          <t>NSC</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>274.1</v>
+        <v>312.92</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -2578,22 +2551,22 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>32.7</v>
+        <v>34.3</v>
       </c>
       <c r="J23" t="n">
-        <v>34.1</v>
+        <v>33.9</v>
       </c>
       <c r="K23" t="n">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="L23" t="n">
-        <v>1.72</v>
+        <v>1.43</v>
       </c>
       <c r="M23" t="n">
-        <v>19.4</v>
+        <v>16.4</v>
       </c>
       <c r="N23" t="n">
-        <v>24.8</v>
+        <v>19.7</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2601,7 +2574,7 @@
         </is>
       </c>
       <c r="P23" t="n">
-        <v>49.2</v>
+        <v>47</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -2610,21 +2583,113 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>APD</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>278.49</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>32.2</v>
+      </c>
+      <c r="J24" t="n">
+        <v>33.9</v>
+      </c>
+      <c r="K24" t="n">
+        <v>78</v>
+      </c>
+      <c r="L24" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="M24" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="N24" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P24" t="n">
+        <v>43.2</v>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 30.09.2026 19:03 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V24"/>
+  <dimension ref="A1:V25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -577,15 +577,15 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>AZN</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>732.72</v>
+        <v>162.35</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -600,41 +600,44 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>81.5</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>63.7</v>
+        <v>46.1</v>
       </c>
       <c r="K2" t="n">
-        <v>96</v>
+        <v>16</v>
       </c>
       <c r="L2" t="n">
-        <v>4.11</v>
+        <v>1.88</v>
       </c>
       <c r="M2" t="n">
-        <v>45.8</v>
+        <v>23</v>
+      </c>
+      <c r="N2" t="n">
+        <v>20.4</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>61.7</v>
+        <v>42</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -643,12 +646,12 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -656,7 +659,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr"/>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V2" t="inlineStr">
         <is>
           <t>No</t>
@@ -666,15 +673,15 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>422.36</v>
+        <v>67.18000000000001</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -689,36 +696,36 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>80.40000000000001</v>
+        <v>79.5</v>
       </c>
       <c r="J3" t="n">
-        <v>60.3</v>
+        <v>42.8</v>
       </c>
       <c r="K3" t="n">
-        <v>90</v>
+        <v>3</v>
       </c>
       <c r="L3" t="n">
-        <v>2.36</v>
+        <v>1.95</v>
       </c>
       <c r="M3" t="n">
-        <v>39.7</v>
+        <v>20.3</v>
       </c>
       <c r="N3" t="n">
-        <v>91.90000000000001</v>
+        <v>33.7</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -726,91 +733,95 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>61.3</v>
+        <v>49.9</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>FIRED</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Squeeze Fired, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>510.67</v>
+        <v>421.42</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>75.09999999999999</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="J4" t="n">
         <v>59.3</v>
       </c>
       <c r="K4" t="n">
-        <v>7</v>
+        <v>89</v>
       </c>
       <c r="L4" t="n">
-        <v>2.43</v>
+        <v>2.28</v>
       </c>
       <c r="M4" t="n">
-        <v>21.9</v>
+        <v>39.6</v>
       </c>
       <c r="N4" t="n">
-        <v>11.7</v>
+        <v>91.5</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -818,11 +829,11 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>63.1</v>
+        <v>61.1</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -832,19 +843,15 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
         <is>
           <t>No</t>
@@ -858,7 +865,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>322.21</v>
+        <v>330.92</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -887,34 +894,34 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>70</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>58.2</v>
+        <v>62.9</v>
       </c>
       <c r="K5" t="n">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="L5" t="n">
-        <v>3.42</v>
+        <v>3.44</v>
       </c>
       <c r="M5" t="n">
-        <v>43.3</v>
+        <v>43</v>
       </c>
       <c r="N5" t="n">
-        <v>63.2</v>
+        <v>62.5</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>48.6</v>
+        <v>50.6</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -946,15 +953,15 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MET</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>95.42</v>
+        <v>733.41</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -969,36 +976,36 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>65</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>45.4</v>
+        <v>63.1</v>
       </c>
       <c r="K6" t="n">
-        <v>6</v>
+        <v>94</v>
       </c>
       <c r="L6" t="n">
-        <v>2.03</v>
+        <v>3.96</v>
       </c>
       <c r="M6" t="n">
-        <v>19.6</v>
+        <v>47.1</v>
       </c>
       <c r="N6" t="n">
-        <v>22.7</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1006,11 +1013,11 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>62.4</v>
+        <v>61.8</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1028,11 +1035,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+      <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr">
         <is>
           <t>No</t>
@@ -1042,59 +1045,59 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>TMO</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>31.05</v>
+        <v>679.33</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>64</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>48</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="K7" t="n">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="L7" t="n">
-        <v>2.52</v>
+        <v>2.22</v>
       </c>
       <c r="M7" t="n">
         <v>24.4</v>
       </c>
       <c r="N7" t="n">
-        <v>45.3</v>
+        <v>31.8</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1102,7 +1105,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>53.1</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1111,12 +1114,12 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -1124,11 +1127,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr">
         <is>
           <t>No</t>
@@ -1138,15 +1137,15 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>AIG</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>609.1799999999999</v>
+        <v>74.68000000000001</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1161,48 +1160,48 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>62.8</v>
+        <v>61.3</v>
       </c>
       <c r="J8" t="n">
-        <v>65.8</v>
+        <v>46.9</v>
       </c>
       <c r="K8" t="n">
-        <v>84</v>
+        <v>18</v>
       </c>
       <c r="L8" t="n">
-        <v>4.04</v>
+        <v>2.09</v>
       </c>
       <c r="M8" t="n">
-        <v>55.1</v>
+        <v>17.6</v>
       </c>
       <c r="N8" t="n">
-        <v>30</v>
+        <v>18.7</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>67.59999999999999</v>
+        <v>45.7</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -1212,7 +1211,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -1220,7 +1219,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr"/>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V8" t="inlineStr">
         <is>
           <t>No</t>
@@ -1234,7 +1237,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>614.55</v>
+        <v>599.2</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1267,22 +1270,22 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>60</v>
+        <v>59.8</v>
       </c>
       <c r="J9" t="n">
-        <v>16.4</v>
+        <v>15.9</v>
       </c>
       <c r="K9" t="n">
         <v>100</v>
       </c>
       <c r="L9" t="n">
-        <v>10.73</v>
+        <v>10.25</v>
       </c>
       <c r="M9" t="n">
-        <v>98.40000000000001</v>
+        <v>97.2</v>
       </c>
       <c r="N9" t="n">
-        <v>100</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1290,7 +1293,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>28.2</v>
+        <v>27.9</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1312,95 +1315,91 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BKNG</t>
+          <t>MET</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>163.31</v>
+        <v>94.37</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I10" t="n">
         <v>59.8</v>
       </c>
       <c r="J10" t="n">
-        <v>33.4</v>
+        <v>41.4</v>
       </c>
       <c r="K10" t="n">
-        <v>87</v>
+        <v>8</v>
       </c>
       <c r="L10" t="n">
-        <v>3.68</v>
+        <v>1.97</v>
       </c>
       <c r="M10" t="n">
-        <v>36.9</v>
+        <v>19.8</v>
       </c>
       <c r="N10" t="n">
-        <v>50</v>
+        <v>23.9</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>40.1</v>
+        <v>59.9</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1408,7 +1407,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr"/>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V10" t="inlineStr">
         <is>
           <t>No</t>
@@ -1422,7 +1425,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>157.73</v>
+        <v>161.21</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1451,23 +1454,26 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>57.8</v>
+        <v>59.5</v>
       </c>
       <c r="J11" t="n">
-        <v>39.5</v>
+        <v>44.3</v>
       </c>
       <c r="K11" t="n">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="L11" t="n">
-        <v>3.57</v>
+        <v>3.48</v>
       </c>
       <c r="M11" t="n">
-        <v>41.1</v>
+        <v>36.6</v>
+      </c>
+      <c r="N11" t="n">
+        <v>42.5</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1475,7 +1481,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1484,17 +1490,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
@@ -1507,30 +1513,30 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CMG</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>32.12</v>
+        <v>610.2</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1544,30 +1550,30 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>56.8</v>
+        <v>58</v>
       </c>
       <c r="J12" t="n">
-        <v>36.5</v>
+        <v>66</v>
       </c>
       <c r="K12" t="n">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="L12" t="n">
-        <v>3.92</v>
+        <v>3.87</v>
       </c>
       <c r="M12" t="n">
-        <v>35.9</v>
+        <v>53.1</v>
       </c>
       <c r="N12" t="n">
-        <v>33.4</v>
+        <v>26.8</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>44.7</v>
+        <v>67.8</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1576,12 +1582,12 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -1599,11 +1605,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AON</t>
+          <t>BKNG</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>274.93</v>
+        <v>162.6</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1636,22 +1642,22 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>54.2</v>
+        <v>57.7</v>
       </c>
       <c r="J13" t="n">
-        <v>25.9</v>
+        <v>33.1</v>
       </c>
       <c r="K13" t="n">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="L13" t="n">
-        <v>2.71</v>
+        <v>3.62</v>
       </c>
       <c r="M13" t="n">
-        <v>36.1</v>
+        <v>36.3</v>
       </c>
       <c r="N13" t="n">
-        <v>89.7</v>
+        <v>48.3</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1659,7 +1665,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>29</v>
+        <v>39.9</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1668,17 +1674,17 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U13" t="inlineStr"/>
@@ -1691,11 +1697,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>DASH</t>
+          <t>AON</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>186.19</v>
+        <v>277.22</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1724,26 +1730,26 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>51.8</v>
+        <v>54.8</v>
       </c>
       <c r="J14" t="n">
-        <v>38.5</v>
+        <v>28.4</v>
       </c>
       <c r="K14" t="n">
-        <v>74</v>
+        <v>90</v>
       </c>
       <c r="L14" t="n">
-        <v>4.52</v>
+        <v>2.58</v>
       </c>
       <c r="M14" t="n">
-        <v>41.4</v>
+        <v>36.4</v>
       </c>
       <c r="N14" t="n">
-        <v>35.8</v>
+        <v>91</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1751,7 +1757,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>47.2</v>
+        <v>29.5</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1760,17 +1766,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
@@ -1783,11 +1789,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>CMG</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>49.53</v>
+        <v>31.91</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1820,30 +1826,30 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>50.3</v>
+        <v>53.7</v>
       </c>
       <c r="J15" t="n">
-        <v>34.5</v>
+        <v>34.8</v>
       </c>
       <c r="K15" t="n">
-        <v>83</v>
+        <v>97</v>
       </c>
       <c r="L15" t="n">
-        <v>3.4</v>
+        <v>3.66</v>
       </c>
       <c r="M15" t="n">
-        <v>35.5</v>
+        <v>35.7</v>
       </c>
       <c r="N15" t="n">
-        <v>40.6</v>
+        <v>32.8</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>47.5</v>
+        <v>44.2</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1865,25 +1871,21 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>FDX</t>
+          <t>XEL</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>287.91</v>
+        <v>70.78</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1916,30 +1918,30 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>49.1</v>
+        <v>51</v>
       </c>
       <c r="J16" t="n">
-        <v>34.9</v>
+        <v>36.6</v>
       </c>
       <c r="K16" t="n">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="L16" t="n">
-        <v>2.45</v>
+        <v>1.8</v>
       </c>
       <c r="M16" t="n">
-        <v>25.1</v>
+        <v>18.3</v>
       </c>
       <c r="N16" t="n">
-        <v>29</v>
+        <v>42.8</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>42.9</v>
+        <v>37.3</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1948,17 +1950,17 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
@@ -1971,11 +1973,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SYK</t>
+          <t>CMCSA</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>276.93</v>
+        <v>21.91</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -2004,23 +2006,26 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>48.3</v>
+        <v>50.6</v>
       </c>
       <c r="J17" t="n">
-        <v>37.2</v>
+        <v>30.3</v>
       </c>
       <c r="K17" t="n">
-        <v>78</v>
+        <v>99</v>
       </c>
       <c r="L17" t="n">
-        <v>2.57</v>
+        <v>2.85</v>
       </c>
       <c r="M17" t="n">
-        <v>34.8</v>
+        <v>30.6</v>
+      </c>
+      <c r="N17" t="n">
+        <v>30</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2028,7 +2033,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>34.8</v>
+        <v>36.8</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2037,17 +2042,17 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
@@ -2060,11 +2065,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SBUX</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>95.22</v>
+        <v>48.94</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2097,30 +2102,30 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>48.2</v>
+        <v>49.1</v>
       </c>
       <c r="J18" t="n">
-        <v>33.7</v>
+        <v>32.7</v>
       </c>
       <c r="K18" t="n">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L18" t="n">
-        <v>2.14</v>
+        <v>3.27</v>
       </c>
       <c r="M18" t="n">
-        <v>20.3</v>
+        <v>35.2</v>
       </c>
       <c r="N18" t="n">
-        <v>3.1</v>
+        <v>39.3</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>42.9</v>
+        <v>46.6</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2129,17 +2134,17 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
@@ -2152,11 +2157,11 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>BKR</t>
+          <t>SYK</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>55.98</v>
+        <v>275.5</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2185,35 +2190,35 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>46</v>
+        <v>48.9</v>
       </c>
       <c r="J19" t="n">
+        <v>36.9</v>
+      </c>
+      <c r="K19" t="n">
+        <v>73</v>
+      </c>
+      <c r="L19" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="M19" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="N19" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P19" t="n">
         <v>34.1</v>
       </c>
-      <c r="K19" t="n">
-        <v>87</v>
-      </c>
-      <c r="L19" t="n">
-        <v>2.64</v>
-      </c>
-      <c r="M19" t="n">
-        <v>27</v>
-      </c>
-      <c r="N19" t="n">
-        <v>29.8</v>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="P19" t="n">
-        <v>44.8</v>
-      </c>
       <c r="Q19" t="inlineStr">
         <is>
           <t>OFF</t>
@@ -2221,17 +2226,17 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U19" t="inlineStr"/>
@@ -2244,11 +2249,11 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>AXP</t>
+          <t>SBUX</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>305.5</v>
+        <v>94.86</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2281,22 +2286,22 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>41.7</v>
+        <v>47.8</v>
       </c>
       <c r="J20" t="n">
-        <v>34.3</v>
+        <v>33.1</v>
       </c>
       <c r="K20" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="L20" t="n">
-        <v>1.86</v>
+        <v>2.03</v>
       </c>
       <c r="M20" t="n">
-        <v>20.3</v>
+        <v>19.9</v>
       </c>
       <c r="N20" t="n">
-        <v>15.1</v>
+        <v>1.5</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2304,7 +2309,7 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>38.8</v>
+        <v>42.3</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2336,11 +2341,11 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ROP</t>
+          <t>FDX</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>348.98</v>
+        <v>284.85</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2373,27 +2378,30 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>38.8</v>
+        <v>45</v>
       </c>
       <c r="J21" t="n">
-        <v>25.5</v>
+        <v>33.1</v>
       </c>
       <c r="K21" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="L21" t="n">
-        <v>2.62</v>
+        <v>2.35</v>
       </c>
       <c r="M21" t="n">
-        <v>34.9</v>
+        <v>25.1</v>
+      </c>
+      <c r="N21" t="n">
+        <v>29</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>41.4</v>
+        <v>41.5</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2425,11 +2433,11 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>VRSK</t>
+          <t>BKR</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>164.99</v>
+        <v>55.11</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -2462,19 +2470,22 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>37</v>
+        <v>44.6</v>
       </c>
       <c r="J22" t="n">
-        <v>32.9</v>
+        <v>31.4</v>
       </c>
       <c r="K22" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L22" t="n">
-        <v>3.06</v>
+        <v>2.71</v>
       </c>
       <c r="M22" t="n">
-        <v>41.9</v>
+        <v>27.2</v>
+      </c>
+      <c r="N22" t="n">
+        <v>30.8</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -2482,7 +2493,7 @@
         </is>
       </c>
       <c r="P22" t="n">
-        <v>37.5</v>
+        <v>43.6</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
@@ -2504,21 +2515,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U22" t="inlineStr"/>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>NSC</t>
+          <t>AXP</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>312.92</v>
+        <v>304.69</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -2547,34 +2562,34 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>34.3</v>
+        <v>40.8</v>
       </c>
       <c r="J23" t="n">
-        <v>33.9</v>
+        <v>33.6</v>
       </c>
       <c r="K23" t="n">
-        <v>58</v>
+        <v>84</v>
       </c>
       <c r="L23" t="n">
-        <v>1.43</v>
+        <v>1.78</v>
       </c>
       <c r="M23" t="n">
-        <v>16.4</v>
+        <v>20</v>
       </c>
       <c r="N23" t="n">
-        <v>19.7</v>
+        <v>14.2</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>47</v>
+        <v>38.5</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -2583,17 +2598,17 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U23" t="inlineStr"/>
@@ -2606,11 +2621,11 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>APD</t>
+          <t>ROP</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>278.49</v>
+        <v>350.3</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -2639,26 +2654,26 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I24" t="n">
-        <v>32.2</v>
+        <v>37.6</v>
       </c>
       <c r="J24" t="n">
-        <v>33.9</v>
+        <v>26.6</v>
       </c>
       <c r="K24" t="n">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="L24" t="n">
-        <v>1.82</v>
+        <v>2.5</v>
       </c>
       <c r="M24" t="n">
-        <v>17.6</v>
+        <v>24.2</v>
       </c>
       <c r="N24" t="n">
-        <v>7.9</v>
+        <v>35.3</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2666,7 +2681,7 @@
         </is>
       </c>
       <c r="P24" t="n">
-        <v>43.2</v>
+        <v>41.7</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -2690,6 +2705,95 @@
       </c>
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>APD</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>281.47</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>34</v>
+      </c>
+      <c r="J25" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="K25" t="n">
+        <v>75</v>
+      </c>
+      <c r="L25" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="M25" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P25" t="n">
+        <v>44.7</v>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 01.10.2026 19:23 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V25"/>
+  <dimension ref="A1:V26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -448,8 +448,8 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="7" customWidth="1" min="11" max="11"/>
-    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="6" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
@@ -577,15 +577,15 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AZN</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>162.35</v>
+        <v>410.52</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -600,44 +600,44 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>81.09999999999999</v>
+        <v>78.5</v>
       </c>
       <c r="J2" t="n">
-        <v>46.1</v>
+        <v>52</v>
       </c>
       <c r="K2" t="n">
-        <v>16</v>
+        <v>87</v>
       </c>
       <c r="L2" t="n">
-        <v>1.88</v>
+        <v>2.48</v>
       </c>
       <c r="M2" t="n">
-        <v>23</v>
+        <v>38.4</v>
       </c>
       <c r="N2" t="n">
-        <v>20.4</v>
+        <v>86.2</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>42</v>
+        <v>58.5</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -646,12 +646,12 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -661,42 +661,42 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Squeeze Expanding</t>
+          <t>Divergence</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>67.18000000000001</v>
+        <v>138.49</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -710,22 +710,22 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>79.5</v>
+        <v>77.5</v>
       </c>
       <c r="J3" t="n">
-        <v>42.8</v>
+        <v>55</v>
       </c>
       <c r="K3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L3" t="n">
-        <v>1.95</v>
+        <v>4.26</v>
       </c>
       <c r="M3" t="n">
-        <v>20.3</v>
+        <v>55.5</v>
       </c>
       <c r="N3" t="n">
-        <v>33.7</v>
+        <v>47.5</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -733,51 +733,51 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>49.9</v>
+        <v>59.1</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>FIRED</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Squeeze Fired, Divergence, Squeeze Expanding</t>
+          <t>Squeeze Expanding</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>421.42</v>
+        <v>66.81999999999999</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -792,36 +792,36 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>76.90000000000001</v>
+        <v>75</v>
       </c>
       <c r="J4" t="n">
-        <v>59.3</v>
+        <v>40.9</v>
       </c>
       <c r="K4" t="n">
-        <v>89</v>
+        <v>5</v>
       </c>
       <c r="L4" t="n">
-        <v>2.28</v>
+        <v>1.92</v>
       </c>
       <c r="M4" t="n">
-        <v>39.6</v>
+        <v>19.9</v>
       </c>
       <c r="N4" t="n">
-        <v>91.5</v>
+        <v>32.5</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -829,7 +829,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>61.1</v>
+        <v>49.2</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -838,12 +838,12 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -851,69 +851,73 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr"/>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>TEAM</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>330.92</v>
+        <v>190.48</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>76.90000000000001</v>
+        <v>71</v>
       </c>
       <c r="J5" t="n">
-        <v>62.9</v>
+        <v>58.1</v>
       </c>
       <c r="K5" t="n">
-        <v>82</v>
+        <v>6</v>
       </c>
       <c r="L5" t="n">
-        <v>3.44</v>
+        <v>5.1</v>
       </c>
       <c r="M5" t="n">
-        <v>43</v>
+        <v>57</v>
       </c>
       <c r="N5" t="n">
-        <v>62.5</v>
+        <v>35.1</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -921,7 +925,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>50.6</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -930,12 +934,12 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -943,7 +947,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr"/>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V5" t="inlineStr">
         <is>
           <t>No</t>
@@ -957,7 +965,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>733.41</v>
+        <v>728.4400000000001</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -990,22 +998,22 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>75.90000000000001</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>63.1</v>
+        <v>61.6</v>
       </c>
       <c r="K6" t="n">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="L6" t="n">
-        <v>3.96</v>
+        <v>3.72</v>
       </c>
       <c r="M6" t="n">
-        <v>47.1</v>
+        <v>47.5</v>
       </c>
       <c r="N6" t="n">
-        <v>75.40000000000001</v>
+        <v>76.7</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1013,7 +1021,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>61.8</v>
+        <v>61.1</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1045,15 +1053,15 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TMO</t>
+          <t>AIG</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>679.33</v>
+        <v>75.09</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -1068,48 +1076,48 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>66.90000000000001</v>
+        <v>68.8</v>
       </c>
       <c r="J7" t="n">
-        <v>73.59999999999999</v>
+        <v>49.1</v>
       </c>
       <c r="K7" t="n">
-        <v>88</v>
+        <v>17</v>
       </c>
       <c r="L7" t="n">
-        <v>2.22</v>
+        <v>1.96</v>
       </c>
       <c r="M7" t="n">
-        <v>24.4</v>
+        <v>17.9</v>
       </c>
       <c r="N7" t="n">
-        <v>31.8</v>
+        <v>20</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>74.09999999999999</v>
+        <v>47</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1119,7 +1127,7 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -1127,7 +1135,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr"/>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V7" t="inlineStr">
         <is>
           <t>No</t>
@@ -1137,11 +1149,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AIG</t>
+          <t>AZN</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>74.68000000000001</v>
+        <v>158.13</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1170,26 +1182,26 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>61.3</v>
+        <v>63.8</v>
       </c>
       <c r="J8" t="n">
-        <v>46.9</v>
+        <v>39.6</v>
       </c>
       <c r="K8" t="n">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="L8" t="n">
-        <v>2.09</v>
+        <v>2.02</v>
       </c>
       <c r="M8" t="n">
-        <v>17.6</v>
+        <v>22.3</v>
       </c>
       <c r="N8" t="n">
-        <v>18.7</v>
+        <v>17.5</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1197,21 +1209,21 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>45.7</v>
+        <v>39.5</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -1221,23 +1233,23 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>Divergence</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>FICO</t>
+          <t>ABNB</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>599.2</v>
+        <v>160.54</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1266,34 +1278,34 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>59.8</v>
+        <v>58.6</v>
       </c>
       <c r="J9" t="n">
-        <v>15.9</v>
+        <v>43.4</v>
       </c>
       <c r="K9" t="n">
-        <v>100</v>
+        <v>77</v>
       </c>
       <c r="L9" t="n">
-        <v>10.25</v>
+        <v>3.36</v>
       </c>
       <c r="M9" t="n">
-        <v>97.2</v>
+        <v>35.9</v>
       </c>
       <c r="N9" t="n">
-        <v>99.59999999999999</v>
+        <v>40.5</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>27.9</v>
+        <v>53.6</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1302,17 +1314,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
@@ -1325,15 +1337,15 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>MET</t>
+          <t>TMO</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>94.37</v>
+        <v>658.71</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1348,36 +1360,36 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>59.8</v>
+        <v>57.4</v>
       </c>
       <c r="J10" t="n">
-        <v>41.4</v>
+        <v>59</v>
       </c>
       <c r="K10" t="n">
-        <v>8</v>
+        <v>82</v>
       </c>
       <c r="L10" t="n">
-        <v>1.97</v>
+        <v>2.4</v>
       </c>
       <c r="M10" t="n">
-        <v>19.8</v>
+        <v>23.4</v>
       </c>
       <c r="N10" t="n">
-        <v>23.9</v>
+        <v>27.7</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1385,11 +1397,11 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>59.9</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -1409,42 +1421,42 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>Divergence</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ABNB</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>161.21</v>
+        <v>615.5599999999999</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1458,22 +1470,22 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>59.5</v>
+        <v>57.1</v>
       </c>
       <c r="J11" t="n">
-        <v>44.3</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="K11" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="L11" t="n">
-        <v>3.48</v>
+        <v>3.71</v>
       </c>
       <c r="M11" t="n">
-        <v>36.6</v>
+        <v>51.3</v>
       </c>
       <c r="N11" t="n">
-        <v>42.5</v>
+        <v>23.9</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1481,7 +1493,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>54</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1495,12 +1507,12 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
@@ -1513,30 +1525,30 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>BKNG</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>610.2</v>
+        <v>160.93</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1546,34 +1558,34 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>58</v>
+        <v>54.3</v>
       </c>
       <c r="J12" t="n">
-        <v>66</v>
+        <v>31.9</v>
       </c>
       <c r="K12" t="n">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="L12" t="n">
-        <v>3.87</v>
+        <v>3.63</v>
       </c>
       <c r="M12" t="n">
-        <v>53.1</v>
+        <v>35.2</v>
       </c>
       <c r="N12" t="n">
-        <v>26.8</v>
+        <v>45.3</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>67.8</v>
+        <v>39.2</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1582,12 +1594,12 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -1605,11 +1617,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BKNG</t>
+          <t>AON</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>162.6</v>
+        <v>276.49</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1642,22 +1654,22 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>57.7</v>
+        <v>52.5</v>
       </c>
       <c r="J13" t="n">
-        <v>33.1</v>
+        <v>27.8</v>
       </c>
       <c r="K13" t="n">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="L13" t="n">
-        <v>3.62</v>
+        <v>2.5</v>
       </c>
       <c r="M13" t="n">
-        <v>36.3</v>
+        <v>35.8</v>
       </c>
       <c r="N13" t="n">
-        <v>48.3</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1665,7 +1677,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>39.9</v>
+        <v>29.4</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1697,11 +1709,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AON</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>277.22</v>
+        <v>83.45999999999999</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1734,22 +1746,22 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>54.8</v>
+        <v>51.8</v>
       </c>
       <c r="J14" t="n">
-        <v>28.4</v>
+        <v>33.2</v>
       </c>
       <c r="K14" t="n">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="L14" t="n">
-        <v>2.58</v>
+        <v>1.56</v>
       </c>
       <c r="M14" t="n">
-        <v>36.4</v>
+        <v>14.2</v>
       </c>
       <c r="N14" t="n">
-        <v>91</v>
+        <v>15.6</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1757,7 +1769,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>29.5</v>
+        <v>33.8</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1789,11 +1801,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CMG</t>
+          <t>CMCSA</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>31.91</v>
+        <v>21.76</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1826,22 +1838,22 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>53.7</v>
+        <v>49.4</v>
       </c>
       <c r="J15" t="n">
-        <v>34.8</v>
+        <v>28.3</v>
       </c>
       <c r="K15" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="L15" t="n">
-        <v>3.66</v>
+        <v>2.75</v>
       </c>
       <c r="M15" t="n">
-        <v>35.7</v>
+        <v>29.7</v>
       </c>
       <c r="N15" t="n">
-        <v>32.8</v>
+        <v>26.9</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1849,7 +1861,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>44.2</v>
+        <v>36.4</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1881,15 +1893,15 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>XEL</t>
+          <t>PSX</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>70.78</v>
+        <v>263.95</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -1904,44 +1916,41 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>51</v>
+        <v>47.8</v>
       </c>
       <c r="J16" t="n">
-        <v>36.6</v>
+        <v>62.5</v>
       </c>
       <c r="K16" t="n">
-        <v>99</v>
+        <v>12</v>
       </c>
       <c r="L16" t="n">
-        <v>1.8</v>
+        <v>3.37</v>
       </c>
       <c r="M16" t="n">
-        <v>18.3</v>
-      </c>
-      <c r="N16" t="n">
-        <v>42.8</v>
+        <v>45.2</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>37.3</v>
+        <v>72.7</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1950,20 +1959,24 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V16" t="inlineStr">
         <is>
           <t>No</t>
@@ -1973,11 +1986,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CMCSA</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>21.91</v>
+        <v>48.66</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -2010,30 +2023,30 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>50.6</v>
+        <v>46.8</v>
       </c>
       <c r="J17" t="n">
-        <v>30.3</v>
+        <v>31.9</v>
       </c>
       <c r="K17" t="n">
-        <v>99</v>
+        <v>86</v>
       </c>
       <c r="L17" t="n">
-        <v>2.85</v>
+        <v>3.14</v>
       </c>
       <c r="M17" t="n">
-        <v>30.6</v>
+        <v>35.3</v>
       </c>
       <c r="N17" t="n">
-        <v>30</v>
+        <v>39.7</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>36.8</v>
+        <v>46.2</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2065,11 +2078,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>CMG</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>48.94</v>
+        <v>32.06</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2102,30 +2115,30 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>49.1</v>
+        <v>46.3</v>
       </c>
       <c r="J18" t="n">
-        <v>32.7</v>
+        <v>36.2</v>
       </c>
       <c r="K18" t="n">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="L18" t="n">
-        <v>3.27</v>
+        <v>3.37</v>
       </c>
       <c r="M18" t="n">
-        <v>35.2</v>
+        <v>33.6</v>
       </c>
       <c r="N18" t="n">
-        <v>39.3</v>
+        <v>28.2</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>46.6</v>
+        <v>44.5</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2157,11 +2170,11 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SYK</t>
+          <t>FDX</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>275.5</v>
+        <v>286.12</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2190,34 +2203,34 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>48.9</v>
+        <v>45.6</v>
       </c>
       <c r="J19" t="n">
-        <v>36.9</v>
+        <v>34.5</v>
       </c>
       <c r="K19" t="n">
-        <v>73</v>
+        <v>95</v>
       </c>
       <c r="L19" t="n">
-        <v>2.55</v>
+        <v>2.23</v>
       </c>
       <c r="M19" t="n">
-        <v>35.4</v>
+        <v>25.1</v>
       </c>
       <c r="N19" t="n">
-        <v>63.5</v>
+        <v>29.3</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>34.1</v>
+        <v>42</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2226,17 +2239,17 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U19" t="inlineStr"/>
@@ -2253,7 +2266,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>94.86</v>
+        <v>94.25</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2282,26 +2295,26 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>47.8</v>
+        <v>45.6</v>
       </c>
       <c r="J20" t="n">
-        <v>33.1</v>
+        <v>32.4</v>
       </c>
       <c r="K20" t="n">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="L20" t="n">
-        <v>2.03</v>
+        <v>2.02</v>
       </c>
       <c r="M20" t="n">
-        <v>19.9</v>
+        <v>20.2</v>
       </c>
       <c r="N20" t="n">
-        <v>1.5</v>
+        <v>2.8</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2309,7 +2322,7 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>42.3</v>
+        <v>41.6</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2341,11 +2354,11 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>FDX</t>
+          <t>BKR</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>284.85</v>
+        <v>55.83</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2374,34 +2387,34 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>45</v>
+        <v>44.3</v>
       </c>
       <c r="J21" t="n">
-        <v>33.1</v>
+        <v>36.5</v>
       </c>
       <c r="K21" t="n">
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="L21" t="n">
-        <v>2.35</v>
+        <v>2.75</v>
       </c>
       <c r="M21" t="n">
-        <v>25.1</v>
+        <v>28.1</v>
       </c>
       <c r="N21" t="n">
-        <v>29</v>
+        <v>35.3</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>41.5</v>
+        <v>44.5</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2433,11 +2446,11 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BKR</t>
+          <t>TMUS</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>55.11</v>
+        <v>161.74</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -2470,22 +2483,22 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>44.6</v>
+        <v>43.8</v>
       </c>
       <c r="J22" t="n">
-        <v>31.4</v>
+        <v>33.9</v>
       </c>
       <c r="K22" t="n">
-        <v>85</v>
+        <v>98</v>
       </c>
       <c r="L22" t="n">
-        <v>2.71</v>
+        <v>2.47</v>
       </c>
       <c r="M22" t="n">
-        <v>27.2</v>
+        <v>29.1</v>
       </c>
       <c r="N22" t="n">
-        <v>30.8</v>
+        <v>34.3</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -2493,7 +2506,7 @@
         </is>
       </c>
       <c r="P22" t="n">
-        <v>43.6</v>
+        <v>34.3</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
@@ -2515,14 +2528,10 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U22" t="inlineStr"/>
       <c r="V22" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2533,7 +2542,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>304.69</v>
+        <v>300.8</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -2566,22 +2575,22 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>40.8</v>
+        <v>42.5</v>
       </c>
       <c r="J23" t="n">
-        <v>33.6</v>
+        <v>30.7</v>
       </c>
       <c r="K23" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="L23" t="n">
-        <v>1.78</v>
+        <v>1.91</v>
       </c>
       <c r="M23" t="n">
         <v>20</v>
       </c>
       <c r="N23" t="n">
-        <v>14.2</v>
+        <v>14.1</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2589,7 +2598,7 @@
         </is>
       </c>
       <c r="P23" t="n">
-        <v>38.5</v>
+        <v>37.1</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -2611,10 +2620,14 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U23" t="inlineStr"/>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2625,7 +2638,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>350.3</v>
+        <v>362.4</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -2658,22 +2671,22 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>37.6</v>
+        <v>42.5</v>
       </c>
       <c r="J24" t="n">
-        <v>26.6</v>
+        <v>39.2</v>
       </c>
       <c r="K24" t="n">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="L24" t="n">
-        <v>2.5</v>
+        <v>2.62</v>
       </c>
       <c r="M24" t="n">
-        <v>24.2</v>
+        <v>24.7</v>
       </c>
       <c r="N24" t="n">
-        <v>35.3</v>
+        <v>36.7</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2681,7 +2694,7 @@
         </is>
       </c>
       <c r="P24" t="n">
-        <v>41.7</v>
+        <v>45.2</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -2690,17 +2703,17 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U24" t="inlineStr"/>
@@ -2713,11 +2726,11 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>APD</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>281.47</v>
+        <v>68.11</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -2746,23 +2759,26 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="J25" t="n">
-        <v>38.5</v>
+        <v>32.9</v>
       </c>
       <c r="K25" t="n">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="L25" t="n">
-        <v>1.72</v>
+        <v>2.77</v>
       </c>
       <c r="M25" t="n">
-        <v>28.5</v>
+        <v>33.5</v>
+      </c>
+      <c r="N25" t="n">
+        <v>43</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2770,7 +2786,7 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>44.7</v>
+        <v>34.5</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
@@ -2794,6 +2810,98 @@
       </c>
       <c r="U25" t="inlineStr"/>
       <c r="V25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>CHTR</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>112.1</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="J26" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="K26" t="n">
+        <v>91</v>
+      </c>
+      <c r="L26" t="n">
+        <v>4.64</v>
+      </c>
+      <c r="M26" t="n">
+        <v>55.9</v>
+      </c>
+      <c r="N26" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P26" t="n">
+        <v>31.6</v>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr"/>
+      <c r="V26" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 02.10.2026 19:07 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V26"/>
+  <dimension ref="A1:V41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -448,7 +448,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
     <col width="6" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>ILMN</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>410.52</v>
+        <v>270.7</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,22 +614,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>78.5</v>
+        <v>79.7</v>
       </c>
       <c r="J2" t="n">
-        <v>52</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="K2" t="n">
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="L2" t="n">
-        <v>2.48</v>
+        <v>4.17</v>
       </c>
       <c r="M2" t="n">
-        <v>38.4</v>
+        <v>50</v>
       </c>
       <c r="N2" t="n">
-        <v>86.2</v>
+        <v>43.2</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>58.5</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -651,7 +651,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -659,14 +659,10 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -677,7 +673,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>138.49</v>
+        <v>134.88</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -710,13 +706,13 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>77.5</v>
+        <v>78.3</v>
       </c>
       <c r="J3" t="n">
-        <v>55</v>
+        <v>50.9</v>
       </c>
       <c r="K3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L3" t="n">
         <v>4.26</v>
@@ -725,7 +721,7 @@
         <v>55.5</v>
       </c>
       <c r="N3" t="n">
-        <v>47.5</v>
+        <v>47.4</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -733,21 +729,21 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>59.1</v>
+        <v>57.4</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -757,7 +753,7 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Squeeze Expanding</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -769,11 +765,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>ROST</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>66.81999999999999</v>
+        <v>227.79</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -806,22 +802,22 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>75</v>
+        <v>76.7</v>
       </c>
       <c r="J4" t="n">
-        <v>40.9</v>
+        <v>42.3</v>
       </c>
       <c r="K4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L4" t="n">
-        <v>1.92</v>
+        <v>2.16</v>
       </c>
       <c r="M4" t="n">
-        <v>19.9</v>
+        <v>23.8</v>
       </c>
       <c r="N4" t="n">
-        <v>32.5</v>
+        <v>38.3</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -829,7 +825,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>49.2</v>
+        <v>51.4</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -843,7 +839,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -865,30 +861,30 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TEAM</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>190.48</v>
+        <v>67.22</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -902,22 +898,22 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="J5" t="n">
-        <v>58.1</v>
+        <v>43.6</v>
       </c>
       <c r="K5" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L5" t="n">
-        <v>5.1</v>
+        <v>1.82</v>
       </c>
       <c r="M5" t="n">
-        <v>57</v>
+        <v>19.5</v>
       </c>
       <c r="N5" t="n">
-        <v>35.1</v>
+        <v>31</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -925,7 +921,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>70.59999999999999</v>
+        <v>50</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -961,68 +957,65 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>TEAM</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>728.4400000000001</v>
+        <v>187.46</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I6" t="n">
+        <v>74.90000000000001</v>
+      </c>
+      <c r="J6" t="n">
+        <v>55.7</v>
+      </c>
+      <c r="K6" t="n">
+        <v>5</v>
+      </c>
+      <c r="L6" t="n">
+        <v>4.85</v>
+      </c>
+      <c r="M6" t="n">
+        <v>72.90000000000001</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
         <v>69.90000000000001</v>
       </c>
-      <c r="J6" t="n">
-        <v>61.6</v>
-      </c>
-      <c r="K6" t="n">
-        <v>89</v>
-      </c>
-      <c r="L6" t="n">
-        <v>3.72</v>
-      </c>
-      <c r="M6" t="n">
-        <v>47.5</v>
-      </c>
-      <c r="N6" t="n">
-        <v>76.7</v>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P6" t="n">
-        <v>61.1</v>
-      </c>
       <c r="Q6" t="inlineStr">
         <is>
           <t>OFF</t>
@@ -1040,7 +1033,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
@@ -1053,30 +1046,30 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AIG</t>
+          <t>ABBV</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>75.09</v>
+        <v>262.85</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1090,44 +1083,44 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>68.8</v>
+        <v>73.5</v>
       </c>
       <c r="J7" t="n">
-        <v>49.1</v>
+        <v>53.8</v>
       </c>
       <c r="K7" t="n">
+        <v>14</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="M7" t="n">
         <v>17</v>
       </c>
-      <c r="L7" t="n">
-        <v>1.96</v>
-      </c>
-      <c r="M7" t="n">
-        <v>17.9</v>
-      </c>
       <c r="N7" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>47</v>
+        <v>62.3</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -1137,23 +1130,23 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>TTM Squeeze</t>
+          <t>Divergence, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AZN</t>
+          <t>AIG</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>158.13</v>
+        <v>75.25</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1182,26 +1175,26 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>63.8</v>
+        <v>70</v>
       </c>
       <c r="J8" t="n">
-        <v>39.6</v>
+        <v>49.8</v>
       </c>
       <c r="K8" t="n">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="L8" t="n">
-        <v>2.02</v>
+        <v>1.97</v>
       </c>
       <c r="M8" t="n">
-        <v>22.3</v>
+        <v>18.1</v>
       </c>
       <c r="N8" t="n">
-        <v>17.5</v>
+        <v>21.2</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1209,21 +1202,21 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>39.5</v>
+        <v>47.4</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -1233,42 +1226,42 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ABNB</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>160.54</v>
+        <v>728.0599999999999</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1278,26 +1271,26 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>58.6</v>
+        <v>61.9</v>
       </c>
       <c r="J9" t="n">
-        <v>43.4</v>
+        <v>61.5</v>
       </c>
       <c r="K9" t="n">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="L9" t="n">
-        <v>3.36</v>
+        <v>3.51</v>
       </c>
       <c r="M9" t="n">
-        <v>35.9</v>
+        <v>47.5</v>
       </c>
       <c r="N9" t="n">
-        <v>40.5</v>
+        <v>76.7</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1305,7 +1298,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>53.6</v>
+        <v>61.1</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1314,12 +1307,12 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1337,15 +1330,15 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TMO</t>
+          <t>AZN</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>658.71</v>
+        <v>156.99</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1360,44 +1353,44 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>57.4</v>
+        <v>58.2</v>
       </c>
       <c r="J10" t="n">
-        <v>59</v>
+        <v>38</v>
       </c>
       <c r="K10" t="n">
-        <v>82</v>
+        <v>38</v>
       </c>
       <c r="L10" t="n">
-        <v>2.4</v>
+        <v>1.99</v>
       </c>
       <c r="M10" t="n">
-        <v>23.4</v>
+        <v>22.5</v>
       </c>
       <c r="N10" t="n">
-        <v>27.7</v>
+        <v>18.4</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>68.90000000000001</v>
+        <v>38.9</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1411,12 +1404,12 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1437,7 +1430,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>615.5599999999999</v>
+        <v>632.13</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1470,22 +1463,22 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>57.1</v>
+        <v>57.9</v>
       </c>
       <c r="J11" t="n">
-        <v>66.90000000000001</v>
+        <v>69.8</v>
       </c>
       <c r="K11" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="L11" t="n">
-        <v>3.71</v>
+        <v>3.76</v>
       </c>
       <c r="M11" t="n">
-        <v>51.3</v>
+        <v>51.5</v>
       </c>
       <c r="N11" t="n">
-        <v>23.9</v>
+        <v>24.3</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1493,7 +1486,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>68.59999999999999</v>
+        <v>71.2</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1525,11 +1518,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BKNG</t>
+          <t>PNC</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>160.93</v>
+        <v>221.24</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1558,34 +1551,34 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>54.3</v>
+        <v>57.2</v>
       </c>
       <c r="J12" t="n">
-        <v>31.9</v>
+        <v>28.3</v>
       </c>
       <c r="K12" t="n">
-        <v>72</v>
+        <v>99</v>
       </c>
       <c r="L12" t="n">
-        <v>3.63</v>
+        <v>2.02</v>
       </c>
       <c r="M12" t="n">
-        <v>35.2</v>
+        <v>17.9</v>
       </c>
       <c r="N12" t="n">
-        <v>45.3</v>
+        <v>19</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>39.2</v>
+        <v>41.8</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1617,11 +1610,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AON</t>
+          <t>D</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>276.49</v>
+        <v>61.22</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1654,22 +1647,22 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>52.5</v>
+        <v>54.5</v>
       </c>
       <c r="J13" t="n">
-        <v>27.8</v>
+        <v>34.3</v>
       </c>
       <c r="K13" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="L13" t="n">
-        <v>2.5</v>
+        <v>1.78</v>
       </c>
       <c r="M13" t="n">
-        <v>35.8</v>
+        <v>13.8</v>
       </c>
       <c r="N13" t="n">
-        <v>88.40000000000001</v>
+        <v>2.9</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1677,7 +1670,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>29.4</v>
+        <v>40.2</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1709,11 +1702,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>NEE</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>83.45999999999999</v>
+        <v>76.76000000000001</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1746,22 +1739,22 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>51.8</v>
+        <v>53.7</v>
       </c>
       <c r="J14" t="n">
-        <v>33.2</v>
+        <v>32.7</v>
       </c>
       <c r="K14" t="n">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="L14" t="n">
-        <v>1.56</v>
+        <v>1.77</v>
       </c>
       <c r="M14" t="n">
-        <v>14.2</v>
+        <v>15.2</v>
       </c>
       <c r="N14" t="n">
-        <v>15.6</v>
+        <v>12.9</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1769,7 +1762,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>33.8</v>
+        <v>33.9</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1801,11 +1794,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CMCSA</t>
+          <t>AON</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>21.76</v>
+        <v>270.95</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1838,22 +1831,19 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>49.4</v>
+        <v>53.3</v>
       </c>
       <c r="J15" t="n">
-        <v>28.3</v>
+        <v>25.4</v>
       </c>
       <c r="K15" t="n">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="L15" t="n">
-        <v>2.75</v>
+        <v>2.58</v>
       </c>
       <c r="M15" t="n">
-        <v>29.7</v>
-      </c>
-      <c r="N15" t="n">
-        <v>26.9</v>
+        <v>32</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1861,7 +1851,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>36.4</v>
+        <v>28.2</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1883,25 +1873,29 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr"/>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PSX</t>
+          <t>PAYX</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>263.95</v>
+        <v>99.09</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -1916,41 +1910,41 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>47.8</v>
+        <v>52.4</v>
       </c>
       <c r="J16" t="n">
-        <v>62.5</v>
+        <v>25.4</v>
       </c>
       <c r="K16" t="n">
-        <v>12</v>
+        <v>98</v>
       </c>
       <c r="L16" t="n">
-        <v>3.37</v>
+        <v>2.99</v>
       </c>
       <c r="M16" t="n">
-        <v>45.2</v>
+        <v>31.8</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>72.7</v>
+        <v>40.4</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1964,7 +1958,7 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
@@ -1972,11 +1966,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr">
         <is>
           <t>No</t>
@@ -1986,11 +1976,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>XLF</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>48.66</v>
+        <v>53.51</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -2023,22 +2013,19 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>46.8</v>
+        <v>52.1</v>
       </c>
       <c r="J17" t="n">
-        <v>31.9</v>
+        <v>27.7</v>
       </c>
       <c r="K17" t="n">
-        <v>86</v>
+        <v>99</v>
       </c>
       <c r="L17" t="n">
-        <v>3.14</v>
+        <v>1.31</v>
       </c>
       <c r="M17" t="n">
-        <v>35.3</v>
-      </c>
-      <c r="N17" t="n">
-        <v>39.7</v>
+        <v>17.1</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2046,7 +2033,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>46.2</v>
+        <v>44.4</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2078,11 +2065,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CMG</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>32.06</v>
+        <v>83.68000000000001</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2115,22 +2102,22 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>46.3</v>
+        <v>51.1</v>
       </c>
       <c r="J18" t="n">
-        <v>36.2</v>
+        <v>34.9</v>
       </c>
       <c r="K18" t="n">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="L18" t="n">
-        <v>3.37</v>
+        <v>1.5</v>
       </c>
       <c r="M18" t="n">
-        <v>33.6</v>
+        <v>14.2</v>
       </c>
       <c r="N18" t="n">
-        <v>28.2</v>
+        <v>15.8</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -2138,7 +2125,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>44.5</v>
+        <v>34.5</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2147,17 +2134,17 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
@@ -2170,11 +2157,11 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>FDX</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>286.12</v>
+        <v>191.09</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2207,30 +2194,27 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>45.6</v>
+        <v>49.5</v>
       </c>
       <c r="J19" t="n">
-        <v>34.5</v>
+        <v>31.7</v>
       </c>
       <c r="K19" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="L19" t="n">
-        <v>2.23</v>
+        <v>2.35</v>
       </c>
       <c r="M19" t="n">
-        <v>25.1</v>
-      </c>
-      <c r="N19" t="n">
-        <v>29.3</v>
+        <v>34.4</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>42</v>
+        <v>42.3</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2262,11 +2246,11 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SBUX</t>
+          <t>SRE</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>94.25</v>
+        <v>78.39</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2295,26 +2279,26 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>45.6</v>
+        <v>49.4</v>
       </c>
       <c r="J20" t="n">
-        <v>32.4</v>
+        <v>37.9</v>
       </c>
       <c r="K20" t="n">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="L20" t="n">
-        <v>2.02</v>
+        <v>1.74</v>
       </c>
       <c r="M20" t="n">
-        <v>20.2</v>
+        <v>25.6</v>
       </c>
       <c r="N20" t="n">
-        <v>2.8</v>
+        <v>84.7</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2322,7 +2306,7 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>41.6</v>
+        <v>35.6</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2331,17 +2315,17 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U20" t="inlineStr"/>
@@ -2354,11 +2338,11 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>BKR</t>
+          <t>CMCSA</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>55.83</v>
+        <v>21.5</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2387,26 +2371,26 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>44.3</v>
+        <v>49.2</v>
       </c>
       <c r="J21" t="n">
-        <v>36.5</v>
+        <v>26.7</v>
       </c>
       <c r="K21" t="n">
-        <v>74</v>
+        <v>95</v>
       </c>
       <c r="L21" t="n">
-        <v>2.75</v>
+        <v>2.74</v>
       </c>
       <c r="M21" t="n">
-        <v>28.1</v>
+        <v>29.6</v>
       </c>
       <c r="N21" t="n">
-        <v>35.3</v>
+        <v>26.8</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2414,7 +2398,7 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>44.5</v>
+        <v>35.7</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2446,15 +2430,15 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>TMUS</t>
+          <t>PSX</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>161.74</v>
+        <v>265.98</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -2469,44 +2453,44 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>43.8</v>
+        <v>48.5</v>
       </c>
       <c r="J22" t="n">
-        <v>33.9</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="K22" t="n">
-        <v>98</v>
+        <v>13</v>
       </c>
       <c r="L22" t="n">
-        <v>2.47</v>
+        <v>3.49</v>
       </c>
       <c r="M22" t="n">
-        <v>29.1</v>
+        <v>27</v>
       </c>
       <c r="N22" t="n">
-        <v>34.3</v>
+        <v>22.1</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P22" t="n">
-        <v>34.3</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
@@ -2520,7 +2504,7 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
@@ -2528,7 +2512,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U22" t="inlineStr"/>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V22" t="inlineStr">
         <is>
           <t>No</t>
@@ -2538,11 +2526,11 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>AXP</t>
+          <t>EXC</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>300.8</v>
+        <v>40.65</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -2575,19 +2563,19 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>42.5</v>
+        <v>48.1</v>
       </c>
       <c r="J23" t="n">
-        <v>30.7</v>
+        <v>32</v>
       </c>
       <c r="K23" t="n">
-        <v>85</v>
+        <v>98</v>
       </c>
       <c r="L23" t="n">
-        <v>1.91</v>
+        <v>1.67</v>
       </c>
       <c r="M23" t="n">
-        <v>20</v>
+        <v>15.6</v>
       </c>
       <c r="N23" t="n">
         <v>14.1</v>
@@ -2598,7 +2586,7 @@
         </is>
       </c>
       <c r="P23" t="n">
-        <v>37.1</v>
+        <v>34.7</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -2607,38 +2595,34 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr"/>
       <c r="V23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ROP</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>362.4</v>
+        <v>48.95</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -2671,30 +2655,30 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>42.5</v>
+        <v>47.9</v>
       </c>
       <c r="J24" t="n">
-        <v>39.2</v>
+        <v>33.8</v>
       </c>
       <c r="K24" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="L24" t="n">
-        <v>2.62</v>
+        <v>3.17</v>
       </c>
       <c r="M24" t="n">
-        <v>24.7</v>
+        <v>35.4</v>
       </c>
       <c r="N24" t="n">
-        <v>36.7</v>
+        <v>40.1</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P24" t="n">
-        <v>45.2</v>
+        <v>46.6</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -2703,17 +2687,17 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U24" t="inlineStr"/>
@@ -2726,30 +2710,30 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>TMO</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>68.11</v>
+        <v>654.16</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2759,34 +2743,34 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>41</v>
+        <v>47.9</v>
       </c>
       <c r="J25" t="n">
-        <v>32.9</v>
+        <v>56.4</v>
       </c>
       <c r="K25" t="n">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="L25" t="n">
-        <v>2.77</v>
+        <v>2.37</v>
       </c>
       <c r="M25" t="n">
-        <v>33.5</v>
+        <v>23.7</v>
       </c>
       <c r="N25" t="n">
-        <v>43</v>
+        <v>28.6</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P25" t="n">
-        <v>34.5</v>
+        <v>67.7</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
@@ -2800,12 +2784,12 @@
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U25" t="inlineStr"/>
@@ -2818,11 +2802,11 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CHTR</t>
+          <t>USB</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>112.1</v>
+        <v>57.6</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -2855,30 +2839,30 @@
         </is>
       </c>
       <c r="I26" t="n">
-        <v>36.7</v>
+        <v>47.1</v>
       </c>
       <c r="J26" t="n">
-        <v>30.8</v>
+        <v>34.8</v>
       </c>
       <c r="K26" t="n">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="L26" t="n">
-        <v>4.64</v>
+        <v>1.9</v>
       </c>
       <c r="M26" t="n">
-        <v>55.9</v>
+        <v>19.1</v>
       </c>
       <c r="N26" t="n">
-        <v>49.5</v>
+        <v>20.8</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P26" t="n">
-        <v>31.6</v>
+        <v>47.2</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
@@ -2902,6 +2886,1380 @@
       </c>
       <c r="U26" t="inlineStr"/>
       <c r="V26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>224.16</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="J27" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="K27" t="n">
+        <v>99</v>
+      </c>
+      <c r="L27" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="M27" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="N27" t="n">
+        <v>49.4</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="P27" t="n">
+        <v>42.6</v>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr"/>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>BKNG</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>159.12</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>46.1</v>
+      </c>
+      <c r="J28" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="K28" t="n">
+        <v>64</v>
+      </c>
+      <c r="L28" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="M28" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="N28" t="n">
+        <v>45.4</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P28" t="n">
+        <v>38.6</v>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>DUK</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>113.91</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="J29" t="n">
+        <v>31</v>
+      </c>
+      <c r="K29" t="n">
+        <v>97</v>
+      </c>
+      <c r="L29" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="M29" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P29" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr"/>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>TMUS</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>164</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>45.3</v>
+      </c>
+      <c r="J30" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="K30" t="n">
+        <v>95</v>
+      </c>
+      <c r="L30" t="n">
+        <v>2.42</v>
+      </c>
+      <c r="M30" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="N30" t="n">
+        <v>35.6</v>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P30" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr"/>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>CMG</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>32.12</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>44</v>
+      </c>
+      <c r="J31" t="n">
+        <v>37.4</v>
+      </c>
+      <c r="K31" t="n">
+        <v>83</v>
+      </c>
+      <c r="L31" t="n">
+        <v>3.29</v>
+      </c>
+      <c r="M31" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="N31" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P31" t="n">
+        <v>44.7</v>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr"/>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>FDX</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>288.49</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>42.1</v>
+      </c>
+      <c r="J32" t="n">
+        <v>37.3</v>
+      </c>
+      <c r="K32" t="n">
+        <v>85</v>
+      </c>
+      <c r="L32" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="M32" t="n">
+        <v>41.8</v>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P32" t="n">
+        <v>43.2</v>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr"/>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>GS</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>902.74</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>42</v>
+      </c>
+      <c r="J33" t="n">
+        <v>32.2</v>
+      </c>
+      <c r="K33" t="n">
+        <v>99</v>
+      </c>
+      <c r="L33" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="M33" t="n">
+        <v>28</v>
+      </c>
+      <c r="N33" t="n">
+        <v>26.1</v>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P33" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr"/>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>BKR</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>55.96</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="J34" t="n">
+        <v>37.4</v>
+      </c>
+      <c r="K34" t="n">
+        <v>70</v>
+      </c>
+      <c r="L34" t="n">
+        <v>2.61</v>
+      </c>
+      <c r="M34" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="N34" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="P34" t="n">
+        <v>44.7</v>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr"/>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>CPRT</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>41.2</v>
+      </c>
+      <c r="J35" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="K35" t="n">
+        <v>97</v>
+      </c>
+      <c r="L35" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="M35" t="n">
+        <v>32.8</v>
+      </c>
+      <c r="N35" t="n">
+        <v>56.6</v>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P35" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr"/>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>SBUX</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>94.56</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="J36" t="n">
+        <v>34.7</v>
+      </c>
+      <c r="K36" t="n">
+        <v>60</v>
+      </c>
+      <c r="L36" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="M36" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="N36" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P36" t="n">
+        <v>42</v>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr"/>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>331.48</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>39.8</v>
+      </c>
+      <c r="J37" t="n">
+        <v>33.8</v>
+      </c>
+      <c r="K37" t="n">
+        <v>84</v>
+      </c>
+      <c r="L37" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="M37" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="N37" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P37" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr"/>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>ROP</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>355.6</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="J38" t="n">
+        <v>35.6</v>
+      </c>
+      <c r="K38" t="n">
+        <v>69</v>
+      </c>
+      <c r="L38" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="M38" t="n">
+        <v>25</v>
+      </c>
+      <c r="N38" t="n">
+        <v>37.3</v>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P38" t="n">
+        <v>43.1</v>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr"/>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>AXP</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>302.96</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="J39" t="n">
+        <v>33.1</v>
+      </c>
+      <c r="K39" t="n">
+        <v>78</v>
+      </c>
+      <c r="L39" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="M39" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="N39" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P39" t="n">
+        <v>37.9</v>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr"/>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>67.11</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="J40" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="K40" t="n">
+        <v>85</v>
+      </c>
+      <c r="L40" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="M40" t="n">
+        <v>33.7</v>
+      </c>
+      <c r="N40" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P40" t="n">
+        <v>33.7</v>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr"/>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>CHTR</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>109.15</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="J41" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="K41" t="n">
+        <v>91</v>
+      </c>
+      <c r="L41" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="M41" t="n">
+        <v>55.4</v>
+      </c>
+      <c r="N41" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P41" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr"/>
+      <c r="V41" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 05.10.2026 21:26 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>270.7</v>
+        <v>293.69</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,22 +614,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>79.7</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>69.59999999999999</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="K2" t="n">
         <v>100</v>
       </c>
       <c r="L2" t="n">
-        <v>4.17</v>
+        <v>4.55</v>
       </c>
       <c r="M2" t="n">
-        <v>50</v>
+        <v>53.6</v>
       </c>
       <c r="N2" t="n">
-        <v>43.2</v>
+        <v>49.8</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>78.40000000000001</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -669,11 +669,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>134.88</v>
+        <v>112.82</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -706,22 +706,22 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>78.3</v>
+        <v>80.3</v>
       </c>
       <c r="J3" t="n">
-        <v>50.9</v>
+        <v>59.5</v>
       </c>
       <c r="K3" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="L3" t="n">
-        <v>4.26</v>
+        <v>2.13</v>
       </c>
       <c r="M3" t="n">
-        <v>55.5</v>
+        <v>26.7</v>
       </c>
       <c r="N3" t="n">
-        <v>47.4</v>
+        <v>29.3</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -729,21 +729,21 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>57.4</v>
+        <v>57.6</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -753,7 +753,7 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>TTM Squeeze</t>
+          <t>Squeeze Expanding</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -765,30 +765,30 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ROST</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>227.79</v>
+        <v>136.08</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -802,22 +802,22 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>76.7</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>42.3</v>
+        <v>52.2</v>
       </c>
       <c r="K4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L4" t="n">
-        <v>2.16</v>
+        <v>4.14</v>
       </c>
       <c r="M4" t="n">
-        <v>23.8</v>
+        <v>55.6</v>
       </c>
       <c r="N4" t="n">
-        <v>38.3</v>
+        <v>47.6</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -825,11 +825,11 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>51.4</v>
+        <v>57.9</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -839,7 +839,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -849,42 +849,42 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>Divergence, Squeeze Expanding</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>TEAM</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>67.22</v>
+        <v>196.65</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -898,22 +898,22 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>75</v>
+        <v>78.2</v>
       </c>
       <c r="J5" t="n">
-        <v>43.6</v>
+        <v>61.3</v>
       </c>
       <c r="K5" t="n">
         <v>8</v>
       </c>
       <c r="L5" t="n">
-        <v>1.82</v>
+        <v>4.76</v>
       </c>
       <c r="M5" t="n">
-        <v>19.5</v>
+        <v>57.9</v>
       </c>
       <c r="N5" t="n">
-        <v>31</v>
+        <v>35.9</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -921,7 +921,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>50</v>
+        <v>72</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -930,12 +930,12 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -957,11 +957,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TEAM</t>
+          <t>ABBV</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>187.46</v>
+        <v>265.76</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -994,19 +994,22 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>74.90000000000001</v>
+        <v>75</v>
       </c>
       <c r="J6" t="n">
-        <v>55.7</v>
+        <v>58.4</v>
       </c>
       <c r="K6" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L6" t="n">
-        <v>4.85</v>
+        <v>1.97</v>
       </c>
       <c r="M6" t="n">
-        <v>72.90000000000001</v>
+        <v>16.9</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1014,7 +1017,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>69.90000000000001</v>
+        <v>63.6</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1023,12 +1026,12 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1046,30 +1049,30 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ABBV</t>
+          <t>ROST</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>262.85</v>
+        <v>226.37</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1083,22 +1086,19 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>73.5</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="J7" t="n">
-        <v>53.8</v>
+        <v>40.4</v>
       </c>
       <c r="K7" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="L7" t="n">
-        <v>1.83</v>
+        <v>2.26</v>
       </c>
       <c r="M7" t="n">
-        <v>17</v>
-      </c>
-      <c r="N7" t="n">
-        <v>0</v>
+        <v>29.9</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1106,7 +1106,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>62.3</v>
+        <v>50.5</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -1142,15 +1142,15 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AIG</t>
+          <t>WBD</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>75.25</v>
+        <v>30.95</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1165,48 +1165,45 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>70</v>
+        <v>67.3</v>
       </c>
       <c r="J8" t="n">
-        <v>49.8</v>
+        <v>75.2</v>
       </c>
       <c r="K8" t="n">
-        <v>17</v>
+        <v>99</v>
       </c>
       <c r="L8" t="n">
-        <v>1.97</v>
+        <v>0.75</v>
       </c>
       <c r="M8" t="n">
-        <v>18.1</v>
-      </c>
-      <c r="N8" t="n">
-        <v>21.2</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>47.4</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -1216,7 +1213,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -1224,11 +1221,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+      <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
           <t>No</t>
@@ -1238,30 +1231,30 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>AMP</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>728.0599999999999</v>
+        <v>494.94</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1275,30 +1268,30 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>61.9</v>
+        <v>59.1</v>
       </c>
       <c r="J9" t="n">
-        <v>61.5</v>
+        <v>33.7</v>
       </c>
       <c r="K9" t="n">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="L9" t="n">
-        <v>3.51</v>
+        <v>2.53</v>
       </c>
       <c r="M9" t="n">
-        <v>47.5</v>
+        <v>24.4</v>
       </c>
       <c r="N9" t="n">
-        <v>76.7</v>
+        <v>33.6</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>61.1</v>
+        <v>46</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1312,12 +1305,12 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
@@ -1330,15 +1323,15 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AZN</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>156.99</v>
+        <v>741.9</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1353,12 +1346,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1367,30 +1360,30 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>58.2</v>
+        <v>57.2</v>
       </c>
       <c r="J10" t="n">
-        <v>38</v>
+        <v>64</v>
       </c>
       <c r="K10" t="n">
-        <v>38</v>
+        <v>77</v>
       </c>
       <c r="L10" t="n">
-        <v>1.99</v>
+        <v>3.34</v>
       </c>
       <c r="M10" t="n">
-        <v>22.5</v>
+        <v>47.6</v>
       </c>
       <c r="N10" t="n">
-        <v>18.4</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>38.9</v>
+        <v>62.3</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1404,52 +1397,48 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>CCI</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>632.13</v>
+        <v>67.58</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1459,34 +1448,34 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>57.9</v>
+        <v>55.4</v>
       </c>
       <c r="J11" t="n">
-        <v>69.8</v>
+        <v>34.7</v>
       </c>
       <c r="K11" t="n">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="L11" t="n">
-        <v>3.76</v>
+        <v>2.79</v>
       </c>
       <c r="M11" t="n">
-        <v>51.5</v>
+        <v>22.1</v>
       </c>
       <c r="N11" t="n">
-        <v>24.3</v>
+        <v>21.8</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>71.2</v>
+        <v>32.9</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1495,12 +1484,12 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1518,11 +1507,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PNC</t>
+          <t>XLF</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>221.24</v>
+        <v>53.88</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1555,22 +1544,19 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>57.2</v>
+        <v>55.4</v>
       </c>
       <c r="J12" t="n">
-        <v>28.3</v>
+        <v>33.4</v>
       </c>
       <c r="K12" t="n">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="L12" t="n">
-        <v>2.02</v>
+        <v>1.29</v>
       </c>
       <c r="M12" t="n">
-        <v>17.9</v>
-      </c>
-      <c r="N12" t="n">
-        <v>19</v>
+        <v>18.3</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1578,7 +1564,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>41.8</v>
+        <v>46.4</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1587,17 +1573,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
@@ -1610,11 +1596,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>NEE</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>61.22</v>
+        <v>76.28</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1647,22 +1633,22 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>54.5</v>
+        <v>54.4</v>
       </c>
       <c r="J13" t="n">
-        <v>34.3</v>
+        <v>31.2</v>
       </c>
       <c r="K13" t="n">
         <v>86</v>
       </c>
       <c r="L13" t="n">
-        <v>1.78</v>
+        <v>1.73</v>
       </c>
       <c r="M13" t="n">
-        <v>13.8</v>
+        <v>14.7</v>
       </c>
       <c r="N13" t="n">
-        <v>2.9</v>
+        <v>11.2</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1670,7 +1656,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>40.2</v>
+        <v>33.3</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1702,11 +1688,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>NEE</t>
+          <t>CMG</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>76.76000000000001</v>
+        <v>30.85</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1739,22 +1725,22 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>53.7</v>
+        <v>54.3</v>
       </c>
       <c r="J14" t="n">
-        <v>32.7</v>
+        <v>31.4</v>
       </c>
       <c r="K14" t="n">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="L14" t="n">
-        <v>1.77</v>
+        <v>3.9</v>
       </c>
       <c r="M14" t="n">
-        <v>15.2</v>
+        <v>32.4</v>
       </c>
       <c r="N14" t="n">
-        <v>12.9</v>
+        <v>25.4</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1762,7 +1748,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>33.9</v>
+        <v>42.4</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1771,34 +1757,38 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr"/>
-      <c r="V14" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>AON</t>
+          <t>PNC</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>270.95</v>
+        <v>220.28</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1831,27 +1821,30 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>53.3</v>
+        <v>53.8</v>
       </c>
       <c r="J15" t="n">
-        <v>25.4</v>
+        <v>26.9</v>
       </c>
       <c r="K15" t="n">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="L15" t="n">
-        <v>2.58</v>
+        <v>1.94</v>
       </c>
       <c r="M15" t="n">
-        <v>32</v>
+        <v>17.7</v>
+      </c>
+      <c r="N15" t="n">
+        <v>17.6</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>28.2</v>
+        <v>41.2</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1873,25 +1866,21 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PAYX</t>
+          <t>D</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>99.09</v>
+        <v>61.02</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1924,19 +1913,22 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>52.4</v>
+        <v>53.7</v>
       </c>
       <c r="J16" t="n">
-        <v>25.4</v>
+        <v>33.7</v>
       </c>
       <c r="K16" t="n">
-        <v>98</v>
+        <v>83</v>
       </c>
       <c r="L16" t="n">
-        <v>2.99</v>
+        <v>1.74</v>
       </c>
       <c r="M16" t="n">
-        <v>31.8</v>
+        <v>13.6</v>
+      </c>
+      <c r="N16" t="n">
+        <v>2</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1944,7 +1936,7 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>40.4</v>
+        <v>39.8</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1953,17 +1945,17 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
@@ -1976,11 +1968,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>XLF</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>53.51</v>
+        <v>83.79000000000001</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -2013,27 +2005,27 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>52.1</v>
+        <v>53.3</v>
       </c>
       <c r="J17" t="n">
-        <v>27.7</v>
+        <v>35.8</v>
       </c>
       <c r="K17" t="n">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="L17" t="n">
-        <v>1.31</v>
+        <v>1.49</v>
       </c>
       <c r="M17" t="n">
-        <v>17.1</v>
+        <v>24.9</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>44.4</v>
+        <v>34.8</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2042,17 +2034,17 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
@@ -2065,11 +2057,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>EXC</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>83.68000000000001</v>
+        <v>40.82</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2102,30 +2094,30 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>51.1</v>
+        <v>52.8</v>
       </c>
       <c r="J18" t="n">
-        <v>34.9</v>
+        <v>34.8</v>
       </c>
       <c r="K18" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="L18" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="M18" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="N18" t="n">
         <v>1.5</v>
       </c>
-      <c r="M18" t="n">
-        <v>14.2</v>
-      </c>
-      <c r="N18" t="n">
-        <v>15.8</v>
-      </c>
       <c r="O18" t="inlineStr">
         <is>
           <t>Bearish</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>34.5</v>
+        <v>35.6</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2157,15 +2149,15 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>PSX</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>191.09</v>
+        <v>269.72</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -2180,33 +2172,36 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>49.5</v>
+        <v>52.3</v>
       </c>
       <c r="J19" t="n">
-        <v>31.7</v>
+        <v>67</v>
       </c>
       <c r="K19" t="n">
-        <v>99</v>
+        <v>15</v>
       </c>
       <c r="L19" t="n">
-        <v>2.35</v>
+        <v>3.45</v>
       </c>
       <c r="M19" t="n">
-        <v>34.4</v>
+        <v>27.2</v>
+      </c>
+      <c r="N19" t="n">
+        <v>24</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -2214,7 +2209,7 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>42.3</v>
+        <v>74</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2223,12 +2218,12 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
@@ -2236,7 +2231,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr"/>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V19" t="inlineStr">
         <is>
           <t>No</t>
@@ -2246,11 +2245,11 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SRE</t>
+          <t>WFC</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>78.39</v>
+        <v>81.44</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2283,22 +2282,22 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>49.4</v>
+        <v>50.9</v>
       </c>
       <c r="J20" t="n">
-        <v>37.9</v>
+        <v>38.7</v>
       </c>
       <c r="K20" t="n">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="L20" t="n">
-        <v>1.74</v>
+        <v>2.15</v>
       </c>
       <c r="M20" t="n">
-        <v>25.6</v>
+        <v>23.7</v>
       </c>
       <c r="N20" t="n">
-        <v>84.7</v>
+        <v>42.2</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2306,7 +2305,7 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>35.6</v>
+        <v>45.8</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2315,17 +2314,17 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U20" t="inlineStr"/>
@@ -2338,11 +2337,11 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CMCSA</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>21.5</v>
+        <v>50.28</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2371,34 +2370,34 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>49.2</v>
+        <v>50.7</v>
       </c>
       <c r="J21" t="n">
-        <v>26.7</v>
+        <v>41.8</v>
       </c>
       <c r="K21" t="n">
-        <v>95</v>
+        <v>79</v>
       </c>
       <c r="L21" t="n">
-        <v>2.74</v>
+        <v>3.16</v>
       </c>
       <c r="M21" t="n">
-        <v>29.6</v>
+        <v>36.6</v>
       </c>
       <c r="N21" t="n">
-        <v>26.8</v>
+        <v>45.5</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>35.7</v>
+        <v>49</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2430,15 +2429,15 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>PSX</t>
+          <t>BAC</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>265.98</v>
+        <v>54</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -2453,44 +2452,44 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>48.5</v>
+        <v>50</v>
       </c>
       <c r="J22" t="n">
-        <v>64.09999999999999</v>
+        <v>24.8</v>
       </c>
       <c r="K22" t="n">
-        <v>13</v>
+        <v>98</v>
       </c>
       <c r="L22" t="n">
-        <v>3.49</v>
+        <v>1.92</v>
       </c>
       <c r="M22" t="n">
-        <v>27</v>
+        <v>22.6</v>
       </c>
       <c r="N22" t="n">
-        <v>22.1</v>
+        <v>54.7</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P22" t="n">
-        <v>73.09999999999999</v>
+        <v>42.2</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
@@ -2504,7 +2503,7 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
@@ -2512,11 +2511,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t>Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U22" t="inlineStr"/>
       <c r="V22" t="inlineStr">
         <is>
           <t>No</t>
@@ -2526,11 +2521,11 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>EXC</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>40.65</v>
+        <v>190.19</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -2563,30 +2558,30 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>48.1</v>
+        <v>50</v>
       </c>
       <c r="J23" t="n">
-        <v>32</v>
+        <v>29.9</v>
       </c>
       <c r="K23" t="n">
         <v>98</v>
       </c>
       <c r="L23" t="n">
-        <v>1.67</v>
+        <v>2.29</v>
       </c>
       <c r="M23" t="n">
-        <v>15.6</v>
+        <v>20.8</v>
       </c>
       <c r="N23" t="n">
-        <v>14.1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>34.7</v>
+        <v>41.7</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -2595,17 +2590,17 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U23" t="inlineStr"/>
@@ -2618,11 +2613,11 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>AON</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>48.95</v>
+        <v>272.05</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -2651,34 +2646,34 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I24" t="n">
-        <v>47.9</v>
+        <v>49.7</v>
       </c>
       <c r="J24" t="n">
-        <v>33.8</v>
+        <v>27.9</v>
       </c>
       <c r="K24" t="n">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="L24" t="n">
-        <v>3.17</v>
+        <v>2.52</v>
       </c>
       <c r="M24" t="n">
-        <v>35.4</v>
+        <v>35.7</v>
       </c>
       <c r="N24" t="n">
-        <v>40.1</v>
+        <v>88</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P24" t="n">
-        <v>46.6</v>
+        <v>29.3</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -2687,17 +2682,17 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U24" t="inlineStr"/>
@@ -2710,30 +2705,30 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>TMO</t>
+          <t>SRE</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>654.16</v>
+        <v>78.16</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2743,34 +2738,34 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>47.9</v>
+        <v>49.7</v>
       </c>
       <c r="J25" t="n">
-        <v>56.4</v>
+        <v>37</v>
       </c>
       <c r="K25" t="n">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="L25" t="n">
-        <v>2.37</v>
+        <v>1.69</v>
       </c>
       <c r="M25" t="n">
-        <v>23.7</v>
+        <v>21.1</v>
       </c>
       <c r="N25" t="n">
-        <v>28.6</v>
+        <v>56.7</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P25" t="n">
-        <v>67.7</v>
+        <v>35.3</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
@@ -2779,12 +2774,12 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
@@ -2802,11 +2797,11 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>USB</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>57.6</v>
+        <v>224.71</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -2839,30 +2834,30 @@
         </is>
       </c>
       <c r="I26" t="n">
-        <v>47.1</v>
+        <v>49.5</v>
       </c>
       <c r="J26" t="n">
-        <v>34.8</v>
+        <v>30.1</v>
       </c>
       <c r="K26" t="n">
-        <v>84</v>
+        <v>98</v>
       </c>
       <c r="L26" t="n">
-        <v>1.9</v>
+        <v>2.27</v>
       </c>
       <c r="M26" t="n">
-        <v>19.1</v>
+        <v>25.3</v>
       </c>
       <c r="N26" t="n">
-        <v>20.8</v>
+        <v>50</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P26" t="n">
-        <v>47.2</v>
+        <v>43.1</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
@@ -2894,11 +2889,11 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ALL</t>
+          <t>PAYX</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>224.16</v>
+        <v>99.78</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -2931,30 +2926,30 @@
         </is>
       </c>
       <c r="I27" t="n">
-        <v>46.4</v>
+        <v>49.2</v>
       </c>
       <c r="J27" t="n">
-        <v>28.7</v>
+        <v>27.9</v>
       </c>
       <c r="K27" t="n">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="L27" t="n">
-        <v>2.23</v>
+        <v>2.79</v>
       </c>
       <c r="M27" t="n">
-        <v>25.2</v>
+        <v>33.3</v>
       </c>
       <c r="N27" t="n">
-        <v>49.4</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P27" t="n">
-        <v>42.6</v>
+        <v>41.3</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
@@ -2986,11 +2981,11 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>BKNG</t>
+          <t>DUK</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>159.12</v>
+        <v>113.84</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -3019,26 +3014,26 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I28" t="n">
-        <v>46.1</v>
+        <v>46.6</v>
       </c>
       <c r="J28" t="n">
-        <v>30.5</v>
+        <v>31.5</v>
       </c>
       <c r="K28" t="n">
-        <v>64</v>
+        <v>96</v>
       </c>
       <c r="L28" t="n">
-        <v>3.5</v>
+        <v>1.26</v>
       </c>
       <c r="M28" t="n">
-        <v>35.2</v>
+        <v>11.4</v>
       </c>
       <c r="N28" t="n">
-        <v>45.4</v>
+        <v>0</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -3046,7 +3041,7 @@
         </is>
       </c>
       <c r="P28" t="n">
-        <v>38.6</v>
+        <v>36.5</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
@@ -3078,11 +3073,11 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>DUK</t>
+          <t>TMUS</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>113.91</v>
+        <v>164.64</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -3115,19 +3110,22 @@
         </is>
       </c>
       <c r="I29" t="n">
-        <v>45.9</v>
+        <v>44.7</v>
       </c>
       <c r="J29" t="n">
-        <v>31</v>
+        <v>39.8</v>
       </c>
       <c r="K29" t="n">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="L29" t="n">
-        <v>1.32</v>
+        <v>2.29</v>
       </c>
       <c r="M29" t="n">
-        <v>20.4</v>
+        <v>29.3</v>
+      </c>
+      <c r="N29" t="n">
+        <v>34.9</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -3135,7 +3133,7 @@
         </is>
       </c>
       <c r="P29" t="n">
-        <v>36.4</v>
+        <v>36.2</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
@@ -3167,11 +3165,11 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>TMUS</t>
+          <t>CMCSA</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>164</v>
+        <v>21.57</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -3204,22 +3202,22 @@
         </is>
       </c>
       <c r="I30" t="n">
-        <v>45.3</v>
+        <v>44.5</v>
       </c>
       <c r="J30" t="n">
-        <v>38.5</v>
+        <v>27.1</v>
       </c>
       <c r="K30" t="n">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="L30" t="n">
-        <v>2.42</v>
+        <v>2.56</v>
       </c>
       <c r="M30" t="n">
-        <v>29.5</v>
+        <v>28.9</v>
       </c>
       <c r="N30" t="n">
-        <v>35.6</v>
+        <v>24.3</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -3227,7 +3225,7 @@
         </is>
       </c>
       <c r="P30" t="n">
-        <v>35.4</v>
+        <v>35.9</v>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
@@ -3259,11 +3257,11 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CMG</t>
+          <t>FDX</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>32.12</v>
+        <v>289.13</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -3292,34 +3290,34 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I31" t="n">
-        <v>44</v>
+        <v>43.5</v>
       </c>
       <c r="J31" t="n">
-        <v>37.4</v>
+        <v>38.5</v>
       </c>
       <c r="K31" t="n">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="L31" t="n">
-        <v>3.29</v>
+        <v>2.13</v>
       </c>
       <c r="M31" t="n">
-        <v>33.3</v>
+        <v>25.6</v>
       </c>
       <c r="N31" t="n">
-        <v>27.4</v>
+        <v>31.1</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P31" t="n">
-        <v>44.7</v>
+        <v>43.6</v>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
@@ -3328,17 +3326,17 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U31" t="inlineStr"/>
@@ -3351,11 +3349,11 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>FDX</t>
+          <t>USB</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>288.49</v>
+        <v>57.27</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -3384,23 +3382,26 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I32" t="n">
-        <v>42.1</v>
+        <v>43.1</v>
       </c>
       <c r="J32" t="n">
-        <v>37.3</v>
+        <v>32.9</v>
       </c>
       <c r="K32" t="n">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="L32" t="n">
-        <v>2.09</v>
+        <v>1.82</v>
       </c>
       <c r="M32" t="n">
-        <v>41.8</v>
+        <v>19</v>
+      </c>
+      <c r="N32" t="n">
+        <v>19.9</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -3408,7 +3409,7 @@
         </is>
       </c>
       <c r="P32" t="n">
-        <v>43.2</v>
+        <v>46.3</v>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
@@ -3417,17 +3418,17 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U32" t="inlineStr"/>
@@ -3440,11 +3441,11 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>GS</t>
+          <t>SCHW</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>902.74</v>
+        <v>97.95999999999999</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -3480,27 +3481,27 @@
         <v>42</v>
       </c>
       <c r="J33" t="n">
-        <v>32.2</v>
+        <v>35.1</v>
       </c>
       <c r="K33" t="n">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="L33" t="n">
-        <v>2.41</v>
+        <v>2.11</v>
       </c>
       <c r="M33" t="n">
-        <v>28</v>
+        <v>25.9</v>
       </c>
       <c r="N33" t="n">
-        <v>26.1</v>
+        <v>52.2</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P33" t="n">
-        <v>38.3</v>
+        <v>46.7</v>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
@@ -3532,11 +3533,11 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>BKR</t>
+          <t>ROP</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>55.96</v>
+        <v>363.38</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -3569,30 +3570,30 @@
         </is>
       </c>
       <c r="I34" t="n">
-        <v>41.6</v>
+        <v>41.8</v>
       </c>
       <c r="J34" t="n">
-        <v>37.4</v>
+        <v>43</v>
       </c>
       <c r="K34" t="n">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="L34" t="n">
-        <v>2.61</v>
+        <v>2.65</v>
       </c>
       <c r="M34" t="n">
-        <v>27.2</v>
+        <v>26.4</v>
       </c>
       <c r="N34" t="n">
-        <v>30.8</v>
+        <v>41.5</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P34" t="n">
-        <v>44.7</v>
+        <v>46.2</v>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
@@ -3601,17 +3602,17 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U34" t="inlineStr"/>
@@ -3624,11 +3625,11 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>27.3</v>
+        <v>893.46</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -3661,22 +3662,22 @@
         </is>
       </c>
       <c r="I35" t="n">
-        <v>41.2</v>
+        <v>41.7</v>
       </c>
       <c r="J35" t="n">
-        <v>31.5</v>
+        <v>30.5</v>
       </c>
       <c r="K35" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="L35" t="n">
-        <v>2.6</v>
+        <v>2.38</v>
       </c>
       <c r="M35" t="n">
-        <v>32.8</v>
+        <v>25.3</v>
       </c>
       <c r="N35" t="n">
-        <v>56.6</v>
+        <v>14.9</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
@@ -3684,7 +3685,7 @@
         </is>
       </c>
       <c r="P35" t="n">
-        <v>35.3</v>
+        <v>37.2</v>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
@@ -3716,11 +3717,11 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SBUX</t>
+          <t>JPM</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>94.56</v>
+        <v>332.38</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -3749,34 +3750,34 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I36" t="n">
-        <v>40.6</v>
+        <v>41.4</v>
       </c>
       <c r="J36" t="n">
-        <v>34.7</v>
+        <v>34.5</v>
       </c>
       <c r="K36" t="n">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="L36" t="n">
-        <v>1.9</v>
+        <v>1.78</v>
       </c>
       <c r="M36" t="n">
-        <v>20.4</v>
+        <v>17.2</v>
       </c>
       <c r="N36" t="n">
-        <v>3.7</v>
+        <v>22.6</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P36" t="n">
-        <v>42</v>
+        <v>49.4</v>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
@@ -3785,17 +3786,17 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U36" t="inlineStr"/>
@@ -3808,11 +3809,11 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>JPM</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>331.48</v>
+        <v>27.65</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -3845,30 +3846,30 @@
         </is>
       </c>
       <c r="I37" t="n">
-        <v>39.8</v>
+        <v>41.1</v>
       </c>
       <c r="J37" t="n">
-        <v>33.8</v>
+        <v>35.8</v>
       </c>
       <c r="K37" t="n">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="L37" t="n">
-        <v>1.92</v>
+        <v>2.64</v>
       </c>
       <c r="M37" t="n">
-        <v>17.2</v>
+        <v>33.4</v>
       </c>
       <c r="N37" t="n">
-        <v>22.7</v>
+        <v>58.3</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P37" t="n">
-        <v>48.9</v>
+        <v>36.9</v>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
@@ -3900,11 +3901,11 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ROP</t>
+          <t>PCAR</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>355.6</v>
+        <v>109.36</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -3933,26 +3934,26 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I38" t="n">
-        <v>39.7</v>
+        <v>39</v>
       </c>
       <c r="J38" t="n">
-        <v>35.6</v>
+        <v>21.4</v>
       </c>
       <c r="K38" t="n">
-        <v>69</v>
+        <v>92</v>
       </c>
       <c r="L38" t="n">
-        <v>2.66</v>
+        <v>2.25</v>
       </c>
       <c r="M38" t="n">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="N38" t="n">
-        <v>37.3</v>
+        <v>0</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
@@ -3960,7 +3961,7 @@
         </is>
       </c>
       <c r="P38" t="n">
-        <v>43.1</v>
+        <v>35.9</v>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
@@ -3996,7 +3997,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>302.96</v>
+        <v>304.02</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -4029,22 +4030,22 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>39.3</v>
+        <v>38.3</v>
       </c>
       <c r="J39" t="n">
-        <v>33.1</v>
+        <v>34.9</v>
       </c>
       <c r="K39" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="L39" t="n">
-        <v>1.81</v>
+        <v>1.73</v>
       </c>
       <c r="M39" t="n">
-        <v>18.9</v>
+        <v>18.3</v>
       </c>
       <c r="N39" t="n">
-        <v>9.199999999999999</v>
+        <v>6.5</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
@@ -4052,7 +4053,7 @@
         </is>
       </c>
       <c r="P39" t="n">
-        <v>37.9</v>
+        <v>38.6</v>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
@@ -4084,11 +4085,11 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>CHTR</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>67.11</v>
+        <v>107.77</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -4121,22 +4122,22 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>36.5</v>
+        <v>36.1</v>
       </c>
       <c r="J40" t="n">
-        <v>31.1</v>
+        <v>27.4</v>
       </c>
       <c r="K40" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="L40" t="n">
-        <v>2.66</v>
+        <v>4.67</v>
       </c>
       <c r="M40" t="n">
-        <v>33.7</v>
+        <v>54.9</v>
       </c>
       <c r="N40" t="n">
-        <v>43.5</v>
+        <v>48.1</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
@@ -4144,7 +4145,7 @@
         </is>
       </c>
       <c r="P40" t="n">
-        <v>33.7</v>
+        <v>30.5</v>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
@@ -4176,11 +4177,11 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CHTR</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>109.15</v>
+        <v>67.5</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -4213,22 +4214,22 @@
         </is>
       </c>
       <c r="I41" t="n">
-        <v>34.9</v>
+        <v>35.5</v>
       </c>
       <c r="J41" t="n">
-        <v>28.3</v>
+        <v>32.8</v>
       </c>
       <c r="K41" t="n">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="L41" t="n">
-        <v>4.6</v>
+        <v>2.48</v>
       </c>
       <c r="M41" t="n">
-        <v>55.4</v>
+        <v>33.9</v>
       </c>
       <c r="N41" t="n">
-        <v>48.9</v>
+        <v>44</v>
       </c>
       <c r="O41" t="inlineStr">
         <is>
@@ -4236,7 +4237,7 @@
         </is>
       </c>
       <c r="P41" t="n">
-        <v>30.8</v>
+        <v>34.4</v>
       </c>
       <c r="Q41" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Scan 06.10.2026 19:24 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -448,7 +448,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
     <col width="6" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>293.69</v>
+        <v>275.43</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,22 +614,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>90.59999999999999</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>76.59999999999999</v>
+        <v>63.9</v>
       </c>
       <c r="K2" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L2" t="n">
-        <v>4.55</v>
+        <v>5.99</v>
       </c>
       <c r="M2" t="n">
-        <v>53.6</v>
+        <v>57.5</v>
       </c>
       <c r="N2" t="n">
-        <v>49.8</v>
+        <v>56.8</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>81.40000000000001</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -646,34 +646,38 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>ABBV</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>112.82</v>
+        <v>267.15</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -706,22 +710,22 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>80.3</v>
+        <v>80</v>
       </c>
       <c r="J3" t="n">
-        <v>59.5</v>
+        <v>60.4</v>
       </c>
       <c r="K3" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="L3" t="n">
-        <v>2.13</v>
+        <v>2.1</v>
       </c>
       <c r="M3" t="n">
-        <v>26.7</v>
+        <v>17</v>
       </c>
       <c r="N3" t="n">
-        <v>29.3</v>
+        <v>0.3</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -729,11 +733,11 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>57.6</v>
+        <v>64.2</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -743,17 +747,17 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Squeeze Expanding</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -765,11 +769,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>136.08</v>
+        <v>118.19</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -798,26 +802,23 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>80.09999999999999</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>52.2</v>
+        <v>68.8</v>
       </c>
       <c r="K4" t="n">
-        <v>1</v>
+        <v>39</v>
       </c>
       <c r="L4" t="n">
-        <v>4.14</v>
+        <v>2.38</v>
       </c>
       <c r="M4" t="n">
-        <v>55.6</v>
-      </c>
-      <c r="N4" t="n">
-        <v>47.6</v>
+        <v>31.5</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -825,21 +826,21 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>57.9</v>
+        <v>62</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -847,11 +848,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+      <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
         <is>
           <t>No</t>
@@ -861,30 +858,30 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TEAM</t>
+          <t>EW</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>196.65</v>
+        <v>86.44</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -898,22 +895,22 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>78.2</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>61.3</v>
+        <v>46.3</v>
       </c>
       <c r="K5" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="L5" t="n">
-        <v>4.76</v>
+        <v>2.37</v>
       </c>
       <c r="M5" t="n">
-        <v>57.9</v>
+        <v>23.9</v>
       </c>
       <c r="N5" t="n">
-        <v>35.9</v>
+        <v>40.8</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -921,11 +918,11 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>72</v>
+        <v>50.1</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -935,7 +932,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -945,7 +942,7 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>Squeeze Expanding</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
@@ -957,30 +954,30 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ABBV</t>
+          <t>DXCM</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>265.76</v>
+        <v>83.31</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -994,22 +991,22 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>75</v>
+        <v>69.3</v>
       </c>
       <c r="J6" t="n">
-        <v>58.4</v>
+        <v>38.7</v>
       </c>
       <c r="K6" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="L6" t="n">
-        <v>1.97</v>
+        <v>2.66</v>
       </c>
       <c r="M6" t="n">
-        <v>16.9</v>
+        <v>24.4</v>
       </c>
       <c r="N6" t="n">
-        <v>0</v>
+        <v>7.7</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1017,7 +1014,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>63.6</v>
+        <v>54.9</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1026,12 +1023,12 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1039,25 +1036,29 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr"/>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ROST</t>
+          <t>WBD</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>226.37</v>
+        <v>30.95</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -1072,33 +1073,33 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>71.59999999999999</v>
+        <v>67.3</v>
       </c>
       <c r="J7" t="n">
-        <v>40.4</v>
+        <v>75.2</v>
       </c>
       <c r="K7" t="n">
-        <v>10</v>
+        <v>99</v>
       </c>
       <c r="L7" t="n">
-        <v>2.26</v>
+        <v>0.75</v>
       </c>
       <c r="M7" t="n">
-        <v>29.9</v>
+        <v>4.7</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1106,7 +1107,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>50.5</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1115,12 +1116,12 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -1128,29 +1129,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>WBD</t>
+          <t>ROST</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>30.95</v>
+        <v>222.5</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1165,33 +1162,36 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>67.3</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="J8" t="n">
-        <v>75.2</v>
+        <v>35.9</v>
       </c>
       <c r="K8" t="n">
-        <v>99</v>
+        <v>11</v>
       </c>
       <c r="L8" t="n">
-        <v>0.75</v>
+        <v>2.3</v>
       </c>
       <c r="M8" t="n">
-        <v>9.800000000000001</v>
+        <v>19.8</v>
+      </c>
+      <c r="N8" t="n">
+        <v>23.3</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1199,7 +1199,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>71.09999999999999</v>
+        <v>48.4</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1208,12 +1208,12 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -1221,21 +1221,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr"/>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AMP</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>494.94</v>
+        <v>84.83</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1268,30 +1272,30 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>59.1</v>
+        <v>58</v>
       </c>
       <c r="J9" t="n">
-        <v>33.7</v>
+        <v>43.9</v>
       </c>
       <c r="K9" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="L9" t="n">
-        <v>2.53</v>
+        <v>1.47</v>
       </c>
       <c r="M9" t="n">
-        <v>24.4</v>
+        <v>12.2</v>
       </c>
       <c r="N9" t="n">
-        <v>33.6</v>
+        <v>0</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>46</v>
+        <v>37.9</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1300,17 +1304,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
@@ -1323,30 +1327,30 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>NEE</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>741.9</v>
+        <v>77.48</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1356,34 +1360,34 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>57.2</v>
+        <v>56.8</v>
       </c>
       <c r="J10" t="n">
-        <v>64</v>
+        <v>39.8</v>
       </c>
       <c r="K10" t="n">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="L10" t="n">
-        <v>3.34</v>
+        <v>1.7</v>
       </c>
       <c r="M10" t="n">
-        <v>47.6</v>
+        <v>15.5</v>
       </c>
       <c r="N10" t="n">
-        <v>76.90000000000001</v>
+        <v>14.4</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>62.3</v>
+        <v>35.9</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1392,12 +1396,12 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1415,11 +1419,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CCI</t>
+          <t>EXC</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>67.58</v>
+        <v>41.28</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1452,22 +1456,22 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>55.4</v>
+        <v>56.2</v>
       </c>
       <c r="J11" t="n">
-        <v>34.7</v>
+        <v>41.7</v>
       </c>
       <c r="K11" t="n">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="L11" t="n">
-        <v>2.79</v>
+        <v>1.65</v>
       </c>
       <c r="M11" t="n">
-        <v>22.1</v>
+        <v>13.6</v>
       </c>
       <c r="N11" t="n">
-        <v>21.8</v>
+        <v>0.6</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1475,7 +1479,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>32.9</v>
+        <v>38</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1484,17 +1488,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
@@ -1507,11 +1511,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>XLF</t>
+          <t>AMP</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>53.88</v>
+        <v>494.44</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1544,19 +1548,22 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>55.4</v>
+        <v>55.9</v>
       </c>
       <c r="J12" t="n">
         <v>33.4</v>
       </c>
       <c r="K12" t="n">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="L12" t="n">
-        <v>1.29</v>
+        <v>2.42</v>
       </c>
       <c r="M12" t="n">
-        <v>18.3</v>
+        <v>24.1</v>
+      </c>
+      <c r="N12" t="n">
+        <v>32.1</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1564,7 +1571,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>46.4</v>
+        <v>45.8</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1573,17 +1580,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
@@ -1596,11 +1603,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>NEE</t>
+          <t>XLF</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>76.28</v>
+        <v>53.99</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1633,30 +1640,27 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>54.4</v>
+        <v>54.9</v>
       </c>
       <c r="J13" t="n">
-        <v>31.2</v>
+        <v>35</v>
       </c>
       <c r="K13" t="n">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="L13" t="n">
-        <v>1.73</v>
+        <v>1.22</v>
       </c>
       <c r="M13" t="n">
-        <v>14.7</v>
-      </c>
-      <c r="N13" t="n">
-        <v>11.2</v>
+        <v>17.4</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>33.3</v>
+        <v>47</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1688,11 +1692,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CMG</t>
+          <t>CCI</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>30.85</v>
+        <v>68.19</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1725,22 +1729,22 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>54.3</v>
+        <v>53.8</v>
       </c>
       <c r="J14" t="n">
-        <v>31.4</v>
+        <v>38.3</v>
       </c>
       <c r="K14" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="L14" t="n">
-        <v>3.9</v>
+        <v>2.62</v>
       </c>
       <c r="M14" t="n">
-        <v>32.4</v>
+        <v>22</v>
       </c>
       <c r="N14" t="n">
-        <v>25.4</v>
+        <v>21.3</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1748,7 +1752,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>42.4</v>
+        <v>34.2</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1757,38 +1761,34 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PNC</t>
+          <t>SRE</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>220.28</v>
+        <v>79.23999999999999</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1821,30 +1821,30 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>53.8</v>
+        <v>53</v>
       </c>
       <c r="J15" t="n">
-        <v>26.9</v>
+        <v>43.4</v>
       </c>
       <c r="K15" t="n">
-        <v>98</v>
+        <v>81</v>
       </c>
       <c r="L15" t="n">
-        <v>1.94</v>
+        <v>1.68</v>
       </c>
       <c r="M15" t="n">
-        <v>17.7</v>
+        <v>20.6</v>
       </c>
       <c r="N15" t="n">
-        <v>17.6</v>
+        <v>53.6</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>41.2</v>
+        <v>37.5</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1853,17 +1853,17 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U15" t="inlineStr"/>
@@ -1876,11 +1876,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>PNC</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>61.02</v>
+        <v>220.06</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1913,30 +1913,30 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>53.7</v>
+        <v>51.4</v>
       </c>
       <c r="J16" t="n">
-        <v>33.7</v>
+        <v>26.7</v>
       </c>
       <c r="K16" t="n">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="L16" t="n">
-        <v>1.74</v>
+        <v>1.86</v>
       </c>
       <c r="M16" t="n">
-        <v>13.6</v>
+        <v>17.6</v>
       </c>
       <c r="N16" t="n">
-        <v>2</v>
+        <v>17.2</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>39.8</v>
+        <v>41.1</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1945,17 +1945,17 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
@@ -1968,11 +1968,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>PAYX</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>83.79000000000001</v>
+        <v>100.93</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -2005,19 +2005,22 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>53.3</v>
+        <v>50.9</v>
       </c>
       <c r="J17" t="n">
-        <v>35.8</v>
+        <v>31.5</v>
       </c>
       <c r="K17" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="L17" t="n">
-        <v>1.49</v>
+        <v>2.63</v>
       </c>
       <c r="M17" t="n">
-        <v>24.9</v>
+        <v>33.3</v>
+      </c>
+      <c r="N17" t="n">
+        <v>77.40000000000001</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2025,7 +2028,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>34.8</v>
+        <v>42.6</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2057,11 +2060,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>EXC</t>
+          <t>WFC</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>40.82</v>
+        <v>81.58</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2094,22 +2097,22 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>52.8</v>
+        <v>50.7</v>
       </c>
       <c r="J18" t="n">
-        <v>34.8</v>
+        <v>39.5</v>
       </c>
       <c r="K18" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="L18" t="n">
-        <v>1.71</v>
+        <v>2.01</v>
       </c>
       <c r="M18" t="n">
-        <v>13.7</v>
+        <v>23.5</v>
       </c>
       <c r="N18" t="n">
-        <v>1.5</v>
+        <v>40.9</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -2117,7 +2120,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>35.6</v>
+        <v>46.1</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2126,17 +2129,17 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
@@ -2149,15 +2152,15 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PSX</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>269.72</v>
+        <v>49.89</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -2172,36 +2175,36 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>52.3</v>
+        <v>50.5</v>
       </c>
       <c r="J19" t="n">
-        <v>67</v>
+        <v>40.3</v>
       </c>
       <c r="K19" t="n">
-        <v>15</v>
+        <v>75</v>
       </c>
       <c r="L19" t="n">
-        <v>3.45</v>
+        <v>3.07</v>
       </c>
       <c r="M19" t="n">
-        <v>27.2</v>
+        <v>36.6</v>
       </c>
       <c r="N19" t="n">
-        <v>24</v>
+        <v>45.5</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -2209,7 +2212,7 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>74</v>
+        <v>48.4</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2218,12 +2221,12 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
@@ -2231,11 +2234,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr">
         <is>
           <t>No</t>
@@ -2245,11 +2244,11 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>WFC</t>
+          <t>BAC</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>81.44</v>
+        <v>54.07</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2282,30 +2281,30 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>50.9</v>
+        <v>50.2</v>
       </c>
       <c r="J20" t="n">
-        <v>38.7</v>
+        <v>25.5</v>
       </c>
       <c r="K20" t="n">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="L20" t="n">
-        <v>2.15</v>
+        <v>1.8</v>
       </c>
       <c r="M20" t="n">
-        <v>23.7</v>
+        <v>22.2</v>
       </c>
       <c r="N20" t="n">
-        <v>42.2</v>
+        <v>52.4</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>45.8</v>
+        <v>42.5</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2337,11 +2336,11 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>CMG</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>50.28</v>
+        <v>30.88</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2374,30 +2373,30 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>50.7</v>
+        <v>49.4</v>
       </c>
       <c r="J21" t="n">
-        <v>41.8</v>
+        <v>31.6</v>
       </c>
       <c r="K21" t="n">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="L21" t="n">
-        <v>3.16</v>
+        <v>3.74</v>
       </c>
       <c r="M21" t="n">
-        <v>36.6</v>
+        <v>30.6</v>
       </c>
       <c r="N21" t="n">
-        <v>45.5</v>
+        <v>21.4</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>49</v>
+        <v>42.5</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2429,30 +2428,30 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BAC</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>54</v>
+        <v>743.6900000000001</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2462,34 +2461,34 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>50</v>
+        <v>49.4</v>
       </c>
       <c r="J22" t="n">
-        <v>24.8</v>
+        <v>64.3</v>
       </c>
       <c r="K22" t="n">
-        <v>98</v>
+        <v>65</v>
       </c>
       <c r="L22" t="n">
-        <v>1.92</v>
+        <v>3.08</v>
       </c>
       <c r="M22" t="n">
-        <v>22.6</v>
+        <v>47.6</v>
       </c>
       <c r="N22" t="n">
-        <v>54.7</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P22" t="n">
-        <v>42.2</v>
+        <v>62.4</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
@@ -2503,12 +2502,12 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U22" t="inlineStr"/>
@@ -2521,11 +2520,11 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>DUK</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>190.19</v>
+        <v>114.56</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -2558,30 +2557,30 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>50</v>
+        <v>49.3</v>
       </c>
       <c r="J23" t="n">
-        <v>29.9</v>
+        <v>36.9</v>
       </c>
       <c r="K23" t="n">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="L23" t="n">
-        <v>2.29</v>
+        <v>1.25</v>
       </c>
       <c r="M23" t="n">
-        <v>20.8</v>
+        <v>10.1</v>
       </c>
       <c r="N23" t="n">
-        <v>9.699999999999999</v>
+        <v>0</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>41.7</v>
+        <v>37.8</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -2590,17 +2589,17 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U23" t="inlineStr"/>
@@ -2613,11 +2612,11 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AON</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>272.05</v>
+        <v>191.3</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -2646,34 +2645,34 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I24" t="n">
-        <v>49.7</v>
+        <v>49.1</v>
       </c>
       <c r="J24" t="n">
-        <v>27.9</v>
+        <v>32.6</v>
       </c>
       <c r="K24" t="n">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="L24" t="n">
-        <v>2.52</v>
+        <v>2.18</v>
       </c>
       <c r="M24" t="n">
-        <v>35.7</v>
+        <v>21</v>
       </c>
       <c r="N24" t="n">
-        <v>88</v>
+        <v>10.4</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P24" t="n">
-        <v>29.3</v>
+        <v>42.7</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -2705,11 +2704,11 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SRE</t>
+          <t>D</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>78.16</v>
+        <v>61.62</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -2738,26 +2737,23 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>49.7</v>
+        <v>48.7</v>
       </c>
       <c r="J25" t="n">
-        <v>37</v>
+        <v>39.5</v>
       </c>
       <c r="K25" t="n">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="L25" t="n">
-        <v>1.69</v>
+        <v>1.65</v>
       </c>
       <c r="M25" t="n">
-        <v>21.1</v>
-      </c>
-      <c r="N25" t="n">
-        <v>56.7</v>
+        <v>21.9</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2765,7 +2761,7 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>35.3</v>
+        <v>41.6</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
@@ -2801,7 +2797,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>224.71</v>
+        <v>223.51</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -2834,22 +2830,22 @@
         </is>
       </c>
       <c r="I26" t="n">
-        <v>49.5</v>
+        <v>47.5</v>
       </c>
       <c r="J26" t="n">
-        <v>30.1</v>
+        <v>29.2</v>
       </c>
       <c r="K26" t="n">
         <v>98</v>
       </c>
       <c r="L26" t="n">
-        <v>2.27</v>
+        <v>2.16</v>
       </c>
       <c r="M26" t="n">
-        <v>25.3</v>
+        <v>23.8</v>
       </c>
       <c r="N26" t="n">
-        <v>50</v>
+        <v>41.5</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -2857,7 +2853,7 @@
         </is>
       </c>
       <c r="P26" t="n">
-        <v>43.1</v>
+        <v>42.3</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
@@ -2889,11 +2885,11 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>PAYX</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>99.78</v>
+        <v>125.64</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -2926,22 +2922,22 @@
         </is>
       </c>
       <c r="I27" t="n">
-        <v>49.2</v>
+        <v>47.2</v>
       </c>
       <c r="J27" t="n">
-        <v>27.9</v>
+        <v>25.6</v>
       </c>
       <c r="K27" t="n">
         <v>97</v>
       </c>
       <c r="L27" t="n">
-        <v>2.79</v>
+        <v>1.73</v>
       </c>
       <c r="M27" t="n">
-        <v>33.3</v>
+        <v>13.9</v>
       </c>
       <c r="N27" t="n">
-        <v>77.59999999999999</v>
+        <v>0</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -2949,7 +2945,7 @@
         </is>
       </c>
       <c r="P27" t="n">
-        <v>41.3</v>
+        <v>30.9</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
@@ -2981,11 +2977,11 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>DUK</t>
+          <t>MCD</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>113.84</v>
+        <v>232.25</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -3021,19 +3017,19 @@
         <v>46.6</v>
       </c>
       <c r="J28" t="n">
-        <v>31.5</v>
+        <v>26.2</v>
       </c>
       <c r="K28" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L28" t="n">
-        <v>1.26</v>
+        <v>1.73</v>
       </c>
       <c r="M28" t="n">
-        <v>11.4</v>
+        <v>20.3</v>
       </c>
       <c r="N28" t="n">
-        <v>0</v>
+        <v>52.6</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -3041,7 +3037,7 @@
         </is>
       </c>
       <c r="P28" t="n">
-        <v>36.5</v>
+        <v>24.5</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
@@ -3073,11 +3069,11 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>TMUS</t>
+          <t>AON</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>164.64</v>
+        <v>272.92</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -3106,26 +3102,23 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I29" t="n">
-        <v>44.7</v>
+        <v>45.5</v>
       </c>
       <c r="J29" t="n">
-        <v>39.8</v>
+        <v>28.9</v>
       </c>
       <c r="K29" t="n">
-        <v>93</v>
+        <v>76</v>
       </c>
       <c r="L29" t="n">
-        <v>2.29</v>
+        <v>2.41</v>
       </c>
       <c r="M29" t="n">
-        <v>29.3</v>
-      </c>
-      <c r="N29" t="n">
-        <v>34.9</v>
+        <v>33.3</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -3133,7 +3126,7 @@
         </is>
       </c>
       <c r="P29" t="n">
-        <v>36.2</v>
+        <v>29.8</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
@@ -3165,11 +3158,11 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CMCSA</t>
+          <t>TMUS</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>21.57</v>
+        <v>165.38</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -3202,22 +3195,22 @@
         </is>
       </c>
       <c r="I30" t="n">
-        <v>44.5</v>
+        <v>45.2</v>
       </c>
       <c r="J30" t="n">
-        <v>27.1</v>
+        <v>41.3</v>
       </c>
       <c r="K30" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="L30" t="n">
-        <v>2.56</v>
+        <v>2.18</v>
       </c>
       <c r="M30" t="n">
-        <v>28.9</v>
+        <v>29.4</v>
       </c>
       <c r="N30" t="n">
-        <v>24.3</v>
+        <v>35.1</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -3225,7 +3218,7 @@
         </is>
       </c>
       <c r="P30" t="n">
-        <v>35.9</v>
+        <v>36.9</v>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
@@ -3234,17 +3227,17 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U30" t="inlineStr"/>
@@ -3257,11 +3250,11 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>FDX</t>
+          <t>CMCSA</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>289.13</v>
+        <v>21.52</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -3290,34 +3283,34 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I31" t="n">
-        <v>43.5</v>
+        <v>43.8</v>
       </c>
       <c r="J31" t="n">
-        <v>38.5</v>
+        <v>26.8</v>
       </c>
       <c r="K31" t="n">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="L31" t="n">
-        <v>2.13</v>
+        <v>2.49</v>
       </c>
       <c r="M31" t="n">
-        <v>25.6</v>
+        <v>28.7</v>
       </c>
       <c r="N31" t="n">
-        <v>31.1</v>
+        <v>23.5</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P31" t="n">
-        <v>43.6</v>
+        <v>35.7</v>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
@@ -3326,17 +3319,17 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U31" t="inlineStr"/>
@@ -3349,11 +3342,11 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>USB</t>
+          <t>FDX</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>57.27</v>
+        <v>288.44</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -3386,22 +3379,22 @@
         </is>
       </c>
       <c r="I32" t="n">
-        <v>43.1</v>
+        <v>42.8</v>
       </c>
       <c r="J32" t="n">
-        <v>32.9</v>
+        <v>37.9</v>
       </c>
       <c r="K32" t="n">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="L32" t="n">
-        <v>1.82</v>
+        <v>2</v>
       </c>
       <c r="M32" t="n">
-        <v>19</v>
+        <v>23.9</v>
       </c>
       <c r="N32" t="n">
-        <v>19.9</v>
+        <v>24.5</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -3409,7 +3402,7 @@
         </is>
       </c>
       <c r="P32" t="n">
-        <v>46.3</v>
+        <v>43.3</v>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
@@ -3418,17 +3411,17 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U32" t="inlineStr"/>
@@ -3445,7 +3438,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>97.95999999999999</v>
+        <v>97.12</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -3478,30 +3471,30 @@
         </is>
       </c>
       <c r="I33" t="n">
-        <v>42</v>
+        <v>42.5</v>
       </c>
       <c r="J33" t="n">
-        <v>35.1</v>
+        <v>33.3</v>
       </c>
       <c r="K33" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="L33" t="n">
-        <v>2.11</v>
+        <v>2.1</v>
       </c>
       <c r="M33" t="n">
-        <v>25.9</v>
+        <v>25.4</v>
       </c>
       <c r="N33" t="n">
-        <v>52.2</v>
+        <v>49.7</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P33" t="n">
-        <v>46.7</v>
+        <v>45.4</v>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
@@ -3533,11 +3526,11 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ROP</t>
+          <t>USB</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>363.38</v>
+        <v>57.24</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -3570,30 +3563,30 @@
         </is>
       </c>
       <c r="I34" t="n">
-        <v>41.8</v>
+        <v>41.6</v>
       </c>
       <c r="J34" t="n">
-        <v>43</v>
+        <v>32.8</v>
       </c>
       <c r="K34" t="n">
-        <v>57</v>
+        <v>76</v>
       </c>
       <c r="L34" t="n">
-        <v>2.65</v>
+        <v>1.75</v>
       </c>
       <c r="M34" t="n">
-        <v>26.4</v>
+        <v>18.9</v>
       </c>
       <c r="N34" t="n">
-        <v>41.5</v>
+        <v>18.9</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P34" t="n">
-        <v>46.2</v>
+        <v>46.3</v>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
@@ -3602,17 +3595,17 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U34" t="inlineStr"/>
@@ -3625,11 +3618,11 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>GS</t>
+          <t>JPM</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>893.46</v>
+        <v>331.53</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -3662,30 +3655,30 @@
         </is>
       </c>
       <c r="I35" t="n">
-        <v>41.7</v>
+        <v>40.8</v>
       </c>
       <c r="J35" t="n">
-        <v>30.5</v>
+        <v>33.7</v>
       </c>
       <c r="K35" t="n">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="L35" t="n">
-        <v>2.38</v>
+        <v>1.66</v>
       </c>
       <c r="M35" t="n">
-        <v>25.3</v>
+        <v>16.5</v>
       </c>
       <c r="N35" t="n">
-        <v>14.9</v>
+        <v>18.7</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P35" t="n">
-        <v>37.2</v>
+        <v>48.9</v>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
@@ -3717,11 +3710,11 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>JPM</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>332.38</v>
+        <v>898.76</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -3754,30 +3747,30 @@
         </is>
       </c>
       <c r="I36" t="n">
-        <v>41.4</v>
+        <v>40.6</v>
       </c>
       <c r="J36" t="n">
-        <v>34.5</v>
+        <v>32.7</v>
       </c>
       <c r="K36" t="n">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="L36" t="n">
-        <v>1.78</v>
+        <v>2.24</v>
       </c>
       <c r="M36" t="n">
-        <v>17.2</v>
+        <v>25.5</v>
       </c>
       <c r="N36" t="n">
-        <v>22.6</v>
+        <v>15.6</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P36" t="n">
-        <v>49.4</v>
+        <v>37.8</v>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
@@ -3813,7 +3806,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>27.65</v>
+        <v>26.8</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -3846,22 +3839,22 @@
         </is>
       </c>
       <c r="I37" t="n">
-        <v>41.1</v>
+        <v>39.8</v>
       </c>
       <c r="J37" t="n">
-        <v>35.8</v>
+        <v>31.2</v>
       </c>
       <c r="K37" t="n">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L37" t="n">
-        <v>2.64</v>
+        <v>2.82</v>
       </c>
       <c r="M37" t="n">
-        <v>33.4</v>
+        <v>34</v>
       </c>
       <c r="N37" t="n">
-        <v>58.3</v>
+        <v>60.3</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
@@ -3869,7 +3862,7 @@
         </is>
       </c>
       <c r="P37" t="n">
-        <v>36.9</v>
+        <v>34.2</v>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
@@ -3891,10 +3884,14 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U37" t="inlineStr"/>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V37" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3905,7 +3902,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>109.36</v>
+        <v>109.11</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -3938,22 +3935,22 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>39</v>
+        <v>38.9</v>
       </c>
       <c r="J38" t="n">
-        <v>21.4</v>
+        <v>21</v>
       </c>
       <c r="K38" t="n">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="L38" t="n">
-        <v>2.25</v>
+        <v>2.15</v>
       </c>
       <c r="M38" t="n">
         <v>16</v>
       </c>
       <c r="N38" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
@@ -3961,7 +3958,7 @@
         </is>
       </c>
       <c r="P38" t="n">
-        <v>35.9</v>
+        <v>35.7</v>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
@@ -3993,11 +3990,11 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>AXP</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>304.02</v>
+        <v>68.37</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -4026,26 +4023,26 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I39" t="n">
         <v>38.3</v>
       </c>
       <c r="J39" t="n">
-        <v>34.9</v>
+        <v>36.2</v>
       </c>
       <c r="K39" t="n">
-        <v>75</v>
+        <v>89</v>
       </c>
       <c r="L39" t="n">
-        <v>1.73</v>
+        <v>2.36</v>
       </c>
       <c r="M39" t="n">
-        <v>18.3</v>
+        <v>34.2</v>
       </c>
       <c r="N39" t="n">
-        <v>6.5</v>
+        <v>44.8</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
@@ -4053,7 +4050,7 @@
         </is>
       </c>
       <c r="P39" t="n">
-        <v>38.6</v>
+        <v>35.8</v>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
@@ -4062,17 +4059,17 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U39" t="inlineStr"/>
@@ -4089,7 +4086,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>107.77</v>
+        <v>108.9</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -4122,22 +4119,19 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>36.1</v>
+        <v>36.9</v>
       </c>
       <c r="J40" t="n">
-        <v>27.4</v>
+        <v>29.3</v>
       </c>
       <c r="K40" t="n">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="L40" t="n">
-        <v>4.67</v>
+        <v>4.63</v>
       </c>
       <c r="M40" t="n">
-        <v>54.9</v>
-      </c>
-      <c r="N40" t="n">
-        <v>48.1</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
@@ -4145,7 +4139,7 @@
         </is>
       </c>
       <c r="P40" t="n">
-        <v>30.5</v>
+        <v>30.8</v>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
@@ -4177,11 +4171,11 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>VZ</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>67.5</v>
+        <v>45.69</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -4214,30 +4208,30 @@
         </is>
       </c>
       <c r="I41" t="n">
-        <v>35.5</v>
+        <v>36.4</v>
       </c>
       <c r="J41" t="n">
-        <v>32.8</v>
+        <v>33.2</v>
       </c>
       <c r="K41" t="n">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="L41" t="n">
-        <v>2.48</v>
+        <v>1.7</v>
       </c>
       <c r="M41" t="n">
-        <v>33.9</v>
+        <v>19.1</v>
       </c>
       <c r="N41" t="n">
-        <v>44</v>
+        <v>22.1</v>
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P41" t="n">
-        <v>34.4</v>
+        <v>47.2</v>
       </c>
       <c r="Q41" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Scan 07.10.2026 19:51 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V41"/>
+  <dimension ref="A1:V34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>275.43</v>
+        <v>266.93</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,22 +614,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>86.59999999999999</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>63.9</v>
+        <v>59</v>
       </c>
       <c r="K2" t="n">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="L2" t="n">
-        <v>5.99</v>
+        <v>6.18</v>
       </c>
       <c r="M2" t="n">
-        <v>57.5</v>
+        <v>58.9</v>
       </c>
       <c r="N2" t="n">
-        <v>56.8</v>
+        <v>60.5</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>79.09999999999999</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -659,85 +659,81 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ABBV</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>267.15</v>
+        <v>410.3</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>80</v>
+        <v>72.3</v>
       </c>
       <c r="J3" t="n">
+        <v>64</v>
+      </c>
+      <c r="K3" t="n">
+        <v>99</v>
+      </c>
+      <c r="L3" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="M3" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="N3" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
         <v>60.4</v>
       </c>
-      <c r="K3" t="n">
-        <v>1</v>
-      </c>
-      <c r="L3" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="M3" t="n">
-        <v>17</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P3" t="n">
-        <v>64.2</v>
-      </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -752,47 +748,47 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>EW</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>118.19</v>
+        <v>85.61</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -802,23 +798,26 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>73.09999999999999</v>
+        <v>69.8</v>
       </c>
       <c r="J4" t="n">
-        <v>68.8</v>
+        <v>43.6</v>
       </c>
       <c r="K4" t="n">
-        <v>39</v>
+        <v>14</v>
       </c>
       <c r="L4" t="n">
-        <v>2.38</v>
+        <v>2.41</v>
       </c>
       <c r="M4" t="n">
-        <v>31.5</v>
+        <v>23.9</v>
+      </c>
+      <c r="N4" t="n">
+        <v>41.1</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -826,29 +825,33 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>62</v>
+        <v>48.9</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V4" t="inlineStr">
         <is>
           <t>No</t>
@@ -858,11 +861,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>EW</t>
+          <t>DXCM</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>86.44</v>
+        <v>84.23999999999999</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -895,22 +898,22 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>70.90000000000001</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="J5" t="n">
-        <v>46.3</v>
+        <v>42.4</v>
       </c>
       <c r="K5" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="L5" t="n">
-        <v>2.37</v>
+        <v>2.7</v>
       </c>
       <c r="M5" t="n">
-        <v>23.9</v>
+        <v>24</v>
       </c>
       <c r="N5" t="n">
-        <v>40.8</v>
+        <v>6.5</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -918,21 +921,21 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>50.1</v>
+        <v>56.2</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -940,11 +943,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
           <t>No</t>
@@ -954,67 +953,67 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DXCM</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>83.31</v>
+        <v>85.62</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>69.3</v>
+        <v>63.2</v>
       </c>
       <c r="J6" t="n">
-        <v>38.7</v>
+        <v>48.8</v>
       </c>
       <c r="K6" t="n">
-        <v>6</v>
+        <v>88</v>
       </c>
       <c r="L6" t="n">
-        <v>2.66</v>
+        <v>1.46</v>
       </c>
       <c r="M6" t="n">
-        <v>24.4</v>
+        <v>13.1</v>
       </c>
       <c r="N6" t="n">
-        <v>7.7</v>
+        <v>8</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>54.9</v>
+        <v>40.1</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1023,57 +1022,53 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>WBD</t>
+          <t>NEE</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>30.95</v>
+        <v>77.05</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1083,31 +1078,34 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>67.3</v>
+        <v>62.4</v>
       </c>
       <c r="J7" t="n">
-        <v>75.2</v>
+        <v>38.7</v>
       </c>
       <c r="K7" t="n">
-        <v>99</v>
+        <v>80</v>
       </c>
       <c r="L7" t="n">
-        <v>0.75</v>
+        <v>1.82</v>
       </c>
       <c r="M7" t="n">
-        <v>4.7</v>
+        <v>16.3</v>
+      </c>
+      <c r="N7" t="n">
+        <v>17.5</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>71.09999999999999</v>
+        <v>34.7</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1121,12 +1119,12 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
@@ -1139,67 +1137,67 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ROST</t>
+          <t>EXC</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>222.5</v>
+        <v>41.56</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>64.90000000000001</v>
+        <v>60.8</v>
       </c>
       <c r="J8" t="n">
-        <v>35.9</v>
+        <v>45.4</v>
       </c>
       <c r="K8" t="n">
-        <v>11</v>
+        <v>86</v>
       </c>
       <c r="L8" t="n">
-        <v>2.3</v>
+        <v>1.62</v>
       </c>
       <c r="M8" t="n">
-        <v>19.8</v>
+        <v>14.7</v>
       </c>
       <c r="N8" t="n">
-        <v>23.3</v>
+        <v>8</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>48.4</v>
+        <v>39.4</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1208,38 +1206,34 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>CCI</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>84.83</v>
+        <v>68.97</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1272,22 +1266,22 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>58</v>
+        <v>59.4</v>
       </c>
       <c r="J9" t="n">
-        <v>43.9</v>
+        <v>42.7</v>
       </c>
       <c r="K9" t="n">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="L9" t="n">
-        <v>1.47</v>
+        <v>2.6</v>
       </c>
       <c r="M9" t="n">
-        <v>12.2</v>
+        <v>22.4</v>
       </c>
       <c r="N9" t="n">
-        <v>0</v>
+        <v>22.8</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1295,7 +1289,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>37.9</v>
+        <v>35.9</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1327,11 +1321,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>NEE</t>
+          <t>SRE</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>77.48</v>
+        <v>79.83</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1360,26 +1354,26 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>56.8</v>
+        <v>56.9</v>
       </c>
       <c r="J10" t="n">
-        <v>39.8</v>
+        <v>46.4</v>
       </c>
       <c r="K10" t="n">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="L10" t="n">
-        <v>1.7</v>
+        <v>1.65</v>
       </c>
       <c r="M10" t="n">
-        <v>15.5</v>
+        <v>21.3</v>
       </c>
       <c r="N10" t="n">
-        <v>14.4</v>
+        <v>58.1</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1387,7 +1381,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>35.9</v>
+        <v>38.9</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1419,11 +1413,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>EXC</t>
+          <t>AMP</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>41.28</v>
+        <v>490.52</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1456,22 +1450,19 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>56.2</v>
+        <v>56.4</v>
       </c>
       <c r="J11" t="n">
-        <v>41.7</v>
+        <v>32.4</v>
       </c>
       <c r="K11" t="n">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="L11" t="n">
-        <v>1.65</v>
+        <v>2.42</v>
       </c>
       <c r="M11" t="n">
-        <v>13.6</v>
-      </c>
-      <c r="N11" t="n">
-        <v>0.6</v>
+        <v>31.6</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1479,7 +1470,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>38</v>
+        <v>44.6</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1488,17 +1479,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
@@ -1511,11 +1502,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AMP</t>
+          <t>D</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>494.44</v>
+        <v>61.49</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1544,34 +1535,34 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>55.9</v>
+        <v>56.4</v>
       </c>
       <c r="J12" t="n">
-        <v>33.4</v>
+        <v>39.7</v>
       </c>
       <c r="K12" t="n">
-        <v>91</v>
+        <v>76</v>
       </c>
       <c r="L12" t="n">
-        <v>2.42</v>
+        <v>1.73</v>
       </c>
       <c r="M12" t="n">
-        <v>24.1</v>
+        <v>14.5</v>
       </c>
       <c r="N12" t="n">
-        <v>32.1</v>
+        <v>6.3</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>45.8</v>
+        <v>41.1</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1580,17 +1571,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
@@ -1607,7 +1598,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>53.99</v>
+        <v>53.75</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1640,27 +1631,27 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>54.9</v>
+        <v>55.3</v>
       </c>
       <c r="J13" t="n">
-        <v>35</v>
+        <v>33.3</v>
       </c>
       <c r="K13" t="n">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="L13" t="n">
-        <v>1.22</v>
+        <v>1.21</v>
       </c>
       <c r="M13" t="n">
-        <v>17.4</v>
+        <v>17.3</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>47</v>
+        <v>45.8</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1692,11 +1683,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CCI</t>
+          <t>WFC</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>68.19</v>
+        <v>80.37</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1729,22 +1720,22 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>53.8</v>
+        <v>54.4</v>
       </c>
       <c r="J14" t="n">
-        <v>38.3</v>
+        <v>35.5</v>
       </c>
       <c r="K14" t="n">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="L14" t="n">
-        <v>2.62</v>
+        <v>2.17</v>
       </c>
       <c r="M14" t="n">
-        <v>22</v>
+        <v>23.8</v>
       </c>
       <c r="N14" t="n">
-        <v>21.3</v>
+        <v>42.5</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1752,7 +1743,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>34.2</v>
+        <v>44</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1761,17 +1752,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
@@ -1784,11 +1775,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SRE</t>
+          <t>PAYX</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>79.23999999999999</v>
+        <v>101.69</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1821,22 +1812,19 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>53</v>
+        <v>53.7</v>
       </c>
       <c r="J15" t="n">
-        <v>43.4</v>
+        <v>33.8</v>
       </c>
       <c r="K15" t="n">
-        <v>81</v>
+        <v>97</v>
       </c>
       <c r="L15" t="n">
-        <v>1.68</v>
+        <v>2.47</v>
       </c>
       <c r="M15" t="n">
-        <v>20.6</v>
-      </c>
-      <c r="N15" t="n">
-        <v>53.6</v>
+        <v>29.4</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1844,7 +1832,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>37.5</v>
+        <v>43.5</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1876,11 +1864,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PNC</t>
+          <t>DUK</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>220.06</v>
+        <v>115.56</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1913,30 +1901,30 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>51.4</v>
+        <v>53.5</v>
       </c>
       <c r="J16" t="n">
-        <v>26.7</v>
+        <v>43.2</v>
       </c>
       <c r="K16" t="n">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="L16" t="n">
-        <v>1.86</v>
+        <v>1.24</v>
       </c>
       <c r="M16" t="n">
-        <v>17.6</v>
+        <v>11.1</v>
       </c>
       <c r="N16" t="n">
-        <v>17.2</v>
+        <v>0</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>41.1</v>
+        <v>40</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1945,17 +1933,17 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
@@ -1968,81 +1956,81 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PAYX</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>100.93</v>
+        <v>657.72</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>50.9</v>
+        <v>52.8</v>
       </c>
       <c r="J17" t="n">
-        <v>31.5</v>
+        <v>44.2</v>
       </c>
       <c r="K17" t="n">
-        <v>97</v>
+        <v>7</v>
       </c>
       <c r="L17" t="n">
-        <v>2.63</v>
+        <v>2.99</v>
       </c>
       <c r="M17" t="n">
-        <v>33.3</v>
+        <v>28.8</v>
       </c>
       <c r="N17" t="n">
-        <v>77.40000000000001</v>
+        <v>40.9</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>42.6</v>
+        <v>57.2</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>FIRED</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
@@ -2050,21 +2038,25 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr"/>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>Squeeze Fired, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>WFC</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>81.58</v>
+        <v>189.46</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2097,30 +2089,30 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>50.7</v>
+        <v>52.6</v>
       </c>
       <c r="J18" t="n">
-        <v>39.5</v>
+        <v>30.2</v>
       </c>
       <c r="K18" t="n">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="L18" t="n">
-        <v>2.01</v>
+        <v>2.32</v>
       </c>
       <c r="M18" t="n">
-        <v>23.5</v>
+        <v>20.4</v>
       </c>
       <c r="N18" t="n">
-        <v>40.9</v>
+        <v>7.8</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>46.1</v>
+        <v>41.3</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2152,11 +2144,11 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>PNC</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>49.89</v>
+        <v>217.84</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2185,34 +2177,34 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>50.5</v>
+        <v>51.3</v>
       </c>
       <c r="J19" t="n">
-        <v>40.3</v>
+        <v>24.4</v>
       </c>
       <c r="K19" t="n">
-        <v>75</v>
+        <v>96</v>
       </c>
       <c r="L19" t="n">
-        <v>3.07</v>
+        <v>1.87</v>
       </c>
       <c r="M19" t="n">
-        <v>36.6</v>
+        <v>17.7</v>
       </c>
       <c r="N19" t="n">
-        <v>45.5</v>
+        <v>17.6</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>48.4</v>
+        <v>39.8</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2234,10 +2226,14 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr"/>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2248,7 +2244,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>54.07</v>
+        <v>53.55</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2281,30 +2277,30 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>50.2</v>
+        <v>50.5</v>
       </c>
       <c r="J20" t="n">
-        <v>25.5</v>
+        <v>23.8</v>
       </c>
       <c r="K20" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="L20" t="n">
-        <v>1.8</v>
+        <v>1.87</v>
       </c>
       <c r="M20" t="n">
         <v>22.2</v>
       </c>
       <c r="N20" t="n">
-        <v>52.4</v>
+        <v>52.3</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>42.5</v>
+        <v>41.1</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2336,11 +2332,11 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CMG</t>
+          <t>TMUS</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>30.88</v>
+        <v>168.47</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2373,22 +2369,22 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>49.4</v>
+        <v>50.3</v>
       </c>
       <c r="J21" t="n">
-        <v>31.6</v>
+        <v>47.1</v>
       </c>
       <c r="K21" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="L21" t="n">
-        <v>3.74</v>
+        <v>2.2</v>
       </c>
       <c r="M21" t="n">
-        <v>30.6</v>
+        <v>29.9</v>
       </c>
       <c r="N21" t="n">
-        <v>21.4</v>
+        <v>36.7</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2396,7 +2392,7 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>42.5</v>
+        <v>39.7</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2405,17 +2401,17 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U21" t="inlineStr"/>
@@ -2428,30 +2424,30 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>743.6900000000001</v>
+        <v>123.71</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2461,34 +2457,34 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>49.4</v>
+        <v>49</v>
       </c>
       <c r="J22" t="n">
-        <v>64.3</v>
+        <v>22.2</v>
       </c>
       <c r="K22" t="n">
-        <v>65</v>
+        <v>97</v>
       </c>
       <c r="L22" t="n">
-        <v>3.08</v>
+        <v>1.83</v>
       </c>
       <c r="M22" t="n">
-        <v>47.6</v>
+        <v>13.9</v>
       </c>
       <c r="N22" t="n">
-        <v>76.90000000000001</v>
+        <v>0</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P22" t="n">
-        <v>62.4</v>
+        <v>29.3</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
@@ -2502,29 +2498,33 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr"/>
-      <c r="V22" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>DUK</t>
+          <t>MCD</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>114.56</v>
+        <v>230.96</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -2557,22 +2557,22 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>49.3</v>
+        <v>46.8</v>
       </c>
       <c r="J23" t="n">
-        <v>36.9</v>
+        <v>25</v>
       </c>
       <c r="K23" t="n">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="L23" t="n">
-        <v>1.25</v>
+        <v>1.68</v>
       </c>
       <c r="M23" t="n">
-        <v>10.1</v>
+        <v>20.1</v>
       </c>
       <c r="N23" t="n">
-        <v>0</v>
+        <v>50.7</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="P23" t="n">
-        <v>37.8</v>
+        <v>23.9</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -2589,17 +2589,17 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U23" t="inlineStr"/>
@@ -2612,11 +2612,11 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>191.3</v>
+        <v>224.32</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -2649,30 +2649,30 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>49.1</v>
+        <v>46.6</v>
       </c>
       <c r="J24" t="n">
-        <v>32.6</v>
+        <v>29.8</v>
       </c>
       <c r="K24" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="L24" t="n">
-        <v>2.18</v>
+        <v>2</v>
       </c>
       <c r="M24" t="n">
-        <v>21</v>
+        <v>23.8</v>
       </c>
       <c r="N24" t="n">
-        <v>10.4</v>
+        <v>41.5</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P24" t="n">
-        <v>42.7</v>
+        <v>42.8</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -2704,11 +2704,11 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>CMCSA</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>61.62</v>
+        <v>21.01</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -2737,23 +2737,26 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>48.7</v>
+        <v>46.5</v>
       </c>
       <c r="J25" t="n">
-        <v>39.5</v>
+        <v>23.4</v>
       </c>
       <c r="K25" t="n">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="L25" t="n">
-        <v>1.65</v>
+        <v>2.64</v>
       </c>
       <c r="M25" t="n">
-        <v>21.9</v>
+        <v>29</v>
+      </c>
+      <c r="N25" t="n">
+        <v>24.6</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2761,7 +2764,7 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>41.6</v>
+        <v>34.3</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
@@ -2770,34 +2773,38 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="U25" t="inlineStr"/>
-      <c r="V25" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ALL</t>
+          <t>SCHW</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>223.51</v>
+        <v>95.69</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -2830,30 +2837,30 @@
         </is>
       </c>
       <c r="I26" t="n">
-        <v>47.5</v>
+        <v>44.2</v>
       </c>
       <c r="J26" t="n">
-        <v>29.2</v>
+        <v>30.5</v>
       </c>
       <c r="K26" t="n">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="L26" t="n">
         <v>2.16</v>
       </c>
       <c r="M26" t="n">
-        <v>23.8</v>
+        <v>25.5</v>
       </c>
       <c r="N26" t="n">
-        <v>41.5</v>
+        <v>49.9</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P26" t="n">
-        <v>42.3</v>
+        <v>43.3</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
@@ -2885,11 +2892,11 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>FANG</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>125.64</v>
+        <v>184.27</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -2922,30 +2929,30 @@
         </is>
       </c>
       <c r="I27" t="n">
-        <v>47.2</v>
+        <v>42</v>
       </c>
       <c r="J27" t="n">
-        <v>25.6</v>
+        <v>38.5</v>
       </c>
       <c r="K27" t="n">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="L27" t="n">
-        <v>1.73</v>
+        <v>2.49</v>
       </c>
       <c r="M27" t="n">
-        <v>13.9</v>
+        <v>30.6</v>
       </c>
       <c r="N27" t="n">
-        <v>0</v>
+        <v>39.5</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P27" t="n">
-        <v>30.9</v>
+        <v>47.6</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
@@ -2977,11 +2984,11 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>MCD</t>
+          <t>CMG</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>232.25</v>
+        <v>30.77</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -3010,26 +3017,26 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I28" t="n">
-        <v>46.6</v>
+        <v>41.9</v>
       </c>
       <c r="J28" t="n">
-        <v>26.2</v>
+        <v>31.2</v>
       </c>
       <c r="K28" t="n">
-        <v>97</v>
+        <v>69</v>
       </c>
       <c r="L28" t="n">
-        <v>1.73</v>
+        <v>3.49</v>
       </c>
       <c r="M28" t="n">
-        <v>20.3</v>
+        <v>30.5</v>
       </c>
       <c r="N28" t="n">
-        <v>52.6</v>
+        <v>21.1</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -3037,7 +3044,7 @@
         </is>
       </c>
       <c r="P28" t="n">
-        <v>24.5</v>
+        <v>42.3</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
@@ -3046,17 +3053,17 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U28" t="inlineStr"/>
@@ -3069,11 +3076,11 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>AON</t>
+          <t>JPM</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>272.92</v>
+        <v>329.44</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -3102,31 +3109,34 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I29" t="n">
-        <v>45.5</v>
+        <v>41.9</v>
       </c>
       <c r="J29" t="n">
-        <v>28.9</v>
+        <v>33.7</v>
       </c>
       <c r="K29" t="n">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="L29" t="n">
-        <v>2.41</v>
+        <v>1.7</v>
       </c>
       <c r="M29" t="n">
-        <v>33.3</v>
+        <v>16.6</v>
+      </c>
+      <c r="N29" t="n">
+        <v>18.9</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P29" t="n">
-        <v>29.8</v>
+        <v>48.6</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
@@ -3135,17 +3145,17 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U29" t="inlineStr"/>
@@ -3158,11 +3168,11 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>TMUS</t>
+          <t>CHTR</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>165.38</v>
+        <v>107.9</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -3195,22 +3205,22 @@
         </is>
       </c>
       <c r="I30" t="n">
-        <v>45.2</v>
+        <v>41.8</v>
       </c>
       <c r="J30" t="n">
-        <v>41.3</v>
+        <v>28.4</v>
       </c>
       <c r="K30" t="n">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="L30" t="n">
-        <v>2.18</v>
+        <v>4.73</v>
       </c>
       <c r="M30" t="n">
-        <v>29.4</v>
+        <v>53.6</v>
       </c>
       <c r="N30" t="n">
-        <v>35.1</v>
+        <v>46.3</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -3218,7 +3228,7 @@
         </is>
       </c>
       <c r="P30" t="n">
-        <v>36.9</v>
+        <v>30.5</v>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
@@ -3227,17 +3237,17 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U30" t="inlineStr"/>
@@ -3250,11 +3260,11 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CMCSA</t>
+          <t>PCAR</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>21.52</v>
+        <v>106.86</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -3287,22 +3297,22 @@
         </is>
       </c>
       <c r="I31" t="n">
-        <v>43.8</v>
+        <v>40.4</v>
       </c>
       <c r="J31" t="n">
-        <v>26.8</v>
+        <v>17.7</v>
       </c>
       <c r="K31" t="n">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="L31" t="n">
-        <v>2.49</v>
+        <v>2.26</v>
       </c>
       <c r="M31" t="n">
-        <v>28.7</v>
+        <v>16.8</v>
       </c>
       <c r="N31" t="n">
-        <v>23.5</v>
+        <v>4.1</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
@@ -3310,7 +3320,7 @@
         </is>
       </c>
       <c r="P31" t="n">
-        <v>35.7</v>
+        <v>33.7</v>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
@@ -3332,21 +3342,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U31" t="inlineStr"/>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>FDX</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>288.44</v>
+        <v>886.99</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -3375,34 +3389,34 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I32" t="n">
-        <v>42.8</v>
+        <v>39.6</v>
       </c>
       <c r="J32" t="n">
-        <v>37.9</v>
+        <v>30</v>
       </c>
       <c r="K32" t="n">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="L32" t="n">
-        <v>2</v>
+        <v>2.39</v>
       </c>
       <c r="M32" t="n">
-        <v>23.9</v>
+        <v>24.2</v>
       </c>
       <c r="N32" t="n">
-        <v>24.5</v>
+        <v>10.5</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P32" t="n">
-        <v>43.3</v>
+        <v>36.4</v>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
@@ -3411,34 +3425,38 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="U32" t="inlineStr"/>
-      <c r="V32" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SCHW</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>97.12</v>
+        <v>26.72</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -3471,30 +3489,30 @@
         </is>
       </c>
       <c r="I33" t="n">
-        <v>42.5</v>
+        <v>38.2</v>
       </c>
       <c r="J33" t="n">
-        <v>33.3</v>
+        <v>30.8</v>
       </c>
       <c r="K33" t="n">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="L33" t="n">
-        <v>2.1</v>
+        <v>2.76</v>
       </c>
       <c r="M33" t="n">
-        <v>25.4</v>
+        <v>33.9</v>
       </c>
       <c r="N33" t="n">
-        <v>49.7</v>
+        <v>59.8</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P33" t="n">
-        <v>45.4</v>
+        <v>34</v>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
@@ -3526,11 +3544,11 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>USB</t>
+          <t>VZ</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>57.24</v>
+        <v>46.02</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -3559,26 +3577,26 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I34" t="n">
-        <v>41.6</v>
+        <v>37.6</v>
       </c>
       <c r="J34" t="n">
-        <v>32.8</v>
+        <v>36.1</v>
       </c>
       <c r="K34" t="n">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="L34" t="n">
-        <v>1.75</v>
+        <v>1.65</v>
       </c>
       <c r="M34" t="n">
-        <v>18.9</v>
+        <v>19.2</v>
       </c>
       <c r="N34" t="n">
-        <v>18.9</v>
+        <v>22.3</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
@@ -3586,7 +3604,7 @@
         </is>
       </c>
       <c r="P34" t="n">
-        <v>46.3</v>
+        <v>48.2</v>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
@@ -3610,651 +3628,6 @@
       </c>
       <c r="U34" t="inlineStr"/>
       <c r="V34" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>JPM</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>331.53</v>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I35" t="n">
-        <v>40.8</v>
-      </c>
-      <c r="J35" t="n">
-        <v>33.7</v>
-      </c>
-      <c r="K35" t="n">
-        <v>84</v>
-      </c>
-      <c r="L35" t="n">
-        <v>1.66</v>
-      </c>
-      <c r="M35" t="n">
-        <v>16.5</v>
-      </c>
-      <c r="N35" t="n">
-        <v>18.7</v>
-      </c>
-      <c r="O35" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P35" t="n">
-        <v>48.9</v>
-      </c>
-      <c r="Q35" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R35" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S35" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T35" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U35" t="inlineStr"/>
-      <c r="V35" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>GS</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>898.76</v>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D36" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I36" t="n">
-        <v>40.6</v>
-      </c>
-      <c r="J36" t="n">
-        <v>32.7</v>
-      </c>
-      <c r="K36" t="n">
-        <v>92</v>
-      </c>
-      <c r="L36" t="n">
-        <v>2.24</v>
-      </c>
-      <c r="M36" t="n">
-        <v>25.5</v>
-      </c>
-      <c r="N36" t="n">
-        <v>15.6</v>
-      </c>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P36" t="n">
-        <v>37.8</v>
-      </c>
-      <c r="Q36" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R36" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S36" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T36" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U36" t="inlineStr"/>
-      <c r="V36" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>CPRT</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>26.8</v>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I37" t="n">
-        <v>39.8</v>
-      </c>
-      <c r="J37" t="n">
-        <v>31.2</v>
-      </c>
-      <c r="K37" t="n">
-        <v>86</v>
-      </c>
-      <c r="L37" t="n">
-        <v>2.82</v>
-      </c>
-      <c r="M37" t="n">
-        <v>34</v>
-      </c>
-      <c r="N37" t="n">
-        <v>60.3</v>
-      </c>
-      <c r="O37" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P37" t="n">
-        <v>34.2</v>
-      </c>
-      <c r="Q37" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R37" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S37" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T37" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U37" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
-      <c r="V37" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>PCAR</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>109.11</v>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I38" t="n">
-        <v>38.9</v>
-      </c>
-      <c r="J38" t="n">
-        <v>21</v>
-      </c>
-      <c r="K38" t="n">
-        <v>91</v>
-      </c>
-      <c r="L38" t="n">
-        <v>2.15</v>
-      </c>
-      <c r="M38" t="n">
-        <v>16</v>
-      </c>
-      <c r="N38" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="O38" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P38" t="n">
-        <v>35.7</v>
-      </c>
-      <c r="Q38" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R38" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S38" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T38" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U38" t="inlineStr"/>
-      <c r="V38" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>NFLX</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>68.37</v>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I39" t="n">
-        <v>38.3</v>
-      </c>
-      <c r="J39" t="n">
-        <v>36.2</v>
-      </c>
-      <c r="K39" t="n">
-        <v>89</v>
-      </c>
-      <c r="L39" t="n">
-        <v>2.36</v>
-      </c>
-      <c r="M39" t="n">
-        <v>34.2</v>
-      </c>
-      <c r="N39" t="n">
-        <v>44.8</v>
-      </c>
-      <c r="O39" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P39" t="n">
-        <v>35.8</v>
-      </c>
-      <c r="Q39" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R39" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S39" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T39" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U39" t="inlineStr"/>
-      <c r="V39" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>CHTR</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>108.9</v>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I40" t="n">
-        <v>36.9</v>
-      </c>
-      <c r="J40" t="n">
-        <v>29.3</v>
-      </c>
-      <c r="K40" t="n">
-        <v>89</v>
-      </c>
-      <c r="L40" t="n">
-        <v>4.63</v>
-      </c>
-      <c r="M40" t="n">
-        <v>76.09999999999999</v>
-      </c>
-      <c r="O40" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P40" t="n">
-        <v>30.8</v>
-      </c>
-      <c r="Q40" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R40" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S40" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T40" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U40" t="inlineStr"/>
-      <c r="V40" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>VZ</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>45.69</v>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D41" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I41" t="n">
-        <v>36.4</v>
-      </c>
-      <c r="J41" t="n">
-        <v>33.2</v>
-      </c>
-      <c r="K41" t="n">
-        <v>84</v>
-      </c>
-      <c r="L41" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="M41" t="n">
-        <v>19.1</v>
-      </c>
-      <c r="N41" t="n">
-        <v>22.1</v>
-      </c>
-      <c r="O41" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P41" t="n">
-        <v>47.2</v>
-      </c>
-      <c r="Q41" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R41" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S41" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T41" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U41" t="inlineStr"/>
-      <c r="V41" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 08.10.2026 19:46 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V34"/>
+  <dimension ref="A1:V33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -577,15 +577,15 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ILMN</t>
+          <t>TSN</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>266.93</v>
+        <v>52.41</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -600,44 +600,44 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>76.90000000000001</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>59</v>
+        <v>49.5</v>
       </c>
       <c r="K2" t="n">
-        <v>94</v>
+        <v>6</v>
       </c>
       <c r="L2" t="n">
-        <v>6.18</v>
+        <v>1.73</v>
       </c>
       <c r="M2" t="n">
-        <v>58.9</v>
+        <v>26.9</v>
       </c>
       <c r="N2" t="n">
-        <v>60.5</v>
+        <v>39.9</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>75.40000000000001</v>
+        <v>39</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -646,17 +646,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
@@ -669,67 +669,67 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>ZTS</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>410.3</v>
+        <v>73.34999999999999</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>72.3</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>64</v>
+        <v>54.3</v>
       </c>
       <c r="K3" t="n">
-        <v>99</v>
+        <v>14</v>
       </c>
       <c r="L3" t="n">
-        <v>2.71</v>
+        <v>2.47</v>
       </c>
       <c r="M3" t="n">
-        <v>31.4</v>
+        <v>24.1</v>
       </c>
       <c r="N3" t="n">
-        <v>20.9</v>
+        <v>11.5</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>60.4</v>
+        <v>35.5</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -743,7 +743,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -753,23 +753,23 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>Squeeze Expanding</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>EW</t>
+          <t>FCX</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>85.61</v>
+        <v>70.86</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -802,22 +802,22 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>69.8</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>43.6</v>
+        <v>47.5</v>
       </c>
       <c r="K4" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="L4" t="n">
-        <v>2.41</v>
+        <v>3.51</v>
       </c>
       <c r="M4" t="n">
-        <v>23.9</v>
+        <v>36.8</v>
       </c>
       <c r="N4" t="n">
-        <v>41.1</v>
+        <v>23.2</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -825,7 +825,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>48.9</v>
+        <v>56.5</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -861,30 +861,30 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DXCM</t>
+          <t>ADP</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>84.23999999999999</v>
+        <v>271.54</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -898,22 +898,22 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>68.59999999999999</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="J5" t="n">
-        <v>42.4</v>
+        <v>56.1</v>
       </c>
       <c r="K5" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="L5" t="n">
-        <v>2.7</v>
+        <v>2.16</v>
       </c>
       <c r="M5" t="n">
-        <v>24</v>
+        <v>23.6</v>
       </c>
       <c r="N5" t="n">
-        <v>6.5</v>
+        <v>34.3</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -921,7 +921,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>56.2</v>
+        <v>59.7</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -930,12 +930,12 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -943,7 +943,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr"/>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V5" t="inlineStr">
         <is>
           <t>No</t>
@@ -953,30 +957,30 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>85.62</v>
+        <v>348.26</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -990,30 +994,27 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>63.2</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="J6" t="n">
-        <v>48.8</v>
+        <v>64</v>
       </c>
       <c r="K6" t="n">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="L6" t="n">
-        <v>1.46</v>
+        <v>3.28</v>
       </c>
       <c r="M6" t="n">
-        <v>13.1</v>
-      </c>
-      <c r="N6" t="n">
-        <v>8</v>
+        <v>49.8</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>40.1</v>
+        <v>54.2</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1027,33 +1028,37 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>NEE</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>77.05</v>
+        <v>155.61</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -1068,48 +1073,48 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>62.4</v>
+        <v>70.5</v>
       </c>
       <c r="J7" t="n">
-        <v>38.7</v>
+        <v>53.6</v>
       </c>
       <c r="K7" t="n">
-        <v>80</v>
+        <v>9</v>
       </c>
       <c r="L7" t="n">
-        <v>1.82</v>
+        <v>2.18</v>
       </c>
       <c r="M7" t="n">
-        <v>16.3</v>
+        <v>22</v>
       </c>
       <c r="N7" t="n">
-        <v>17.5</v>
+        <v>30.8</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>34.7</v>
+        <v>53.2</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1127,7 +1132,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr"/>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V7" t="inlineStr">
         <is>
           <t>No</t>
@@ -1137,67 +1146,64 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>EXC</t>
+          <t>DXCM</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>41.56</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>60.8</v>
+        <v>70</v>
       </c>
       <c r="J8" t="n">
-        <v>45.4</v>
+        <v>43</v>
       </c>
       <c r="K8" t="n">
-        <v>86</v>
+        <v>7</v>
       </c>
       <c r="L8" t="n">
-        <v>1.62</v>
+        <v>2.55</v>
       </c>
       <c r="M8" t="n">
-        <v>14.7</v>
-      </c>
-      <c r="N8" t="n">
-        <v>8</v>
+        <v>51.8</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>39.4</v>
+        <v>56.3</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1206,20 +1212,24 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V8" t="inlineStr">
         <is>
           <t>No</t>
@@ -1229,30 +1239,30 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CCI</t>
+          <t>ILMN</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>68.97</v>
+        <v>263.39</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1266,30 +1276,30 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>59.4</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="J9" t="n">
-        <v>42.7</v>
+        <v>57</v>
       </c>
       <c r="K9" t="n">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="L9" t="n">
-        <v>2.6</v>
+        <v>6.13</v>
       </c>
       <c r="M9" t="n">
-        <v>22.4</v>
+        <v>59.1</v>
       </c>
       <c r="N9" t="n">
-        <v>22.8</v>
+        <v>60.9</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>35.9</v>
+        <v>73.7</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1298,12 +1308,12 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1321,15 +1331,15 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SRE</t>
+          <t>KO</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>79.83</v>
+        <v>87.81999999999999</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -1344,44 +1354,44 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>56.9</v>
+        <v>67.7</v>
       </c>
       <c r="J10" t="n">
-        <v>46.4</v>
+        <v>53.9</v>
       </c>
       <c r="K10" t="n">
-        <v>75</v>
+        <v>13</v>
       </c>
       <c r="L10" t="n">
-        <v>1.65</v>
+        <v>1.52</v>
       </c>
       <c r="M10" t="n">
-        <v>21.3</v>
+        <v>13.8</v>
       </c>
       <c r="N10" t="n">
-        <v>58.1</v>
+        <v>9.5</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>38.9</v>
+        <v>61.1</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1400,10 +1410,14 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V10" t="inlineStr">
         <is>
           <t>No</t>
@@ -1413,15 +1427,15 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AMP</t>
+          <t>MET</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>490.52</v>
+        <v>98.36</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -1436,63 +1450,70 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>56.4</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>32.4</v>
+        <v>58</v>
       </c>
       <c r="K11" t="n">
-        <v>90</v>
+        <v>14</v>
       </c>
       <c r="L11" t="n">
-        <v>2.42</v>
+        <v>2.13</v>
       </c>
       <c r="M11" t="n">
-        <v>31.6</v>
+        <v>20.9</v>
+      </c>
+      <c r="N11" t="n">
+        <v>31.2</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>44.6</v>
+        <v>65.7</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V11" t="inlineStr">
         <is>
           <t>No</t>
@@ -1502,30 +1523,30 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>61.49</v>
+        <v>404.79</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1535,34 +1556,34 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>56.4</v>
+        <v>67.2</v>
       </c>
       <c r="J12" t="n">
-        <v>39.7</v>
+        <v>59.5</v>
       </c>
       <c r="K12" t="n">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="L12" t="n">
-        <v>1.73</v>
+        <v>2.75</v>
       </c>
       <c r="M12" t="n">
-        <v>14.5</v>
+        <v>31.7</v>
       </c>
       <c r="N12" t="n">
-        <v>6.3</v>
+        <v>21.8</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>41.1</v>
+        <v>58.6</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1571,12 +1592,12 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -1594,11 +1615,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>XLF</t>
+          <t>CCI</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>53.75</v>
+        <v>68.70999999999999</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1631,27 +1652,30 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>55.3</v>
+        <v>62.1</v>
       </c>
       <c r="J13" t="n">
-        <v>33.3</v>
+        <v>41.7</v>
       </c>
       <c r="K13" t="n">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="L13" t="n">
-        <v>1.21</v>
+        <v>2.62</v>
       </c>
       <c r="M13" t="n">
-        <v>17.3</v>
+        <v>22.3</v>
+      </c>
+      <c r="N13" t="n">
+        <v>22.5</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>45.8</v>
+        <v>35.3</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1687,7 +1711,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>80.37</v>
+        <v>82.06</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1720,30 +1744,30 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>54.4</v>
+        <v>60.8</v>
       </c>
       <c r="J14" t="n">
-        <v>35.5</v>
+        <v>43.8</v>
       </c>
       <c r="K14" t="n">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="L14" t="n">
-        <v>2.17</v>
+        <v>2.24</v>
       </c>
       <c r="M14" t="n">
-        <v>23.8</v>
+        <v>24.8</v>
       </c>
       <c r="N14" t="n">
-        <v>42.5</v>
+        <v>48.4</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>44</v>
+        <v>46.8</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1752,17 +1776,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
@@ -1775,11 +1799,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PAYX</t>
+          <t>XLF</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>101.69</v>
+        <v>54.24</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1812,27 +1836,30 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>53.7</v>
+        <v>60.1</v>
       </c>
       <c r="J15" t="n">
-        <v>33.8</v>
+        <v>40.4</v>
       </c>
       <c r="K15" t="n">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="L15" t="n">
-        <v>2.47</v>
+        <v>1.25</v>
       </c>
       <c r="M15" t="n">
-        <v>29.4</v>
+        <v>12.7</v>
+      </c>
+      <c r="N15" t="n">
+        <v>25.5</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>43.5</v>
+        <v>48.2</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1864,11 +1891,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>DUK</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>115.56</v>
+        <v>127.6</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1901,22 +1928,22 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>53.5</v>
+        <v>58.7</v>
       </c>
       <c r="J16" t="n">
-        <v>43.2</v>
+        <v>40.3</v>
       </c>
       <c r="K16" t="n">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="L16" t="n">
-        <v>1.24</v>
+        <v>1.97</v>
       </c>
       <c r="M16" t="n">
-        <v>11.1</v>
+        <v>17.3</v>
       </c>
       <c r="N16" t="n">
-        <v>0</v>
+        <v>21.6</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1924,7 +1951,7 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>40</v>
+        <v>34.3</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1956,11 +1983,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>EW</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>657.72</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -1993,34 +2020,34 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>52.8</v>
+        <v>58.5</v>
       </c>
       <c r="J17" t="n">
-        <v>44.2</v>
+        <v>38.7</v>
       </c>
       <c r="K17" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="L17" t="n">
-        <v>2.99</v>
+        <v>2.66</v>
       </c>
       <c r="M17" t="n">
-        <v>28.8</v>
+        <v>24.5</v>
       </c>
       <c r="N17" t="n">
-        <v>40.9</v>
+        <v>44.8</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>57.2</v>
+        <v>46.5</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>FIRED</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -2030,7 +2057,7 @@
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
@@ -2040,7 +2067,7 @@
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>Squeeze Fired, Divergence, Squeeze Expanding</t>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
@@ -2052,11 +2079,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>MCD</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>189.46</v>
+        <v>237.06</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2089,30 +2116,30 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>52.6</v>
+        <v>57.8</v>
       </c>
       <c r="J18" t="n">
-        <v>30.2</v>
+        <v>39.4</v>
       </c>
       <c r="K18" t="n">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="L18" t="n">
-        <v>2.32</v>
+        <v>1.85</v>
       </c>
       <c r="M18" t="n">
-        <v>20.4</v>
+        <v>22</v>
       </c>
       <c r="N18" t="n">
-        <v>7.8</v>
+        <v>64.3</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>41.3</v>
+        <v>29.2</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2121,17 +2148,17 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
@@ -2144,11 +2171,11 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PNC</t>
+          <t>AMP</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>217.84</v>
+        <v>497.9</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2181,30 +2208,30 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>51.3</v>
+        <v>56.9</v>
       </c>
       <c r="J19" t="n">
-        <v>24.4</v>
+        <v>38.3</v>
       </c>
       <c r="K19" t="n">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="L19" t="n">
-        <v>1.87</v>
+        <v>2.38</v>
       </c>
       <c r="M19" t="n">
-        <v>17.7</v>
+        <v>24.9</v>
       </c>
       <c r="N19" t="n">
-        <v>17.6</v>
+        <v>35.6</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>39.8</v>
+        <v>46.9</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2213,38 +2240,34 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>BAC</t>
+          <t>PNC</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>53.55</v>
+        <v>219.28</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2277,22 +2300,22 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>50.5</v>
+        <v>52.9</v>
       </c>
       <c r="J20" t="n">
-        <v>23.8</v>
+        <v>28.9</v>
       </c>
       <c r="K20" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="L20" t="n">
-        <v>1.87</v>
+        <v>1.89</v>
       </c>
       <c r="M20" t="n">
-        <v>22.2</v>
+        <v>17.9</v>
       </c>
       <c r="N20" t="n">
-        <v>52.3</v>
+        <v>18.9</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2300,7 +2323,7 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>41.1</v>
+        <v>40.6</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2332,11 +2355,11 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TMUS</t>
+          <t>BAC</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>168.47</v>
+        <v>53.38</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2365,26 +2388,26 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>50.3</v>
+        <v>52.8</v>
       </c>
       <c r="J21" t="n">
-        <v>47.1</v>
+        <v>23.2</v>
       </c>
       <c r="K21" t="n">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="L21" t="n">
-        <v>2.2</v>
+        <v>1.95</v>
       </c>
       <c r="M21" t="n">
-        <v>29.9</v>
+        <v>22.2</v>
       </c>
       <c r="N21" t="n">
-        <v>36.7</v>
+        <v>52.5</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2392,7 +2415,7 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>39.7</v>
+        <v>40.8</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2401,17 +2424,17 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U21" t="inlineStr"/>
@@ -2424,11 +2447,11 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>123.71</v>
+        <v>230.55</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -2461,30 +2484,30 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>49</v>
+        <v>52.8</v>
       </c>
       <c r="J22" t="n">
-        <v>22.2</v>
+        <v>41.3</v>
       </c>
       <c r="K22" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="L22" t="n">
-        <v>1.83</v>
+        <v>2.12</v>
       </c>
       <c r="M22" t="n">
-        <v>13.9</v>
+        <v>25</v>
       </c>
       <c r="N22" t="n">
-        <v>0</v>
+        <v>48.5</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P22" t="n">
-        <v>29.3</v>
+        <v>46.9</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
@@ -2493,38 +2516,34 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr"/>
       <c r="V22" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MCD</t>
+          <t>PCAR</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>230.96</v>
+        <v>109.43</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -2557,22 +2576,22 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>46.8</v>
+        <v>50</v>
       </c>
       <c r="J23" t="n">
-        <v>25</v>
+        <v>30.9</v>
       </c>
       <c r="K23" t="n">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="L23" t="n">
-        <v>1.68</v>
+        <v>2.4</v>
       </c>
       <c r="M23" t="n">
-        <v>20.1</v>
+        <v>18.9</v>
       </c>
       <c r="N23" t="n">
-        <v>50.7</v>
+        <v>15.2</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2580,7 +2599,7 @@
         </is>
       </c>
       <c r="P23" t="n">
-        <v>23.9</v>
+        <v>36</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -2589,17 +2608,17 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U23" t="inlineStr"/>
@@ -2612,11 +2631,11 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ALL</t>
+          <t>FANG</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>224.32</v>
+        <v>191.72</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -2649,30 +2668,30 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>46.6</v>
+        <v>49.6</v>
       </c>
       <c r="J24" t="n">
-        <v>29.8</v>
+        <v>50.8</v>
       </c>
       <c r="K24" t="n">
-        <v>96</v>
+        <v>82</v>
       </c>
       <c r="L24" t="n">
-        <v>2</v>
+        <v>2.63</v>
       </c>
       <c r="M24" t="n">
-        <v>23.8</v>
+        <v>33</v>
       </c>
       <c r="N24" t="n">
-        <v>41.5</v>
+        <v>53.1</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P24" t="n">
-        <v>42.8</v>
+        <v>51.2</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -2704,11 +2723,11 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CMCSA</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>21.01</v>
+        <v>187.27</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -2741,30 +2760,30 @@
         </is>
       </c>
       <c r="I25" t="n">
-        <v>46.5</v>
+        <v>49</v>
       </c>
       <c r="J25" t="n">
-        <v>23.4</v>
+        <v>27.8</v>
       </c>
       <c r="K25" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="L25" t="n">
-        <v>2.64</v>
+        <v>2.29</v>
       </c>
       <c r="M25" t="n">
-        <v>29</v>
+        <v>20.4</v>
       </c>
       <c r="N25" t="n">
-        <v>24.6</v>
+        <v>7.8</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P25" t="n">
-        <v>34.3</v>
+        <v>39.9</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
@@ -2786,81 +2805,77 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U25" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U25" t="inlineStr"/>
       <c r="V25" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SCHW</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>95.69</v>
+        <v>652.23</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>44.2</v>
+        <v>48.4</v>
       </c>
       <c r="J26" t="n">
-        <v>30.5</v>
+        <v>42.3</v>
       </c>
       <c r="K26" t="n">
-        <v>88</v>
+        <v>11</v>
       </c>
       <c r="L26" t="n">
-        <v>2.16</v>
+        <v>3</v>
       </c>
       <c r="M26" t="n">
-        <v>25.5</v>
+        <v>29</v>
       </c>
       <c r="N26" t="n">
-        <v>49.9</v>
+        <v>41.7</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P26" t="n">
-        <v>43.3</v>
+        <v>56</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
@@ -2874,7 +2889,7 @@
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
@@ -2882,21 +2897,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U26" t="inlineStr"/>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>FANG</t>
+          <t>CMCSA</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>184.27</v>
+        <v>21.11</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -2929,30 +2948,30 @@
         </is>
       </c>
       <c r="I27" t="n">
-        <v>42</v>
+        <v>46.1</v>
       </c>
       <c r="J27" t="n">
-        <v>38.5</v>
+        <v>28.5</v>
       </c>
       <c r="K27" t="n">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="L27" t="n">
         <v>2.49</v>
       </c>
       <c r="M27" t="n">
-        <v>30.6</v>
+        <v>28.8</v>
       </c>
       <c r="N27" t="n">
-        <v>39.5</v>
+        <v>23.9</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P27" t="n">
-        <v>47.6</v>
+        <v>35.5</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
@@ -2961,17 +2980,17 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U27" t="inlineStr"/>
@@ -2984,11 +3003,11 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CMG</t>
+          <t>SCHW</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>30.77</v>
+        <v>97.06999999999999</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -3017,34 +3036,34 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I28" t="n">
-        <v>41.9</v>
+        <v>44.9</v>
       </c>
       <c r="J28" t="n">
-        <v>31.2</v>
+        <v>36.4</v>
       </c>
       <c r="K28" t="n">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="L28" t="n">
-        <v>3.49</v>
+        <v>2.09</v>
       </c>
       <c r="M28" t="n">
-        <v>30.5</v>
+        <v>25.4</v>
       </c>
       <c r="N28" t="n">
-        <v>21.1</v>
+        <v>49.7</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P28" t="n">
-        <v>42.3</v>
+        <v>45.3</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
@@ -3076,11 +3095,11 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>JPM</t>
+          <t>CHTR</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>329.44</v>
+        <v>109.25</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -3113,30 +3132,30 @@
         </is>
       </c>
       <c r="I29" t="n">
-        <v>41.9</v>
+        <v>44.3</v>
       </c>
       <c r="J29" t="n">
-        <v>33.7</v>
+        <v>31.8</v>
       </c>
       <c r="K29" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="L29" t="n">
-        <v>1.7</v>
+        <v>4.78</v>
       </c>
       <c r="M29" t="n">
-        <v>16.6</v>
+        <v>54.4</v>
       </c>
       <c r="N29" t="n">
-        <v>18.9</v>
+        <v>47.5</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P29" t="n">
-        <v>48.6</v>
+        <v>30.8</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
@@ -3145,17 +3164,17 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U29" t="inlineStr"/>
@@ -3168,11 +3187,11 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CHTR</t>
+          <t>JPM</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>107.9</v>
+        <v>331.64</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -3201,34 +3220,34 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I30" t="n">
-        <v>41.8</v>
+        <v>43.5</v>
       </c>
       <c r="J30" t="n">
-        <v>28.4</v>
+        <v>37.6</v>
       </c>
       <c r="K30" t="n">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="L30" t="n">
-        <v>4.73</v>
+        <v>1.73</v>
       </c>
       <c r="M30" t="n">
-        <v>53.6</v>
+        <v>16.7</v>
       </c>
       <c r="N30" t="n">
-        <v>46.3</v>
+        <v>20</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P30" t="n">
-        <v>30.5</v>
+        <v>49.9</v>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
@@ -3260,11 +3279,11 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>PCAR</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>106.86</v>
+        <v>27.51</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -3293,26 +3312,26 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I31" t="n">
-        <v>40.4</v>
+        <v>41.2</v>
       </c>
       <c r="J31" t="n">
-        <v>17.7</v>
+        <v>39.5</v>
       </c>
       <c r="K31" t="n">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="L31" t="n">
-        <v>2.26</v>
+        <v>2.83</v>
       </c>
       <c r="M31" t="n">
-        <v>16.8</v>
+        <v>35.6</v>
       </c>
       <c r="N31" t="n">
-        <v>4.1</v>
+        <v>65.3</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
@@ -3320,7 +3339,7 @@
         </is>
       </c>
       <c r="P31" t="n">
-        <v>33.7</v>
+        <v>36.4</v>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
@@ -3329,38 +3348,34 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U31" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr"/>
       <c r="V31" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>GS</t>
+          <t>VZ</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>886.99</v>
+        <v>46.4</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -3389,34 +3404,34 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I32" t="n">
-        <v>39.6</v>
+        <v>40.9</v>
       </c>
       <c r="J32" t="n">
-        <v>30</v>
+        <v>41.4</v>
       </c>
       <c r="K32" t="n">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="L32" t="n">
-        <v>2.39</v>
+        <v>1.71</v>
       </c>
       <c r="M32" t="n">
-        <v>24.2</v>
+        <v>19.8</v>
       </c>
       <c r="N32" t="n">
-        <v>10.5</v>
+        <v>24.5</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P32" t="n">
-        <v>36.4</v>
+        <v>49.4</v>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
@@ -3438,25 +3453,21 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U32" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U32" t="inlineStr"/>
       <c r="V32" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>26.72</v>
+        <v>881.59</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -3485,26 +3496,23 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I33" t="n">
-        <v>38.2</v>
+        <v>36.1</v>
       </c>
       <c r="J33" t="n">
-        <v>30.8</v>
+        <v>29</v>
       </c>
       <c r="K33" t="n">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="L33" t="n">
-        <v>2.76</v>
+        <v>2.25</v>
       </c>
       <c r="M33" t="n">
-        <v>33.9</v>
-      </c>
-      <c r="N33" t="n">
-        <v>59.8</v>
+        <v>35.3</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
@@ -3512,7 +3520,7 @@
         </is>
       </c>
       <c r="P33" t="n">
-        <v>34</v>
+        <v>35.8</v>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
@@ -3536,98 +3544,6 @@
       </c>
       <c r="U33" t="inlineStr"/>
       <c r="V33" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>VZ</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>46.02</v>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>37.6</v>
-      </c>
-      <c r="J34" t="n">
-        <v>36.1</v>
-      </c>
-      <c r="K34" t="n">
-        <v>82</v>
-      </c>
-      <c r="L34" t="n">
-        <v>1.65</v>
-      </c>
-      <c r="M34" t="n">
-        <v>19.2</v>
-      </c>
-      <c r="N34" t="n">
-        <v>22.3</v>
-      </c>
-      <c r="O34" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P34" t="n">
-        <v>48.2</v>
-      </c>
-      <c r="Q34" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R34" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S34" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T34" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U34" t="inlineStr"/>
-      <c r="V34" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 09.10.2026 19:23 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,11 +435,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V33"/>
+  <dimension ref="A1:V34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>52.41</v>
+        <v>53.13</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,22 +614,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>91.40000000000001</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>49.5</v>
+        <v>54.7</v>
       </c>
       <c r="K2" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="L2" t="n">
-        <v>1.73</v>
+        <v>1.72</v>
       </c>
       <c r="M2" t="n">
-        <v>26.9</v>
+        <v>26.7</v>
       </c>
       <c r="N2" t="n">
-        <v>39.9</v>
+        <v>38.6</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>39</v>
+        <v>41.3</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -659,7 +659,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr"/>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V2" t="inlineStr">
         <is>
           <t>No</t>
@@ -669,11 +673,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ZTS</t>
+          <t>PDD</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>73.34999999999999</v>
+        <v>81.19</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -706,22 +710,22 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>86.59999999999999</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="J3" t="n">
-        <v>54.3</v>
+        <v>55.5</v>
       </c>
       <c r="K3" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="L3" t="n">
-        <v>2.47</v>
+        <v>2.34</v>
       </c>
       <c r="M3" t="n">
-        <v>24.1</v>
+        <v>25.1</v>
       </c>
       <c r="N3" t="n">
-        <v>11.5</v>
+        <v>15.1</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -729,7 +733,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>35.5</v>
+        <v>43.2</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -765,30 +769,30 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>FCX</t>
+          <t>ADP</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>70.86</v>
+        <v>271.82</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -802,22 +806,22 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>80.59999999999999</v>
+        <v>84.2</v>
       </c>
       <c r="J4" t="n">
-        <v>47.5</v>
+        <v>56.5</v>
       </c>
       <c r="K4" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="L4" t="n">
-        <v>3.51</v>
+        <v>2.02</v>
       </c>
       <c r="M4" t="n">
-        <v>36.8</v>
+        <v>23</v>
       </c>
       <c r="N4" t="n">
-        <v>23.2</v>
+        <v>31.7</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -825,31 +829,31 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>56.5</v>
+        <v>59.8</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>Squeeze Expanding</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -861,11 +865,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>FCX</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>271.54</v>
+        <v>73.73</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -898,22 +902,22 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>77.09999999999999</v>
+        <v>84</v>
       </c>
       <c r="J5" t="n">
-        <v>56.1</v>
+        <v>56.2</v>
       </c>
       <c r="K5" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="L5" t="n">
-        <v>2.16</v>
+        <v>3.44</v>
       </c>
       <c r="M5" t="n">
-        <v>23.6</v>
+        <v>38.4</v>
       </c>
       <c r="N5" t="n">
-        <v>34.3</v>
+        <v>27.8</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -921,11 +925,11 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>59.7</v>
+        <v>60.2</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -935,17 +939,17 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>Squeeze Expanding</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
@@ -957,64 +961,67 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>ZTS</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>348.26</v>
+        <v>74.45</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>74.59999999999999</v>
+        <v>83.5</v>
       </c>
       <c r="J6" t="n">
-        <v>64</v>
+        <v>58.4</v>
       </c>
       <c r="K6" t="n">
-        <v>99</v>
+        <v>28</v>
       </c>
       <c r="L6" t="n">
-        <v>3.28</v>
+        <v>2.4</v>
       </c>
       <c r="M6" t="n">
-        <v>49.8</v>
+        <v>22.7</v>
+      </c>
+      <c r="N6" t="n">
+        <v>8.9</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>54.2</v>
+        <v>37.4</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1028,7 +1035,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1036,25 +1043,21 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>BLK</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>155.61</v>
+        <v>1085.89</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1087,30 +1090,30 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>70.5</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>53.6</v>
+        <v>52.1</v>
       </c>
       <c r="K7" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="L7" t="n">
-        <v>2.18</v>
+        <v>2.07</v>
       </c>
       <c r="M7" t="n">
         <v>22</v>
       </c>
       <c r="N7" t="n">
-        <v>30.8</v>
+        <v>11.1</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>53.2</v>
+        <v>52.1</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1146,30 +1149,30 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>DXCM</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>84.40000000000001</v>
+        <v>156.49</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1183,19 +1186,22 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>70</v>
+        <v>79.2</v>
       </c>
       <c r="J8" t="n">
-        <v>43</v>
+        <v>55.6</v>
       </c>
       <c r="K8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L8" t="n">
-        <v>2.55</v>
+        <v>2.05</v>
       </c>
       <c r="M8" t="n">
-        <v>51.8</v>
+        <v>22</v>
+      </c>
+      <c r="N8" t="n">
+        <v>30.7</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1203,31 +1209,31 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>56.3</v>
+        <v>54</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>Squeeze Expanding</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
@@ -1239,59 +1245,59 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ILMN</t>
+          <t>UNH</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>263.39</v>
+        <v>382.41</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>68.40000000000001</v>
+        <v>76.8</v>
       </c>
       <c r="J9" t="n">
-        <v>57</v>
+        <v>52.5</v>
       </c>
       <c r="K9" t="n">
-        <v>91</v>
+        <v>4</v>
       </c>
       <c r="L9" t="n">
-        <v>6.13</v>
+        <v>2.54</v>
       </c>
       <c r="M9" t="n">
-        <v>59.1</v>
+        <v>21.1</v>
       </c>
       <c r="N9" t="n">
-        <v>60.9</v>
+        <v>4.6</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1299,21 +1305,21 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>73.7</v>
+        <v>52</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1321,7 +1327,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr"/>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V9" t="inlineStr">
         <is>
           <t>No</t>
@@ -1335,7 +1345,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>87.81999999999999</v>
+        <v>88.31</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1368,22 +1378,22 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>67.7</v>
+        <v>73.5</v>
       </c>
       <c r="J10" t="n">
-        <v>53.9</v>
+        <v>56.4</v>
       </c>
       <c r="K10" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="L10" t="n">
-        <v>1.52</v>
+        <v>1.46</v>
       </c>
       <c r="M10" t="n">
-        <v>13.8</v>
+        <v>13.4</v>
       </c>
       <c r="N10" t="n">
-        <v>9.5</v>
+        <v>7.4</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1391,7 +1401,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>61.1</v>
+        <v>61.9</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1427,15 +1437,15 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MET</t>
+          <t>TLT</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>98.36</v>
+        <v>77.84999999999999</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -1450,48 +1460,45 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>67.40000000000001</v>
+        <v>71.5</v>
       </c>
       <c r="J11" t="n">
-        <v>58</v>
+        <v>35.9</v>
       </c>
       <c r="K11" t="n">
-        <v>14</v>
+        <v>99</v>
       </c>
       <c r="L11" t="n">
-        <v>2.13</v>
+        <v>1.03</v>
       </c>
       <c r="M11" t="n">
-        <v>20.9</v>
-      </c>
-      <c r="N11" t="n">
-        <v>31.2</v>
+        <v>13.7</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>65.7</v>
+        <v>31.7</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1501,7 +1508,7 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1509,11 +1516,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr">
         <is>
           <t>No</t>
@@ -1523,11 +1526,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>404.79</v>
+        <v>351.11</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1560,22 +1563,22 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>67.2</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="J12" t="n">
-        <v>59.5</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="K12" t="n">
         <v>98</v>
       </c>
       <c r="L12" t="n">
-        <v>2.75</v>
+        <v>3.09</v>
       </c>
       <c r="M12" t="n">
-        <v>31.7</v>
+        <v>43.2</v>
       </c>
       <c r="N12" t="n">
-        <v>21.8</v>
+        <v>63.1</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1583,7 +1586,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>58.6</v>
+        <v>54.9</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1592,17 +1595,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
@@ -1615,30 +1618,30 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CCI</t>
+          <t>ILMN</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>68.70999999999999</v>
+        <v>275.98</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1652,30 +1655,30 @@
         </is>
       </c>
       <c r="I13" t="n">
+        <v>68.3</v>
+      </c>
+      <c r="J13" t="n">
         <v>62.1</v>
       </c>
-      <c r="J13" t="n">
-        <v>41.7</v>
-      </c>
       <c r="K13" t="n">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="L13" t="n">
-        <v>2.62</v>
+        <v>5.64</v>
       </c>
       <c r="M13" t="n">
-        <v>22.3</v>
+        <v>59.9</v>
       </c>
       <c r="N13" t="n">
-        <v>22.5</v>
+        <v>62.5</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>35.3</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1684,12 +1687,12 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -1707,15 +1710,15 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>WFC</t>
+          <t>MET</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>82.06</v>
+        <v>98.22</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -1730,48 +1733,48 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>60.8</v>
+        <v>67.2</v>
       </c>
       <c r="J14" t="n">
-        <v>43.8</v>
+        <v>57.3</v>
       </c>
       <c r="K14" t="n">
-        <v>94</v>
+        <v>17</v>
       </c>
       <c r="L14" t="n">
-        <v>2.24</v>
+        <v>2.16</v>
       </c>
       <c r="M14" t="n">
-        <v>24.8</v>
+        <v>21</v>
       </c>
       <c r="N14" t="n">
-        <v>48.4</v>
+        <v>32</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>46.8</v>
+        <v>65.5</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -1781,7 +1784,7 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -1789,7 +1792,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr"/>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V14" t="inlineStr">
         <is>
           <t>No</t>
@@ -1799,11 +1806,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>XLF</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>54.24</v>
+        <v>126.05</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1836,30 +1843,30 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>60.1</v>
+        <v>66</v>
       </c>
       <c r="J15" t="n">
-        <v>40.4</v>
+        <v>37.5</v>
       </c>
       <c r="K15" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="L15" t="n">
-        <v>1.25</v>
+        <v>2.21</v>
       </c>
       <c r="M15" t="n">
-        <v>12.7</v>
+        <v>18.4</v>
       </c>
       <c r="N15" t="n">
-        <v>25.5</v>
+        <v>28.8</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>48.2</v>
+        <v>31.4</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1891,11 +1898,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>WFC</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>127.6</v>
+        <v>84.02</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1924,34 +1931,34 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>58.7</v>
+        <v>65.7</v>
       </c>
       <c r="J16" t="n">
-        <v>40.3</v>
+        <v>51.5</v>
       </c>
       <c r="K16" t="n">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="L16" t="n">
-        <v>1.97</v>
+        <v>2.29</v>
       </c>
       <c r="M16" t="n">
-        <v>17.3</v>
+        <v>25.8</v>
       </c>
       <c r="N16" t="n">
-        <v>21.6</v>
+        <v>54.5</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>34.3</v>
+        <v>49.8</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1983,15 +1990,15 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>EW</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>83.98999999999999</v>
+        <v>404.91</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -2006,48 +2013,48 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>58.5</v>
+        <v>63.7</v>
       </c>
       <c r="J17" t="n">
-        <v>38.7</v>
+        <v>59.6</v>
       </c>
       <c r="K17" t="n">
-        <v>17</v>
+        <v>98</v>
       </c>
       <c r="L17" t="n">
-        <v>2.66</v>
+        <v>2.76</v>
       </c>
       <c r="M17" t="n">
-        <v>24.5</v>
+        <v>31.6</v>
       </c>
       <c r="N17" t="n">
-        <v>44.8</v>
+        <v>21.5</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>46.5</v>
+        <v>58.7</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -2057,7 +2064,7 @@
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
@@ -2067,7 +2074,7 @@
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+          <t>Divergence</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
@@ -2079,11 +2086,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>MCD</t>
+          <t>XLF</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>237.06</v>
+        <v>54.81</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2112,34 +2119,31 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>57.8</v>
+        <v>58.4</v>
       </c>
       <c r="J18" t="n">
-        <v>39.4</v>
+        <v>47.2</v>
       </c>
       <c r="K18" t="n">
-        <v>94</v>
+        <v>69</v>
       </c>
       <c r="L18" t="n">
-        <v>1.85</v>
+        <v>1.23</v>
       </c>
       <c r="M18" t="n">
-        <v>22</v>
-      </c>
-      <c r="N18" t="n">
-        <v>64.3</v>
+        <v>17.6</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>29.2</v>
+        <v>50.8</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2171,11 +2175,11 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>AMP</t>
+          <t>MCD</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>497.9</v>
+        <v>235.85</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2208,30 +2212,30 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>56.9</v>
+        <v>57.8</v>
       </c>
       <c r="J19" t="n">
-        <v>38.3</v>
+        <v>37.7</v>
       </c>
       <c r="K19" t="n">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="L19" t="n">
-        <v>2.38</v>
+        <v>1.8</v>
       </c>
       <c r="M19" t="n">
-        <v>24.9</v>
+        <v>20.9</v>
       </c>
       <c r="N19" t="n">
-        <v>35.6</v>
+        <v>56.7</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>46.9</v>
+        <v>28.1</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2263,11 +2267,11 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PNC</t>
+          <t>AMP</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>219.28</v>
+        <v>500.61</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2300,30 +2304,30 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>52.9</v>
+        <v>55.3</v>
       </c>
       <c r="J20" t="n">
-        <v>28.9</v>
+        <v>40.3</v>
       </c>
       <c r="K20" t="n">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="L20" t="n">
-        <v>1.89</v>
+        <v>2.22</v>
       </c>
       <c r="M20" t="n">
-        <v>17.9</v>
+        <v>25.1</v>
       </c>
       <c r="N20" t="n">
-        <v>18.9</v>
+        <v>36.5</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>40.6</v>
+        <v>47.7</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2332,17 +2336,17 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U20" t="inlineStr"/>
@@ -2355,11 +2359,11 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>BAC</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>53.38</v>
+        <v>230.01</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2392,30 +2396,30 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>52.8</v>
+        <v>53.1</v>
       </c>
       <c r="J21" t="n">
-        <v>23.2</v>
+        <v>40.7</v>
       </c>
       <c r="K21" t="n">
         <v>92</v>
       </c>
       <c r="L21" t="n">
-        <v>1.95</v>
+        <v>1.98</v>
       </c>
       <c r="M21" t="n">
-        <v>22.2</v>
+        <v>24.8</v>
       </c>
       <c r="N21" t="n">
-        <v>52.5</v>
+        <v>47.2</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>40.8</v>
+        <v>46.6</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2424,17 +2428,17 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U21" t="inlineStr"/>
@@ -2447,11 +2451,11 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ALL</t>
+          <t>BAC</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>230.55</v>
+        <v>54.36</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -2480,34 +2484,34 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>52.8</v>
+        <v>52.5</v>
       </c>
       <c r="J22" t="n">
-        <v>41.3</v>
+        <v>32.4</v>
       </c>
       <c r="K22" t="n">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="L22" t="n">
-        <v>2.12</v>
+        <v>1.91</v>
       </c>
       <c r="M22" t="n">
-        <v>25</v>
+        <v>22.6</v>
       </c>
       <c r="N22" t="n">
-        <v>48.5</v>
+        <v>54.9</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P22" t="n">
-        <v>46.9</v>
+        <v>43.2</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
@@ -2539,11 +2543,11 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>PCAR</t>
+          <t>FANG</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>109.43</v>
+        <v>192.48</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -2572,34 +2576,34 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>50</v>
+        <v>51.4</v>
       </c>
       <c r="J23" t="n">
-        <v>30.9</v>
+        <v>51.9</v>
       </c>
       <c r="K23" t="n">
-        <v>91</v>
+        <v>74</v>
       </c>
       <c r="L23" t="n">
-        <v>2.4</v>
+        <v>2.47</v>
       </c>
       <c r="M23" t="n">
-        <v>18.9</v>
+        <v>33</v>
       </c>
       <c r="N23" t="n">
-        <v>15.2</v>
+        <v>53</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>36</v>
+        <v>51.6</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -2631,11 +2635,11 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>FANG</t>
+          <t>CHTR</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>191.72</v>
+        <v>103.68</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -2668,30 +2672,30 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>49.6</v>
+        <v>51.1</v>
       </c>
       <c r="J24" t="n">
-        <v>50.8</v>
+        <v>28.1</v>
       </c>
       <c r="K24" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="L24" t="n">
-        <v>2.63</v>
+        <v>5.3</v>
       </c>
       <c r="M24" t="n">
-        <v>33</v>
+        <v>55.6</v>
       </c>
       <c r="N24" t="n">
-        <v>53.1</v>
+        <v>49.2</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P24" t="n">
-        <v>51.2</v>
+        <v>29.4</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -2700,34 +2704,38 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="U24" t="inlineStr"/>
-      <c r="V24" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>PCAR</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>187.27</v>
+        <v>108.32</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -2760,30 +2768,30 @@
         </is>
       </c>
       <c r="I25" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J25" t="n">
-        <v>27.8</v>
+        <v>29.3</v>
       </c>
       <c r="K25" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="L25" t="n">
-        <v>2.29</v>
+        <v>2.4</v>
       </c>
       <c r="M25" t="n">
-        <v>20.4</v>
+        <v>18.8</v>
       </c>
       <c r="N25" t="n">
-        <v>7.8</v>
+        <v>14.4</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P25" t="n">
-        <v>39.9</v>
+        <v>35</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
@@ -2792,17 +2800,17 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U25" t="inlineStr"/>
@@ -2815,67 +2823,67 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>CMCSA</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>652.23</v>
+        <v>20.65</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>48.4</v>
+        <v>47.9</v>
       </c>
       <c r="J26" t="n">
-        <v>42.3</v>
+        <v>26.1</v>
       </c>
       <c r="K26" t="n">
-        <v>11</v>
+        <v>78</v>
       </c>
       <c r="L26" t="n">
-        <v>3</v>
+        <v>2.67</v>
       </c>
       <c r="M26" t="n">
-        <v>29</v>
+        <v>28.9</v>
       </c>
       <c r="N26" t="n">
-        <v>41.7</v>
+        <v>24.2</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P26" t="n">
-        <v>56</v>
+        <v>34.1</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
@@ -2889,7 +2897,7 @@
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
@@ -2897,25 +2905,21 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U26" t="inlineStr">
-        <is>
-          <t>Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U26" t="inlineStr"/>
       <c r="V26" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CMCSA</t>
+          <t>TTD</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>21.11</v>
+        <v>12.06</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -2948,22 +2952,22 @@
         </is>
       </c>
       <c r="I27" t="n">
-        <v>46.1</v>
+        <v>47.2</v>
       </c>
       <c r="J27" t="n">
-        <v>28.5</v>
+        <v>35</v>
       </c>
       <c r="K27" t="n">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="L27" t="n">
-        <v>2.49</v>
+        <v>3.56</v>
       </c>
       <c r="M27" t="n">
-        <v>28.8</v>
+        <v>39.9</v>
       </c>
       <c r="N27" t="n">
-        <v>23.9</v>
+        <v>19.1</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -2971,7 +2975,7 @@
         </is>
       </c>
       <c r="P27" t="n">
-        <v>35.5</v>
+        <v>27.4</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
@@ -2980,17 +2984,17 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U27" t="inlineStr"/>
@@ -3003,11 +3007,11 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SCHW</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>97.06999999999999</v>
+        <v>190.31</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -3036,34 +3040,34 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I28" t="n">
-        <v>44.9</v>
+        <v>45.8</v>
       </c>
       <c r="J28" t="n">
-        <v>36.4</v>
+        <v>35.1</v>
       </c>
       <c r="K28" t="n">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="L28" t="n">
-        <v>2.09</v>
+        <v>2.19</v>
       </c>
       <c r="M28" t="n">
-        <v>25.4</v>
+        <v>21</v>
       </c>
       <c r="N28" t="n">
-        <v>49.7</v>
+        <v>10.6</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P28" t="n">
-        <v>45.3</v>
+        <v>41.8</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
@@ -3072,17 +3076,17 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U28" t="inlineStr"/>
@@ -3095,11 +3099,11 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CHTR</t>
+          <t>PNC</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>109.25</v>
+        <v>219.97</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -3128,34 +3132,34 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I29" t="n">
-        <v>44.3</v>
+        <v>44.7</v>
       </c>
       <c r="J29" t="n">
-        <v>31.8</v>
+        <v>30.9</v>
       </c>
       <c r="K29" t="n">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="L29" t="n">
-        <v>4.78</v>
+        <v>1.78</v>
       </c>
       <c r="M29" t="n">
-        <v>54.4</v>
+        <v>18.1</v>
       </c>
       <c r="N29" t="n">
-        <v>47.5</v>
+        <v>19.8</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P29" t="n">
-        <v>30.8</v>
+        <v>41</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
@@ -3187,11 +3191,11 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>JPM</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>331.64</v>
+        <v>27.28</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -3224,30 +3228,30 @@
         </is>
       </c>
       <c r="I30" t="n">
-        <v>43.5</v>
+        <v>42.4</v>
       </c>
       <c r="J30" t="n">
-        <v>37.6</v>
+        <v>38</v>
       </c>
       <c r="K30" t="n">
         <v>78</v>
       </c>
       <c r="L30" t="n">
-        <v>1.73</v>
+        <v>2.8</v>
       </c>
       <c r="M30" t="n">
-        <v>16.7</v>
+        <v>35.4</v>
       </c>
       <c r="N30" t="n">
-        <v>20</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P30" t="n">
-        <v>49.9</v>
+        <v>35.4</v>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
@@ -3256,17 +3260,17 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U30" t="inlineStr"/>
@@ -3279,11 +3283,11 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>SCHW</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>27.51</v>
+        <v>97.09</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -3316,30 +3320,30 @@
         </is>
       </c>
       <c r="I31" t="n">
-        <v>41.2</v>
+        <v>41.5</v>
       </c>
       <c r="J31" t="n">
-        <v>39.5</v>
+        <v>36.5</v>
       </c>
       <c r="K31" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="L31" t="n">
-        <v>2.83</v>
+        <v>1.95</v>
       </c>
       <c r="M31" t="n">
-        <v>35.6</v>
+        <v>25.2</v>
       </c>
       <c r="N31" t="n">
-        <v>65.3</v>
+        <v>48.6</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P31" t="n">
-        <v>36.4</v>
+        <v>45.3</v>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
@@ -3371,11 +3375,11 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>VZ</t>
+          <t>JPM</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>46.4</v>
+        <v>333.51</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -3411,19 +3415,19 @@
         <v>40.9</v>
       </c>
       <c r="J32" t="n">
-        <v>41.4</v>
+        <v>40.9</v>
       </c>
       <c r="K32" t="n">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="L32" t="n">
-        <v>1.71</v>
+        <v>1.61</v>
       </c>
       <c r="M32" t="n">
-        <v>19.8</v>
+        <v>16.8</v>
       </c>
       <c r="N32" t="n">
-        <v>24.5</v>
+        <v>20.6</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -3431,7 +3435,7 @@
         </is>
       </c>
       <c r="P32" t="n">
-        <v>49.4</v>
+        <v>51</v>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
@@ -3440,17 +3444,17 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U32" t="inlineStr"/>
@@ -3463,87 +3467,186 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>625.6799999999999</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="J33" t="n">
+        <v>34.6</v>
+      </c>
+      <c r="K33" t="n">
+        <v>29</v>
+      </c>
+      <c r="L33" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="M33" t="n">
+        <v>31</v>
+      </c>
+      <c r="N33" t="n">
+        <v>49</v>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P33" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>GS</t>
         </is>
       </c>
-      <c r="B33" t="n">
-        <v>881.59</v>
-      </c>
-      <c r="C33" t="inlineStr">
+      <c r="B34" t="n">
+        <v>898.28</v>
+      </c>
+      <c r="C34" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>Credit Put</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>7-21 DTE</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="H34" t="inlineStr">
         <is>
           <t>NEUTRAL</t>
         </is>
       </c>
-      <c r="I33" t="n">
+      <c r="I34" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="J34" t="n">
         <v>36.1</v>
       </c>
-      <c r="J33" t="n">
-        <v>29</v>
-      </c>
-      <c r="K33" t="n">
-        <v>79</v>
-      </c>
-      <c r="L33" t="n">
-        <v>2.25</v>
-      </c>
-      <c r="M33" t="n">
-        <v>35.3</v>
-      </c>
-      <c r="O33" t="inlineStr">
+      <c r="K34" t="n">
+        <v>46</v>
+      </c>
+      <c r="L34" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="M34" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="N34" t="n">
+        <v>13</v>
+      </c>
+      <c r="O34" t="inlineStr">
         <is>
           <t>Bearish</t>
         </is>
       </c>
-      <c r="P33" t="n">
-        <v>35.8</v>
-      </c>
-      <c r="Q33" t="inlineStr">
+      <c r="P34" t="n">
+        <v>37.8</v>
+      </c>
+      <c r="Q34" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S33" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T33" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U33" t="inlineStr"/>
-      <c r="V33" t="inlineStr">
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr"/>
+      <c r="V34" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 12.10.2026 22:02 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -31,10 +31,10 @@
       <sz val="11"/>
     </font>
     <font>
-      <color rgb="00ef4444"/>
+      <color rgb="0022c55e"/>
     </font>
     <font>
-      <color rgb="0022c55e"/>
+      <color rgb="00ef4444"/>
     </font>
   </fonts>
   <fills count="3">
@@ -435,11 +435,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V34"/>
+  <dimension ref="A1:V28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TSN</t>
+          <t>ADP</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>53.13</v>
+        <v>273.81</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -590,17 +590,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -614,30 +614,30 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>92.59999999999999</v>
+        <v>91.7</v>
       </c>
       <c r="J2" t="n">
-        <v>54.7</v>
+        <v>58.7</v>
       </c>
       <c r="K2" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="L2" t="n">
-        <v>1.72</v>
+        <v>1.91</v>
       </c>
       <c r="M2" t="n">
-        <v>26.7</v>
+        <v>23</v>
       </c>
       <c r="N2" t="n">
-        <v>38.6</v>
+        <v>31.6</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>41.3</v>
+        <v>60.6</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -659,11 +659,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
         <is>
           <t>No</t>
@@ -677,14 +673,14 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>81.19</v>
+        <v>80.92</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -710,16 +706,16 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>84.90000000000001</v>
+        <v>88.7</v>
       </c>
       <c r="J3" t="n">
-        <v>55.5</v>
+        <v>54.3</v>
       </c>
       <c r="K3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L3" t="n">
-        <v>2.34</v>
+        <v>2.23</v>
       </c>
       <c r="M3" t="n">
         <v>25.1</v>
@@ -733,7 +729,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>43.2</v>
+        <v>43</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -769,18 +765,18 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>FCX</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>271.82</v>
+        <v>73.29000000000001</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -806,22 +802,22 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>84.2</v>
+        <v>85.8</v>
       </c>
       <c r="J4" t="n">
-        <v>56.5</v>
+        <v>54.8</v>
       </c>
       <c r="K4" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="L4" t="n">
-        <v>2.02</v>
+        <v>3.16</v>
       </c>
       <c r="M4" t="n">
-        <v>23</v>
+        <v>37.8</v>
       </c>
       <c r="N4" t="n">
-        <v>31.7</v>
+        <v>25.9</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -829,11 +825,11 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>59.8</v>
+        <v>59.5</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -843,17 +839,17 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>Squeeze Expanding</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -865,18 +861,18 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>FCX</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>73.73</v>
+        <v>157.42</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -902,22 +898,19 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>84</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>56.2</v>
+        <v>57.6</v>
       </c>
       <c r="K5" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L5" t="n">
-        <v>3.44</v>
+        <v>1.88</v>
       </c>
       <c r="M5" t="n">
-        <v>38.4</v>
-      </c>
-      <c r="N5" t="n">
-        <v>27.8</v>
+        <v>36.5</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -925,7 +918,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>60.2</v>
+        <v>54.8</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -939,7 +932,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -961,11 +954,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ZTS</t>
+          <t>BKR</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>74.45</v>
+        <v>56.18</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -974,17 +967,17 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -994,38 +987,38 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>83.5</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="J6" t="n">
-        <v>58.4</v>
+        <v>42.4</v>
       </c>
       <c r="K6" t="n">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="L6" t="n">
-        <v>2.4</v>
+        <v>2.58</v>
       </c>
       <c r="M6" t="n">
-        <v>22.7</v>
+        <v>30.1</v>
       </c>
       <c r="N6" t="n">
-        <v>8.9</v>
+        <v>46.1</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>37.4</v>
+        <v>45.2</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1043,7 +1036,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr"/>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V6" t="inlineStr">
         <is>
           <t>No</t>
@@ -1053,18 +1050,18 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BLK</t>
+          <t>KO</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1085.89</v>
+        <v>89.79000000000001</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -1090,22 +1087,19 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>81.40000000000001</v>
+        <v>79.3</v>
       </c>
       <c r="J7" t="n">
-        <v>52.1</v>
+        <v>63</v>
       </c>
       <c r="K7" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="L7" t="n">
-        <v>2.07</v>
+        <v>1.51</v>
       </c>
       <c r="M7" t="n">
-        <v>22</v>
-      </c>
-      <c r="N7" t="n">
-        <v>11.1</v>
+        <v>23.4</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1113,11 +1107,11 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>52.1</v>
+        <v>64.5</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1132,12 +1126,12 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>Squeeze Expanding</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
@@ -1149,59 +1143,59 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>SNPS</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>156.49</v>
+        <v>502.51</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>79.2</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="J8" t="n">
-        <v>55.6</v>
+        <v>70.7</v>
       </c>
       <c r="K8" t="n">
-        <v>6</v>
+        <v>99</v>
       </c>
       <c r="L8" t="n">
-        <v>2.05</v>
+        <v>3.68</v>
       </c>
       <c r="M8" t="n">
-        <v>22</v>
+        <v>54.2</v>
       </c>
       <c r="N8" t="n">
-        <v>30.7</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1209,11 +1203,11 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>54</v>
+        <v>59.3</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -1223,19 +1217,15 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
           <t>No</t>
@@ -1245,18 +1235,18 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>UNH</t>
+          <t>ZTS</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>382.41</v>
+        <v>75.65000000000001</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -1278,38 +1268,38 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>76.8</v>
+        <v>77.2</v>
       </c>
       <c r="J9" t="n">
-        <v>52.5</v>
+        <v>62.2</v>
       </c>
       <c r="K9" t="n">
-        <v>4</v>
+        <v>54</v>
       </c>
       <c r="L9" t="n">
-        <v>2.54</v>
+        <v>2.35</v>
       </c>
       <c r="M9" t="n">
-        <v>21.1</v>
+        <v>21.5</v>
       </c>
       <c r="N9" t="n">
-        <v>4.6</v>
+        <v>6.6</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>52</v>
+        <v>39.3</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1324,14 +1314,10 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
           <t>No</t>
@@ -1341,11 +1327,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>88.31</v>
+        <v>137.39</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1354,17 +1340,17 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1378,30 +1364,30 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>73.5</v>
+        <v>74.5</v>
       </c>
       <c r="J10" t="n">
-        <v>56.4</v>
+        <v>44.9</v>
       </c>
       <c r="K10" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="L10" t="n">
-        <v>1.46</v>
+        <v>4.46</v>
       </c>
       <c r="M10" t="n">
-        <v>13.4</v>
+        <v>50.9</v>
       </c>
       <c r="N10" t="n">
-        <v>7.4</v>
+        <v>28.1</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>61.9</v>
+        <v>42.8</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1425,12 +1411,12 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>Squeeze Expanding</t>
+          <t>Divergence, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1441,14 +1427,14 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>77.84999999999999</v>
+        <v>78.05</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -1474,19 +1460,22 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>71.5</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>35.9</v>
+        <v>38.2</v>
       </c>
       <c r="K11" t="n">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="L11" t="n">
-        <v>1.03</v>
+        <v>0.93</v>
       </c>
       <c r="M11" t="n">
-        <v>13.7</v>
+        <v>9.5</v>
+      </c>
+      <c r="N11" t="n">
+        <v>53.5</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1494,7 +1483,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>31.7</v>
+        <v>32.8</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1526,18 +1515,18 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>ILMN</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>351.11</v>
+        <v>276.67</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -1563,22 +1552,22 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>68.90000000000001</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="J12" t="n">
-        <v>65.40000000000001</v>
+        <v>61.9</v>
       </c>
       <c r="K12" t="n">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="L12" t="n">
-        <v>3.09</v>
+        <v>5.43</v>
       </c>
       <c r="M12" t="n">
-        <v>43.2</v>
+        <v>57.8</v>
       </c>
       <c r="N12" t="n">
-        <v>63.1</v>
+        <v>58.8</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1586,7 +1575,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>54.9</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1595,17 +1584,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
@@ -1618,59 +1607,59 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ILMN</t>
+          <t>MET</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>275.98</v>
+        <v>100.17</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>68.3</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="J13" t="n">
-        <v>62.1</v>
+        <v>63.3</v>
       </c>
       <c r="K13" t="n">
-        <v>89</v>
+        <v>37</v>
       </c>
       <c r="L13" t="n">
-        <v>5.64</v>
+        <v>2.08</v>
       </c>
       <c r="M13" t="n">
-        <v>59.9</v>
+        <v>21.6</v>
       </c>
       <c r="N13" t="n">
-        <v>62.5</v>
+        <v>35.9</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1678,21 +1667,21 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>79.09999999999999</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>FIRED</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -1700,7 +1689,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr"/>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>Squeeze Fired</t>
+        </is>
+      </c>
       <c r="V13" t="inlineStr">
         <is>
           <t>No</t>
@@ -1710,59 +1703,59 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MET</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>98.22</v>
+        <v>348.42</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>67.2</v>
+        <v>64.7</v>
       </c>
       <c r="J14" t="n">
-        <v>57.3</v>
+        <v>62.5</v>
       </c>
       <c r="K14" t="n">
-        <v>17</v>
+        <v>96</v>
       </c>
       <c r="L14" t="n">
-        <v>2.16</v>
+        <v>2.98</v>
       </c>
       <c r="M14" t="n">
-        <v>21</v>
+        <v>43</v>
       </c>
       <c r="N14" t="n">
-        <v>32</v>
+        <v>62.5</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1770,11 +1763,11 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>65.5</v>
+        <v>54.1</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -1789,14 +1782,10 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr">
         <is>
           <t>No</t>
@@ -1810,14 +1799,14 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>126.05</v>
+        <v>126.68</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -1839,26 +1828,26 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>66</v>
+        <v>62.5</v>
       </c>
       <c r="J15" t="n">
-        <v>37.5</v>
+        <v>39.9</v>
       </c>
       <c r="K15" t="n">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="L15" t="n">
-        <v>2.21</v>
+        <v>2.05</v>
       </c>
       <c r="M15" t="n">
-        <v>18.4</v>
+        <v>18.2</v>
       </c>
       <c r="N15" t="n">
-        <v>28.8</v>
+        <v>27.8</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1866,7 +1855,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>31.4</v>
+        <v>32.7</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1898,11 +1887,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>WFC</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>84.02</v>
+        <v>406.24</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1911,17 +1900,17 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1931,26 +1920,23 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>65.7</v>
+        <v>58.2</v>
       </c>
       <c r="J16" t="n">
-        <v>51.5</v>
+        <v>60.6</v>
       </c>
       <c r="K16" t="n">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="L16" t="n">
-        <v>2.29</v>
+        <v>2.68</v>
       </c>
       <c r="M16" t="n">
-        <v>25.8</v>
-      </c>
-      <c r="N16" t="n">
-        <v>54.5</v>
+        <v>40</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1958,7 +1944,7 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>49.8</v>
+        <v>59.1</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1967,12 +1953,12 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
@@ -1990,11 +1976,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>MCD</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>404.91</v>
+        <v>235.65</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -2003,17 +1989,17 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2027,30 +2013,27 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>63.7</v>
+        <v>58.1</v>
       </c>
       <c r="J17" t="n">
-        <v>59.6</v>
+        <v>37.9</v>
       </c>
       <c r="K17" t="n">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="L17" t="n">
-        <v>2.76</v>
+        <v>1.76</v>
       </c>
       <c r="M17" t="n">
-        <v>31.6</v>
-      </c>
-      <c r="N17" t="n">
-        <v>21.5</v>
+        <v>24.8</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>58.7</v>
+        <v>27.9</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2059,12 +2042,12 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
@@ -2072,32 +2055,28 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>XLF</t>
+          <t>VZ</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>54.81</v>
+        <v>42.78</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -2119,31 +2098,34 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>58.4</v>
+        <v>56.6</v>
       </c>
       <c r="J18" t="n">
-        <v>47.2</v>
+        <v>32.2</v>
       </c>
       <c r="K18" t="n">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="L18" t="n">
-        <v>1.23</v>
+        <v>3.03</v>
       </c>
       <c r="M18" t="n">
-        <v>17.6</v>
+        <v>32.3</v>
+      </c>
+      <c r="N18" t="n">
+        <v>72</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>50.8</v>
+        <v>42.6</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2152,17 +2134,17 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
@@ -2175,18 +2157,18 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MCD</t>
+          <t>AMP</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>235.85</v>
+        <v>500.02</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -2208,34 +2190,34 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>57.8</v>
+        <v>54.9</v>
       </c>
       <c r="J19" t="n">
-        <v>37.7</v>
+        <v>40</v>
       </c>
       <c r="K19" t="n">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="L19" t="n">
-        <v>1.8</v>
+        <v>2.16</v>
       </c>
       <c r="M19" t="n">
-        <v>20.9</v>
+        <v>24.9</v>
       </c>
       <c r="N19" t="n">
-        <v>56.7</v>
+        <v>35.8</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>28.1</v>
+        <v>47.5</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2267,18 +2249,18 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>AMP</t>
+          <t>BAC</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>500.61</v>
+        <v>54.58</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -2300,26 +2282,26 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>55.3</v>
+        <v>53.5</v>
       </c>
       <c r="J20" t="n">
-        <v>40.3</v>
+        <v>34.6</v>
       </c>
       <c r="K20" t="n">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="L20" t="n">
-        <v>2.22</v>
+        <v>1.83</v>
       </c>
       <c r="M20" t="n">
-        <v>25.1</v>
+        <v>21.7</v>
       </c>
       <c r="N20" t="n">
-        <v>36.5</v>
+        <v>49.1</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2327,7 +2309,7 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>47.7</v>
+        <v>43.9</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2359,18 +2341,18 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ALL</t>
+          <t>NOC</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>230.01</v>
+        <v>485</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -2396,30 +2378,30 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>53.1</v>
+        <v>48.9</v>
       </c>
       <c r="J21" t="n">
-        <v>40.7</v>
+        <v>38.2</v>
       </c>
       <c r="K21" t="n">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="L21" t="n">
-        <v>1.98</v>
+        <v>2.15</v>
       </c>
       <c r="M21" t="n">
-        <v>24.8</v>
+        <v>22.6</v>
       </c>
       <c r="N21" t="n">
-        <v>47.2</v>
+        <v>40.1</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>46.6</v>
+        <v>37.1</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2451,18 +2433,18 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BAC</t>
+          <t>PCAR</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>54.36</v>
+        <v>108.13</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -2488,30 +2470,30 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>52.5</v>
+        <v>46.1</v>
       </c>
       <c r="J22" t="n">
-        <v>32.4</v>
+        <v>29.2</v>
       </c>
       <c r="K22" t="n">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="L22" t="n">
-        <v>1.91</v>
+        <v>2.31</v>
       </c>
       <c r="M22" t="n">
-        <v>22.6</v>
+        <v>18.9</v>
       </c>
       <c r="N22" t="n">
-        <v>54.9</v>
+        <v>15.1</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P22" t="n">
-        <v>43.2</v>
+        <v>34.9</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
@@ -2543,18 +2525,18 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>FANG</t>
+          <t>CHTR</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>192.48</v>
+        <v>102.48</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -2576,34 +2558,31 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>51.4</v>
+        <v>45.6</v>
       </c>
       <c r="J23" t="n">
-        <v>51.9</v>
+        <v>27.3</v>
       </c>
       <c r="K23" t="n">
-        <v>74</v>
+        <v>87</v>
       </c>
       <c r="L23" t="n">
-        <v>2.47</v>
+        <v>5.03</v>
       </c>
       <c r="M23" t="n">
-        <v>33</v>
-      </c>
-      <c r="N23" t="n">
-        <v>53</v>
+        <v>78.8</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>51.6</v>
+        <v>29.1</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -2612,17 +2591,17 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U23" t="inlineStr"/>
@@ -2635,18 +2614,18 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CHTR</t>
+          <t>TTD</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>103.68</v>
+        <v>11.94</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -2668,26 +2647,23 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I24" t="n">
-        <v>51.1</v>
+        <v>45.6</v>
       </c>
       <c r="J24" t="n">
-        <v>28.1</v>
+        <v>33.7</v>
       </c>
       <c r="K24" t="n">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="L24" t="n">
-        <v>5.3</v>
+        <v>3.61</v>
       </c>
       <c r="M24" t="n">
-        <v>55.6</v>
-      </c>
-      <c r="N24" t="n">
-        <v>49.2</v>
+        <v>74</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2695,7 +2671,7 @@
         </is>
       </c>
       <c r="P24" t="n">
-        <v>29.4</v>
+        <v>27.2</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -2717,32 +2693,28 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U24" t="inlineStr"/>
       <c r="V24" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>PCAR</t>
+          <t>CMCSA</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>108.32</v>
+        <v>20.68</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -2764,26 +2736,26 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>50</v>
+        <v>44.2</v>
       </c>
       <c r="J25" t="n">
-        <v>29.3</v>
+        <v>26.6</v>
       </c>
       <c r="K25" t="n">
-        <v>87</v>
+        <v>72</v>
       </c>
       <c r="L25" t="n">
-        <v>2.4</v>
+        <v>2.54</v>
       </c>
       <c r="M25" t="n">
-        <v>18.8</v>
+        <v>27.3</v>
       </c>
       <c r="N25" t="n">
-        <v>14.4</v>
+        <v>18.9</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2791,7 +2763,7 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>35</v>
+        <v>34.3</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
@@ -2823,18 +2795,18 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CMCSA</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>20.65</v>
+        <v>190.02</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -2860,30 +2832,30 @@
         </is>
       </c>
       <c r="I26" t="n">
-        <v>47.9</v>
+        <v>44</v>
       </c>
       <c r="J26" t="n">
-        <v>26.1</v>
+        <v>34.4</v>
       </c>
       <c r="K26" t="n">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="L26" t="n">
-        <v>2.67</v>
+        <v>2.1</v>
       </c>
       <c r="M26" t="n">
-        <v>28.9</v>
+        <v>20.9</v>
       </c>
       <c r="N26" t="n">
-        <v>24.2</v>
+        <v>10.1</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P26" t="n">
-        <v>34.1</v>
+        <v>41.6</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
@@ -2892,17 +2864,17 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U26" t="inlineStr"/>
@@ -2915,18 +2887,18 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>TTD</t>
+          <t>PNC</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>12.06</v>
+        <v>221.26</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -2948,34 +2920,34 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I27" t="n">
-        <v>47.2</v>
+        <v>41.6</v>
       </c>
       <c r="J27" t="n">
-        <v>35</v>
+        <v>35.3</v>
       </c>
       <c r="K27" t="n">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="L27" t="n">
-        <v>3.56</v>
+        <v>1.66</v>
       </c>
       <c r="M27" t="n">
-        <v>39.9</v>
+        <v>18.4</v>
       </c>
       <c r="N27" t="n">
-        <v>19.1</v>
+        <v>21.6</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P27" t="n">
-        <v>27.4</v>
+        <v>42.4</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
@@ -2984,17 +2956,17 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U27" t="inlineStr"/>
@@ -3007,18 +2979,18 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>SCHW</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>190.31</v>
+        <v>97.06</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D28" s="3" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
@@ -3044,30 +3016,30 @@
         </is>
       </c>
       <c r="I28" t="n">
-        <v>45.8</v>
+        <v>41.3</v>
       </c>
       <c r="J28" t="n">
-        <v>35.1</v>
+        <v>36.8</v>
       </c>
       <c r="K28" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="L28" t="n">
-        <v>2.19</v>
+        <v>1.85</v>
       </c>
       <c r="M28" t="n">
-        <v>21</v>
+        <v>24.3</v>
       </c>
       <c r="N28" t="n">
-        <v>10.6</v>
+        <v>43.5</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P28" t="n">
-        <v>41.8</v>
+        <v>45.3</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
@@ -3091,562 +3063,6 @@
       </c>
       <c r="U28" t="inlineStr"/>
       <c r="V28" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>PNC</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>219.97</v>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>44.7</v>
-      </c>
-      <c r="J29" t="n">
-        <v>30.9</v>
-      </c>
-      <c r="K29" t="n">
-        <v>75</v>
-      </c>
-      <c r="L29" t="n">
-        <v>1.78</v>
-      </c>
-      <c r="M29" t="n">
-        <v>18.1</v>
-      </c>
-      <c r="N29" t="n">
-        <v>19.8</v>
-      </c>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="P29" t="n">
-        <v>41</v>
-      </c>
-      <c r="Q29" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R29" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S29" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T29" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U29" t="inlineStr"/>
-      <c r="V29" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>CPRT</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>27.28</v>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I30" t="n">
-        <v>42.4</v>
-      </c>
-      <c r="J30" t="n">
-        <v>38</v>
-      </c>
-      <c r="K30" t="n">
-        <v>78</v>
-      </c>
-      <c r="L30" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="M30" t="n">
-        <v>35.4</v>
-      </c>
-      <c r="N30" t="n">
-        <v>64.59999999999999</v>
-      </c>
-      <c r="O30" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P30" t="n">
-        <v>35.4</v>
-      </c>
-      <c r="Q30" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R30" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S30" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T30" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U30" t="inlineStr"/>
-      <c r="V30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>SCHW</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>97.09</v>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I31" t="n">
-        <v>41.5</v>
-      </c>
-      <c r="J31" t="n">
-        <v>36.5</v>
-      </c>
-      <c r="K31" t="n">
-        <v>80</v>
-      </c>
-      <c r="L31" t="n">
-        <v>1.95</v>
-      </c>
-      <c r="M31" t="n">
-        <v>25.2</v>
-      </c>
-      <c r="N31" t="n">
-        <v>48.6</v>
-      </c>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="P31" t="n">
-        <v>45.3</v>
-      </c>
-      <c r="Q31" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R31" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S31" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T31" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U31" t="inlineStr"/>
-      <c r="V31" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>JPM</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>333.51</v>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I32" t="n">
-        <v>40.9</v>
-      </c>
-      <c r="J32" t="n">
-        <v>40.9</v>
-      </c>
-      <c r="K32" t="n">
-        <v>73</v>
-      </c>
-      <c r="L32" t="n">
-        <v>1.61</v>
-      </c>
-      <c r="M32" t="n">
-        <v>16.8</v>
-      </c>
-      <c r="N32" t="n">
-        <v>20.6</v>
-      </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P32" t="n">
-        <v>51</v>
-      </c>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R32" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S32" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T32" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U32" t="inlineStr"/>
-      <c r="V32" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>625.6799999999999</v>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I33" t="n">
-        <v>30.2</v>
-      </c>
-      <c r="J33" t="n">
-        <v>34.6</v>
-      </c>
-      <c r="K33" t="n">
-        <v>29</v>
-      </c>
-      <c r="L33" t="n">
-        <v>3.45</v>
-      </c>
-      <c r="M33" t="n">
-        <v>31</v>
-      </c>
-      <c r="N33" t="n">
-        <v>49</v>
-      </c>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P33" t="n">
-        <v>51.5</v>
-      </c>
-      <c r="Q33" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S33" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T33" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U33" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
-      <c r="V33" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>GS</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>898.28</v>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>27.3</v>
-      </c>
-      <c r="J34" t="n">
-        <v>36.1</v>
-      </c>
-      <c r="K34" t="n">
-        <v>46</v>
-      </c>
-      <c r="L34" t="n">
-        <v>2.22</v>
-      </c>
-      <c r="M34" t="n">
-        <v>24.8</v>
-      </c>
-      <c r="N34" t="n">
-        <v>13</v>
-      </c>
-      <c r="O34" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P34" t="n">
-        <v>37.8</v>
-      </c>
-      <c r="Q34" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R34" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S34" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T34" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U34" t="inlineStr"/>
-      <c r="V34" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 13.10.2026 20:09 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V28"/>
+  <dimension ref="A1:V21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>FCX</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>273.81</v>
+        <v>72.43000000000001</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,22 +614,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>91.7</v>
+        <v>87.2</v>
       </c>
       <c r="J2" t="n">
-        <v>58.7</v>
+        <v>51.8</v>
       </c>
       <c r="K2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L2" t="n">
-        <v>1.91</v>
+        <v>3.1</v>
       </c>
       <c r="M2" t="n">
-        <v>23</v>
+        <v>37.8</v>
       </c>
       <c r="N2" t="n">
-        <v>31.6</v>
+        <v>26.1</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,11 +637,11 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>60.6</v>
+        <v>58.1</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -651,15 +651,19 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V2" t="inlineStr">
         <is>
           <t>No</t>
@@ -669,30 +673,30 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PDD</t>
+          <t>BKR</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>80.92</v>
+        <v>56.45</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -706,34 +710,34 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>88.7</v>
+        <v>83.7</v>
       </c>
       <c r="J3" t="n">
-        <v>54.3</v>
+        <v>43.9</v>
       </c>
       <c r="K3" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L3" t="n">
-        <v>2.23</v>
+        <v>2.48</v>
       </c>
       <c r="M3" t="n">
-        <v>25.1</v>
+        <v>29.5</v>
       </c>
       <c r="N3" t="n">
-        <v>15.1</v>
+        <v>42.9</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>43</v>
+        <v>45.7</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -753,7 +757,7 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Squeeze Expanding</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -765,11 +769,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>FCX</t>
+          <t>PDD</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>73.29000000000001</v>
+        <v>81.95999999999999</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -802,34 +806,34 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>85.8</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>54.8</v>
+        <v>57.5</v>
       </c>
       <c r="K4" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="L4" t="n">
-        <v>3.16</v>
+        <v>2.4</v>
       </c>
       <c r="M4" t="n">
-        <v>37.8</v>
+        <v>24.8</v>
       </c>
       <c r="N4" t="n">
-        <v>25.9</v>
+        <v>14.3</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>59.5</v>
+        <v>44.2</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -839,17 +843,17 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>TTM Squeeze</t>
+          <t>Squeeze Expanding</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -861,15 +865,15 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>FICO</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>157.42</v>
+        <v>722.42</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -884,45 +888,48 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>85.40000000000001</v>
+        <v>77.8</v>
       </c>
       <c r="J5" t="n">
-        <v>57.6</v>
+        <v>39.4</v>
       </c>
       <c r="K5" t="n">
-        <v>6</v>
+        <v>95</v>
       </c>
       <c r="L5" t="n">
-        <v>1.88</v>
+        <v>7.43</v>
       </c>
       <c r="M5" t="n">
-        <v>36.5</v>
+        <v>109.9</v>
+      </c>
+      <c r="N5" t="n">
+        <v>100</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>54.8</v>
+        <v>33.4</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -940,11 +947,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
           <t>No</t>
@@ -954,71 +957,68 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BKR</t>
+          <t>TLT</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>56.18</v>
+        <v>78.37</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>81.09999999999999</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>42.4</v>
+        <v>42.1</v>
       </c>
       <c r="K6" t="n">
-        <v>2</v>
+        <v>94</v>
       </c>
       <c r="L6" t="n">
-        <v>2.58</v>
+        <v>0.89</v>
       </c>
       <c r="M6" t="n">
-        <v>30.1</v>
-      </c>
-      <c r="N6" t="n">
-        <v>46.1</v>
+        <v>13.4</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>45.2</v>
+        <v>34.6</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1033,14 +1033,10 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr">
         <is>
           <t>No</t>
@@ -1050,30 +1046,30 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>89.79000000000001</v>
+        <v>143.27</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1087,27 +1083,30 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>79.3</v>
+        <v>76.2</v>
       </c>
       <c r="J7" t="n">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="K7" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="L7" t="n">
-        <v>1.51</v>
+        <v>4.52</v>
       </c>
       <c r="M7" t="n">
-        <v>23.4</v>
+        <v>52.4</v>
+      </c>
+      <c r="N7" t="n">
+        <v>32.8</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>64.5</v>
+        <v>45.1</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1147,7 +1146,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>502.51</v>
+        <v>494.51</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1180,22 +1179,22 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>78.59999999999999</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="J8" t="n">
-        <v>70.7</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="K8" t="n">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="L8" t="n">
-        <v>3.68</v>
+        <v>3.6</v>
       </c>
       <c r="M8" t="n">
-        <v>54.2</v>
+        <v>54.5</v>
       </c>
       <c r="N8" t="n">
-        <v>65.40000000000001</v>
+        <v>66</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1203,7 +1202,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>59.3</v>
+        <v>57.9</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1235,67 +1234,67 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ZTS</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>75.65000000000001</v>
+        <v>478.06</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>77.2</v>
+        <v>73.5</v>
       </c>
       <c r="J9" t="n">
-        <v>62.2</v>
+        <v>66.2</v>
       </c>
       <c r="K9" t="n">
-        <v>54</v>
+        <v>98</v>
       </c>
       <c r="L9" t="n">
-        <v>2.35</v>
+        <v>2.34</v>
       </c>
       <c r="M9" t="n">
-        <v>21.5</v>
+        <v>20.9</v>
       </c>
       <c r="N9" t="n">
-        <v>6.6</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>39.3</v>
+        <v>57.3</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1309,7 +1308,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1327,11 +1326,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>DLR</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>137.39</v>
+        <v>178.18</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1364,34 +1363,31 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>74.5</v>
+        <v>71.5</v>
       </c>
       <c r="J10" t="n">
-        <v>44.9</v>
+        <v>45.3</v>
       </c>
       <c r="K10" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L10" t="n">
-        <v>4.46</v>
+        <v>2.46</v>
       </c>
       <c r="M10" t="n">
-        <v>50.9</v>
-      </c>
-      <c r="N10" t="n">
-        <v>28.1</v>
+        <v>36.6</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>42.8</v>
+        <v>46.7</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -1411,42 +1407,42 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>Divergence, Squeeze Expanding</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TLT</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>78.05</v>
+        <v>334.2</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1460,30 +1456,30 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>74.40000000000001</v>
+        <v>62.2</v>
       </c>
       <c r="J11" t="n">
-        <v>38.2</v>
+        <v>52.6</v>
       </c>
       <c r="K11" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="L11" t="n">
-        <v>0.93</v>
+        <v>3.29</v>
       </c>
       <c r="M11" t="n">
-        <v>9.5</v>
+        <v>44.7</v>
       </c>
       <c r="N11" t="n">
-        <v>53.5</v>
+        <v>67.5</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>32.8</v>
+        <v>50.6</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1492,12 +1488,12 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1505,21 +1501,25 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr"/>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ILMN</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>276.67</v>
+        <v>414.7</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1552,22 +1552,22 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>67.90000000000001</v>
+        <v>58.8</v>
       </c>
       <c r="J12" t="n">
-        <v>61.9</v>
+        <v>65.3</v>
       </c>
       <c r="K12" t="n">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="L12" t="n">
-        <v>5.43</v>
+        <v>2.75</v>
       </c>
       <c r="M12" t="n">
-        <v>57.8</v>
+        <v>30</v>
       </c>
       <c r="N12" t="n">
-        <v>58.8</v>
+        <v>16.7</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1575,7 +1575,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>78.59999999999999</v>
+        <v>61</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1584,17 +1584,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
@@ -1607,15 +1607,15 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MET</t>
+          <t>MCD</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>100.17</v>
+        <v>235.87</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1630,48 +1630,48 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>65.09999999999999</v>
+        <v>57.1</v>
       </c>
       <c r="J13" t="n">
-        <v>63.3</v>
+        <v>38.4</v>
       </c>
       <c r="K13" t="n">
-        <v>37</v>
+        <v>88</v>
       </c>
       <c r="L13" t="n">
-        <v>2.08</v>
+        <v>1.71</v>
       </c>
       <c r="M13" t="n">
-        <v>21.6</v>
+        <v>20</v>
       </c>
       <c r="N13" t="n">
-        <v>35.9</v>
+        <v>50.3</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>67.90000000000001</v>
+        <v>28.2</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>FIRED</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -1681,7 +1681,7 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -1689,11 +1689,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>Squeeze Fired</t>
-        </is>
-      </c>
+      <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr">
         <is>
           <t>No</t>
@@ -1703,11 +1699,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>ILMN</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>348.42</v>
+        <v>271.17</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1736,26 +1732,26 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>64.7</v>
+        <v>54.6</v>
       </c>
       <c r="J14" t="n">
-        <v>62.5</v>
+        <v>58.6</v>
       </c>
       <c r="K14" t="n">
-        <v>96</v>
+        <v>58</v>
       </c>
       <c r="L14" t="n">
-        <v>2.98</v>
+        <v>5.26</v>
       </c>
       <c r="M14" t="n">
-        <v>43</v>
+        <v>58.2</v>
       </c>
       <c r="N14" t="n">
-        <v>62.5</v>
+        <v>60.9</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1763,7 +1759,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>54.1</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1772,17 +1768,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
@@ -1799,7 +1795,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>126.68</v>
+        <v>127.3</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1832,22 +1828,22 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>62.5</v>
+        <v>54.5</v>
       </c>
       <c r="J15" t="n">
-        <v>39.9</v>
+        <v>42</v>
       </c>
       <c r="K15" t="n">
-        <v>77</v>
+        <v>56</v>
       </c>
       <c r="L15" t="n">
-        <v>2.05</v>
+        <v>2.02</v>
       </c>
       <c r="M15" t="n">
-        <v>18.2</v>
+        <v>18.4</v>
       </c>
       <c r="N15" t="n">
-        <v>27.8</v>
+        <v>28.6</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1855,7 +1851,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>32.7</v>
+        <v>34</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1887,30 +1883,30 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>VZ</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>406.24</v>
+        <v>43.53</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1920,31 +1916,34 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>58.2</v>
+        <v>51.9</v>
       </c>
       <c r="J16" t="n">
-        <v>60.6</v>
+        <v>37.4</v>
       </c>
       <c r="K16" t="n">
-        <v>91</v>
+        <v>67</v>
       </c>
       <c r="L16" t="n">
-        <v>2.68</v>
+        <v>2.89</v>
       </c>
       <c r="M16" t="n">
-        <v>40</v>
+        <v>32.9</v>
+      </c>
+      <c r="N16" t="n">
+        <v>74.3</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>59.1</v>
+        <v>44.8</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1958,12 +1957,12 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
@@ -1976,11 +1975,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>MCD</t>
+          <t>KHC</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>235.65</v>
+        <v>22.43</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -2013,19 +2012,22 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>58.1</v>
+        <v>48.6</v>
       </c>
       <c r="J17" t="n">
-        <v>37.9</v>
+        <v>36.5</v>
       </c>
       <c r="K17" t="n">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="L17" t="n">
-        <v>1.76</v>
+        <v>2.37</v>
       </c>
       <c r="M17" t="n">
-        <v>24.8</v>
+        <v>19.9</v>
+      </c>
+      <c r="N17" t="n">
+        <v>23.7</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2033,7 +2035,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>27.9</v>
+        <v>41.2</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2065,11 +2067,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>VZ</t>
+          <t>CHTR</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>42.78</v>
+        <v>106.95</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2102,22 +2104,22 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>56.6</v>
+        <v>46.9</v>
       </c>
       <c r="J18" t="n">
-        <v>32.2</v>
+        <v>34.8</v>
       </c>
       <c r="K18" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L18" t="n">
-        <v>3.03</v>
+        <v>4.94</v>
       </c>
       <c r="M18" t="n">
-        <v>32.3</v>
+        <v>56.4</v>
       </c>
       <c r="N18" t="n">
-        <v>72</v>
+        <v>50.3</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -2125,7 +2127,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>42.6</v>
+        <v>31.5</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2134,17 +2136,17 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
@@ -2157,11 +2159,11 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>AMP</t>
+          <t>NOC</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>500.02</v>
+        <v>481.26</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2190,34 +2192,34 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>54.9</v>
+        <v>44.7</v>
       </c>
       <c r="J19" t="n">
-        <v>40</v>
+        <v>36.4</v>
       </c>
       <c r="K19" t="n">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="L19" t="n">
-        <v>2.16</v>
+        <v>2.1</v>
       </c>
       <c r="M19" t="n">
-        <v>24.9</v>
+        <v>22.6</v>
       </c>
       <c r="N19" t="n">
-        <v>35.8</v>
+        <v>40.2</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>47.5</v>
+        <v>36.1</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2249,11 +2251,11 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>BAC</t>
+          <t>TTD</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>54.58</v>
+        <v>12.17</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2286,30 +2288,30 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>53.5</v>
+        <v>44.6</v>
       </c>
       <c r="J20" t="n">
-        <v>34.6</v>
+        <v>38.2</v>
       </c>
       <c r="K20" t="n">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="L20" t="n">
-        <v>1.83</v>
+        <v>3.66</v>
       </c>
       <c r="M20" t="n">
-        <v>21.7</v>
+        <v>40.1</v>
       </c>
       <c r="N20" t="n">
-        <v>49.1</v>
+        <v>19.3</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>43.9</v>
+        <v>27.9</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2341,11 +2343,11 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>NOC</t>
+          <t>PCAR</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>485</v>
+        <v>107.98</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2374,26 +2376,26 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>48.9</v>
+        <v>40.4</v>
       </c>
       <c r="J21" t="n">
-        <v>38.2</v>
+        <v>28.9</v>
       </c>
       <c r="K21" t="n">
-        <v>96</v>
+        <v>56</v>
       </c>
       <c r="L21" t="n">
-        <v>2.15</v>
+        <v>2.32</v>
       </c>
       <c r="M21" t="n">
-        <v>22.6</v>
+        <v>18.9</v>
       </c>
       <c r="N21" t="n">
-        <v>40.1</v>
+        <v>14.9</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2401,7 +2403,7 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>37.1</v>
+        <v>34.7</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2425,644 +2427,6 @@
       </c>
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>PCAR</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>108.13</v>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>46.1</v>
-      </c>
-      <c r="J22" t="n">
-        <v>29.2</v>
-      </c>
-      <c r="K22" t="n">
-        <v>76</v>
-      </c>
-      <c r="L22" t="n">
-        <v>2.31</v>
-      </c>
-      <c r="M22" t="n">
-        <v>18.9</v>
-      </c>
-      <c r="N22" t="n">
-        <v>15.1</v>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P22" t="n">
-        <v>34.9</v>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T22" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr"/>
-      <c r="V22" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>CHTR</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>102.48</v>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>45.6</v>
-      </c>
-      <c r="J23" t="n">
-        <v>27.3</v>
-      </c>
-      <c r="K23" t="n">
-        <v>87</v>
-      </c>
-      <c r="L23" t="n">
-        <v>5.03</v>
-      </c>
-      <c r="M23" t="n">
-        <v>78.8</v>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P23" t="n">
-        <v>29.1</v>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>TTD</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>11.94</v>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>45.6</v>
-      </c>
-      <c r="J24" t="n">
-        <v>33.7</v>
-      </c>
-      <c r="K24" t="n">
-        <v>75</v>
-      </c>
-      <c r="L24" t="n">
-        <v>3.61</v>
-      </c>
-      <c r="M24" t="n">
-        <v>74</v>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P24" t="n">
-        <v>27.2</v>
-      </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S24" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T24" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U24" t="inlineStr"/>
-      <c r="V24" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>CMCSA</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>20.68</v>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>44.2</v>
-      </c>
-      <c r="J25" t="n">
-        <v>26.6</v>
-      </c>
-      <c r="K25" t="n">
-        <v>72</v>
-      </c>
-      <c r="L25" t="n">
-        <v>2.54</v>
-      </c>
-      <c r="M25" t="n">
-        <v>27.3</v>
-      </c>
-      <c r="N25" t="n">
-        <v>18.9</v>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P25" t="n">
-        <v>34.3</v>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S25" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T25" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U25" t="inlineStr"/>
-      <c r="V25" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>MS</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>190.02</v>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>44</v>
-      </c>
-      <c r="J26" t="n">
-        <v>34.4</v>
-      </c>
-      <c r="K26" t="n">
-        <v>72</v>
-      </c>
-      <c r="L26" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="M26" t="n">
-        <v>20.9</v>
-      </c>
-      <c r="N26" t="n">
-        <v>10.1</v>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="P26" t="n">
-        <v>41.6</v>
-      </c>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R26" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S26" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T26" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U26" t="inlineStr"/>
-      <c r="V26" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>PNC</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>221.26</v>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>41.6</v>
-      </c>
-      <c r="J27" t="n">
-        <v>35.3</v>
-      </c>
-      <c r="K27" t="n">
-        <v>63</v>
-      </c>
-      <c r="L27" t="n">
-        <v>1.66</v>
-      </c>
-      <c r="M27" t="n">
-        <v>18.4</v>
-      </c>
-      <c r="N27" t="n">
-        <v>21.6</v>
-      </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="P27" t="n">
-        <v>42.4</v>
-      </c>
-      <c r="Q27" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R27" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S27" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T27" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U27" t="inlineStr"/>
-      <c r="V27" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>SCHW</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>97.06</v>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>41.3</v>
-      </c>
-      <c r="J28" t="n">
-        <v>36.8</v>
-      </c>
-      <c r="K28" t="n">
-        <v>77</v>
-      </c>
-      <c r="L28" t="n">
-        <v>1.85</v>
-      </c>
-      <c r="M28" t="n">
-        <v>24.3</v>
-      </c>
-      <c r="N28" t="n">
-        <v>43.5</v>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="P28" t="n">
-        <v>45.3</v>
-      </c>
-      <c r="Q28" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S28" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U28" t="inlineStr"/>
-      <c r="V28" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 14.10.2026 18:27 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,11 +435,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V21"/>
+  <dimension ref="A1:V20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -577,15 +577,15 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>FCX</t>
+          <t>TLT</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>72.43000000000001</v>
+        <v>79</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -600,48 +600,48 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>87.2</v>
+        <v>86.2</v>
       </c>
       <c r="J2" t="n">
-        <v>51.8</v>
+        <v>48.9</v>
       </c>
       <c r="K2" t="n">
-        <v>1</v>
+        <v>93</v>
       </c>
       <c r="L2" t="n">
-        <v>3.1</v>
+        <v>0.98</v>
       </c>
       <c r="M2" t="n">
-        <v>37.8</v>
+        <v>10</v>
       </c>
       <c r="N2" t="n">
-        <v>26.1</v>
+        <v>63.3</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>58.1</v>
+        <v>37.9</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -651,7 +651,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -659,11 +659,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+      <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
         <is>
           <t>No</t>
@@ -673,30 +669,30 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BKR</t>
+          <t>LLY</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>56.45</v>
+        <v>1214.61</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -710,30 +706,30 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>83.7</v>
+        <v>79.3</v>
       </c>
       <c r="J3" t="n">
-        <v>43.9</v>
+        <v>61.6</v>
       </c>
       <c r="K3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L3" t="n">
-        <v>2.48</v>
+        <v>2.94</v>
       </c>
       <c r="M3" t="n">
-        <v>29.5</v>
+        <v>22.8</v>
       </c>
       <c r="N3" t="n">
-        <v>42.9</v>
+        <v>10.3</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>45.7</v>
+        <v>59.1</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -747,12 +743,12 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -769,30 +765,30 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PDD</t>
+          <t>FCX</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>81.95999999999999</v>
+        <v>69.15000000000001</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -806,59 +802,59 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>83.40000000000001</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>57.5</v>
+        <v>42.4</v>
       </c>
       <c r="K4" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="L4" t="n">
-        <v>2.4</v>
+        <v>3.54</v>
       </c>
       <c r="M4" t="n">
-        <v>24.8</v>
+        <v>38</v>
       </c>
       <c r="N4" t="n">
-        <v>14.3</v>
+        <v>26.6</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>44.2</v>
+        <v>53.3</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>Squeeze Expanding</t>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -869,7 +865,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>722.42</v>
+        <v>712.5</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -902,22 +898,22 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>77.8</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>39.4</v>
+        <v>38.6</v>
       </c>
       <c r="K5" t="n">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="L5" t="n">
-        <v>7.43</v>
+        <v>6.95</v>
       </c>
       <c r="M5" t="n">
-        <v>109.9</v>
+        <v>109.6</v>
       </c>
       <c r="N5" t="n">
-        <v>100</v>
+        <v>99.7</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -925,7 +921,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>33.4</v>
+        <v>32.8</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -957,56 +953,59 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TLT</t>
+          <t>BKR</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>78.37</v>
+        <v>55.22</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>76.90000000000001</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>42.1</v>
+        <v>38.9</v>
       </c>
       <c r="K6" t="n">
-        <v>94</v>
+        <v>5</v>
       </c>
       <c r="L6" t="n">
-        <v>0.89</v>
+        <v>2.72</v>
       </c>
       <c r="M6" t="n">
-        <v>13.4</v>
+        <v>29.9</v>
+      </c>
+      <c r="N6" t="n">
+        <v>45.1</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1014,11 +1013,11 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>34.6</v>
+        <v>43.7</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1033,28 +1032,32 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>143.27</v>
+        <v>468.12</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -1069,44 +1072,44 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>76.2</v>
+        <v>72.8</v>
       </c>
       <c r="J7" t="n">
-        <v>51</v>
+        <v>56.9</v>
       </c>
       <c r="K7" t="n">
-        <v>9</v>
+        <v>96</v>
       </c>
       <c r="L7" t="n">
-        <v>4.52</v>
+        <v>2.53</v>
       </c>
       <c r="M7" t="n">
-        <v>52.4</v>
+        <v>21.7</v>
       </c>
       <c r="N7" t="n">
-        <v>32.8</v>
+        <v>13.6</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>45.1</v>
+        <v>53.8</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1115,24 +1118,20 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr">
         <is>
           <t>No</t>
@@ -1146,7 +1145,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>494.51</v>
+        <v>479.15</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1179,22 +1178,22 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>74.09999999999999</v>
+        <v>68.8</v>
       </c>
       <c r="J8" t="n">
-        <v>66.59999999999999</v>
+        <v>59.4</v>
       </c>
       <c r="K8" t="n">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="L8" t="n">
-        <v>3.6</v>
+        <v>3.75</v>
       </c>
       <c r="M8" t="n">
-        <v>54.5</v>
+        <v>52.5</v>
       </c>
       <c r="N8" t="n">
-        <v>66</v>
+        <v>60.8</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1202,7 +1201,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>57.9</v>
+        <v>55.5</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1211,17 +1210,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
@@ -1234,15 +1233,15 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>NKE</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>478.06</v>
+        <v>34.82</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -1257,44 +1256,44 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>73.5</v>
+        <v>68.2</v>
       </c>
       <c r="J9" t="n">
-        <v>66.2</v>
+        <v>40.4</v>
       </c>
       <c r="K9" t="n">
-        <v>98</v>
+        <v>12</v>
       </c>
       <c r="L9" t="n">
-        <v>2.34</v>
+        <v>2.98</v>
       </c>
       <c r="M9" t="n">
-        <v>20.9</v>
+        <v>22.6</v>
       </c>
       <c r="N9" t="n">
-        <v>9.300000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>57.3</v>
+        <v>30.3</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1308,7 +1307,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1316,7 +1315,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr"/>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V9" t="inlineStr">
         <is>
           <t>No</t>
@@ -1326,11 +1329,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>DLR</t>
+          <t>DASH</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>178.18</v>
+        <v>180.82</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1363,41 +1366,44 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>71.5</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="J10" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="K10" t="n">
+        <v>9</v>
+      </c>
+      <c r="L10" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="M10" t="n">
+        <v>44.1</v>
+      </c>
+      <c r="N10" t="n">
+        <v>41.8</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P10" t="n">
         <v>45.3</v>
       </c>
-      <c r="K10" t="n">
-        <v>10</v>
-      </c>
-      <c r="L10" t="n">
-        <v>2.46</v>
-      </c>
-      <c r="M10" t="n">
-        <v>36.6</v>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="P10" t="n">
-        <v>46.7</v>
-      </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1407,42 +1413,42 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>Divergence, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>MCD</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>334.2</v>
+        <v>237.4</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1456,30 +1462,30 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>62.2</v>
+        <v>61</v>
       </c>
       <c r="J11" t="n">
-        <v>52.6</v>
+        <v>41.8</v>
       </c>
       <c r="K11" t="n">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="L11" t="n">
-        <v>3.29</v>
+        <v>1.66</v>
       </c>
       <c r="M11" t="n">
-        <v>44.7</v>
+        <v>20.2</v>
       </c>
       <c r="N11" t="n">
-        <v>67.5</v>
+        <v>51.7</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>50.6</v>
+        <v>29.7</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1488,12 +1494,12 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1501,29 +1507,25 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>414.7</v>
+        <v>130</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -1538,44 +1540,44 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>58.8</v>
+        <v>57.5</v>
       </c>
       <c r="J12" t="n">
-        <v>65.3</v>
+        <v>40.2</v>
       </c>
       <c r="K12" t="n">
-        <v>84</v>
+        <v>13</v>
       </c>
       <c r="L12" t="n">
-        <v>2.75</v>
+        <v>5.68</v>
       </c>
       <c r="M12" t="n">
-        <v>30</v>
+        <v>56.9</v>
       </c>
       <c r="N12" t="n">
-        <v>16.7</v>
+        <v>46.2</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>61</v>
+        <v>40.4</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1584,12 +1586,12 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -1597,69 +1599,73 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr"/>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MCD</t>
+          <t>DLR</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>235.87</v>
+        <v>173.09</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>57.1</v>
+        <v>55</v>
       </c>
       <c r="J13" t="n">
-        <v>38.4</v>
+        <v>39.1</v>
       </c>
       <c r="K13" t="n">
-        <v>88</v>
+        <v>21</v>
       </c>
       <c r="L13" t="n">
-        <v>1.71</v>
+        <v>2.65</v>
       </c>
       <c r="M13" t="n">
-        <v>20</v>
+        <v>27.8</v>
       </c>
       <c r="N13" t="n">
-        <v>50.3</v>
+        <v>31.6</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1667,21 +1673,21 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>28.2</v>
+        <v>43.5</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>FIRED</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -1689,21 +1695,25 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr"/>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>Squeeze Fired, Divergence</t>
+        </is>
+      </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ILMN</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>271.17</v>
+        <v>403.72</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1736,30 +1746,30 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>54.6</v>
+        <v>53.3</v>
       </c>
       <c r="J14" t="n">
-        <v>58.6</v>
+        <v>56</v>
       </c>
       <c r="K14" t="n">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="L14" t="n">
-        <v>5.26</v>
+        <v>2.89</v>
       </c>
       <c r="M14" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="N14" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P14" t="n">
         <v>58.2</v>
-      </c>
-      <c r="N14" t="n">
-        <v>60.9</v>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P14" t="n">
-        <v>75.59999999999999</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1791,11 +1801,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>VZ</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>127.3</v>
+        <v>44.24</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1828,30 +1838,30 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>54.5</v>
+        <v>51.9</v>
       </c>
       <c r="J15" t="n">
         <v>42</v>
       </c>
       <c r="K15" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="L15" t="n">
-        <v>2.02</v>
+        <v>2.77</v>
       </c>
       <c r="M15" t="n">
-        <v>18.4</v>
+        <v>33.3</v>
       </c>
       <c r="N15" t="n">
-        <v>28.6</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>34</v>
+        <v>46.7</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1883,30 +1893,30 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>VZ</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>43.53</v>
+        <v>327.9</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1916,34 +1926,34 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>51.9</v>
+        <v>51.4</v>
       </c>
       <c r="J16" t="n">
-        <v>37.4</v>
+        <v>48.8</v>
       </c>
       <c r="K16" t="n">
-        <v>67</v>
+        <v>86</v>
       </c>
       <c r="L16" t="n">
-        <v>2.89</v>
+        <v>3.24</v>
       </c>
       <c r="M16" t="n">
-        <v>32.9</v>
+        <v>39</v>
       </c>
       <c r="N16" t="n">
-        <v>74.3</v>
+        <v>50.2</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>44.8</v>
+        <v>49.2</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1957,12 +1967,12 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
@@ -1979,7 +1989,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>22.43</v>
+        <v>22.73</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -2012,22 +2022,22 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>48.6</v>
+        <v>50.6</v>
       </c>
       <c r="J17" t="n">
-        <v>36.5</v>
+        <v>41.9</v>
       </c>
       <c r="K17" t="n">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="L17" t="n">
-        <v>2.37</v>
+        <v>2.35</v>
       </c>
       <c r="M17" t="n">
-        <v>19.9</v>
+        <v>20.3</v>
       </c>
       <c r="N17" t="n">
-        <v>23.7</v>
+        <v>25.2</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2035,7 +2045,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>41.2</v>
+        <v>43.4</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2067,11 +2077,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CHTR</t>
+          <t>NOC</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>106.95</v>
+        <v>496.82</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2100,26 +2110,26 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>46.9</v>
+        <v>48.5</v>
       </c>
       <c r="J18" t="n">
-        <v>34.8</v>
+        <v>47.2</v>
       </c>
       <c r="K18" t="n">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="L18" t="n">
-        <v>4.94</v>
+        <v>2.21</v>
       </c>
       <c r="M18" t="n">
-        <v>56.4</v>
+        <v>24.7</v>
       </c>
       <c r="N18" t="n">
-        <v>50.3</v>
+        <v>49.6</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -2127,7 +2137,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>31.5</v>
+        <v>40</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2159,30 +2169,30 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>NOC</t>
+          <t>ILMN</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>481.26</v>
+        <v>269.26</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2192,34 +2202,34 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>44.7</v>
+        <v>46.9</v>
       </c>
       <c r="J19" t="n">
-        <v>36.4</v>
+        <v>57.5</v>
       </c>
       <c r="K19" t="n">
-        <v>86</v>
+        <v>47</v>
       </c>
       <c r="L19" t="n">
-        <v>2.1</v>
+        <v>5.06</v>
       </c>
       <c r="M19" t="n">
-        <v>22.6</v>
+        <v>57.2</v>
       </c>
       <c r="N19" t="n">
-        <v>40.2</v>
+        <v>59</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>36.1</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2228,12 +2238,12 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
@@ -2251,11 +2261,11 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TTD</t>
+          <t>CHTR</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>12.17</v>
+        <v>104.07</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2288,22 +2298,22 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>44.6</v>
+        <v>43.5</v>
       </c>
       <c r="J20" t="n">
-        <v>38.2</v>
+        <v>32.5</v>
       </c>
       <c r="K20" t="n">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="L20" t="n">
-        <v>3.66</v>
+        <v>4.9</v>
       </c>
       <c r="M20" t="n">
-        <v>40.1</v>
+        <v>55.9</v>
       </c>
       <c r="N20" t="n">
-        <v>19.3</v>
+        <v>49.6</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2311,7 +2321,7 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>27.9</v>
+        <v>29.8</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2335,98 +2345,6 @@
       </c>
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>PCAR</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>107.98</v>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>40.4</v>
-      </c>
-      <c r="J21" t="n">
-        <v>28.9</v>
-      </c>
-      <c r="K21" t="n">
-        <v>56</v>
-      </c>
-      <c r="L21" t="n">
-        <v>2.32</v>
-      </c>
-      <c r="M21" t="n">
-        <v>18.9</v>
-      </c>
-      <c r="N21" t="n">
-        <v>14.9</v>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P21" t="n">
-        <v>34.7</v>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U21" t="inlineStr"/>
-      <c r="V21" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 15.10.2026 18:09 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V20"/>
+  <dimension ref="A1:V14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -458,7 +458,7 @@
     <col width="15" customWidth="1" min="18" max="18"/>
     <col width="11" customWidth="1" min="19" max="19"/>
     <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="25" customWidth="1" min="21" max="21"/>
+    <col width="19" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TLT</t>
+          <t>FICO</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>79</v>
+        <v>755.47</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,22 +614,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>86.2</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>48.9</v>
+        <v>43.9</v>
       </c>
       <c r="K2" t="n">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="L2" t="n">
-        <v>0.98</v>
+        <v>6.51</v>
       </c>
       <c r="M2" t="n">
-        <v>10</v>
+        <v>111</v>
       </c>
       <c r="N2" t="n">
-        <v>63.3</v>
+        <v>100</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>37.9</v>
+        <v>35.4</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -669,30 +669,30 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LLY</t>
+          <t>DASH</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1214.61</v>
+        <v>190.93</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -706,34 +706,34 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>79.3</v>
+        <v>75</v>
       </c>
       <c r="J3" t="n">
-        <v>61.6</v>
+        <v>46.8</v>
       </c>
       <c r="K3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L3" t="n">
-        <v>2.94</v>
+        <v>4.17</v>
       </c>
       <c r="M3" t="n">
-        <v>22.8</v>
+        <v>44.3</v>
       </c>
       <c r="N3" t="n">
-        <v>10.3</v>
+        <v>42.2</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>59.1</v>
+        <v>48.9</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -743,19 +743,15 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr">
         <is>
           <t>No</t>
@@ -765,81 +761,81 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>FCX</t>
+          <t>MCD</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>69.15000000000001</v>
+        <v>242.96</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>78.59999999999999</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>42.4</v>
+        <v>52.2</v>
       </c>
       <c r="K4" t="n">
-        <v>2</v>
+        <v>73</v>
       </c>
       <c r="L4" t="n">
-        <v>3.54</v>
+        <v>1.83</v>
       </c>
       <c r="M4" t="n">
-        <v>38</v>
+        <v>21.4</v>
       </c>
       <c r="N4" t="n">
-        <v>26.6</v>
+        <v>60</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>53.3</v>
+        <v>34.7</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -847,29 +843,25 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>FICO</t>
+          <t>LLY</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>712.5</v>
+        <v>1264.91</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -884,48 +876,48 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>77.90000000000001</v>
+        <v>70</v>
       </c>
       <c r="J5" t="n">
-        <v>38.6</v>
+        <v>69.5</v>
       </c>
       <c r="K5" t="n">
-        <v>93</v>
+        <v>27</v>
       </c>
       <c r="L5" t="n">
-        <v>6.95</v>
+        <v>3.15</v>
       </c>
       <c r="M5" t="n">
-        <v>109.6</v>
+        <v>25.6</v>
       </c>
       <c r="N5" t="n">
-        <v>99.7</v>
+        <v>19.2</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>32.8</v>
+        <v>62.7</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>FIRED</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -935,7 +927,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -943,7 +935,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr"/>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Squeeze Fired</t>
+        </is>
+      </c>
       <c r="V5" t="inlineStr">
         <is>
           <t>No</t>
@@ -953,15 +949,15 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BKR</t>
+          <t>SNPS</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>55.22</v>
+        <v>462.31</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -976,68 +972,68 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>73.90000000000001</v>
+        <v>67.2</v>
       </c>
       <c r="J6" t="n">
-        <v>38.9</v>
+        <v>52.7</v>
       </c>
       <c r="K6" t="n">
-        <v>5</v>
+        <v>93</v>
       </c>
       <c r="L6" t="n">
-        <v>2.72</v>
+        <v>4.1</v>
       </c>
       <c r="M6" t="n">
-        <v>29.9</v>
+        <v>53.8</v>
       </c>
       <c r="N6" t="n">
-        <v>45.1</v>
+        <v>64.2</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>43.7</v>
+        <v>53.1</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+          <t>Divergence</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
@@ -1053,7 +1049,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>468.12</v>
+        <v>453.6</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1086,22 +1082,22 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>72.8</v>
+        <v>66.5</v>
       </c>
       <c r="J7" t="n">
-        <v>56.9</v>
+        <v>46.4</v>
       </c>
       <c r="K7" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="L7" t="n">
-        <v>2.53</v>
+        <v>2.98</v>
       </c>
       <c r="M7" t="n">
-        <v>21.7</v>
+        <v>24.1</v>
       </c>
       <c r="N7" t="n">
-        <v>13.6</v>
+        <v>26.8</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1109,7 +1105,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>53.8</v>
+        <v>49.4</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1131,25 +1127,29 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr"/>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SNPS</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>479.15</v>
+        <v>133.79</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -1164,48 +1164,48 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>68.8</v>
+        <v>61.7</v>
       </c>
       <c r="J8" t="n">
-        <v>59.4</v>
+        <v>43.7</v>
       </c>
       <c r="K8" t="n">
-        <v>95</v>
+        <v>11</v>
       </c>
       <c r="L8" t="n">
-        <v>3.75</v>
+        <v>5.52</v>
       </c>
       <c r="M8" t="n">
-        <v>52.5</v>
+        <v>56.1</v>
       </c>
       <c r="N8" t="n">
-        <v>60.8</v>
+        <v>43.7</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>55.5</v>
+        <v>41.6</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -1215,7 +1215,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -1223,7 +1223,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr"/>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V8" t="inlineStr">
         <is>
           <t>No</t>
@@ -1233,59 +1237,59 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>NKE</t>
+          <t>KHC</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>34.82</v>
+        <v>23.25</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>68.2</v>
+        <v>59.6</v>
       </c>
       <c r="J9" t="n">
-        <v>40.4</v>
+        <v>50</v>
       </c>
       <c r="K9" t="n">
-        <v>12</v>
+        <v>78</v>
       </c>
       <c r="L9" t="n">
-        <v>2.98</v>
+        <v>2.52</v>
       </c>
       <c r="M9" t="n">
-        <v>22.6</v>
+        <v>21.1</v>
       </c>
       <c r="N9" t="n">
-        <v>0.1</v>
+        <v>28.8</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1293,7 +1297,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>30.3</v>
+        <v>46.8</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1312,14 +1316,10 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
           <t>No</t>
@@ -1329,11 +1329,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>DASH</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>180.82</v>
+        <v>368.65</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1366,30 +1366,30 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>68.09999999999999</v>
+        <v>55.7</v>
       </c>
       <c r="J10" t="n">
-        <v>37.5</v>
+        <v>44.1</v>
       </c>
       <c r="K10" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L10" t="n">
-        <v>4.4</v>
+        <v>4.81</v>
       </c>
       <c r="M10" t="n">
-        <v>44.1</v>
+        <v>56.1</v>
       </c>
       <c r="N10" t="n">
-        <v>41.8</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>45.3</v>
+        <v>58.6</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1403,7 +1403,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1413,23 +1413,23 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>Divergence, Squeeze Expanding</t>
+          <t>Squeeze Expanding</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MCD</t>
+          <t>NOC</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>237.4</v>
+        <v>498.02</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1458,26 +1458,26 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>61</v>
+        <v>52.1</v>
       </c>
       <c r="J11" t="n">
-        <v>41.8</v>
+        <v>48</v>
       </c>
       <c r="K11" t="n">
-        <v>86</v>
+        <v>63</v>
       </c>
       <c r="L11" t="n">
-        <v>1.66</v>
+        <v>2.27</v>
       </c>
       <c r="M11" t="n">
-        <v>20.2</v>
+        <v>24.1</v>
       </c>
       <c r="N11" t="n">
-        <v>51.7</v>
+        <v>46.8</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>29.7</v>
+        <v>40.4</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1517,15 +1517,15 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>130</v>
+        <v>399.99</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -1540,44 +1540,44 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>57.5</v>
+        <v>45.7</v>
       </c>
       <c r="J12" t="n">
-        <v>40.2</v>
+        <v>53.2</v>
       </c>
       <c r="K12" t="n">
-        <v>13</v>
+        <v>57</v>
       </c>
       <c r="L12" t="n">
-        <v>5.68</v>
+        <v>3.05</v>
       </c>
       <c r="M12" t="n">
-        <v>56.9</v>
+        <v>30.9</v>
       </c>
       <c r="N12" t="n">
-        <v>46.2</v>
+        <v>19.4</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>40.4</v>
+        <v>57</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1591,57 +1591,53 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr">
+        <is>
           <t>No</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V12" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DLR</t>
+          <t>CHTR</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>173.09</v>
+        <v>108.67</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1650,22 +1646,22 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>55</v>
+        <v>41.8</v>
       </c>
       <c r="J13" t="n">
-        <v>39.1</v>
+        <v>38.8</v>
       </c>
       <c r="K13" t="n">
-        <v>21</v>
+        <v>67</v>
       </c>
       <c r="L13" t="n">
-        <v>2.65</v>
+        <v>4.63</v>
       </c>
       <c r="M13" t="n">
-        <v>27.8</v>
+        <v>49.4</v>
       </c>
       <c r="N13" t="n">
-        <v>31.6</v>
+        <v>40.3</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1673,21 +1669,21 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>43.5</v>
+        <v>32.5</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>FIRED</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -1695,29 +1691,25 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>Squeeze Fired, Divergence</t>
-        </is>
-      </c>
+      <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>DLR</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>403.72</v>
+        <v>171.17</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -1732,12 +1724,12 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1746,30 +1738,30 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>53.3</v>
+        <v>38.8</v>
       </c>
       <c r="J14" t="n">
-        <v>56</v>
+        <v>37.2</v>
       </c>
       <c r="K14" t="n">
-        <v>75</v>
+        <v>42</v>
       </c>
       <c r="L14" t="n">
-        <v>2.89</v>
+        <v>2.79</v>
       </c>
       <c r="M14" t="n">
-        <v>30.6</v>
+        <v>28.3</v>
       </c>
       <c r="N14" t="n">
-        <v>18.6</v>
+        <v>33.7</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>58.2</v>
+        <v>42.4</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1783,570 +1775,22 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr"/>
-      <c r="V14" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>VZ</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>44.24</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>51.9</v>
-      </c>
-      <c r="J15" t="n">
-        <v>42</v>
-      </c>
-      <c r="K15" t="n">
-        <v>57</v>
-      </c>
-      <c r="L15" t="n">
-        <v>2.77</v>
-      </c>
-      <c r="M15" t="n">
-        <v>33.3</v>
-      </c>
-      <c r="N15" t="n">
-        <v>75.90000000000001</v>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="P15" t="n">
-        <v>46.7</v>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U15" t="inlineStr"/>
-      <c r="V15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>CDNS</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>327.9</v>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>51.4</v>
-      </c>
-      <c r="J16" t="n">
-        <v>48.8</v>
-      </c>
-      <c r="K16" t="n">
-        <v>86</v>
-      </c>
-      <c r="L16" t="n">
-        <v>3.24</v>
-      </c>
-      <c r="M16" t="n">
-        <v>39</v>
-      </c>
-      <c r="N16" t="n">
-        <v>50.2</v>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="P16" t="n">
-        <v>49.2</v>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr"/>
-      <c r="V16" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>KHC</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>22.73</v>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>50.6</v>
-      </c>
-      <c r="J17" t="n">
-        <v>41.9</v>
-      </c>
-      <c r="K17" t="n">
-        <v>86</v>
-      </c>
-      <c r="L17" t="n">
-        <v>2.35</v>
-      </c>
-      <c r="M17" t="n">
-        <v>20.3</v>
-      </c>
-      <c r="N17" t="n">
-        <v>25.2</v>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P17" t="n">
-        <v>43.4</v>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T17" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>NOC</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>496.82</v>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>48.5</v>
-      </c>
-      <c r="J18" t="n">
-        <v>47.2</v>
-      </c>
-      <c r="K18" t="n">
-        <v>70</v>
-      </c>
-      <c r="L18" t="n">
-        <v>2.21</v>
-      </c>
-      <c r="M18" t="n">
-        <v>24.7</v>
-      </c>
-      <c r="N18" t="n">
-        <v>49.6</v>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P18" t="n">
-        <v>40</v>
-      </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S18" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T18" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>ILMN</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>269.26</v>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>46.9</v>
-      </c>
-      <c r="J19" t="n">
-        <v>57.5</v>
-      </c>
-      <c r="K19" t="n">
-        <v>47</v>
-      </c>
-      <c r="L19" t="n">
-        <v>5.06</v>
-      </c>
-      <c r="M19" t="n">
-        <v>57.2</v>
-      </c>
-      <c r="N19" t="n">
-        <v>59</v>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P19" t="n">
-        <v>74.59999999999999</v>
-      </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T19" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U19" t="inlineStr"/>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>CHTR</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>104.07</v>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>43.5</v>
-      </c>
-      <c r="J20" t="n">
-        <v>32.5</v>
-      </c>
-      <c r="K20" t="n">
-        <v>74</v>
-      </c>
-      <c r="L20" t="n">
-        <v>4.9</v>
-      </c>
-      <c r="M20" t="n">
-        <v>55.9</v>
-      </c>
-      <c r="N20" t="n">
-        <v>49.6</v>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P20" t="n">
-        <v>29.8</v>
-      </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S20" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T20" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U20" t="inlineStr"/>
-      <c r="V20" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan 16.10.2026 17:55 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V14"/>
+  <dimension ref="A1:V11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -458,7 +458,7 @@
     <col width="15" customWidth="1" min="18" max="18"/>
     <col width="11" customWidth="1" min="19" max="19"/>
     <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="19" customWidth="1" min="21" max="21"/>
+    <col width="25" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>755.47</v>
+        <v>759.4299999999999</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,22 +614,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>78.90000000000001</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>43.9</v>
+        <v>44.6</v>
       </c>
       <c r="K2" t="n">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="L2" t="n">
-        <v>6.51</v>
+        <v>6.22</v>
       </c>
       <c r="M2" t="n">
-        <v>111</v>
+        <v>111.8</v>
       </c>
       <c r="N2" t="n">
-        <v>100</v>
+        <v>99.7</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>35.4</v>
+        <v>35.6</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -669,11 +669,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DASH</t>
+          <t>GFS</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>190.93</v>
+        <v>47.05</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -706,70 +706,74 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>75</v>
+        <v>76.3</v>
       </c>
       <c r="J3" t="n">
-        <v>46.8</v>
+        <v>46.7</v>
       </c>
       <c r="K3" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="L3" t="n">
-        <v>4.17</v>
+        <v>5.11</v>
       </c>
       <c r="M3" t="n">
-        <v>44.3</v>
+        <v>46.4</v>
       </c>
       <c r="N3" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
         <v>42.2</v>
       </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P3" t="n">
-        <v>48.9</v>
-      </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MCD</t>
+          <t>LLY</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>242.96</v>
+        <v>1258.19</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -784,12 +788,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -798,34 +802,34 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>71.59999999999999</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>52.2</v>
+        <v>68.7</v>
       </c>
       <c r="K4" t="n">
-        <v>73</v>
+        <v>35</v>
       </c>
       <c r="L4" t="n">
-        <v>1.83</v>
+        <v>2.99</v>
       </c>
       <c r="M4" t="n">
-        <v>21.4</v>
+        <v>24.1</v>
       </c>
       <c r="N4" t="n">
-        <v>60</v>
+        <v>14.6</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>34.7</v>
+        <v>62.3</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>FIRED</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -835,7 +839,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -843,7 +847,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr"/>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Squeeze Fired</t>
+        </is>
+      </c>
       <c r="V4" t="inlineStr">
         <is>
           <t>No</t>
@@ -853,30 +861,30 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LLY</t>
+          <t>DASH</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1264.91</v>
+        <v>187.61</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -886,38 +894,38 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>70</v>
+        <v>69.2</v>
       </c>
       <c r="J5" t="n">
-        <v>69.5</v>
+        <v>44.4</v>
       </c>
       <c r="K5" t="n">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="L5" t="n">
-        <v>3.15</v>
+        <v>4.37</v>
       </c>
       <c r="M5" t="n">
-        <v>25.6</v>
+        <v>45.8</v>
       </c>
       <c r="N5" t="n">
-        <v>19.2</v>
+        <v>45.3</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>62.7</v>
+        <v>47.6</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>FIRED</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -927,37 +935,37 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>Squeeze Fired</t>
-        </is>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SNPS</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>462.31</v>
+        <v>341.85</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -972,36 +980,36 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>67.2</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="J6" t="n">
-        <v>52.7</v>
+        <v>45.5</v>
       </c>
       <c r="K6" t="n">
-        <v>93</v>
+        <v>12</v>
       </c>
       <c r="L6" t="n">
-        <v>4.1</v>
+        <v>2.63</v>
       </c>
       <c r="M6" t="n">
-        <v>53.8</v>
+        <v>23.1</v>
       </c>
       <c r="N6" t="n">
-        <v>64.2</v>
+        <v>22.3</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1009,11 +1017,11 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>53.1</v>
+        <v>49.9</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1033,7 +1041,7 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
@@ -1045,59 +1053,59 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>BLK</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>453.6</v>
+        <v>1128.54</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>66.5</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="J7" t="n">
-        <v>46.4</v>
+        <v>62.7</v>
       </c>
       <c r="K7" t="n">
-        <v>93</v>
+        <v>19</v>
       </c>
       <c r="L7" t="n">
-        <v>2.98</v>
+        <v>2.6</v>
       </c>
       <c r="M7" t="n">
-        <v>24.1</v>
+        <v>23.9</v>
       </c>
       <c r="N7" t="n">
-        <v>26.8</v>
+        <v>22.9</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1105,21 +1113,21 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>49.4</v>
+        <v>57</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>FIRED</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -1129,23 +1137,23 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>Squeeze Fired, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>133.79</v>
+        <v>338.09</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1178,30 +1186,30 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>61.7</v>
+        <v>66.8</v>
       </c>
       <c r="J8" t="n">
-        <v>43.7</v>
+        <v>45</v>
       </c>
       <c r="K8" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="L8" t="n">
-        <v>5.52</v>
+        <v>2.6</v>
       </c>
       <c r="M8" t="n">
-        <v>56.1</v>
+        <v>22.3</v>
       </c>
       <c r="N8" t="n">
-        <v>43.7</v>
+        <v>18.5</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>41.6</v>
+        <v>49.4</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1225,71 +1233,71 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>TTM Squeeze</t>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>KHC</t>
+          <t>TTWO</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>23.25</v>
+        <v>204.6</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>59.6</v>
+        <v>65.5</v>
       </c>
       <c r="J9" t="n">
-        <v>50</v>
+        <v>45.2</v>
       </c>
       <c r="K9" t="n">
-        <v>78</v>
+        <v>2</v>
       </c>
       <c r="L9" t="n">
-        <v>2.52</v>
+        <v>3.62</v>
       </c>
       <c r="M9" t="n">
-        <v>21.1</v>
+        <v>33.4</v>
       </c>
       <c r="N9" t="n">
-        <v>28.8</v>
+        <v>50.2</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1297,11 +1305,11 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>46.8</v>
+        <v>41.4</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1316,10 +1324,14 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V9" t="inlineStr">
         <is>
           <t>No</t>
@@ -1329,11 +1341,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>368.65</v>
+        <v>128.82</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1366,34 +1378,34 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>55.7</v>
+        <v>53.8</v>
       </c>
       <c r="J10" t="n">
-        <v>44.1</v>
+        <v>40.4</v>
       </c>
       <c r="K10" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="L10" t="n">
-        <v>4.81</v>
+        <v>5.68</v>
       </c>
       <c r="M10" t="n">
-        <v>56.1</v>
+        <v>54.6</v>
       </c>
       <c r="N10" t="n">
-        <v>65.59999999999999</v>
+        <v>39.3</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>58.6</v>
+        <v>40</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>FIRED</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -1403,57 +1415,57 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>Squeeze Expanding</t>
+          <t>Squeeze Fired, Divergence, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>NOC</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>498.02</v>
+        <v>341.72</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1462,30 +1474,30 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>52.1</v>
+        <v>32.5</v>
       </c>
       <c r="J11" t="n">
-        <v>48</v>
+        <v>36.9</v>
       </c>
       <c r="K11" t="n">
-        <v>63</v>
+        <v>21</v>
       </c>
       <c r="L11" t="n">
-        <v>2.27</v>
+        <v>5.91</v>
       </c>
       <c r="M11" t="n">
-        <v>24.1</v>
+        <v>60.7</v>
       </c>
       <c r="N11" t="n">
-        <v>46.8</v>
+        <v>74.8</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>40.4</v>
+        <v>53.8</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1494,301 +1506,25 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V11" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>ADI</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>399.99</v>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
-        <v>45.7</v>
-      </c>
-      <c r="J12" t="n">
-        <v>53.2</v>
-      </c>
-      <c r="K12" t="n">
-        <v>57</v>
-      </c>
-      <c r="L12" t="n">
-        <v>3.05</v>
-      </c>
-      <c r="M12" t="n">
-        <v>30.9</v>
-      </c>
-      <c r="N12" t="n">
-        <v>19.4</v>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P12" t="n">
-        <v>57</v>
-      </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S12" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr"/>
-      <c r="V12" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>CHTR</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>108.67</v>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Credit Put</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>41.8</v>
-      </c>
-      <c r="J13" t="n">
-        <v>38.8</v>
-      </c>
-      <c r="K13" t="n">
-        <v>67</v>
-      </c>
-      <c r="L13" t="n">
-        <v>4.63</v>
-      </c>
-      <c r="M13" t="n">
-        <v>49.4</v>
-      </c>
-      <c r="N13" t="n">
-        <v>40.3</v>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P13" t="n">
-        <v>32.5</v>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T13" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr"/>
-      <c r="V13" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>DLR</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>171.17</v>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>38.8</v>
-      </c>
-      <c r="J14" t="n">
-        <v>37.2</v>
-      </c>
-      <c r="K14" t="n">
-        <v>42</v>
-      </c>
-      <c r="L14" t="n">
-        <v>2.79</v>
-      </c>
-      <c r="M14" t="n">
-        <v>28.3</v>
-      </c>
-      <c r="N14" t="n">
-        <v>33.7</v>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P14" t="n">
-        <v>42.4</v>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S14" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T14" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
-      <c r="V14" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>

</xml_diff>

<commit_message>
Scan 19.10.2026 19:45 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -31,10 +31,10 @@
       <sz val="11"/>
     </font>
     <font>
-      <color rgb="0022c55e"/>
+      <color rgb="00ef4444"/>
     </font>
     <font>
-      <color rgb="00ef4444"/>
+      <color rgb="0022c55e"/>
     </font>
   </fonts>
   <fills count="3">
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V11"/>
+  <dimension ref="A1:V6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>FICO</t>
+          <t>VLO</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>759.4299999999999</v>
+        <v>436.4</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -590,17 +590,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -614,30 +614,30 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>81.59999999999999</v>
+        <v>78.2</v>
       </c>
       <c r="J2" t="n">
-        <v>44.6</v>
+        <v>61.4</v>
       </c>
       <c r="K2" t="n">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="L2" t="n">
-        <v>6.22</v>
+        <v>4.09</v>
       </c>
       <c r="M2" t="n">
-        <v>111.8</v>
+        <v>39.8</v>
       </c>
       <c r="N2" t="n">
-        <v>99.7</v>
+        <v>68.5</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>35.6</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -646,12 +646,12 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -659,10 +659,14 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr"/>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -673,14 +677,14 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>47.05</v>
+        <v>46.66</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -706,22 +710,22 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>76.3</v>
+        <v>72.8</v>
       </c>
       <c r="J3" t="n">
-        <v>46.7</v>
+        <v>45.5</v>
       </c>
       <c r="K3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L3" t="n">
-        <v>5.11</v>
+        <v>5.32</v>
       </c>
       <c r="M3" t="n">
-        <v>46.4</v>
+        <v>46.8</v>
       </c>
       <c r="N3" t="n">
-        <v>23.5</v>
+        <v>24.2</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -729,7 +733,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>42.2</v>
+        <v>41.8</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -765,11 +769,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LLY</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1258.19</v>
+        <v>345.66</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -778,17 +782,17 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -798,26 +802,26 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>74.09999999999999</v>
+        <v>71.7</v>
       </c>
       <c r="J4" t="n">
-        <v>68.7</v>
+        <v>49.5</v>
       </c>
       <c r="K4" t="n">
-        <v>35</v>
+        <v>5</v>
       </c>
       <c r="L4" t="n">
-        <v>2.99</v>
+        <v>2.55</v>
       </c>
       <c r="M4" t="n">
-        <v>24.1</v>
+        <v>23.6</v>
       </c>
       <c r="N4" t="n">
-        <v>14.6</v>
+        <v>23.8</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -825,21 +829,21 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>62.3</v>
+        <v>51.4</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>FIRED</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -849,7 +853,7 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>Squeeze Fired</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -861,18 +865,18 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DASH</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>187.61</v>
+        <v>341.48</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -898,70 +902,70 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>69.2</v>
+        <v>71</v>
       </c>
       <c r="J5" t="n">
-        <v>44.4</v>
+        <v>48.8</v>
       </c>
       <c r="K5" t="n">
         <v>6</v>
       </c>
       <c r="L5" t="n">
-        <v>4.37</v>
+        <v>2.51</v>
       </c>
       <c r="M5" t="n">
-        <v>45.8</v>
+        <v>22.7</v>
       </c>
       <c r="N5" t="n">
-        <v>45.3</v>
+        <v>19.8</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>47.6</v>
+        <v>50.8</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
           <t>No</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>BLK</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>341.85</v>
+        <v>1125.77</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -970,17 +974,17 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -990,26 +994,26 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>68.09999999999999</v>
+        <v>69.5</v>
       </c>
       <c r="J6" t="n">
-        <v>45.5</v>
+        <v>60.9</v>
       </c>
       <c r="K6" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="L6" t="n">
-        <v>2.63</v>
+        <v>2.49</v>
       </c>
       <c r="M6" t="n">
-        <v>23.1</v>
+        <v>24.2</v>
       </c>
       <c r="N6" t="n">
-        <v>22.3</v>
+        <v>24.5</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1017,516 +1021,32 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>49.9</v>
+        <v>56.4</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>BLK</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>1128.54</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Debit Call</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>SQUEEZE</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>67.59999999999999</v>
-      </c>
-      <c r="J7" t="n">
-        <v>62.7</v>
-      </c>
-      <c r="K7" t="n">
-        <v>19</v>
-      </c>
-      <c r="L7" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="M7" t="n">
-        <v>23.9</v>
-      </c>
-      <c r="N7" t="n">
-        <v>22.9</v>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P7" t="n">
-        <v>57</v>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>FIRED</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>lime</t>
-        </is>
-      </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>Squeeze Fired, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V7" t="inlineStr">
-        <is>
           <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>GOOG</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>338.09</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>SQUEEZE</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>66.8</v>
-      </c>
-      <c r="J8" t="n">
-        <v>45</v>
-      </c>
-      <c r="K8" t="n">
-        <v>14</v>
-      </c>
-      <c r="L8" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="M8" t="n">
-        <v>22.3</v>
-      </c>
-      <c r="N8" t="n">
-        <v>18.5</v>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P8" t="n">
-        <v>49.4</v>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>TTWO</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>204.6</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>SQUEEZE</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>65.5</v>
-      </c>
-      <c r="J9" t="n">
-        <v>45.2</v>
-      </c>
-      <c r="K9" t="n">
-        <v>2</v>
-      </c>
-      <c r="L9" t="n">
-        <v>3.62</v>
-      </c>
-      <c r="M9" t="n">
-        <v>33.4</v>
-      </c>
-      <c r="N9" t="n">
-        <v>50.2</v>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P9" t="n">
-        <v>41.4</v>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>maroon</t>
-        </is>
-      </c>
-      <c r="T9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>ORCL</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>128.82</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>SQUEEZE</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
-        <v>53.8</v>
-      </c>
-      <c r="J10" t="n">
-        <v>40.4</v>
-      </c>
-      <c r="K10" t="n">
-        <v>15</v>
-      </c>
-      <c r="L10" t="n">
-        <v>5.68</v>
-      </c>
-      <c r="M10" t="n">
-        <v>54.6</v>
-      </c>
-      <c r="N10" t="n">
-        <v>39.3</v>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P10" t="n">
-        <v>40</v>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>FIRED</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>Squeeze Fired, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>PANW</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>341.72</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>32.5</v>
-      </c>
-      <c r="J11" t="n">
-        <v>36.9</v>
-      </c>
-      <c r="K11" t="n">
-        <v>21</v>
-      </c>
-      <c r="L11" t="n">
-        <v>5.91</v>
-      </c>
-      <c r="M11" t="n">
-        <v>60.7</v>
-      </c>
-      <c r="N11" t="n">
-        <v>74.8</v>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P11" t="n">
-        <v>53.8</v>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T11" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
-      <c r="V11" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan 20.10.2026 18:25 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -31,10 +31,10 @@
       <sz val="11"/>
     </font>
     <font>
-      <color rgb="00ef4444"/>
+      <color rgb="0022c55e"/>
     </font>
     <font>
-      <color rgb="0022c55e"/>
+      <color rgb="00ef4444"/>
     </font>
   </fonts>
   <fills count="3">
@@ -435,11 +435,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V6"/>
+  <dimension ref="A1:V7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -577,81 +577,81 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>VLO</t>
+          <t>HON</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>436.4</v>
+        <v>212.33</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>78.2</v>
+        <v>84</v>
       </c>
       <c r="J2" t="n">
-        <v>61.4</v>
+        <v>52.7</v>
       </c>
       <c r="K2" t="n">
-        <v>91</v>
+        <v>2</v>
       </c>
       <c r="L2" t="n">
-        <v>4.09</v>
+        <v>1.97</v>
       </c>
       <c r="M2" t="n">
-        <v>39.8</v>
+        <v>16.7</v>
       </c>
       <c r="N2" t="n">
-        <v>68.5</v>
+        <v>9</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>76.09999999999999</v>
+        <v>44.5</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -661,30 +661,30 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GFS</t>
+          <t>MPC</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>46.66</v>
+        <v>473.98</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -696,91 +696,87 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>72.8</v>
+        <v>79.3</v>
       </c>
       <c r="J3" t="n">
-        <v>45.5</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="K3" t="n">
-        <v>3</v>
+        <v>94</v>
       </c>
       <c r="L3" t="n">
-        <v>5.32</v>
+        <v>3.45</v>
       </c>
       <c r="M3" t="n">
-        <v>46.8</v>
+        <v>36.4</v>
       </c>
       <c r="N3" t="n">
-        <v>24.2</v>
+        <v>65.5</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>41.8</v>
+        <v>78.8</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>PH</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>345.66</v>
+        <v>940.6799999999999</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -806,22 +802,22 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>71.7</v>
+        <v>75.2</v>
       </c>
       <c r="J4" t="n">
-        <v>49.5</v>
+        <v>41.3</v>
       </c>
       <c r="K4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L4" t="n">
-        <v>2.55</v>
+        <v>2.14</v>
       </c>
       <c r="M4" t="n">
-        <v>23.6</v>
+        <v>20.2</v>
       </c>
       <c r="N4" t="n">
-        <v>23.8</v>
+        <v>15.2</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -829,7 +825,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>51.4</v>
+        <v>47.9</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -853,30 +849,30 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>TTM Squeeze</t>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>GFS</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>341.48</v>
+        <v>47.57</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -902,30 +898,30 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>71</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>48.8</v>
+        <v>49.1</v>
       </c>
       <c r="K5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L5" t="n">
-        <v>2.51</v>
+        <v>5.45</v>
       </c>
       <c r="M5" t="n">
-        <v>22.7</v>
+        <v>47.8</v>
       </c>
       <c r="N5" t="n">
-        <v>19.8</v>
+        <v>25.8</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>50.8</v>
+        <v>43</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -939,7 +935,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -949,7 +945,7 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>TTM Squeeze</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
@@ -961,11 +957,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BLK</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1125.77</v>
+        <v>340.33</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -974,17 +970,17 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -994,26 +990,26 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>69.5</v>
+        <v>70.8</v>
       </c>
       <c r="J6" t="n">
-        <v>60.9</v>
+        <v>44.7</v>
       </c>
       <c r="K6" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="L6" t="n">
-        <v>2.49</v>
+        <v>2.42</v>
       </c>
       <c r="M6" t="n">
-        <v>24.2</v>
+        <v>23.6</v>
       </c>
       <c r="N6" t="n">
-        <v>24.5</v>
+        <v>24</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1021,30 +1017,130 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>56.4</v>
+        <v>49.4</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr">
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>GOOG</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>336.37</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>69.09999999999999</v>
+      </c>
+      <c r="J7" t="n">
+        <v>44</v>
+      </c>
+      <c r="K7" t="n">
+        <v>7</v>
+      </c>
+      <c r="L7" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="M7" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="N7" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P7" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Scan 21.10.2026 18:31 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -439,7 +439,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>212.33</v>
+        <v>215.11</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,22 +614,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>84</v>
+        <v>87.5</v>
       </c>
       <c r="J2" t="n">
-        <v>52.7</v>
+        <v>57.6</v>
       </c>
       <c r="K2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L2" t="n">
-        <v>1.97</v>
+        <v>1.94</v>
       </c>
       <c r="M2" t="n">
-        <v>16.7</v>
+        <v>16.4</v>
       </c>
       <c r="N2" t="n">
-        <v>9</v>
+        <v>7.9</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>44.5</v>
+        <v>46.2</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -651,7 +651,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -673,15 +673,15 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MPC</t>
+          <t>PH</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>473.98</v>
+        <v>963.1799999999999</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -696,36 +696,36 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>79.3</v>
+        <v>78.2</v>
       </c>
       <c r="J3" t="n">
-        <v>71.59999999999999</v>
+        <v>50.2</v>
       </c>
       <c r="K3" t="n">
-        <v>94</v>
+        <v>3</v>
       </c>
       <c r="L3" t="n">
-        <v>3.45</v>
+        <v>2.12</v>
       </c>
       <c r="M3" t="n">
-        <v>36.4</v>
+        <v>20.5</v>
       </c>
       <c r="N3" t="n">
-        <v>65.5</v>
+        <v>16.7</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -733,11 +733,11 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>78.8</v>
+        <v>51.8</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -747,7 +747,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -755,7 +755,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr"/>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V3" t="inlineStr">
         <is>
           <t>No</t>
@@ -765,15 +769,15 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>MPC</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>940.6799999999999</v>
+        <v>467.88</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -788,36 +792,36 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>75.2</v>
+        <v>74.8</v>
       </c>
       <c r="J4" t="n">
-        <v>41.3</v>
+        <v>66.7</v>
       </c>
       <c r="K4" t="n">
-        <v>4</v>
+        <v>89</v>
       </c>
       <c r="L4" t="n">
-        <v>2.14</v>
+        <v>3.61</v>
       </c>
       <c r="M4" t="n">
-        <v>20.2</v>
+        <v>36.9</v>
       </c>
       <c r="N4" t="n">
-        <v>15.2</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -825,11 +829,11 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>47.9</v>
+        <v>76.8</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -839,7 +843,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -849,7 +853,7 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+          <t>Divergence</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -861,11 +865,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GFS</t>
+          <t>DASH</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>47.57</v>
+        <v>187.31</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -898,22 +902,22 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>70.90000000000001</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="J5" t="n">
-        <v>49.1</v>
+        <v>44.3</v>
       </c>
       <c r="K5" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="L5" t="n">
-        <v>5.45</v>
+        <v>4.27</v>
       </c>
       <c r="M5" t="n">
-        <v>47.8</v>
+        <v>42.1</v>
       </c>
       <c r="N5" t="n">
-        <v>25.8</v>
+        <v>37.3</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -921,7 +925,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>43</v>
+        <v>47.5</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -930,57 +934,57 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>URI</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>340.33</v>
+        <v>1071.65</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -994,22 +998,22 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>70.8</v>
+        <v>60.8</v>
       </c>
       <c r="J6" t="n">
-        <v>44.7</v>
+        <v>56.5</v>
       </c>
       <c r="K6" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L6" t="n">
-        <v>2.42</v>
+        <v>3.3</v>
       </c>
       <c r="M6" t="n">
-        <v>23.6</v>
+        <v>31.3</v>
       </c>
       <c r="N6" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1017,7 +1021,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>49.4</v>
+        <v>54.9</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1026,12 +1030,12 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1041,7 +1045,7 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>TTM Squeeze</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
@@ -1053,11 +1057,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>DXCM</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>336.37</v>
+        <v>81.33</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1090,22 +1094,22 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>69.09999999999999</v>
+        <v>60.2</v>
       </c>
       <c r="J7" t="n">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="K7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L7" t="n">
-        <v>2.4</v>
+        <v>3.55</v>
       </c>
       <c r="M7" t="n">
-        <v>22.8</v>
+        <v>30.7</v>
       </c>
       <c r="N7" t="n">
-        <v>20.2</v>
+        <v>25.2</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1113,7 +1117,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>48.8</v>
+        <v>51.7</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1137,12 +1141,12 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan 22.10.2026 18:27 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V7"/>
+  <dimension ref="A1:V9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>215.11</v>
+        <v>216</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,22 +614,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>87.5</v>
+        <v>81.2</v>
       </c>
       <c r="J2" t="n">
-        <v>57.6</v>
+        <v>59.2</v>
       </c>
       <c r="K2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L2" t="n">
-        <v>1.94</v>
+        <v>2.42</v>
       </c>
       <c r="M2" t="n">
-        <v>16.4</v>
+        <v>15.7</v>
       </c>
       <c r="N2" t="n">
-        <v>7.9</v>
+        <v>5.6</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>46.2</v>
+        <v>46.7</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -673,15 +673,15 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>MCK</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>963.1799999999999</v>
+        <v>1007.95</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -696,36 +696,36 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>78.2</v>
+        <v>69.5</v>
       </c>
       <c r="J3" t="n">
-        <v>50.2</v>
+        <v>69.5</v>
       </c>
       <c r="K3" t="n">
-        <v>3</v>
+        <v>99</v>
       </c>
       <c r="L3" t="n">
-        <v>2.12</v>
+        <v>2.25</v>
       </c>
       <c r="M3" t="n">
-        <v>20.5</v>
+        <v>25.4</v>
       </c>
       <c r="N3" t="n">
-        <v>16.7</v>
+        <v>28.8</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -733,11 +733,11 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>51.8</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -747,7 +747,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -755,11 +755,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+      <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr">
         <is>
           <t>No</t>
@@ -773,7 +769,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>467.88</v>
+        <v>459.61</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -802,20 +798,20 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>74.8</v>
+        <v>67.7</v>
       </c>
       <c r="J4" t="n">
-        <v>66.7</v>
+        <v>61.2</v>
       </c>
       <c r="K4" t="n">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="L4" t="n">
-        <v>3.61</v>
+        <v>3.9</v>
       </c>
       <c r="M4" t="n">
         <v>36.9</v>
@@ -829,7 +825,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>76.8</v>
+        <v>74.3</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -869,7 +865,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>187.31</v>
+        <v>184.25</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -902,22 +898,22 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>72.09999999999999</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="J5" t="n">
-        <v>44.3</v>
+        <v>42.1</v>
       </c>
       <c r="K5" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="L5" t="n">
-        <v>4.27</v>
+        <v>4.31</v>
       </c>
       <c r="M5" t="n">
-        <v>42.1</v>
+        <v>42.5</v>
       </c>
       <c r="N5" t="n">
-        <v>37.3</v>
+        <v>38.2</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -925,7 +921,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>47.5</v>
+        <v>46.3</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -934,27 +930,27 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
           <t>No</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -965,7 +961,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1071.65</v>
+        <v>1094.61</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -998,22 +994,22 @@
         </is>
       </c>
       <c r="I6" t="n">
+        <v>60.6</v>
+      </c>
+      <c r="J6" t="n">
         <v>60.8</v>
       </c>
-      <c r="J6" t="n">
-        <v>56.5</v>
-      </c>
       <c r="K6" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="L6" t="n">
-        <v>3.3</v>
+        <v>3.62</v>
       </c>
       <c r="M6" t="n">
-        <v>31.3</v>
+        <v>29.4</v>
       </c>
       <c r="N6" t="n">
-        <v>16</v>
+        <v>12.1</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1021,7 +1017,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>54.9</v>
+        <v>56.8</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1057,94 +1053,286 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>BKR</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>53.38</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="J7" t="n">
+        <v>35.1</v>
+      </c>
+      <c r="K7" t="n">
+        <v>19</v>
+      </c>
+      <c r="L7" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="M7" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="N7" t="n">
+        <v>31.3</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P7" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>DXCM</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>81.33</v>
-      </c>
-      <c r="C7" t="inlineStr">
+      <c r="B8" t="n">
+        <v>77.61</v>
+      </c>
+      <c r="C8" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>SELL</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Debit Put</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>30-60 DTE</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>SQUEEZE</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>60.2</v>
-      </c>
-      <c r="J7" t="n">
-        <v>38</v>
-      </c>
-      <c r="K7" t="n">
-        <v>6</v>
-      </c>
-      <c r="L7" t="n">
-        <v>3.55</v>
-      </c>
-      <c r="M7" t="n">
-        <v>30.7</v>
-      </c>
-      <c r="N7" t="n">
-        <v>25.2</v>
-      </c>
-      <c r="O7" t="inlineStr">
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="J8" t="n">
+        <v>31.6</v>
+      </c>
+      <c r="K8" t="n">
+        <v>32</v>
+      </c>
+      <c r="L8" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="M8" t="n">
+        <v>33.8</v>
+      </c>
+      <c r="N8" t="n">
+        <v>33.8</v>
+      </c>
+      <c r="O8" t="inlineStr">
         <is>
           <t>Bullish</t>
         </is>
       </c>
-      <c r="P7" t="n">
-        <v>51.7</v>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
+      <c r="P8" t="n">
+        <v>47.7</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>FIRED</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
+      <c r="S8" t="inlineStr">
         <is>
           <t>red</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr">
+      <c r="T8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V7" t="inlineStr">
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Squeeze Fired, Divergence</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>PH</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>881.65</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="J9" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="K9" t="n">
+        <v>44</v>
+      </c>
+      <c r="L9" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="M9" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="N9" t="n">
+        <v>67.90000000000001</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P9" t="n">
+        <v>40.1</v>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>FIRED</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Squeeze Fired, Divergence</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>

</xml_diff>

<commit_message>
Scan 23.10.2026 18:13 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -31,10 +31,10 @@
       <sz val="11"/>
     </font>
     <font>
-      <color rgb="0022c55e"/>
+      <color rgb="00ef4444"/>
     </font>
     <font>
-      <color rgb="00ef4444"/>
+      <color rgb="0022c55e"/>
     </font>
   </fonts>
   <fills count="3">
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V9"/>
+  <dimension ref="A1:V16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -448,7 +448,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
     <col width="6" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
@@ -577,71 +577,71 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>HON</t>
+          <t>CCI</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>216</v>
+        <v>86.70999999999999</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>81.2</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>59.2</v>
+        <v>73</v>
       </c>
       <c r="K2" t="n">
-        <v>6</v>
+        <v>100</v>
       </c>
       <c r="L2" t="n">
-        <v>2.42</v>
+        <v>4.9</v>
       </c>
       <c r="M2" t="n">
-        <v>15.7</v>
+        <v>58.7</v>
       </c>
       <c r="N2" t="n">
-        <v>5.6</v>
+        <v>100</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>46.7</v>
+        <v>59.9</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -656,14 +656,10 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
         <is>
           <t>No</t>
@@ -673,18 +669,18 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MCK</t>
+          <t>XEL</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1007.95</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -710,22 +706,22 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>69.5</v>
+        <v>82.7</v>
       </c>
       <c r="J3" t="n">
-        <v>69.5</v>
+        <v>63.5</v>
       </c>
       <c r="K3" t="n">
         <v>99</v>
       </c>
       <c r="L3" t="n">
-        <v>2.25</v>
+        <v>1.88</v>
       </c>
       <c r="M3" t="n">
-        <v>25.4</v>
+        <v>20.5</v>
       </c>
       <c r="N3" t="n">
-        <v>28.8</v>
+        <v>52.5</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -733,7 +729,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>72.09999999999999</v>
+        <v>53.2</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -755,28 +751,32 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr"/>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MPC</t>
+          <t>ACN</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>459.61</v>
+        <v>246.85</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -798,26 +798,26 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>67.7</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>61.2</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="K4" t="n">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="L4" t="n">
-        <v>3.9</v>
+        <v>4.51</v>
       </c>
       <c r="M4" t="n">
-        <v>36.9</v>
+        <v>67.2</v>
       </c>
       <c r="N4" t="n">
-        <v>68.40000000000001</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -825,7 +825,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>74.3</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -834,17 +834,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -861,18 +861,18 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DASH</t>
+          <t>PCAR</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>184.25</v>
+        <v>107.43</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -898,22 +898,22 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>64.09999999999999</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>42.1</v>
+        <v>35.2</v>
       </c>
       <c r="K5" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="L5" t="n">
-        <v>4.31</v>
+        <v>2.23</v>
       </c>
       <c r="M5" t="n">
-        <v>42.5</v>
+        <v>20.4</v>
       </c>
       <c r="N5" t="n">
-        <v>38.2</v>
+        <v>23.1</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -921,95 +921,95 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>46.3</v>
+        <v>36</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>URI</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1094.61</v>
+        <v>391.05</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>60.6</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>60.8</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="K6" t="n">
-        <v>13</v>
+        <v>99</v>
       </c>
       <c r="L6" t="n">
-        <v>3.62</v>
+        <v>2.07</v>
       </c>
       <c r="M6" t="n">
-        <v>29.4</v>
+        <v>20.1</v>
       </c>
       <c r="N6" t="n">
-        <v>12.1</v>
+        <v>13.8</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1017,21 +1017,21 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>56.8</v>
+        <v>64.5</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1039,11 +1039,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr">
         <is>
           <t>No</t>
@@ -1053,18 +1049,18 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BKR</t>
+          <t>BKNG</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>53.38</v>
+        <v>157.1</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -1090,22 +1086,22 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>54.5</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="J7" t="n">
-        <v>35.1</v>
+        <v>39.2</v>
       </c>
       <c r="K7" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="L7" t="n">
-        <v>3.21</v>
+        <v>3.45</v>
       </c>
       <c r="M7" t="n">
-        <v>27.3</v>
+        <v>30.7</v>
       </c>
       <c r="N7" t="n">
-        <v>31.3</v>
+        <v>33.3</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1113,7 +1109,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>40.9</v>
+        <v>38.6</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1122,17 +1118,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1149,18 +1145,18 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>DXCM</t>
+          <t>AMP</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>77.61</v>
+        <v>490.74</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -1182,81 +1178,81 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>38.2</v>
+        <v>68.7</v>
       </c>
       <c r="J8" t="n">
-        <v>31.6</v>
+        <v>41.8</v>
       </c>
       <c r="K8" t="n">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="L8" t="n">
-        <v>3.76</v>
+        <v>2.28</v>
       </c>
       <c r="M8" t="n">
-        <v>33.8</v>
+        <v>26.5</v>
       </c>
       <c r="N8" t="n">
-        <v>33.8</v>
+        <v>42.6</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>47.7</v>
+        <v>44.8</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>FIRED</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>Squeeze Fired, Divergence</t>
+          <t>TTM Squeeze, Squeeze Expanding</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>DASH</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>881.65</v>
+        <v>182.81</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
@@ -1278,63 +1274,720 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>65.7</v>
+      </c>
+      <c r="J9" t="n">
+        <v>41.3</v>
+      </c>
+      <c r="K9" t="n">
+        <v>15</v>
+      </c>
+      <c r="L9" t="n">
+        <v>4.03</v>
+      </c>
+      <c r="M9" t="n">
+        <v>42.7</v>
+      </c>
+      <c r="N9" t="n">
+        <v>38.7</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P9" t="n">
+        <v>45.8</v>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>FIRED</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Squeeze Fired, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TGT</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>152.66</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Debit Call</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>64.09999999999999</v>
+      </c>
+      <c r="J10" t="n">
+        <v>46</v>
+      </c>
+      <c r="K10" t="n">
+        <v>4</v>
+      </c>
+      <c r="L10" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="M10" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="N10" t="n">
+        <v>29.3</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P10" t="n">
+        <v>59.6</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>MCK</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1000.81</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>62.8</v>
+      </c>
+      <c r="J11" t="n">
+        <v>66.40000000000001</v>
+      </c>
+      <c r="K11" t="n">
+        <v>98</v>
+      </c>
+      <c r="L11" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="M11" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="N11" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P11" t="n">
+        <v>70.90000000000001</v>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TDG</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1100.18</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>62.7</v>
+      </c>
+      <c r="J12" t="n">
+        <v>42.8</v>
+      </c>
+      <c r="K12" t="n">
+        <v>15</v>
+      </c>
+      <c r="L12" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="M12" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="N12" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P12" t="n">
+        <v>40.1</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BKR</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>55.79</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>61.2</v>
+      </c>
+      <c r="J13" t="n">
+        <v>46.6</v>
+      </c>
+      <c r="K13" t="n">
+        <v>7</v>
+      </c>
+      <c r="L13" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="M13" t="n">
+        <v>29.6</v>
+      </c>
+      <c r="N13" t="n">
+        <v>43.4</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>44.7</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>MPC</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>459.34</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
           <t>NEUTRAL</t>
         </is>
       </c>
-      <c r="I9" t="n">
-        <v>28.2</v>
-      </c>
-      <c r="J9" t="n">
-        <v>29.9</v>
-      </c>
-      <c r="K9" t="n">
-        <v>44</v>
-      </c>
-      <c r="L9" t="n">
-        <v>3.23</v>
-      </c>
-      <c r="M9" t="n">
-        <v>30.5</v>
-      </c>
-      <c r="N9" t="n">
-        <v>67.90000000000001</v>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P9" t="n">
-        <v>40.1</v>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>FIRED</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
+      <c r="I14" t="n">
+        <v>59.6</v>
+      </c>
+      <c r="J14" t="n">
+        <v>61</v>
+      </c>
+      <c r="K14" t="n">
+        <v>72</v>
+      </c>
+      <c r="L14" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="M14" t="n">
+        <v>37</v>
+      </c>
+      <c r="N14" t="n">
+        <v>68.7</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P14" t="n">
+        <v>74.3</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr">
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>URI</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1096.76</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Debit Call</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>54.4</v>
+      </c>
+      <c r="J15" t="n">
+        <v>59.7</v>
+      </c>
+      <c r="K15" t="n">
+        <v>32</v>
+      </c>
+      <c r="L15" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="M15" t="n">
+        <v>31</v>
+      </c>
+      <c r="N15" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P15" t="n">
+        <v>57</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>DXCM</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>78.61</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>37.9</v>
+      </c>
+      <c r="J16" t="n">
+        <v>33.7</v>
+      </c>
+      <c r="K16" t="n">
+        <v>43</v>
+      </c>
+      <c r="L16" t="n">
+        <v>3.48</v>
+      </c>
+      <c r="M16" t="n">
+        <v>51</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P16" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
         <is>
           <t>red</t>
         </is>
       </c>
-      <c r="T9" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>Squeeze Fired, Divergence</t>
-        </is>
-      </c>
-      <c r="V9" t="inlineStr">
-        <is>
-          <t>Yes</t>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan 26.10.2026 19:49 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V16"/>
+  <dimension ref="A1:V24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>86.70999999999999</v>
+        <v>87.31</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,22 +614,19 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>93.59999999999999</v>
+        <v>94.5</v>
       </c>
       <c r="J2" t="n">
-        <v>73</v>
+        <v>73.7</v>
       </c>
       <c r="K2" t="n">
         <v>100</v>
       </c>
       <c r="L2" t="n">
-        <v>4.9</v>
+        <v>4.69</v>
       </c>
       <c r="M2" t="n">
-        <v>58.7</v>
-      </c>
-      <c r="N2" t="n">
-        <v>100</v>
+        <v>38.4</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,7 +634,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>59.9</v>
+        <v>60.6</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -669,11 +666,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>XEL</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>77.59999999999999</v>
+        <v>92.43000000000001</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -706,22 +703,22 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>82.7</v>
+        <v>84.2</v>
       </c>
       <c r="J3" t="n">
-        <v>63.5</v>
+        <v>65.3</v>
       </c>
       <c r="K3" t="n">
         <v>99</v>
       </c>
       <c r="L3" t="n">
-        <v>1.88</v>
+        <v>1.79</v>
       </c>
       <c r="M3" t="n">
-        <v>20.5</v>
+        <v>20.3</v>
       </c>
       <c r="N3" t="n">
-        <v>52.5</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -729,7 +726,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>53.2</v>
+        <v>54.6</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -751,25 +748,21 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ACN</t>
+          <t>AEP</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>246.85</v>
+        <v>128.87</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -802,22 +795,22 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>80.40000000000001</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>71.09999999999999</v>
+        <v>62.9</v>
       </c>
       <c r="K4" t="n">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="L4" t="n">
-        <v>4.51</v>
+        <v>1.84</v>
       </c>
       <c r="M4" t="n">
-        <v>67.2</v>
+        <v>17.9</v>
       </c>
       <c r="N4" t="n">
-        <v>79.09999999999999</v>
+        <v>46.9</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -825,7 +818,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>71.40000000000001</v>
+        <v>54.6</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -847,29 +840,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PCAR</t>
+          <t>XEL</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>107.43</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -884,44 +873,44 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>80.40000000000001</v>
+        <v>77</v>
       </c>
       <c r="J5" t="n">
-        <v>35.2</v>
+        <v>63.3</v>
       </c>
       <c r="K5" t="n">
-        <v>3</v>
+        <v>98</v>
       </c>
       <c r="L5" t="n">
-        <v>2.23</v>
+        <v>1.77</v>
       </c>
       <c r="M5" t="n">
-        <v>20.4</v>
+        <v>19.4</v>
       </c>
       <c r="N5" t="n">
-        <v>23.1</v>
+        <v>44</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>36</v>
+        <v>53</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -935,7 +924,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -943,25 +932,21 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>MNST</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>391.05</v>
+        <v>46.44</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -994,22 +979,22 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>72.90000000000001</v>
+        <v>75.8</v>
       </c>
       <c r="J6" t="n">
-        <v>66.09999999999999</v>
+        <v>60.1</v>
       </c>
       <c r="K6" t="n">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="L6" t="n">
-        <v>2.07</v>
+        <v>2.18</v>
       </c>
       <c r="M6" t="n">
-        <v>20.1</v>
+        <v>22.8</v>
       </c>
       <c r="N6" t="n">
-        <v>13.8</v>
+        <v>26.3</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1017,7 +1002,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>64.5</v>
+        <v>57.2</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1026,17 +1011,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
@@ -1049,15 +1034,15 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BKNG</t>
+          <t>ACN</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>157.1</v>
+        <v>246.82</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -1072,48 +1057,48 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>72.59999999999999</v>
+        <v>75</v>
       </c>
       <c r="J7" t="n">
-        <v>39.2</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="K7" t="n">
-        <v>2</v>
+        <v>85</v>
       </c>
       <c r="L7" t="n">
-        <v>3.45</v>
+        <v>4.36</v>
       </c>
       <c r="M7" t="n">
-        <v>30.7</v>
+        <v>65.2</v>
       </c>
       <c r="N7" t="n">
-        <v>33.3</v>
+        <v>75.3</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>38.6</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1123,7 +1108,7 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -1131,29 +1116,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AMP</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>490.74</v>
+        <v>356.91</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1168,48 +1149,45 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>68.7</v>
+        <v>74.5</v>
       </c>
       <c r="J8" t="n">
-        <v>41.8</v>
+        <v>60.3</v>
       </c>
       <c r="K8" t="n">
-        <v>6</v>
+        <v>91</v>
       </c>
       <c r="L8" t="n">
-        <v>2.28</v>
+        <v>1.88</v>
       </c>
       <c r="M8" t="n">
-        <v>26.5</v>
-      </c>
-      <c r="N8" t="n">
-        <v>42.6</v>
+        <v>21.3</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>44.8</v>
+        <v>61</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -1219,7 +1197,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -1227,11 +1205,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
           <t>No</t>
@@ -1241,15 +1215,15 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DASH</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>182.81</v>
+        <v>614.8</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -1264,48 +1238,48 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>65.7</v>
+        <v>74.3</v>
       </c>
       <c r="J9" t="n">
-        <v>41.3</v>
+        <v>62.8</v>
       </c>
       <c r="K9" t="n">
-        <v>15</v>
+        <v>99</v>
       </c>
       <c r="L9" t="n">
-        <v>4.03</v>
+        <v>1.73</v>
       </c>
       <c r="M9" t="n">
-        <v>42.7</v>
+        <v>18.8</v>
       </c>
       <c r="N9" t="n">
-        <v>38.7</v>
+        <v>20.9</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>45.8</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>FIRED</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1315,7 +1289,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1325,42 +1299,42 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>Squeeze Fired, Squeeze Expanding</t>
+          <t>Divergence</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TGT</t>
+          <t>AMP</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>152.66</v>
+        <v>493.98</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1374,30 +1348,27 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>64.09999999999999</v>
+        <v>73.2</v>
       </c>
       <c r="J10" t="n">
-        <v>46</v>
+        <v>43.8</v>
       </c>
       <c r="K10" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L10" t="n">
-        <v>2.88</v>
+        <v>2.21</v>
       </c>
       <c r="M10" t="n">
-        <v>26.8</v>
-      </c>
-      <c r="N10" t="n">
-        <v>29.3</v>
+        <v>32.8</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>59.6</v>
+        <v>45.9</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1406,12 +1377,12 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1421,23 +1392,23 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Divergence</t>
+          <t>TTM Squeeze</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MCK</t>
+          <t>AIG</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1000.81</v>
+        <v>81.11</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1470,22 +1441,22 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>62.8</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>66.40000000000001</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="K11" t="n">
         <v>98</v>
       </c>
       <c r="L11" t="n">
-        <v>2.14</v>
+        <v>1.76</v>
       </c>
       <c r="M11" t="n">
-        <v>25.7</v>
+        <v>19.9</v>
       </c>
       <c r="N11" t="n">
-        <v>29.4</v>
+        <v>29.1</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1493,7 +1464,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>70.90000000000001</v>
+        <v>61.6</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1525,15 +1496,15 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TDG</t>
+          <t>V</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1100.18</v>
+        <v>404.29</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1548,44 +1519,44 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>62.7</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="J12" t="n">
-        <v>42.8</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="K12" t="n">
-        <v>15</v>
+        <v>99</v>
       </c>
       <c r="L12" t="n">
-        <v>2.8</v>
+        <v>1.66</v>
       </c>
       <c r="M12" t="n">
-        <v>21.3</v>
+        <v>19.4</v>
       </c>
       <c r="N12" t="n">
-        <v>24.7</v>
+        <v>25.8</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>40.1</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1594,12 +1565,12 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -1607,29 +1578,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BKR</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>55.79</v>
+        <v>395.31</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1644,48 +1611,45 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>61.2</v>
+        <v>70.7</v>
       </c>
       <c r="J13" t="n">
-        <v>46.6</v>
+        <v>68.2</v>
       </c>
       <c r="K13" t="n">
-        <v>7</v>
+        <v>100</v>
       </c>
       <c r="L13" t="n">
-        <v>3.26</v>
+        <v>2.04</v>
       </c>
       <c r="M13" t="n">
-        <v>29.6</v>
-      </c>
-      <c r="N13" t="n">
-        <v>43.4</v>
+        <v>32.7</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>44.7</v>
+        <v>65.8</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -1695,7 +1659,7 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -1703,11 +1667,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+      <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr">
         <is>
           <t>No</t>
@@ -1717,15 +1677,15 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MPC</t>
+          <t>BKR</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>459.34</v>
+        <v>55.99</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1740,66 +1700,70 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>59.6</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="J14" t="n">
-        <v>61</v>
+        <v>47.5</v>
       </c>
       <c r="K14" t="n">
-        <v>72</v>
+        <v>4</v>
       </c>
       <c r="L14" t="n">
-        <v>3.65</v>
+        <v>3.1</v>
       </c>
       <c r="M14" t="n">
-        <v>37</v>
+        <v>27.6</v>
       </c>
       <c r="N14" t="n">
-        <v>68.7</v>
+        <v>33</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>74.3</v>
+        <v>45.1</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V14" t="inlineStr">
         <is>
           <t>No</t>
@@ -1809,11 +1773,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>URI</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1096.76</v>
+        <v>298.69</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1842,26 +1806,26 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>54.4</v>
+        <v>67.5</v>
       </c>
       <c r="J15" t="n">
-        <v>59.7</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="K15" t="n">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="L15" t="n">
-        <v>4.06</v>
+        <v>3.46</v>
       </c>
       <c r="M15" t="n">
-        <v>31</v>
+        <v>29.6</v>
       </c>
       <c r="N15" t="n">
-        <v>15.3</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1869,11 +1833,11 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>57</v>
+        <v>59.9</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -1888,12 +1852,12 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>TTM Squeeze</t>
+          <t>Squeeze Expanding</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
@@ -1905,11 +1869,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>DXCM</t>
+          <t>TDG</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>78.61</v>
+        <v>1124.96</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1938,56 +1902,817 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>37.9</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="J16" t="n">
-        <v>33.7</v>
+        <v>50.4</v>
       </c>
       <c r="K16" t="n">
+        <v>16</v>
+      </c>
+      <c r="L16" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="M16" t="n">
+        <v>36.1</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P16" t="n">
         <v>43</v>
       </c>
-      <c r="L16" t="n">
-        <v>3.48</v>
-      </c>
-      <c r="M16" t="n">
-        <v>51</v>
-      </c>
-      <c r="O16" t="inlineStr">
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>INTU</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>338.08</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>67.3</v>
+      </c>
+      <c r="J17" t="n">
+        <v>61</v>
+      </c>
+      <c r="K17" t="n">
+        <v>83</v>
+      </c>
+      <c r="L17" t="n">
+        <v>3.89</v>
+      </c>
+      <c r="M17" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="N17" t="n">
+        <v>30.9</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P17" t="n">
+        <v>49.3</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr"/>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BKNG</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>152.91</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>65.2</v>
+      </c>
+      <c r="J18" t="n">
+        <v>35.1</v>
+      </c>
+      <c r="K18" t="n">
+        <v>9</v>
+      </c>
+      <c r="L18" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="M18" t="n">
+        <v>31.3</v>
+      </c>
+      <c r="N18" t="n">
+        <v>35.1</v>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P18" t="n">
+        <v>36.8</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>CHTR</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>101.24</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>62.6</v>
+      </c>
+      <c r="J19" t="n">
+        <v>35.1</v>
+      </c>
+      <c r="K19" t="n">
+        <v>11</v>
+      </c>
+      <c r="L19" t="n">
+        <v>5.16</v>
+      </c>
+      <c r="M19" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="N19" t="n">
+        <v>34</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P19" t="n">
+        <v>30.7</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>PCAR</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>104.38</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="J20" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="K20" t="n">
+        <v>7</v>
+      </c>
+      <c r="L20" t="n">
+        <v>2.57</v>
+      </c>
+      <c r="M20" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="N20" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P20" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>DDOG</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>281.32</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Debit Call</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>57.6</v>
+      </c>
+      <c r="J21" t="n">
+        <v>57.6</v>
+      </c>
+      <c r="K21" t="n">
+        <v>11</v>
+      </c>
+      <c r="L21" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="M21" t="n">
+        <v>55.7</v>
+      </c>
+      <c r="N21" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="O21" t="inlineStr">
         <is>
           <t>Bullish</t>
         </is>
       </c>
-      <c r="P16" t="n">
-        <v>48.7</v>
-      </c>
-      <c r="Q16" t="inlineStr">
+      <c r="P21" t="n">
+        <v>60.6</v>
+      </c>
+      <c r="Q21" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="R16" t="inlineStr">
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>MCK</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>990.83</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>56.9</v>
+      </c>
+      <c r="J22" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="K22" t="n">
+        <v>96</v>
+      </c>
+      <c r="L22" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="M22" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="N22" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P22" t="n">
+        <v>68.7</v>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="S16" t="inlineStr">
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>TGT</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>148.48</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Debit Call</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>50.7</v>
+      </c>
+      <c r="J23" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="K23" t="n">
+        <v>14</v>
+      </c>
+      <c r="L23" t="n">
+        <v>3.18</v>
+      </c>
+      <c r="M23" t="n">
+        <v>43.6</v>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P23" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
         <is>
           <t>red</t>
         </is>
       </c>
-      <c r="T16" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr"/>
-      <c r="V16" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>MRK</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>140.17</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>41.1</v>
+      </c>
+      <c r="J24" t="n">
+        <v>42</v>
+      </c>
+      <c r="K24" t="n">
+        <v>16</v>
+      </c>
+      <c r="L24" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="M24" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="N24" t="n">
+        <v>34.1</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P24" t="n">
+        <v>56.5</v>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan 27.10.2026 19:19 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V24"/>
+  <dimension ref="A1:V33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -448,7 +448,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
     <col width="6" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CCI</t>
+          <t>XLE</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>87.31</v>
+        <v>68.28</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,19 +614,19 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>94.5</v>
+        <v>82</v>
       </c>
       <c r="J2" t="n">
-        <v>73.7</v>
+        <v>61.6</v>
       </c>
       <c r="K2" t="n">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="L2" t="n">
-        <v>4.69</v>
+        <v>2.24</v>
       </c>
       <c r="M2" t="n">
-        <v>38.4</v>
+        <v>27.2</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -634,7 +634,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>60.6</v>
+        <v>67.2</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -666,11 +666,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>EOG</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>92.43000000000001</v>
+        <v>161.29</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>84.2</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="J3" t="n">
-        <v>65.3</v>
+        <v>69.8</v>
       </c>
       <c r="K3" t="n">
         <v>99</v>
       </c>
       <c r="L3" t="n">
-        <v>1.79</v>
+        <v>2.54</v>
       </c>
       <c r="M3" t="n">
-        <v>20.3</v>
+        <v>30</v>
       </c>
       <c r="N3" t="n">
-        <v>73.40000000000001</v>
+        <v>55.3</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -726,7 +726,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>54.6</v>
+        <v>64.5</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -758,11 +758,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>COP</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>128.87</v>
+        <v>148.08</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -795,22 +795,22 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>77.09999999999999</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>62.9</v>
+        <v>67.7</v>
       </c>
       <c r="K4" t="n">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="L4" t="n">
-        <v>1.84</v>
+        <v>2.58</v>
       </c>
       <c r="M4" t="n">
-        <v>17.9</v>
+        <v>32.5</v>
       </c>
       <c r="N4" t="n">
-        <v>46.9</v>
+        <v>63.7</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -818,7 +818,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>54.6</v>
+        <v>67</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -840,21 +840,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr"/>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>XEL</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>77.59999999999999</v>
+        <v>602.62</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -887,22 +891,22 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>77</v>
+        <v>80.7</v>
       </c>
       <c r="J5" t="n">
-        <v>63.3</v>
+        <v>61.9</v>
       </c>
       <c r="K5" t="n">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="L5" t="n">
-        <v>1.77</v>
+        <v>2.61</v>
       </c>
       <c r="M5" t="n">
-        <v>19.4</v>
+        <v>26.2</v>
       </c>
       <c r="N5" t="n">
-        <v>44</v>
+        <v>38.6</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -910,7 +914,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>53</v>
+        <v>56.3</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -932,21 +936,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr"/>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MNST</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>46.44</v>
+        <v>92.34999999999999</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -979,22 +987,22 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>75.8</v>
+        <v>78.7</v>
       </c>
       <c r="J6" t="n">
-        <v>60.1</v>
+        <v>64.8</v>
       </c>
       <c r="K6" t="n">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="L6" t="n">
-        <v>2.18</v>
+        <v>1.67</v>
       </c>
       <c r="M6" t="n">
-        <v>22.8</v>
+        <v>19.9</v>
       </c>
       <c r="N6" t="n">
-        <v>26.3</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1002,7 +1010,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>57.2</v>
+        <v>54.4</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1034,15 +1042,15 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ACN</t>
+          <t>AMP</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>246.82</v>
+        <v>494.07</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -1057,48 +1065,48 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>75</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="J7" t="n">
-        <v>70.90000000000001</v>
+        <v>43.9</v>
       </c>
       <c r="K7" t="n">
-        <v>85</v>
+        <v>5</v>
       </c>
       <c r="L7" t="n">
-        <v>4.36</v>
+        <v>2.08</v>
       </c>
       <c r="M7" t="n">
-        <v>65.2</v>
+        <v>26.4</v>
       </c>
       <c r="N7" t="n">
-        <v>75.3</v>
+        <v>42.4</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>70.59999999999999</v>
+        <v>45.9</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1108,7 +1116,7 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -1116,7 +1124,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr"/>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V7" t="inlineStr">
         <is>
           <t>No</t>
@@ -1126,11 +1138,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>356.91</v>
+        <v>389.26</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1163,19 +1175,22 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>74.5</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="J8" t="n">
-        <v>60.3</v>
+        <v>62.2</v>
       </c>
       <c r="K8" t="n">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="L8" t="n">
-        <v>1.88</v>
+        <v>2.27</v>
       </c>
       <c r="M8" t="n">
-        <v>21.3</v>
+        <v>20.2</v>
+      </c>
+      <c r="N8" t="n">
+        <v>14.5</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1183,7 +1198,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>61</v>
+        <v>63.6</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1192,34 +1207,38 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>CVX</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>614.8</v>
+        <v>228.62</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1252,22 +1271,19 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>74.3</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="J9" t="n">
-        <v>62.8</v>
+        <v>66.8</v>
       </c>
       <c r="K9" t="n">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="L9" t="n">
-        <v>1.73</v>
+        <v>2.12</v>
       </c>
       <c r="M9" t="n">
-        <v>18.8</v>
-      </c>
-      <c r="N9" t="n">
-        <v>20.9</v>
+        <v>31.2</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1275,7 +1291,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>65.40000000000001</v>
+        <v>67.5</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1284,42 +1300,38 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AMP</t>
+          <t>XOM</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>493.98</v>
+        <v>180.3</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1334,81 +1346,84 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>73.2</v>
+        <v>74</v>
       </c>
       <c r="J10" t="n">
-        <v>43.8</v>
+        <v>65.5</v>
       </c>
       <c r="K10" t="n">
-        <v>6</v>
+        <v>87</v>
       </c>
       <c r="L10" t="n">
-        <v>2.21</v>
+        <v>2.3</v>
       </c>
       <c r="M10" t="n">
-        <v>32.8</v>
+        <v>23.8</v>
+      </c>
+      <c r="N10" t="n">
+        <v>41.5</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>45.9</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>TTM Squeeze</t>
+          <t>Divergence</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AIG</t>
+          <t>ACN</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>81.11</v>
+        <v>235.9</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1437,26 +1452,23 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I11" t="n">
         <v>72.40000000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>64.09999999999999</v>
+        <v>62</v>
       </c>
       <c r="K11" t="n">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="L11" t="n">
-        <v>1.76</v>
+        <v>4.65</v>
       </c>
       <c r="M11" t="n">
-        <v>19.9</v>
-      </c>
-      <c r="N11" t="n">
-        <v>29.1</v>
+        <v>42.7</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1464,7 +1476,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>61.6</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1473,17 +1485,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
@@ -1496,11 +1508,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>MNST</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>404.29</v>
+        <v>45.44</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1533,22 +1545,22 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>71.59999999999999</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="J12" t="n">
-        <v>65.40000000000001</v>
+        <v>52.8</v>
       </c>
       <c r="K12" t="n">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="L12" t="n">
-        <v>1.66</v>
+        <v>2.28</v>
       </c>
       <c r="M12" t="n">
-        <v>19.4</v>
+        <v>23.6</v>
       </c>
       <c r="N12" t="n">
-        <v>25.8</v>
+        <v>29</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1556,7 +1568,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>69.59999999999999</v>
+        <v>53.8</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1565,38 +1577,42 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>TDG</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>395.31</v>
+        <v>1131.44</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1611,41 +1627,44 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>70.7</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="J13" t="n">
-        <v>68.2</v>
+        <v>52.2</v>
       </c>
       <c r="K13" t="n">
-        <v>100</v>
+        <v>17</v>
       </c>
       <c r="L13" t="n">
-        <v>2.04</v>
+        <v>2.49</v>
       </c>
       <c r="M13" t="n">
-        <v>32.7</v>
+        <v>19.2</v>
+      </c>
+      <c r="N13" t="n">
+        <v>14.2</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>65.8</v>
+        <v>43.8</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1667,7 +1686,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr"/>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V13" t="inlineStr">
         <is>
           <t>No</t>
@@ -1677,15 +1700,15 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BKR</t>
+          <t>AEP</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>55.99</v>
+        <v>129.13</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1700,48 +1723,45 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>67.59999999999999</v>
+        <v>70.7</v>
       </c>
       <c r="J14" t="n">
-        <v>47.5</v>
+        <v>63.8</v>
       </c>
       <c r="K14" t="n">
-        <v>4</v>
+        <v>90</v>
       </c>
       <c r="L14" t="n">
-        <v>3.1</v>
+        <v>1.71</v>
       </c>
       <c r="M14" t="n">
-        <v>27.6</v>
-      </c>
-      <c r="N14" t="n">
-        <v>33</v>
+        <v>22.2</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>45.1</v>
+        <v>54.9</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -1751,7 +1771,7 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -1759,11 +1779,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+      <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr">
         <is>
           <t>No</t>
@@ -1777,7 +1793,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>298.69</v>
+        <v>307.32</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1806,26 +1822,26 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>67.5</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="J15" t="n">
-        <v>64.90000000000001</v>
+        <v>69.3</v>
       </c>
       <c r="K15" t="n">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="L15" t="n">
-        <v>3.46</v>
+        <v>3.35</v>
       </c>
       <c r="M15" t="n">
-        <v>29.6</v>
+        <v>30.3</v>
       </c>
       <c r="N15" t="n">
-        <v>9.699999999999999</v>
+        <v>11.4</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1833,7 +1849,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>59.9</v>
+        <v>62.1</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1855,11 +1871,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr">
         <is>
           <t>No</t>
@@ -1869,15 +1881,15 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TDG</t>
+          <t>XEL</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1124.96</v>
+        <v>77.81999999999999</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1892,41 +1904,44 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>67.40000000000001</v>
+        <v>70</v>
       </c>
       <c r="J16" t="n">
-        <v>50.4</v>
+        <v>64.5</v>
       </c>
       <c r="K16" t="n">
-        <v>16</v>
+        <v>97</v>
       </c>
       <c r="L16" t="n">
-        <v>2.65</v>
+        <v>1.68</v>
       </c>
       <c r="M16" t="n">
-        <v>36.1</v>
+        <v>18.7</v>
+      </c>
+      <c r="N16" t="n">
+        <v>38.4</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>43</v>
+        <v>53.5</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1940,7 +1955,7 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
@@ -1948,11 +1963,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr">
         <is>
           <t>No</t>
@@ -1962,11 +1973,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>INTU</t>
+          <t>WMT</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>338.08</v>
+        <v>119.22</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -1999,30 +2010,30 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>67.3</v>
+        <v>69.8</v>
       </c>
       <c r="J17" t="n">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="K17" t="n">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="L17" t="n">
-        <v>3.89</v>
+        <v>2.04</v>
       </c>
       <c r="M17" t="n">
-        <v>42.9</v>
+        <v>23.1</v>
       </c>
       <c r="N17" t="n">
-        <v>30.9</v>
+        <v>35.6</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>49.3</v>
+        <v>56.8</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2054,15 +2065,15 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>BKNG</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>152.91</v>
+        <v>355.06</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -2077,88 +2088,84 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>65.2</v>
+        <v>68.5</v>
       </c>
       <c r="J18" t="n">
-        <v>35.1</v>
+        <v>58.1</v>
       </c>
       <c r="K18" t="n">
-        <v>9</v>
+        <v>89</v>
       </c>
       <c r="L18" t="n">
-        <v>3.51</v>
+        <v>1.8</v>
       </c>
       <c r="M18" t="n">
-        <v>31.3</v>
+        <v>18.7</v>
       </c>
       <c r="N18" t="n">
-        <v>35.1</v>
+        <v>29.8</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>36.8</v>
+        <v>60.2</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U18" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CHTR</t>
+          <t>CDW</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>101.24</v>
+        <v>160.91</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -2173,44 +2180,44 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>62.6</v>
+        <v>68.3</v>
       </c>
       <c r="J19" t="n">
-        <v>35.1</v>
+        <v>63.9</v>
       </c>
       <c r="K19" t="n">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="L19" t="n">
-        <v>5.16</v>
+        <v>3.31</v>
       </c>
       <c r="M19" t="n">
-        <v>44.9</v>
+        <v>39.9</v>
       </c>
       <c r="N19" t="n">
-        <v>34</v>
+        <v>32.6</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>30.7</v>
+        <v>60.8</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2224,7 +2231,7 @@
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
@@ -2232,29 +2239,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PCAR</t>
+          <t>AIG</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>104.38</v>
+        <v>79.56999999999999</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -2269,44 +2272,44 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>60.7</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="J20" t="n">
-        <v>29.2</v>
+        <v>55.4</v>
       </c>
       <c r="K20" t="n">
-        <v>7</v>
+        <v>97</v>
       </c>
       <c r="L20" t="n">
-        <v>2.57</v>
+        <v>1.86</v>
       </c>
       <c r="M20" t="n">
-        <v>21.4</v>
+        <v>20.7</v>
       </c>
       <c r="N20" t="n">
-        <v>28.4</v>
+        <v>33.2</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>33.3</v>
+        <v>56.9</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2320,17 +2323,17 @@
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>Divergence, Squeeze Expanding</t>
+          <t>Divergence</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
@@ -2342,59 +2345,59 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>281.32</v>
+        <v>609.08</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>57.6</v>
+        <v>65.7</v>
       </c>
       <c r="J21" t="n">
-        <v>57.6</v>
+        <v>58.5</v>
       </c>
       <c r="K21" t="n">
-        <v>11</v>
+        <v>97</v>
       </c>
       <c r="L21" t="n">
-        <v>5.75</v>
+        <v>1.68</v>
       </c>
       <c r="M21" t="n">
-        <v>55.7</v>
+        <v>19.1</v>
       </c>
       <c r="N21" t="n">
-        <v>39.9</v>
+        <v>23.1</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2402,7 +2405,7 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>60.6</v>
+        <v>63.5</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2411,24 +2414,20 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t>Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr"/>
       <c r="V21" t="inlineStr">
         <is>
           <t>No</t>
@@ -2438,15 +2437,15 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>MCK</t>
+          <t>CHTR</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>990.83</v>
+        <v>104.64</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -2461,44 +2460,44 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>56.9</v>
+        <v>65.3</v>
       </c>
       <c r="J22" t="n">
-        <v>62.5</v>
+        <v>39.5</v>
       </c>
       <c r="K22" t="n">
-        <v>96</v>
+        <v>11</v>
       </c>
       <c r="L22" t="n">
-        <v>2.17</v>
+        <v>4.91</v>
       </c>
       <c r="M22" t="n">
-        <v>24.5</v>
+        <v>45.2</v>
       </c>
       <c r="N22" t="n">
-        <v>26.6</v>
+        <v>34.4</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P22" t="n">
-        <v>68.7</v>
+        <v>31.7</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
@@ -2507,20 +2506,24 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V22" t="inlineStr">
         <is>
           <t>No</t>
@@ -2530,11 +2533,11 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>TGT</t>
+          <t>DDOG</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>148.48</v>
+        <v>279.97</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -2567,19 +2570,22 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>50.7</v>
+        <v>65.3</v>
       </c>
       <c r="J23" t="n">
-        <v>40.2</v>
+        <v>57.1</v>
       </c>
       <c r="K23" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="L23" t="n">
-        <v>3.18</v>
+        <v>5.41</v>
       </c>
       <c r="M23" t="n">
-        <v>43.6</v>
+        <v>55.5</v>
+      </c>
+      <c r="N23" t="n">
+        <v>39.6</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2587,21 +2593,21 @@
         </is>
       </c>
       <c r="P23" t="n">
-        <v>54.9</v>
+        <v>60.3</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
@@ -2611,106 +2617,943 @@
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+          <t>Squeeze Expanding</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>399.14</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>65.09999999999999</v>
+      </c>
+      <c r="J24" t="n">
+        <v>59.5</v>
+      </c>
+      <c r="K24" t="n">
+        <v>97</v>
+      </c>
+      <c r="L24" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="M24" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="N24" t="n">
+        <v>29.1</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P24" t="n">
+        <v>66.59999999999999</v>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>991.5</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>65</v>
+      </c>
+      <c r="J25" t="n">
+        <v>61.9</v>
+      </c>
+      <c r="K25" t="n">
+        <v>90</v>
+      </c>
+      <c r="L25" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="M25" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="N25" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P25" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>BKNG</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>150.53</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>64.5</v>
+      </c>
+      <c r="J26" t="n">
+        <v>32.9</v>
+      </c>
+      <c r="K26" t="n">
+        <v>13</v>
+      </c>
+      <c r="L26" t="n">
+        <v>3.41</v>
+      </c>
+      <c r="M26" t="n">
+        <v>31</v>
+      </c>
+      <c r="N26" t="n">
+        <v>34.3</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P26" t="n">
+        <v>35.9</v>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>FIRED</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>Squeeze Fired, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>LIN</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>507.49</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>64</v>
+      </c>
+      <c r="J27" t="n">
+        <v>68.90000000000001</v>
+      </c>
+      <c r="K27" t="n">
+        <v>80</v>
+      </c>
+      <c r="L27" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="M27" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="N27" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P27" t="n">
+        <v>56.8</v>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr"/>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>ABBV</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>286.52</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="J28" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="K28" t="n">
+        <v>82</v>
+      </c>
+      <c r="L28" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="M28" t="n">
+        <v>18</v>
+      </c>
+      <c r="N28" t="n">
+        <v>7</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P28" t="n">
+        <v>71.59999999999999</v>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>INTU</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>326.84</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>60.3</v>
+      </c>
+      <c r="J29" t="n">
+        <v>54.4</v>
+      </c>
+      <c r="K29" t="n">
+        <v>76</v>
+      </c>
+      <c r="L29" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="M29" t="n">
+        <v>54.8</v>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P29" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr"/>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>MCK</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>968.6</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>51.1</v>
+      </c>
+      <c r="J30" t="n">
+        <v>54.6</v>
+      </c>
+      <c r="K30" t="n">
+        <v>94</v>
+      </c>
+      <c r="L30" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="M30" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="N30" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P30" t="n">
+        <v>64.09999999999999</v>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr"/>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>ILMN</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>279.8</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Debit Call</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>49.4</v>
+      </c>
+      <c r="J31" t="n">
+        <v>59.8</v>
+      </c>
+      <c r="K31" t="n">
+        <v>12</v>
+      </c>
+      <c r="L31" t="n">
+        <v>5.05</v>
+      </c>
+      <c r="M31" t="n">
+        <v>55.5</v>
+      </c>
+      <c r="N31" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P31" t="n">
+        <v>74.5</v>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>MRK</t>
         </is>
       </c>
-      <c r="B24" t="n">
-        <v>140.17</v>
-      </c>
-      <c r="C24" t="inlineStr">
+      <c r="B32" t="n">
+        <v>141.92</v>
+      </c>
+      <c r="C32" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>SELL</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>Debit Put</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G32" t="inlineStr">
         <is>
           <t>30-60 DTE</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="H32" t="inlineStr">
         <is>
           <t>SQUEEZE</t>
         </is>
       </c>
-      <c r="I24" t="n">
-        <v>41.1</v>
-      </c>
-      <c r="J24" t="n">
-        <v>42</v>
-      </c>
-      <c r="K24" t="n">
-        <v>16</v>
-      </c>
-      <c r="L24" t="n">
-        <v>3.55</v>
-      </c>
-      <c r="M24" t="n">
-        <v>28.4</v>
-      </c>
-      <c r="N24" t="n">
-        <v>34.1</v>
-      </c>
-      <c r="O24" t="inlineStr">
+      <c r="I32" t="n">
+        <v>42.7</v>
+      </c>
+      <c r="J32" t="n">
+        <v>45</v>
+      </c>
+      <c r="K32" t="n">
+        <v>11</v>
+      </c>
+      <c r="L32" t="n">
+        <v>3.32</v>
+      </c>
+      <c r="M32" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="N32" t="n">
+        <v>33.4</v>
+      </c>
+      <c r="O32" t="inlineStr">
         <is>
           <t>Bullish</t>
         </is>
       </c>
-      <c r="P24" t="n">
-        <v>56.5</v>
-      </c>
-      <c r="Q24" t="inlineStr">
+      <c r="P32" t="n">
+        <v>58.4</v>
+      </c>
+      <c r="Q32" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="R24" t="inlineStr">
+      <c r="R32" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="S24" t="inlineStr">
+      <c r="S32" t="inlineStr">
         <is>
           <t>red</t>
         </is>
       </c>
-      <c r="T24" t="inlineStr">
+      <c r="T32" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V24" t="inlineStr">
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>PCAR</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>102.49</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>40</v>
+      </c>
+      <c r="J33" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="K33" t="n">
+        <v>20</v>
+      </c>
+      <c r="L33" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="M33" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="N33" t="n">
+        <v>30</v>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P33" t="n">
+        <v>31.8</v>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>

</xml_diff>

<commit_message>
Scan 28.10.2026 19:25 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,11 +435,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V33"/>
+  <dimension ref="A1:V39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -577,11 +577,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>XLE</t>
+          <t>CCI</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>68.28</v>
+        <v>87.54000000000001</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,19 +614,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>82</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>61.6</v>
+        <v>73.2</v>
       </c>
       <c r="K2" t="n">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="L2" t="n">
-        <v>2.24</v>
+        <v>4.45</v>
       </c>
       <c r="M2" t="n">
-        <v>27.2</v>
+        <v>57.1</v>
+      </c>
+      <c r="N2" t="n">
+        <v>99.2</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -634,7 +637,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>67.2</v>
+        <v>60.8</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -656,21 +659,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr"/>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>EOG</t>
+          <t>DUK</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>161.29</v>
+        <v>123.81</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -703,22 +710,19 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>81.90000000000001</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>69.8</v>
+        <v>62.6</v>
       </c>
       <c r="K3" t="n">
         <v>99</v>
       </c>
       <c r="L3" t="n">
-        <v>2.54</v>
+        <v>1.54</v>
       </c>
       <c r="M3" t="n">
-        <v>30</v>
-      </c>
-      <c r="N3" t="n">
-        <v>55.3</v>
+        <v>22.3</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -726,7 +730,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>64.5</v>
+        <v>53.8</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -758,11 +762,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>COP</t>
+          <t>EXC</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>148.08</v>
+        <v>44.69</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -795,22 +799,22 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>81.40000000000001</v>
+        <v>77.2</v>
       </c>
       <c r="J4" t="n">
-        <v>67.7</v>
+        <v>66.2</v>
       </c>
       <c r="K4" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L4" t="n">
-        <v>2.58</v>
+        <v>1.68</v>
       </c>
       <c r="M4" t="n">
-        <v>32.5</v>
+        <v>21</v>
       </c>
       <c r="N4" t="n">
-        <v>63.7</v>
+        <v>51.4</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -818,7 +822,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>67</v>
+        <v>52.6</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -840,25 +844,21 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>602.62</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -891,22 +891,22 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>80.7</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>61.9</v>
+        <v>60.7</v>
       </c>
       <c r="K5" t="n">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="L5" t="n">
-        <v>2.61</v>
+        <v>1.69</v>
       </c>
       <c r="M5" t="n">
-        <v>26.2</v>
+        <v>20.2</v>
       </c>
       <c r="N5" t="n">
-        <v>38.6</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>56.3</v>
+        <v>52.8</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -936,25 +936,21 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>COP</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>92.34999999999999</v>
+        <v>149.57</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -987,22 +983,22 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>78.7</v>
+        <v>75.2</v>
       </c>
       <c r="J6" t="n">
-        <v>64.8</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="K6" t="n">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="L6" t="n">
-        <v>1.67</v>
+        <v>2.43</v>
       </c>
       <c r="M6" t="n">
-        <v>19.9</v>
+        <v>26.5</v>
       </c>
       <c r="N6" t="n">
-        <v>69.40000000000001</v>
+        <v>18.4</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1010,7 +1006,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>54.4</v>
+        <v>68.5</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1042,15 +1038,15 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AMP</t>
+          <t>BRK-B</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>494.07</v>
+        <v>541.7</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -1065,48 +1061,48 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>77.09999999999999</v>
+        <v>74.3</v>
       </c>
       <c r="J7" t="n">
-        <v>43.9</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="K7" t="n">
-        <v>5</v>
+        <v>98</v>
       </c>
       <c r="L7" t="n">
-        <v>2.08</v>
+        <v>1.21</v>
       </c>
       <c r="M7" t="n">
-        <v>26.4</v>
+        <v>13.4</v>
       </c>
       <c r="N7" t="n">
-        <v>42.4</v>
+        <v>26.5</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>45.9</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1116,7 +1112,7 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -1124,11 +1120,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+      <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr">
         <is>
           <t>No</t>
@@ -1138,15 +1130,15 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>CHTR</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>389.26</v>
+        <v>105.25</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1161,44 +1153,44 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>76.09999999999999</v>
+        <v>74</v>
       </c>
       <c r="J8" t="n">
-        <v>62.2</v>
+        <v>40.3</v>
       </c>
       <c r="K8" t="n">
-        <v>99</v>
+        <v>9</v>
       </c>
       <c r="L8" t="n">
-        <v>2.27</v>
+        <v>4.53</v>
       </c>
       <c r="M8" t="n">
-        <v>20.2</v>
+        <v>44.3</v>
       </c>
       <c r="N8" t="n">
-        <v>14.5</v>
+        <v>33.1</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>63.6</v>
+        <v>31.8</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1207,38 +1199,34 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>maroon</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CVX</t>
+          <t>AEP</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>228.62</v>
+        <v>128.54</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1271,19 +1259,19 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>75.59999999999999</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="J9" t="n">
-        <v>66.8</v>
+        <v>59.8</v>
       </c>
       <c r="K9" t="n">
         <v>87</v>
       </c>
       <c r="L9" t="n">
-        <v>2.12</v>
+        <v>1.85</v>
       </c>
       <c r="M9" t="n">
-        <v>31.2</v>
+        <v>22.5</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1291,7 +1279,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>67.5</v>
+        <v>54.1</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1313,21 +1301,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr"/>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>XOM</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>180.3</v>
+        <v>603.05</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1360,22 +1352,22 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>74</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="J10" t="n">
-        <v>65.5</v>
+        <v>61.9</v>
       </c>
       <c r="K10" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="L10" t="n">
-        <v>2.3</v>
+        <v>2.45</v>
       </c>
       <c r="M10" t="n">
-        <v>23.8</v>
+        <v>26.1</v>
       </c>
       <c r="N10" t="n">
-        <v>41.5</v>
+        <v>38.4</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1383,7 +1375,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>66.90000000000001</v>
+        <v>56.4</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1392,38 +1384,34 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ACN</t>
+          <t>EOG</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>235.9</v>
+        <v>161.52</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1452,23 +1440,26 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>72.40000000000001</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>62</v>
+        <v>69.8</v>
       </c>
       <c r="K11" t="n">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="L11" t="n">
-        <v>4.65</v>
+        <v>2.33</v>
       </c>
       <c r="M11" t="n">
-        <v>42.7</v>
+        <v>24.3</v>
+      </c>
+      <c r="N11" t="n">
+        <v>28.9</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1476,7 +1467,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>65.40000000000001</v>
+        <v>64.7</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1485,17 +1476,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
@@ -1508,11 +1499,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MNST</t>
+          <t>ADP</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>45.44</v>
+        <v>284.21</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1545,22 +1536,22 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>72.40000000000001</v>
+        <v>71.2</v>
       </c>
       <c r="J12" t="n">
-        <v>52.8</v>
+        <v>51.8</v>
       </c>
       <c r="K12" t="n">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="L12" t="n">
-        <v>2.28</v>
+        <v>2.71</v>
       </c>
       <c r="M12" t="n">
-        <v>23.6</v>
+        <v>26.4</v>
       </c>
       <c r="N12" t="n">
-        <v>29</v>
+        <v>47.4</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1568,7 +1559,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>53.8</v>
+        <v>59.6</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1604,15 +1595,15 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TDG</t>
+          <t>XOM</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1131.44</v>
+        <v>182.46</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1627,44 +1618,44 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>71.90000000000001</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="J13" t="n">
-        <v>52.2</v>
+        <v>67.8</v>
       </c>
       <c r="K13" t="n">
-        <v>17</v>
+        <v>84</v>
       </c>
       <c r="L13" t="n">
-        <v>2.49</v>
+        <v>2.24</v>
       </c>
       <c r="M13" t="n">
-        <v>19.2</v>
+        <v>21.4</v>
       </c>
       <c r="N13" t="n">
-        <v>14.2</v>
+        <v>27</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>43.8</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1686,11 +1677,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr">
         <is>
           <t>No</t>
@@ -1700,11 +1687,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>XLE</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>129.13</v>
+        <v>68.68000000000001</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1733,23 +1720,23 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>70.7</v>
+        <v>70.5</v>
       </c>
       <c r="J14" t="n">
-        <v>63.8</v>
+        <v>63</v>
       </c>
       <c r="K14" t="n">
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="L14" t="n">
-        <v>1.71</v>
+        <v>2.09</v>
       </c>
       <c r="M14" t="n">
-        <v>22.2</v>
+        <v>29.3</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1757,7 +1744,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>54.9</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1789,59 +1776,59 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>307.32</v>
+        <v>392.83</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>70.59999999999999</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="J15" t="n">
-        <v>69.3</v>
+        <v>64.7</v>
       </c>
       <c r="K15" t="n">
-        <v>30</v>
+        <v>96</v>
       </c>
       <c r="L15" t="n">
-        <v>3.35</v>
+        <v>2.18</v>
       </c>
       <c r="M15" t="n">
-        <v>30.3</v>
+        <v>19.8</v>
       </c>
       <c r="N15" t="n">
-        <v>11.4</v>
+        <v>11.8</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1849,7 +1836,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>62.1</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1858,17 +1845,17 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U15" t="inlineStr"/>
@@ -1881,11 +1868,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>XEL</t>
+          <t>ACN</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>77.81999999999999</v>
+        <v>243.3</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1914,26 +1901,26 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>70</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="J16" t="n">
-        <v>64.5</v>
+        <v>65</v>
       </c>
       <c r="K16" t="n">
-        <v>97</v>
+        <v>74</v>
       </c>
       <c r="L16" t="n">
-        <v>1.68</v>
+        <v>4.69</v>
       </c>
       <c r="M16" t="n">
-        <v>18.7</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="N16" t="n">
-        <v>38.4</v>
+        <v>78.8</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1941,7 +1928,7 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>53.5</v>
+        <v>68.8</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1950,17 +1937,17 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
@@ -1973,59 +1960,56 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>WMT</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>119.22</v>
+        <v>306.88</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>69.8</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="J17" t="n">
-        <v>66</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="K17" t="n">
-        <v>94</v>
+        <v>50</v>
       </c>
       <c r="L17" t="n">
-        <v>2.04</v>
+        <v>3.16</v>
       </c>
       <c r="M17" t="n">
-        <v>23.1</v>
-      </c>
-      <c r="N17" t="n">
-        <v>35.6</v>
+        <v>40.3</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2033,7 +2017,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>56.8</v>
+        <v>62</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2065,59 +2049,59 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>DDOG</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>355.06</v>
+        <v>276.36</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>68.5</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="J18" t="n">
-        <v>58.1</v>
+        <v>55.2</v>
       </c>
       <c r="K18" t="n">
-        <v>89</v>
+        <v>13</v>
       </c>
       <c r="L18" t="n">
-        <v>1.8</v>
+        <v>5.22</v>
       </c>
       <c r="M18" t="n">
-        <v>18.7</v>
+        <v>55.9</v>
       </c>
       <c r="N18" t="n">
-        <v>29.8</v>
+        <v>40.1</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -2125,7 +2109,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>60.2</v>
+        <v>59.7</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2134,12 +2118,12 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
@@ -2147,7 +2131,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U18" t="inlineStr"/>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V18" t="inlineStr">
         <is>
           <t>No</t>
@@ -2157,11 +2145,11 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CDW</t>
+          <t>XEL</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>160.91</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2197,19 +2185,19 @@
         <v>68.3</v>
       </c>
       <c r="J19" t="n">
-        <v>63.9</v>
+        <v>60</v>
       </c>
       <c r="K19" t="n">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="L19" t="n">
-        <v>3.31</v>
+        <v>1.72</v>
       </c>
       <c r="M19" t="n">
-        <v>39.9</v>
+        <v>19.1</v>
       </c>
       <c r="N19" t="n">
-        <v>32.6</v>
+        <v>41.7</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -2217,7 +2205,7 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>60.8</v>
+        <v>52.2</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2249,11 +2237,11 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>AIG</t>
+          <t>MNST</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>79.56999999999999</v>
+        <v>45.69</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2286,22 +2274,22 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>67.90000000000001</v>
+        <v>67.8</v>
       </c>
       <c r="J20" t="n">
-        <v>55.4</v>
+        <v>54.3</v>
       </c>
       <c r="K20" t="n">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="L20" t="n">
-        <v>1.86</v>
+        <v>2.23</v>
       </c>
       <c r="M20" t="n">
-        <v>20.7</v>
+        <v>23.6</v>
       </c>
       <c r="N20" t="n">
-        <v>33.2</v>
+        <v>29.1</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2309,7 +2297,7 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>56.9</v>
+        <v>54.7</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2331,25 +2319,21 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U20" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>CDW</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>609.08</v>
+        <v>162.27</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2382,22 +2366,22 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>65.7</v>
+        <v>67.3</v>
       </c>
       <c r="J21" t="n">
-        <v>58.5</v>
+        <v>65.5</v>
       </c>
       <c r="K21" t="n">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="L21" t="n">
-        <v>1.68</v>
+        <v>3.14</v>
       </c>
       <c r="M21" t="n">
-        <v>19.1</v>
+        <v>39</v>
       </c>
       <c r="N21" t="n">
-        <v>23.1</v>
+        <v>31.2</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2405,7 +2389,7 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>63.5</v>
+        <v>61.6</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2414,17 +2398,17 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U21" t="inlineStr"/>
@@ -2437,15 +2421,15 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CHTR</t>
+          <t>PG</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>104.64</v>
+        <v>158.62</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -2460,45 +2444,45 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I22" t="n">
+        <v>66.5</v>
+      </c>
+      <c r="J22" t="n">
+        <v>60.4</v>
+      </c>
+      <c r="K22" t="n">
+        <v>97</v>
+      </c>
+      <c r="L22" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="M22" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="N22" t="n">
+        <v>78.2</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P22" t="n">
         <v>65.3</v>
       </c>
-      <c r="J22" t="n">
-        <v>39.5</v>
-      </c>
-      <c r="K22" t="n">
-        <v>11</v>
-      </c>
-      <c r="L22" t="n">
-        <v>4.91</v>
-      </c>
-      <c r="M22" t="n">
-        <v>45.2</v>
-      </c>
-      <c r="N22" t="n">
-        <v>34.4</v>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="P22" t="n">
-        <v>31.7</v>
-      </c>
       <c r="Q22" t="inlineStr">
         <is>
           <t>OFF</t>
@@ -2506,24 +2490,20 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t>Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr"/>
       <c r="V22" t="inlineStr">
         <is>
           <t>No</t>
@@ -2533,59 +2513,59 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>CVX</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>279.97</v>
+        <v>230.49</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>65.3</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="J23" t="n">
-        <v>57.1</v>
+        <v>68.3</v>
       </c>
       <c r="K23" t="n">
-        <v>12</v>
+        <v>83</v>
       </c>
       <c r="L23" t="n">
-        <v>5.41</v>
+        <v>2.02</v>
       </c>
       <c r="M23" t="n">
-        <v>55.5</v>
+        <v>21.5</v>
       </c>
       <c r="N23" t="n">
-        <v>39.6</v>
+        <v>41.8</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2593,7 +2573,7 @@
         </is>
       </c>
       <c r="P23" t="n">
-        <v>60.3</v>
+        <v>69</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -2615,11 +2595,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U23" t="inlineStr"/>
       <c r="V23" t="inlineStr">
         <is>
           <t>No</t>
@@ -2633,7 +2609,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>399.14</v>
+        <v>402.14</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -2666,22 +2642,22 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>65.09999999999999</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="J24" t="n">
-        <v>59.5</v>
+        <v>62.7</v>
       </c>
       <c r="K24" t="n">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="L24" t="n">
-        <v>1.69</v>
+        <v>1.8</v>
       </c>
       <c r="M24" t="n">
-        <v>19.9</v>
+        <v>19.1</v>
       </c>
       <c r="N24" t="n">
-        <v>29.1</v>
+        <v>23.6</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2689,7 +2665,7 @@
         </is>
       </c>
       <c r="P24" t="n">
-        <v>66.59999999999999</v>
+        <v>68.3</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -2711,21 +2687,25 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U24" t="inlineStr"/>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>COST</t>
+          <t>KDP</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>991.5</v>
+        <v>34.8</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -2758,22 +2738,22 @@
         </is>
       </c>
       <c r="I25" t="n">
-        <v>65</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="J25" t="n">
-        <v>61.9</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="K25" t="n">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="L25" t="n">
-        <v>1.64</v>
+        <v>2.04</v>
       </c>
       <c r="M25" t="n">
-        <v>17.1</v>
+        <v>27.5</v>
       </c>
       <c r="N25" t="n">
-        <v>16.1</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2781,7 +2761,7 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>57.7</v>
+        <v>64.5</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
@@ -2790,17 +2770,17 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U25" t="inlineStr"/>
@@ -2813,15 +2793,15 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>BKNG</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>150.53</v>
+        <v>356.64</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -2836,70 +2816,66 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>64.5</v>
+        <v>65</v>
       </c>
       <c r="J26" t="n">
-        <v>32.9</v>
+        <v>59.9</v>
       </c>
       <c r="K26" t="n">
-        <v>13</v>
+        <v>84</v>
       </c>
       <c r="L26" t="n">
-        <v>3.41</v>
+        <v>1.75</v>
       </c>
       <c r="M26" t="n">
-        <v>31</v>
+        <v>18.6</v>
       </c>
       <c r="N26" t="n">
-        <v>34.3</v>
+        <v>29.3</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P26" t="n">
-        <v>35.9</v>
+        <v>60.9</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>FIRED</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U26" t="inlineStr">
-        <is>
-          <t>Squeeze Fired, Squeeze Expanding</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr"/>
       <c r="V26" t="inlineStr">
         <is>
           <t>No</t>
@@ -2909,11 +2885,11 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>APD</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>507.49</v>
+        <v>306.85</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -2942,26 +2918,26 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I27" t="n">
-        <v>64</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="J27" t="n">
-        <v>68.90000000000001</v>
+        <v>68.8</v>
       </c>
       <c r="K27" t="n">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="L27" t="n">
-        <v>1.36</v>
+        <v>1.5</v>
       </c>
       <c r="M27" t="n">
-        <v>13.5</v>
+        <v>17.3</v>
       </c>
       <c r="N27" t="n">
-        <v>16.3</v>
+        <v>7</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -2969,7 +2945,7 @@
         </is>
       </c>
       <c r="P27" t="n">
-        <v>56.8</v>
+        <v>59.5</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
@@ -3001,11 +2977,11 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ABBV</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>286.52</v>
+        <v>612.9299999999999</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -3038,22 +3014,22 @@
         </is>
       </c>
       <c r="I28" t="n">
-        <v>61.1</v>
+        <v>63.9</v>
       </c>
       <c r="J28" t="n">
-        <v>66.7</v>
+        <v>60.7</v>
       </c>
       <c r="K28" t="n">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="L28" t="n">
-        <v>2.12</v>
+        <v>1.69</v>
       </c>
       <c r="M28" t="n">
-        <v>18</v>
+        <v>18.8</v>
       </c>
       <c r="N28" t="n">
-        <v>7</v>
+        <v>20.7</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -3061,7 +3037,7 @@
         </is>
       </c>
       <c r="P28" t="n">
-        <v>71.59999999999999</v>
+        <v>64.8</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
@@ -3070,17 +3046,17 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U28" t="inlineStr"/>
@@ -3093,11 +3069,11 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>INTU</t>
+          <t>EL</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>326.84</v>
+        <v>109.28</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -3126,31 +3102,34 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I29" t="n">
-        <v>60.3</v>
+        <v>63.2</v>
       </c>
       <c r="J29" t="n">
-        <v>54.4</v>
+        <v>67</v>
       </c>
       <c r="K29" t="n">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="L29" t="n">
-        <v>4.1</v>
+        <v>3</v>
       </c>
       <c r="M29" t="n">
-        <v>54.8</v>
+        <v>35.3</v>
+      </c>
+      <c r="N29" t="n">
+        <v>18.9</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P29" t="n">
-        <v>47.1</v>
+        <v>64</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
@@ -3159,17 +3138,17 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U29" t="inlineStr"/>
@@ -3182,11 +3161,11 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>MCK</t>
+          <t>WMT</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>968.6</v>
+        <v>118.76</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -3219,22 +3198,22 @@
         </is>
       </c>
       <c r="I30" t="n">
-        <v>51.1</v>
+        <v>62.3</v>
       </c>
       <c r="J30" t="n">
-        <v>54.6</v>
+        <v>64.2</v>
       </c>
       <c r="K30" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="L30" t="n">
-        <v>2.29</v>
+        <v>1.91</v>
       </c>
       <c r="M30" t="n">
-        <v>25.3</v>
+        <v>23</v>
       </c>
       <c r="N30" t="n">
-        <v>28.5</v>
+        <v>35.3</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -3242,7 +3221,7 @@
         </is>
       </c>
       <c r="P30" t="n">
-        <v>64.09999999999999</v>
+        <v>56.2</v>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
@@ -3251,17 +3230,17 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U30" t="inlineStr"/>
@@ -3274,59 +3253,59 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ILMN</t>
+          <t>ABBV</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>279.8</v>
+        <v>286.81</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I31" t="n">
-        <v>49.4</v>
+        <v>61.5</v>
       </c>
       <c r="J31" t="n">
-        <v>59.8</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="K31" t="n">
-        <v>12</v>
+        <v>79</v>
       </c>
       <c r="L31" t="n">
-        <v>5.05</v>
+        <v>2.2</v>
       </c>
       <c r="M31" t="n">
-        <v>55.5</v>
+        <v>17.9</v>
       </c>
       <c r="N31" t="n">
-        <v>56.2</v>
+        <v>6.7</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
@@ -3334,21 +3313,21 @@
         </is>
       </c>
       <c r="P31" t="n">
-        <v>74.5</v>
+        <v>71.7</v>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
@@ -3358,27 +3337,27 @@
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
+          <t>Divergence</t>
         </is>
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>MRK</t>
+          <t>LIN</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>141.92</v>
+        <v>506.67</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -3393,36 +3372,36 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I32" t="n">
-        <v>42.7</v>
+        <v>60.8</v>
       </c>
       <c r="J32" t="n">
-        <v>45</v>
+        <v>66.7</v>
       </c>
       <c r="K32" t="n">
-        <v>11</v>
+        <v>76</v>
       </c>
       <c r="L32" t="n">
-        <v>3.32</v>
+        <v>1.35</v>
       </c>
       <c r="M32" t="n">
-        <v>28.2</v>
+        <v>13.5</v>
       </c>
       <c r="N32" t="n">
-        <v>33.4</v>
+        <v>16.6</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -3430,33 +3409,29 @@
         </is>
       </c>
       <c r="P32" t="n">
-        <v>58.4</v>
+        <v>56.5</v>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U32" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr"/>
       <c r="V32" t="inlineStr">
         <is>
           <t>No</t>
@@ -3466,96 +3441,653 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>PCAR</t>
+          <t>AIG</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>102.49</v>
+        <v>79.78</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>60.4</v>
+      </c>
+      <c r="J33" t="n">
+        <v>56.3</v>
+      </c>
+      <c r="K33" t="n">
+        <v>95</v>
+      </c>
+      <c r="L33" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="M33" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="N33" t="n">
+        <v>32.8</v>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P33" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr"/>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>983.5700000000001</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>55.3</v>
+      </c>
+      <c r="J34" t="n">
+        <v>57.8</v>
+      </c>
+      <c r="K34" t="n">
+        <v>86</v>
+      </c>
+      <c r="L34" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="M34" t="n">
+        <v>17</v>
+      </c>
+      <c r="N34" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P34" t="n">
+        <v>55.9</v>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr"/>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>INTU</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>327.1</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="J35" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="K35" t="n">
+        <v>71</v>
+      </c>
+      <c r="L35" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="M35" t="n">
+        <v>41.9</v>
+      </c>
+      <c r="N35" t="n">
+        <v>29.1</v>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P35" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr"/>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>ILMN</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>288.39</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Debit Call</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="J36" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="K36" t="n">
+        <v>20</v>
+      </c>
+      <c r="L36" t="n">
+        <v>5.04</v>
+      </c>
+      <c r="M36" t="n">
+        <v>55.5</v>
+      </c>
+      <c r="N36" t="n">
+        <v>57</v>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P36" t="n">
+        <v>75.90000000000001</v>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>ODFL</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>173.77</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>SELL</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>Debit Put</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>30-60 DTE</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>NEUTRAL</t>
-        </is>
-      </c>
-      <c r="I33" t="n">
-        <v>40</v>
-      </c>
-      <c r="J33" t="n">
-        <v>26.2</v>
-      </c>
-      <c r="K33" t="n">
-        <v>20</v>
-      </c>
-      <c r="L33" t="n">
-        <v>3.09</v>
-      </c>
-      <c r="M33" t="n">
-        <v>21.7</v>
-      </c>
-      <c r="N33" t="n">
-        <v>30</v>
-      </c>
-      <c r="O33" t="inlineStr">
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="J37" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="K37" t="n">
+        <v>16</v>
+      </c>
+      <c r="L37" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="M37" t="n">
+        <v>35</v>
+      </c>
+      <c r="O37" t="inlineStr">
         <is>
           <t>Bearish</t>
         </is>
       </c>
-      <c r="P33" t="n">
-        <v>31.8</v>
-      </c>
-      <c r="Q33" t="inlineStr">
+      <c r="P37" t="n">
+        <v>38.6</v>
+      </c>
+      <c r="Q37" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="R33" t="inlineStr">
+      <c r="R37" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="S33" t="inlineStr">
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>MCK</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>961.09</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>42.1</v>
+      </c>
+      <c r="J38" t="n">
+        <v>52.2</v>
+      </c>
+      <c r="K38" t="n">
+        <v>91</v>
+      </c>
+      <c r="L38" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="M38" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="N38" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P38" t="n">
+        <v>62.7</v>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr"/>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>MRK</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>140.57</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="J39" t="n">
+        <v>43</v>
+      </c>
+      <c r="K39" t="n">
+        <v>18</v>
+      </c>
+      <c r="L39" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="M39" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="N39" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P39" t="n">
+        <v>56.9</v>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
         <is>
           <t>red</t>
         </is>
       </c>
-      <c r="T33" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U33" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
-      <c r="V33" t="inlineStr">
+      <c r="T39" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan 29.10.2026 19:29 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V39"/>
+  <dimension ref="A1:V37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -448,7 +448,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
     <col width="6" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>87.54000000000001</v>
+        <v>88.78</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,22 +614,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>93.59999999999999</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>73.2</v>
+        <v>75.3</v>
       </c>
       <c r="K2" t="n">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="L2" t="n">
-        <v>4.45</v>
+        <v>4.17</v>
       </c>
       <c r="M2" t="n">
         <v>57.1</v>
       </c>
       <c r="N2" t="n">
-        <v>99.2</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>60.8</v>
+        <v>62</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -659,25 +659,21 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DUK</t>
+          <t>EXC</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>123.81</v>
+        <v>45.92</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -710,19 +706,22 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>77.59999999999999</v>
+        <v>83.2</v>
       </c>
       <c r="J3" t="n">
-        <v>62.6</v>
+        <v>72.7</v>
       </c>
       <c r="K3" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L3" t="n">
-        <v>1.54</v>
+        <v>1.78</v>
       </c>
       <c r="M3" t="n">
-        <v>22.3</v>
+        <v>22.1</v>
+      </c>
+      <c r="N3" t="n">
+        <v>58.9</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -730,7 +729,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>53.8</v>
+        <v>56.7</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -762,11 +761,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>EXC</t>
+          <t>DUK</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>44.69</v>
+        <v>125.83</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -799,22 +798,22 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>77.2</v>
+        <v>80.5</v>
       </c>
       <c r="J4" t="n">
-        <v>66.2</v>
+        <v>66.7</v>
       </c>
       <c r="K4" t="n">
         <v>99</v>
       </c>
       <c r="L4" t="n">
-        <v>1.68</v>
+        <v>1.58</v>
       </c>
       <c r="M4" t="n">
-        <v>21</v>
+        <v>19.3</v>
       </c>
       <c r="N4" t="n">
-        <v>51.4</v>
+        <v>73.8</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -822,7 +821,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>52.6</v>
+        <v>57</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -854,11 +853,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>XEL</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>91.59999999999999</v>
+        <v>79.2</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -891,22 +890,22 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>75.40000000000001</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>60.7</v>
+        <v>66.7</v>
       </c>
       <c r="K5" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="L5" t="n">
-        <v>1.69</v>
+        <v>1.85</v>
       </c>
       <c r="M5" t="n">
         <v>20.2</v>
       </c>
       <c r="N5" t="n">
-        <v>72.59999999999999</v>
+        <v>50.1</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -914,7 +913,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>52.8</v>
+        <v>56.2</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -946,11 +945,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>COP</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>149.57</v>
+        <v>93.04000000000001</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -983,22 +982,22 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>75.2</v>
+        <v>76</v>
       </c>
       <c r="J6" t="n">
-        <v>69.40000000000001</v>
+        <v>64.8</v>
       </c>
       <c r="K6" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L6" t="n">
-        <v>2.43</v>
+        <v>1.71</v>
       </c>
       <c r="M6" t="n">
-        <v>26.5</v>
+        <v>20.7</v>
       </c>
       <c r="N6" t="n">
-        <v>18.4</v>
+        <v>76.8</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1006,7 +1005,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>68.5</v>
+        <v>55.9</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1038,11 +1037,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BRK-B</t>
+          <t>HD</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>541.7</v>
+        <v>326.98</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1075,30 +1074,30 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>74.3</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="J7" t="n">
-        <v>67.09999999999999</v>
+        <v>66.5</v>
       </c>
       <c r="K7" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L7" t="n">
-        <v>1.21</v>
+        <v>2.22</v>
       </c>
       <c r="M7" t="n">
-        <v>13.4</v>
+        <v>28.9</v>
       </c>
       <c r="N7" t="n">
-        <v>26.5</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>67.59999999999999</v>
+        <v>52</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1130,15 +1129,15 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CHTR</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>105.25</v>
+        <v>616.45</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1153,44 +1152,44 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>74</v>
+        <v>72.7</v>
       </c>
       <c r="J8" t="n">
-        <v>40.3</v>
+        <v>66.3</v>
       </c>
       <c r="K8" t="n">
-        <v>9</v>
+        <v>90</v>
       </c>
       <c r="L8" t="n">
-        <v>4.53</v>
+        <v>2.37</v>
       </c>
       <c r="M8" t="n">
-        <v>44.3</v>
+        <v>26.3</v>
       </c>
       <c r="N8" t="n">
-        <v>33.1</v>
+        <v>38.8</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>31.8</v>
+        <v>59.5</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1204,7 +1203,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>maroon</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -1222,11 +1221,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>BRK-B</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>128.54</v>
+        <v>542.74</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1259,19 +1258,22 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>72.40000000000001</v>
+        <v>72.3</v>
       </c>
       <c r="J9" t="n">
-        <v>59.8</v>
+        <v>67</v>
       </c>
       <c r="K9" t="n">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="L9" t="n">
-        <v>1.85</v>
+        <v>1.26</v>
       </c>
       <c r="M9" t="n">
-        <v>22.5</v>
+        <v>11.8</v>
+      </c>
+      <c r="N9" t="n">
+        <v>13.8</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1279,7 +1281,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>54.1</v>
+        <v>68.2</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1301,25 +1303,21 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>603.05</v>
+        <v>636.53</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1352,22 +1350,22 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>71.59999999999999</v>
+        <v>72.2</v>
       </c>
       <c r="J10" t="n">
-        <v>61.9</v>
+        <v>70.2</v>
       </c>
       <c r="K10" t="n">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="L10" t="n">
-        <v>2.45</v>
+        <v>2.07</v>
       </c>
       <c r="M10" t="n">
-        <v>26.1</v>
+        <v>22</v>
       </c>
       <c r="N10" t="n">
-        <v>38.4</v>
+        <v>42.5</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1375,7 +1373,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>56.4</v>
+        <v>70.8</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1407,11 +1405,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>EOG</t>
+          <t>MDT</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>161.52</v>
+        <v>96.94</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1444,22 +1442,22 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>71.40000000000001</v>
+        <v>70.5</v>
       </c>
       <c r="J11" t="n">
-        <v>69.8</v>
+        <v>62.4</v>
       </c>
       <c r="K11" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L11" t="n">
         <v>2.33</v>
       </c>
       <c r="M11" t="n">
-        <v>24.3</v>
+        <v>27.1</v>
       </c>
       <c r="N11" t="n">
-        <v>28.9</v>
+        <v>49.3</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1467,7 +1465,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>64.7</v>
+        <v>63.8</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1499,11 +1497,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>284.21</v>
+        <v>400.88</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1536,22 +1534,22 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>71.2</v>
+        <v>70.2</v>
       </c>
       <c r="J12" t="n">
-        <v>51.8</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="K12" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="L12" t="n">
-        <v>2.71</v>
+        <v>2.14</v>
       </c>
       <c r="M12" t="n">
-        <v>26.4</v>
+        <v>19.9</v>
       </c>
       <c r="N12" t="n">
-        <v>47.4</v>
+        <v>12.5</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1559,7 +1557,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>59.6</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1568,38 +1566,34 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>XOM</t>
+          <t>CDW</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>182.46</v>
+        <v>165.07</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1632,22 +1626,22 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>70.59999999999999</v>
+        <v>69.2</v>
       </c>
       <c r="J13" t="n">
-        <v>67.8</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="K13" t="n">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="L13" t="n">
-        <v>2.24</v>
+        <v>2.94</v>
       </c>
       <c r="M13" t="n">
-        <v>21.4</v>
+        <v>39.1</v>
       </c>
       <c r="N13" t="n">
-        <v>27</v>
+        <v>31.4</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1655,7 +1649,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>69.09999999999999</v>
+        <v>63.5</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1687,11 +1681,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>XLE</t>
+          <t>V</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>68.68000000000001</v>
+        <v>410.36</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1720,23 +1714,26 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>70.5</v>
+        <v>68.7</v>
       </c>
       <c r="J14" t="n">
-        <v>63</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="K14" t="n">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="L14" t="n">
-        <v>2.09</v>
+        <v>1.91</v>
       </c>
       <c r="M14" t="n">
-        <v>29.3</v>
+        <v>20</v>
+      </c>
+      <c r="N14" t="n">
+        <v>22</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1744,7 +1741,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>68.40000000000001</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1776,11 +1773,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>COP</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>392.83</v>
+        <v>149.68</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1813,22 +1810,22 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>70.40000000000001</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="J15" t="n">
-        <v>64.7</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="K15" t="n">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="L15" t="n">
-        <v>2.18</v>
+        <v>2.3</v>
       </c>
       <c r="M15" t="n">
-        <v>19.8</v>
+        <v>26.4</v>
       </c>
       <c r="N15" t="n">
-        <v>11.8</v>
+        <v>18</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1836,7 +1833,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>65.09999999999999</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1845,17 +1842,17 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U15" t="inlineStr"/>
@@ -1868,11 +1865,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ACN</t>
+          <t>XLP</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>243.3</v>
+        <v>88.12</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1901,26 +1898,23 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>69.40000000000001</v>
+        <v>68.2</v>
       </c>
       <c r="J16" t="n">
-        <v>65</v>
+        <v>61.5</v>
       </c>
       <c r="K16" t="n">
-        <v>74</v>
+        <v>95</v>
       </c>
       <c r="L16" t="n">
-        <v>4.69</v>
+        <v>1.45</v>
       </c>
       <c r="M16" t="n">
-        <v>67.09999999999999</v>
-      </c>
-      <c r="N16" t="n">
-        <v>78.8</v>
+        <v>16.6</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1928,7 +1922,7 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>68.8</v>
+        <v>63.5</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1937,17 +1931,17 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
@@ -1960,56 +1954,59 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>306.88</v>
+        <v>255.07</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>69.40000000000001</v>
+        <v>67.2</v>
       </c>
       <c r="J17" t="n">
-        <v>67.90000000000001</v>
+        <v>61.7</v>
       </c>
       <c r="K17" t="n">
-        <v>50</v>
+        <v>83</v>
       </c>
       <c r="L17" t="n">
-        <v>3.16</v>
+        <v>2.2</v>
       </c>
       <c r="M17" t="n">
-        <v>40.3</v>
+        <v>29.5</v>
+      </c>
+      <c r="N17" t="n">
+        <v>73</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2017,7 +2014,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>62</v>
+        <v>59.5</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2049,67 +2046,64 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>SYK</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>276.36</v>
+        <v>310.12</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>68.40000000000001</v>
+        <v>67</v>
       </c>
       <c r="J18" t="n">
-        <v>55.2</v>
+        <v>64.3</v>
       </c>
       <c r="K18" t="n">
-        <v>13</v>
+        <v>82</v>
       </c>
       <c r="L18" t="n">
-        <v>5.22</v>
+        <v>2.62</v>
       </c>
       <c r="M18" t="n">
-        <v>55.9</v>
-      </c>
-      <c r="N18" t="n">
-        <v>40.1</v>
+        <v>39</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>59.7</v>
+        <v>50</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2118,12 +2112,12 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
@@ -2131,11 +2125,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U18" t="inlineStr">
-        <is>
-          <t>Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr">
         <is>
           <t>No</t>
@@ -2145,11 +2135,11 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>XEL</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>77.23999999999999</v>
+        <v>76.28</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2182,22 +2172,22 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>68.3</v>
+        <v>66.8</v>
       </c>
       <c r="J19" t="n">
-        <v>60</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="K19" t="n">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="L19" t="n">
-        <v>1.72</v>
+        <v>2.22</v>
       </c>
       <c r="M19" t="n">
-        <v>19.1</v>
+        <v>23.8</v>
       </c>
       <c r="N19" t="n">
-        <v>41.7</v>
+        <v>46.2</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -2205,7 +2195,7 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>52.2</v>
+        <v>64.2</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2237,11 +2227,11 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MNST</t>
+          <t>KDP</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>45.69</v>
+        <v>35.22</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2274,22 +2264,22 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>67.8</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="J20" t="n">
-        <v>54.3</v>
+        <v>68.3</v>
       </c>
       <c r="K20" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="L20" t="n">
-        <v>2.23</v>
+        <v>2.02</v>
       </c>
       <c r="M20" t="n">
-        <v>23.6</v>
+        <v>27.1</v>
       </c>
       <c r="N20" t="n">
-        <v>29.1</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2297,7 +2287,7 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>54.7</v>
+        <v>65.7</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2306,17 +2296,17 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U20" t="inlineStr"/>
@@ -2329,11 +2319,11 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CDW</t>
+          <t>WMT</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>162.27</v>
+        <v>121.45</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2366,22 +2356,22 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>67.3</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="J21" t="n">
-        <v>65.5</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="K21" t="n">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="L21" t="n">
-        <v>3.14</v>
+        <v>1.94</v>
       </c>
       <c r="M21" t="n">
-        <v>39</v>
+        <v>23.5</v>
       </c>
       <c r="N21" t="n">
-        <v>31.2</v>
+        <v>37.8</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2389,7 +2379,7 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>61.6</v>
+        <v>59.2</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2421,11 +2411,11 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>158.62</v>
+        <v>360.71</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -2458,22 +2448,22 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>66.5</v>
+        <v>64.8</v>
       </c>
       <c r="J22" t="n">
-        <v>60.4</v>
+        <v>63.1</v>
       </c>
       <c r="K22" t="n">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="L22" t="n">
-        <v>1.93</v>
+        <v>1.74</v>
       </c>
       <c r="M22" t="n">
-        <v>24.5</v>
+        <v>19</v>
       </c>
       <c r="N22" t="n">
-        <v>78.2</v>
+        <v>31.5</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -2481,7 +2471,7 @@
         </is>
       </c>
       <c r="P22" t="n">
-        <v>65.3</v>
+        <v>62.6</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
@@ -2490,17 +2480,17 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U22" t="inlineStr"/>
@@ -2513,11 +2503,11 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CVX</t>
+          <t>APD</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>230.49</v>
+        <v>309.98</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -2550,22 +2540,22 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>66.40000000000001</v>
+        <v>64.5</v>
       </c>
       <c r="J23" t="n">
-        <v>68.3</v>
+        <v>72</v>
       </c>
       <c r="K23" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="L23" t="n">
-        <v>2.02</v>
+        <v>1.5</v>
       </c>
       <c r="M23" t="n">
-        <v>21.5</v>
+        <v>17.3</v>
       </c>
       <c r="N23" t="n">
-        <v>41.8</v>
+        <v>6.9</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2573,7 +2563,7 @@
         </is>
       </c>
       <c r="P23" t="n">
-        <v>69</v>
+        <v>60.9</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -2605,11 +2595,11 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>PG</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>402.14</v>
+        <v>160.54</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -2642,22 +2632,22 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>66.40000000000001</v>
+        <v>64</v>
       </c>
       <c r="J24" t="n">
-        <v>62.7</v>
+        <v>63</v>
       </c>
       <c r="K24" t="n">
         <v>95</v>
       </c>
       <c r="L24" t="n">
-        <v>1.8</v>
+        <v>1.88</v>
       </c>
       <c r="M24" t="n">
-        <v>19.1</v>
+        <v>24.8</v>
       </c>
       <c r="N24" t="n">
-        <v>23.6</v>
+        <v>80.2</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2665,7 +2655,7 @@
         </is>
       </c>
       <c r="P24" t="n">
-        <v>68.3</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -2674,38 +2664,34 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr"/>
       <c r="V24" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>EOG</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>34.8</v>
+        <v>161.07</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -2738,22 +2724,22 @@
         </is>
       </c>
       <c r="I25" t="n">
-        <v>65.59999999999999</v>
+        <v>63.5</v>
       </c>
       <c r="J25" t="n">
-        <v>65.40000000000001</v>
+        <v>69</v>
       </c>
       <c r="K25" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="L25" t="n">
-        <v>2.04</v>
+        <v>2.21</v>
       </c>
       <c r="M25" t="n">
-        <v>27.5</v>
+        <v>24.3</v>
       </c>
       <c r="N25" t="n">
-        <v>67.09999999999999</v>
+        <v>26.4</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2761,7 +2747,7 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>64.5</v>
+        <v>64.3</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
@@ -2793,11 +2779,11 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>ADP</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>356.64</v>
+        <v>285.95</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -2830,22 +2816,22 @@
         </is>
       </c>
       <c r="I26" t="n">
-        <v>65</v>
+        <v>63.3</v>
       </c>
       <c r="J26" t="n">
-        <v>59.9</v>
+        <v>53.3</v>
       </c>
       <c r="K26" t="n">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="L26" t="n">
-        <v>1.75</v>
+        <v>2.63</v>
       </c>
       <c r="M26" t="n">
-        <v>18.6</v>
+        <v>26</v>
       </c>
       <c r="N26" t="n">
-        <v>29.3</v>
+        <v>45.4</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -2853,7 +2839,7 @@
         </is>
       </c>
       <c r="P26" t="n">
-        <v>60.9</v>
+        <v>60.4</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
@@ -2862,17 +2848,17 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U26" t="inlineStr"/>
@@ -2885,11 +2871,11 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>APD</t>
+          <t>XOM</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>306.85</v>
+        <v>182.7</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -2918,26 +2904,26 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I27" t="n">
-        <v>64.90000000000001</v>
+        <v>63.3</v>
       </c>
       <c r="J27" t="n">
-        <v>68.8</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="K27" t="n">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="L27" t="n">
-        <v>1.5</v>
+        <v>2.19</v>
       </c>
       <c r="M27" t="n">
-        <v>17.3</v>
+        <v>21.3</v>
       </c>
       <c r="N27" t="n">
-        <v>7</v>
+        <v>26.2</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -2945,7 +2931,7 @@
         </is>
       </c>
       <c r="P27" t="n">
-        <v>59.5</v>
+        <v>69.3</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
@@ -2977,11 +2963,11 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>XLE</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>612.9299999999999</v>
+        <v>68.45</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -3010,26 +2996,23 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I28" t="n">
-        <v>63.9</v>
+        <v>62.7</v>
       </c>
       <c r="J28" t="n">
-        <v>60.7</v>
+        <v>62.1</v>
       </c>
       <c r="K28" t="n">
-        <v>95</v>
+        <v>66</v>
       </c>
       <c r="L28" t="n">
-        <v>1.69</v>
+        <v>2.06</v>
       </c>
       <c r="M28" t="n">
-        <v>18.8</v>
-      </c>
-      <c r="N28" t="n">
-        <v>20.7</v>
+        <v>27.1</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -3037,7 +3020,7 @@
         </is>
       </c>
       <c r="P28" t="n">
-        <v>64.8</v>
+        <v>67.8</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
@@ -3069,11 +3052,11 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>EL</t>
+          <t>CVX</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>109.28</v>
+        <v>230.92</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -3106,22 +3089,22 @@
         </is>
       </c>
       <c r="I29" t="n">
-        <v>63.2</v>
+        <v>62.1</v>
       </c>
       <c r="J29" t="n">
-        <v>67</v>
+        <v>68.8</v>
       </c>
       <c r="K29" t="n">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="L29" t="n">
-        <v>3</v>
+        <v>1.97</v>
       </c>
       <c r="M29" t="n">
-        <v>35.3</v>
+        <v>21.4</v>
       </c>
       <c r="N29" t="n">
-        <v>18.9</v>
+        <v>41.3</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -3129,7 +3112,7 @@
         </is>
       </c>
       <c r="P29" t="n">
-        <v>64</v>
+        <v>69.3</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
@@ -3161,11 +3144,11 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>WMT</t>
+          <t>AIG</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>118.76</v>
+        <v>81.12</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -3198,22 +3181,22 @@
         </is>
       </c>
       <c r="I30" t="n">
-        <v>62.3</v>
+        <v>60.6</v>
       </c>
       <c r="J30" t="n">
-        <v>64.2</v>
+        <v>61.4</v>
       </c>
       <c r="K30" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="L30" t="n">
-        <v>1.91</v>
+        <v>1.75</v>
       </c>
       <c r="M30" t="n">
-        <v>23</v>
+        <v>20.9</v>
       </c>
       <c r="N30" t="n">
-        <v>35.3</v>
+        <v>34</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -3221,7 +3204,7 @@
         </is>
       </c>
       <c r="P30" t="n">
-        <v>56.2</v>
+        <v>61.6</v>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
@@ -3253,11 +3236,11 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ABBV</t>
+          <t>EL</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>286.81</v>
+        <v>109.26</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -3286,26 +3269,26 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I31" t="n">
-        <v>61.5</v>
+        <v>60.3</v>
       </c>
       <c r="J31" t="n">
         <v>66.90000000000001</v>
       </c>
       <c r="K31" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="L31" t="n">
-        <v>2.2</v>
+        <v>2.93</v>
       </c>
       <c r="M31" t="n">
-        <v>17.9</v>
+        <v>34.7</v>
       </c>
       <c r="N31" t="n">
-        <v>6.7</v>
+        <v>17.5</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
@@ -3313,7 +3296,7 @@
         </is>
       </c>
       <c r="P31" t="n">
-        <v>71.7</v>
+        <v>64</v>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
@@ -3335,29 +3318,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U31" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
+      <c r="U31" t="inlineStr"/>
       <c r="V31" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>506.67</v>
+        <v>229.93</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -3372,36 +3351,36 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I32" t="n">
-        <v>60.8</v>
+        <v>60</v>
       </c>
       <c r="J32" t="n">
-        <v>66.7</v>
+        <v>43</v>
       </c>
       <c r="K32" t="n">
-        <v>76</v>
+        <v>13</v>
       </c>
       <c r="L32" t="n">
-        <v>1.35</v>
+        <v>4.14</v>
       </c>
       <c r="M32" t="n">
-        <v>13.5</v>
+        <v>33.3</v>
       </c>
       <c r="N32" t="n">
-        <v>16.6</v>
+        <v>11.5</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -3409,7 +3388,7 @@
         </is>
       </c>
       <c r="P32" t="n">
-        <v>56.5</v>
+        <v>55.4</v>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
@@ -3418,12 +3397,12 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
@@ -3431,21 +3410,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U32" t="inlineStr"/>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V32" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>AIG</t>
+          <t>ABBV</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>79.78</v>
+        <v>289.46</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -3474,26 +3457,26 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I33" t="n">
-        <v>60.4</v>
+        <v>59.9</v>
       </c>
       <c r="J33" t="n">
-        <v>56.3</v>
+        <v>69</v>
       </c>
       <c r="K33" t="n">
-        <v>95</v>
+        <v>75</v>
       </c>
       <c r="L33" t="n">
-        <v>1.74</v>
+        <v>2.19</v>
       </c>
       <c r="M33" t="n">
-        <v>20.7</v>
+        <v>18.2</v>
       </c>
       <c r="N33" t="n">
-        <v>32.8</v>
+        <v>7.9</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
@@ -3501,7 +3484,7 @@
         </is>
       </c>
       <c r="P33" t="n">
-        <v>57.5</v>
+        <v>72.5</v>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
@@ -3510,17 +3493,17 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U33" t="inlineStr"/>
@@ -3533,30 +3516,30 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>COST</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>983.5700000000001</v>
+        <v>253.26</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Credit Put</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -3570,30 +3553,30 @@
         </is>
       </c>
       <c r="I34" t="n">
-        <v>55.3</v>
+        <v>54.8</v>
       </c>
       <c r="J34" t="n">
-        <v>57.8</v>
+        <v>38.2</v>
       </c>
       <c r="K34" t="n">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="L34" t="n">
-        <v>1.61</v>
+        <v>5.35</v>
       </c>
       <c r="M34" t="n">
-        <v>17</v>
+        <v>59.8</v>
       </c>
       <c r="N34" t="n">
-        <v>15.7</v>
+        <v>25.4</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P34" t="n">
-        <v>55.9</v>
+        <v>43.7</v>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
@@ -3607,12 +3590,12 @@
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U34" t="inlineStr"/>
@@ -3625,35 +3608,35 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>INTU</t>
+          <t>ILMN</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>327.1</v>
+        <v>285.9</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Call</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -3662,44 +3645,44 @@
         </is>
       </c>
       <c r="I35" t="n">
-        <v>53.7</v>
+        <v>51.3</v>
       </c>
       <c r="J35" t="n">
-        <v>54.5</v>
+        <v>61.6</v>
       </c>
       <c r="K35" t="n">
-        <v>71</v>
+        <v>27</v>
       </c>
       <c r="L35" t="n">
-        <v>3.92</v>
+        <v>4.88</v>
       </c>
       <c r="M35" t="n">
-        <v>41.9</v>
+        <v>52.5</v>
       </c>
       <c r="N35" t="n">
-        <v>29.1</v>
+        <v>52.2</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P35" t="n">
-        <v>47.2</v>
+        <v>75.5</v>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
@@ -3707,7 +3690,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U35" t="inlineStr"/>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
       <c r="V35" t="inlineStr">
         <is>
           <t>No</t>
@@ -3717,59 +3704,59 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ILMN</t>
+          <t>COST</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>288.39</v>
+        <v>994.75</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D36" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I36" t="n">
-        <v>51.3</v>
+        <v>50.8</v>
       </c>
       <c r="J36" t="n">
-        <v>63.5</v>
+        <v>61.5</v>
       </c>
       <c r="K36" t="n">
-        <v>20</v>
+        <v>84</v>
       </c>
       <c r="L36" t="n">
-        <v>5.04</v>
+        <v>1.56</v>
       </c>
       <c r="M36" t="n">
-        <v>55.5</v>
+        <v>17.2</v>
       </c>
       <c r="N36" t="n">
-        <v>57</v>
+        <v>18.1</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
@@ -3777,21 +3764,21 @@
         </is>
       </c>
       <c r="P36" t="n">
-        <v>75.90000000000001</v>
+        <v>58.4</v>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
@@ -3799,11 +3786,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="U36" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+      <c r="U36" t="inlineStr"/>
       <c r="V36" t="inlineStr">
         <is>
           <t>No</t>
@@ -3817,7 +3800,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>173.77</v>
+        <v>170.05</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -3846,23 +3829,23 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I37" t="n">
-        <v>47.3</v>
+        <v>34.4</v>
       </c>
       <c r="J37" t="n">
-        <v>37.5</v>
+        <v>34.4</v>
       </c>
       <c r="K37" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="L37" t="n">
-        <v>3.9</v>
+        <v>4.44</v>
       </c>
       <c r="M37" t="n">
-        <v>35</v>
+        <v>34.3</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
@@ -3870,7 +3853,7 @@
         </is>
       </c>
       <c r="P37" t="n">
-        <v>38.6</v>
+        <v>37.1</v>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
@@ -3884,7 +3867,7 @@
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
@@ -3894,200 +3877,12 @@
       </c>
       <c r="U37" t="inlineStr">
         <is>
-          <t>Divergence, Squeeze Expanding</t>
+          <t>Divergence</t>
         </is>
       </c>
       <c r="V37" t="inlineStr">
         <is>
           <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>MCK</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>961.09</v>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>MEAN_REV</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>Credit Call</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>7-21 DTE</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>EXPANSION</t>
-        </is>
-      </c>
-      <c r="I38" t="n">
-        <v>42.1</v>
-      </c>
-      <c r="J38" t="n">
-        <v>52.2</v>
-      </c>
-      <c r="K38" t="n">
-        <v>91</v>
-      </c>
-      <c r="L38" t="n">
-        <v>2.24</v>
-      </c>
-      <c r="M38" t="n">
-        <v>25.1</v>
-      </c>
-      <c r="N38" t="n">
-        <v>28.1</v>
-      </c>
-      <c r="O38" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P38" t="n">
-        <v>62.7</v>
-      </c>
-      <c r="Q38" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="R38" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S38" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="T38" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U38" t="inlineStr"/>
-      <c r="V38" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>MRK</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>140.57</v>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>Debit Put</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>30-60 DTE</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>SQUEEZE</t>
-        </is>
-      </c>
-      <c r="I39" t="n">
-        <v>39.5</v>
-      </c>
-      <c r="J39" t="n">
-        <v>43</v>
-      </c>
-      <c r="K39" t="n">
-        <v>18</v>
-      </c>
-      <c r="L39" t="n">
-        <v>3.21</v>
-      </c>
-      <c r="M39" t="n">
-        <v>28.2</v>
-      </c>
-      <c r="N39" t="n">
-        <v>33.3</v>
-      </c>
-      <c r="O39" t="inlineStr">
-        <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="P39" t="n">
-        <v>56.9</v>
-      </c>
-      <c r="Q39" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="R39" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="S39" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="T39" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U39" t="inlineStr">
-        <is>
-          <t>TTM Squeeze, Squeeze Expanding</t>
-        </is>
-      </c>
-      <c r="V39" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan 30.10.2026 19:05 UTC
</commit_message>
<xml_diff>
--- a/output/scanner_results.xlsx
+++ b/output/scanner_results.xlsx
@@ -435,11 +435,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V37"/>
+  <dimension ref="A1:V56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>88.78</v>
+        <v>89.64</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -614,22 +614,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>92.09999999999999</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>75.3</v>
+        <v>76.3</v>
       </c>
       <c r="K2" t="n">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="L2" t="n">
-        <v>4.17</v>
+        <v>3.87</v>
       </c>
       <c r="M2" t="n">
-        <v>57.1</v>
+        <v>56.9</v>
       </c>
       <c r="N2" t="n">
-        <v>99.09999999999999</v>
+        <v>98.7</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>62</v>
+        <v>62.7</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -669,11 +669,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>EXC</t>
+          <t>TLT</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>45.92</v>
+        <v>81.64</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -706,30 +706,27 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>83.2</v>
+        <v>87.8</v>
       </c>
       <c r="J3" t="n">
-        <v>72.7</v>
+        <v>62.4</v>
       </c>
       <c r="K3" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L3" t="n">
-        <v>1.78</v>
+        <v>0.96</v>
       </c>
       <c r="M3" t="n">
-        <v>22.1</v>
-      </c>
-      <c r="N3" t="n">
-        <v>58.9</v>
+        <v>12.7</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>56.7</v>
+        <v>49.2</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -761,11 +758,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DUK</t>
+          <t>EXC</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>125.83</v>
+        <v>46.43</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -798,22 +795,22 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>80.5</v>
+        <v>87</v>
       </c>
       <c r="J4" t="n">
-        <v>66.7</v>
+        <v>74.8</v>
       </c>
       <c r="K4" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L4" t="n">
-        <v>1.58</v>
+        <v>1.87</v>
       </c>
       <c r="M4" t="n">
-        <v>19.3</v>
+        <v>21.7</v>
       </c>
       <c r="N4" t="n">
-        <v>73.8</v>
+        <v>56.1</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -821,7 +818,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>57</v>
+        <v>58.2</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -853,11 +850,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>XEL</t>
+          <t>DUK</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>79.2</v>
+        <v>128</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -890,22 +887,22 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>76.40000000000001</v>
+        <v>82.2</v>
       </c>
       <c r="J5" t="n">
-        <v>66.7</v>
+        <v>70.8</v>
       </c>
       <c r="K5" t="n">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="L5" t="n">
-        <v>1.85</v>
+        <v>1.57</v>
       </c>
       <c r="M5" t="n">
-        <v>20.2</v>
+        <v>19.6</v>
       </c>
       <c r="N5" t="n">
-        <v>50.1</v>
+        <v>75.7</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -913,7 +910,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>56.2</v>
+        <v>59.7</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -945,11 +942,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>WM</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>93.04000000000001</v>
+        <v>235.11</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -982,22 +979,22 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="J6" t="n">
-        <v>64.8</v>
+        <v>62.1</v>
       </c>
       <c r="K6" t="n">
         <v>95</v>
       </c>
       <c r="L6" t="n">
-        <v>1.71</v>
+        <v>2.57</v>
       </c>
       <c r="M6" t="n">
-        <v>20.7</v>
+        <v>27.6</v>
       </c>
       <c r="N6" t="n">
-        <v>76.8</v>
+        <v>97.5</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1005,7 +1002,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>55.9</v>
+        <v>58.9</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1027,21 +1024,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr"/>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>HD</t>
+          <t>BIIB</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>326.98</v>
+        <v>252.76</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1074,30 +1075,30 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>74.09999999999999</v>
+        <v>80.8</v>
       </c>
       <c r="J7" t="n">
-        <v>66.5</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="K7" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="L7" t="n">
-        <v>2.22</v>
+        <v>3.42</v>
       </c>
       <c r="M7" t="n">
-        <v>28.9</v>
+        <v>29.5</v>
       </c>
       <c r="N7" t="n">
-        <v>77.59999999999999</v>
+        <v>24.6</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>52</v>
+        <v>74.7</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1129,11 +1130,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>SYK</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>616.45</v>
+        <v>292.86</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1162,34 +1163,34 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>72.7</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="J8" t="n">
-        <v>66.3</v>
+        <v>48.7</v>
       </c>
       <c r="K8" t="n">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="L8" t="n">
-        <v>2.37</v>
+        <v>3.75</v>
       </c>
       <c r="M8" t="n">
-        <v>26.3</v>
+        <v>31.6</v>
       </c>
       <c r="N8" t="n">
-        <v>38.8</v>
+        <v>51.9</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>59.5</v>
+        <v>44</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1198,34 +1199,38 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BRK-B</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>542.74</v>
+        <v>78.29000000000001</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1254,26 +1259,23 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>72.3</v>
+        <v>78.8</v>
       </c>
       <c r="J9" t="n">
-        <v>67</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="K9" t="n">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="L9" t="n">
-        <v>1.26</v>
+        <v>2.45</v>
       </c>
       <c r="M9" t="n">
-        <v>11.8</v>
-      </c>
-      <c r="N9" t="n">
-        <v>13.8</v>
+        <v>24</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1281,7 +1283,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>68.2</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1313,11 +1315,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>XEL</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>636.53</v>
+        <v>80.44</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1350,22 +1352,22 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>72.2</v>
+        <v>78.3</v>
       </c>
       <c r="J10" t="n">
         <v>70.2</v>
       </c>
       <c r="K10" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="L10" t="n">
-        <v>2.07</v>
+        <v>1.85</v>
       </c>
       <c r="M10" t="n">
-        <v>22</v>
+        <v>19.5</v>
       </c>
       <c r="N10" t="n">
-        <v>42.5</v>
+        <v>44.5</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1373,7 +1375,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>70.8</v>
+        <v>58.4</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1405,11 +1407,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MDT</t>
+          <t>XLP</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>96.94</v>
+        <v>89.55</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1442,22 +1444,19 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>70.5</v>
+        <v>77.8</v>
       </c>
       <c r="J11" t="n">
-        <v>62.4</v>
+        <v>66</v>
       </c>
       <c r="K11" t="n">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="L11" t="n">
-        <v>2.33</v>
+        <v>1.58</v>
       </c>
       <c r="M11" t="n">
-        <v>27.1</v>
-      </c>
-      <c r="N11" t="n">
-        <v>49.3</v>
+        <v>18.6</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1465,7 +1464,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>63.8</v>
+        <v>66.7</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1497,11 +1496,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>HD</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>400.88</v>
+        <v>329.76</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1534,30 +1533,30 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>70.2</v>
+        <v>75.8</v>
       </c>
       <c r="J12" t="n">
-        <v>68.90000000000001</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="K12" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="L12" t="n">
-        <v>2.14</v>
+        <v>2.23</v>
       </c>
       <c r="M12" t="n">
-        <v>19.9</v>
+        <v>29.3</v>
       </c>
       <c r="N12" t="n">
-        <v>12.5</v>
+        <v>80.5</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>67.40000000000001</v>
+        <v>52.9</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1593,7 +1592,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>165.07</v>
+        <v>147.87</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1626,22 +1625,22 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>69.2</v>
+        <v>75.2</v>
       </c>
       <c r="J13" t="n">
-        <v>67.90000000000001</v>
+        <v>46.1</v>
       </c>
       <c r="K13" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="L13" t="n">
-        <v>2.94</v>
+        <v>4.72</v>
       </c>
       <c r="M13" t="n">
-        <v>39.1</v>
+        <v>49.9</v>
       </c>
       <c r="N13" t="n">
-        <v>31.4</v>
+        <v>48.3</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1649,7 +1648,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>63.5</v>
+        <v>53.6</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1658,34 +1657,38 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>green</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>410.36</v>
+        <v>94.16</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1718,22 +1721,22 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>68.7</v>
+        <v>75</v>
       </c>
       <c r="J14" t="n">
-        <v>67.59999999999999</v>
+        <v>67.8</v>
       </c>
       <c r="K14" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="L14" t="n">
-        <v>1.91</v>
+        <v>1.66</v>
       </c>
       <c r="M14" t="n">
-        <v>20</v>
+        <v>20.2</v>
       </c>
       <c r="N14" t="n">
-        <v>22</v>
+        <v>72.7</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1741,7 +1744,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>72.59999999999999</v>
+        <v>57.8</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1773,11 +1776,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>COP</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>149.68</v>
+        <v>96.22</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1810,22 +1813,22 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>68.40000000000001</v>
+        <v>73.2</v>
       </c>
       <c r="J15" t="n">
-        <v>69.59999999999999</v>
+        <v>64.2</v>
       </c>
       <c r="K15" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="L15" t="n">
-        <v>2.3</v>
+        <v>2.46</v>
       </c>
       <c r="M15" t="n">
         <v>26.4</v>
       </c>
       <c r="N15" t="n">
-        <v>18</v>
+        <v>74.8</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1833,7 +1836,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>68.59999999999999</v>
+        <v>64</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1865,11 +1868,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>XLP</t>
+          <t>BRK-B</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>88.12</v>
+        <v>544.28</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1902,19 +1905,22 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>68.2</v>
+        <v>72.8</v>
       </c>
       <c r="J16" t="n">
-        <v>61.5</v>
+        <v>68</v>
       </c>
       <c r="K16" t="n">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="L16" t="n">
-        <v>1.45</v>
+        <v>1.29</v>
       </c>
       <c r="M16" t="n">
-        <v>16.6</v>
+        <v>11.8</v>
+      </c>
+      <c r="N16" t="n">
+        <v>13.8</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1922,7 +1928,7 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>63.5</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1954,11 +1960,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ALL</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>255.07</v>
+        <v>639.14</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -1991,22 +1997,22 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>67.2</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="J17" t="n">
-        <v>61.7</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="K17" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="L17" t="n">
-        <v>2.2</v>
+        <v>2.01</v>
       </c>
       <c r="M17" t="n">
-        <v>29.5</v>
+        <v>21.8</v>
       </c>
       <c r="N17" t="n">
-        <v>73</v>
+        <v>40.8</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -2014,7 +2020,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>59.5</v>
+        <v>71.2</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2046,11 +2052,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SYK</t>
+          <t>NKE</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>310.12</v>
+        <v>38.72</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2083,19 +2089,22 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>67</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="J18" t="n">
-        <v>64.3</v>
+        <v>62.2</v>
       </c>
       <c r="K18" t="n">
-        <v>82</v>
+        <v>99</v>
       </c>
       <c r="L18" t="n">
-        <v>2.62</v>
+        <v>2.68</v>
       </c>
       <c r="M18" t="n">
-        <v>39</v>
+        <v>28</v>
+      </c>
+      <c r="N18" t="n">
+        <v>18.2</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -2103,7 +2112,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>50</v>
+        <v>43.1</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2135,11 +2144,11 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>MDLZ</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>76.28</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2172,22 +2181,22 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>66.8</v>
+        <v>71</v>
       </c>
       <c r="J19" t="n">
-        <v>66.09999999999999</v>
+        <v>62.1</v>
       </c>
       <c r="K19" t="n">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="L19" t="n">
-        <v>2.22</v>
+        <v>2.32</v>
       </c>
       <c r="M19" t="n">
-        <v>23.8</v>
+        <v>25.7</v>
       </c>
       <c r="N19" t="n">
-        <v>46.2</v>
+        <v>59.5</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -2195,7 +2204,7 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>64.2</v>
+        <v>61.5</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2227,11 +2236,11 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>35.22</v>
+        <v>261.61</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2264,22 +2273,22 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>65.59999999999999</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="J20" t="n">
-        <v>68.3</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="K20" t="n">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="L20" t="n">
-        <v>2.02</v>
+        <v>2.21</v>
       </c>
       <c r="M20" t="n">
-        <v>27.1</v>
+        <v>30.2</v>
       </c>
       <c r="N20" t="n">
-        <v>65.09999999999999</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2287,7 +2296,7 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>65.7</v>
+        <v>62.2</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2319,11 +2328,11 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>WMT</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>121.45</v>
+        <v>622.91</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2356,22 +2365,22 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>65.09999999999999</v>
+        <v>69.7</v>
       </c>
       <c r="J21" t="n">
-        <v>69.40000000000001</v>
+        <v>68.2</v>
       </c>
       <c r="K21" t="n">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="L21" t="n">
-        <v>1.94</v>
+        <v>2.23</v>
       </c>
       <c r="M21" t="n">
-        <v>23.5</v>
+        <v>26.5</v>
       </c>
       <c r="N21" t="n">
-        <v>37.8</v>
+        <v>39.4</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2379,7 +2388,7 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>59.2</v>
+        <v>60.6</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2411,15 +2420,15 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>360.71</v>
+        <v>883.65</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>MEAN_REV</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -2434,44 +2443,44 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Credit Call</t>
+          <t>Debit Put</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>7-21 DTE</t>
+          <t>30-60 DTE</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>SQUEEZE</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>64.8</v>
+        <v>69.5</v>
       </c>
       <c r="J22" t="n">
-        <v>63.1</v>
+        <v>42.5</v>
       </c>
       <c r="K22" t="n">
-        <v>82</v>
+        <v>19</v>
       </c>
       <c r="L22" t="n">
-        <v>1.74</v>
+        <v>2.92</v>
       </c>
       <c r="M22" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="N22" t="n">
-        <v>31.5</v>
+        <v>15.6</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="P22" t="n">
-        <v>62.6</v>
+        <v>36.9</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
@@ -2480,12 +2489,12 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>lime</t>
+          <t>red</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
@@ -2493,21 +2502,25 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U22" t="inlineStr"/>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>APD</t>
+          <t>XOM</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>309.98</v>
+        <v>186.37</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -2536,26 +2549,26 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>EXPANSION</t>
+          <t>NEUTRAL</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>64.5</v>
+        <v>68.8</v>
       </c>
       <c r="J23" t="n">
-        <v>72</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="K23" t="n">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="L23" t="n">
-        <v>1.5</v>
+        <v>2.23</v>
       </c>
       <c r="M23" t="n">
-        <v>17.3</v>
+        <v>21.6</v>
       </c>
       <c r="N23" t="n">
-        <v>6.9</v>
+        <v>28.2</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2563,7 +2576,7 @@
         </is>
       </c>
       <c r="P23" t="n">
-        <v>60.9</v>
+        <v>71.3</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -2595,11 +2608,11 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>MDT</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>160.54</v>
+        <v>96.81999999999999</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -2632,22 +2645,22 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>64</v>
+        <v>68.3</v>
       </c>
       <c r="J24" t="n">
-        <v>63</v>
+        <v>61.7</v>
       </c>
       <c r="K24" t="n">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="L24" t="n">
-        <v>1.88</v>
+        <v>2.25</v>
       </c>
       <c r="M24" t="n">
-        <v>24.8</v>
+        <v>27.1</v>
       </c>
       <c r="N24" t="n">
-        <v>80.2</v>
+        <v>49.4</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2655,7 +2668,7 @@
         </is>
       </c>
       <c r="P24" t="n">
-        <v>68.90000000000001</v>
+        <v>63.7</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -2687,11 +2700,11 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>EOG</t>
+          <t>PG</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>161.07</v>
+        <v>162.36</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -2724,22 +2737,22 @@
         </is>
       </c>
       <c r="I25" t="n">
-        <v>63.5</v>
+        <v>68.2</v>
       </c>
       <c r="J25" t="n">
-        <v>69</v>
+        <v>65.5</v>
       </c>
       <c r="K25" t="n">
         <v>94</v>
       </c>
       <c r="L25" t="n">
-        <v>2.21</v>
+        <v>2</v>
       </c>
       <c r="M25" t="n">
-        <v>24.3</v>
+        <v>24.7</v>
       </c>
       <c r="N25" t="n">
-        <v>26.4</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2747,7 +2760,7 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>64.3</v>
+        <v>71</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
@@ -2779,11 +2792,11 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>V</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>285.95</v>
+        <v>414.75</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -2816,22 +2829,22 @@
         </is>
       </c>
       <c r="I26" t="n">
-        <v>63.3</v>
+        <v>68.2</v>
       </c>
       <c r="J26" t="n">
-        <v>53.3</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="K26" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="L26" t="n">
-        <v>2.63</v>
+        <v>1.84</v>
       </c>
       <c r="M26" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="N26" t="n">
-        <v>45.4</v>
+        <v>21.9</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -2839,7 +2852,7 @@
         </is>
       </c>
       <c r="P26" t="n">
-        <v>60.4</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
@@ -2848,17 +2861,17 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U26" t="inlineStr"/>
@@ -2871,11 +2884,11 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>XOM</t>
+          <t>MNST</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>182.7</v>
+        <v>47.19</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -2904,26 +2917,26 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I27" t="n">
-        <v>63.3</v>
+        <v>68.2</v>
       </c>
       <c r="J27" t="n">
-        <v>68.09999999999999</v>
+        <v>62.3</v>
       </c>
       <c r="K27" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="L27" t="n">
-        <v>2.19</v>
+        <v>2.2</v>
       </c>
       <c r="M27" t="n">
-        <v>21.3</v>
+        <v>24.4</v>
       </c>
       <c r="N27" t="n">
-        <v>26.2</v>
+        <v>31.7</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -2931,7 +2944,7 @@
         </is>
       </c>
       <c r="P27" t="n">
-        <v>69.3</v>
+        <v>59.1</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
@@ -2963,11 +2976,11 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>XLE</t>
+          <t>WMT</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>68.45</v>
+        <v>123.78</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -2996,23 +3009,26 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I28" t="n">
-        <v>62.7</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="J28" t="n">
-        <v>62.1</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="K28" t="n">
-        <v>66</v>
+        <v>88</v>
       </c>
       <c r="L28" t="n">
-        <v>2.06</v>
+        <v>2</v>
       </c>
       <c r="M28" t="n">
-        <v>27.1</v>
+        <v>23.8</v>
+      </c>
+      <c r="N28" t="n">
+        <v>39.6</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -3020,7 +3036,7 @@
         </is>
       </c>
       <c r="P28" t="n">
-        <v>67.8</v>
+        <v>61.2</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
@@ -3029,17 +3045,17 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U28" t="inlineStr"/>
@@ -3052,11 +3068,11 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CVX</t>
+          <t>COP</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>230.92</v>
+        <v>153.23</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -3089,22 +3105,22 @@
         </is>
       </c>
       <c r="I29" t="n">
-        <v>62.1</v>
+        <v>67.8</v>
       </c>
       <c r="J29" t="n">
-        <v>68.8</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="K29" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="L29" t="n">
-        <v>1.97</v>
+        <v>2.28</v>
       </c>
       <c r="M29" t="n">
-        <v>21.4</v>
+        <v>26.5</v>
       </c>
       <c r="N29" t="n">
-        <v>41.3</v>
+        <v>16.2</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -3112,7 +3128,7 @@
         </is>
       </c>
       <c r="P29" t="n">
-        <v>69.3</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
@@ -3144,11 +3160,11 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>AIG</t>
+          <t>VRSK</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>81.12</v>
+        <v>197.31</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -3181,30 +3197,27 @@
         </is>
       </c>
       <c r="I30" t="n">
-        <v>60.6</v>
+        <v>67.7</v>
       </c>
       <c r="J30" t="n">
-        <v>61.4</v>
+        <v>62.5</v>
       </c>
       <c r="K30" t="n">
         <v>94</v>
       </c>
       <c r="L30" t="n">
-        <v>1.75</v>
+        <v>3.34</v>
       </c>
       <c r="M30" t="n">
-        <v>20.9</v>
-      </c>
-      <c r="N30" t="n">
-        <v>34</v>
+        <v>42.7</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P30" t="n">
-        <v>61.6</v>
+        <v>55.9</v>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
@@ -3236,11 +3249,11 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>EL</t>
+          <t>KO</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>109.26</v>
+        <v>94.27</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -3273,22 +3286,22 @@
         </is>
       </c>
       <c r="I31" t="n">
-        <v>60.3</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="J31" t="n">
-        <v>66.90000000000001</v>
+        <v>63.2</v>
       </c>
       <c r="K31" t="n">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="L31" t="n">
-        <v>2.93</v>
+        <v>1.86</v>
       </c>
       <c r="M31" t="n">
-        <v>34.7</v>
+        <v>20.3</v>
       </c>
       <c r="N31" t="n">
-        <v>17.5</v>
+        <v>49.6</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
@@ -3296,7 +3309,7 @@
         </is>
       </c>
       <c r="P31" t="n">
-        <v>64</v>
+        <v>68.8</v>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
@@ -3328,15 +3341,15 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>KDP</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>229.93</v>
+        <v>35.87</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>MEAN_REV</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -3351,36 +3364,36 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Debit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>SQUEEZE</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I32" t="n">
-        <v>60</v>
+        <v>66.7</v>
       </c>
       <c r="J32" t="n">
-        <v>43</v>
+        <v>71.7</v>
       </c>
       <c r="K32" t="n">
-        <v>13</v>
+        <v>94</v>
       </c>
       <c r="L32" t="n">
-        <v>4.14</v>
+        <v>2.06</v>
       </c>
       <c r="M32" t="n">
-        <v>33.3</v>
+        <v>26.7</v>
       </c>
       <c r="N32" t="n">
-        <v>11.5</v>
+        <v>63.1</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -3388,7 +3401,7 @@
         </is>
       </c>
       <c r="P32" t="n">
-        <v>55.4</v>
+        <v>67.2</v>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
@@ -3397,12 +3410,12 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
@@ -3410,25 +3423,21 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U32" t="inlineStr">
-        <is>
-          <t>Divergence, Squeeze Expanding</t>
-        </is>
-      </c>
+      <c r="U32" t="inlineStr"/>
       <c r="V32" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ABBV</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>289.46</v>
+        <v>364.65</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -3461,22 +3470,22 @@
         </is>
       </c>
       <c r="I33" t="n">
-        <v>59.9</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="J33" t="n">
-        <v>69</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="K33" t="n">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="L33" t="n">
-        <v>2.19</v>
+        <v>1.75</v>
       </c>
       <c r="M33" t="n">
-        <v>18.2</v>
+        <v>19.3</v>
       </c>
       <c r="N33" t="n">
-        <v>7.9</v>
+        <v>33.1</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
@@ -3484,7 +3493,7 @@
         </is>
       </c>
       <c r="P33" t="n">
-        <v>72.5</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
@@ -3516,30 +3525,30 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>ADP</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>253.26</v>
+        <v>295.78</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
           <t>MEAN_REV</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Credit Put</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -3553,30 +3562,30 @@
         </is>
       </c>
       <c r="I34" t="n">
-        <v>54.8</v>
+        <v>66</v>
       </c>
       <c r="J34" t="n">
-        <v>38.2</v>
+        <v>60.5</v>
       </c>
       <c r="K34" t="n">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="L34" t="n">
-        <v>5.35</v>
+        <v>2.72</v>
       </c>
       <c r="M34" t="n">
-        <v>59.8</v>
+        <v>27.5</v>
       </c>
       <c r="N34" t="n">
-        <v>25.4</v>
+        <v>52.6</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="P34" t="n">
-        <v>43.7</v>
+        <v>65.2</v>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
@@ -3585,12 +3594,12 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
@@ -3608,59 +3617,59 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ILMN</t>
+          <t>APD</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>285.9</v>
+        <v>313.83</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Debit Call</t>
+          <t>Credit Call</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>30-60 DTE</t>
+          <t>7-21 DTE</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>NEUTRAL</t>
+          <t>EXPANSION</t>
         </is>
       </c>
       <c r="I35" t="n">
-        <v>51.3</v>
+        <v>65.8</v>
       </c>
       <c r="J35" t="n">
-        <v>61.6</v>
+        <v>75</v>
       </c>
       <c r="K35" t="n">
-        <v>27</v>
+        <v>85</v>
       </c>
       <c r="L35" t="n">
-        <v>4.88</v>
+        <v>1.52</v>
       </c>
       <c r="M35" t="n">
-        <v>52.5</v>
+        <v>17.3</v>
       </c>
       <c r="N35" t="n">
-        <v>52.2</v>
+        <v>7</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
@@ -3668,11 +3677,11 @@
         </is>
       </c>
       <c r="P35" t="n">
-        <v>75.5</v>
+        <v>62.5</v>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
@@ -3687,14 +3696,10 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U35" t="inlineStr">
-        <is>
-          <t>TTM Squeeze</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr"/>
       <c r="V35" t="inlineStr">
         <is>
           <t>No</t>
@@ -3704,11 +3709,11 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>COST</t>
+          <t>EOG</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>994.75</v>
+        <v>165.01</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -3741,22 +3746,22 @@
         </is>
       </c>
       <c r="I36" t="n">
-        <v>50.8</v>
+        <v>65.7</v>
       </c>
       <c r="J36" t="n">
-        <v>61.5</v>
+        <v>73.8</v>
       </c>
       <c r="K36" t="n">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="L36" t="n">
-        <v>1.56</v>
+        <v>2.19</v>
       </c>
       <c r="M36" t="n">
-        <v>17.2</v>
+        <v>24.4</v>
       </c>
       <c r="N36" t="n">
-        <v>18.1</v>
+        <v>25</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
@@ -3764,7 +3769,7 @@
         </is>
       </c>
       <c r="P36" t="n">
-        <v>58.4</v>
+        <v>67</v>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
@@ -3773,17 +3778,17 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>lime</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U36" t="inlineStr"/>
@@ -3796,93 +3801,1877 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>MAR</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>400.55</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>65.59999999999999</v>
+      </c>
+      <c r="J37" t="n">
+        <v>68.8</v>
+      </c>
+      <c r="K37" t="n">
+        <v>93</v>
+      </c>
+      <c r="L37" t="n">
+        <v>2.04</v>
+      </c>
+      <c r="M37" t="n">
+        <v>34.7</v>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P37" t="n">
+        <v>67.3</v>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr"/>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>162.28</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>65.3</v>
+      </c>
+      <c r="J38" t="n">
+        <v>37.4</v>
+      </c>
+      <c r="K38" t="n">
+        <v>14</v>
+      </c>
+      <c r="L38" t="n">
+        <v>5.07</v>
+      </c>
+      <c r="M38" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="N38" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P38" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>EL</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>108.16</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>64.5</v>
+      </c>
+      <c r="J39" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="K39" t="n">
+        <v>78</v>
+      </c>
+      <c r="L39" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="M39" t="n">
+        <v>34.8</v>
+      </c>
+      <c r="N39" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P39" t="n">
+        <v>63.1</v>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>CVX</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>234.92</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>64</v>
+      </c>
+      <c r="J40" t="n">
+        <v>72.40000000000001</v>
+      </c>
+      <c r="K40" t="n">
+        <v>81</v>
+      </c>
+      <c r="L40" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="M40" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="N40" t="n">
+        <v>41</v>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P40" t="n">
+        <v>71.8</v>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr"/>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>CTAS</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>221.89</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>62</v>
+      </c>
+      <c r="J41" t="n">
+        <v>63.9</v>
+      </c>
+      <c r="K41" t="n">
+        <v>79</v>
+      </c>
+      <c r="L41" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="M41" t="n">
+        <v>27</v>
+      </c>
+      <c r="N41" t="n">
+        <v>52.7</v>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P41" t="n">
+        <v>67.3</v>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr"/>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>AMP</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>488.53</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>61.3</v>
+      </c>
+      <c r="J42" t="n">
+        <v>42</v>
+      </c>
+      <c r="K42" t="n">
+        <v>11</v>
+      </c>
+      <c r="L42" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="M42" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="N42" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P42" t="n">
+        <v>44.1</v>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>229</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>61</v>
+      </c>
+      <c r="J43" t="n">
+        <v>42.3</v>
+      </c>
+      <c r="K43" t="n">
+        <v>14</v>
+      </c>
+      <c r="L43" t="n">
+        <v>3.93</v>
+      </c>
+      <c r="M43" t="n">
+        <v>32.4</v>
+      </c>
+      <c r="N43" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P43" t="n">
+        <v>55.1</v>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>AIG</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>81.76000000000001</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>60.3</v>
+      </c>
+      <c r="J44" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="K44" t="n">
+        <v>92</v>
+      </c>
+      <c r="L44" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="M44" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="N44" t="n">
+        <v>34.7</v>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P44" t="n">
+        <v>63.1</v>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr"/>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>21.43</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>60.3</v>
+      </c>
+      <c r="J45" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="K45" t="n">
+        <v>94</v>
+      </c>
+      <c r="L45" t="n">
+        <v>3.54</v>
+      </c>
+      <c r="M45" t="n">
+        <v>45.8</v>
+      </c>
+      <c r="N45" t="n">
+        <v>99.2</v>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P45" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr"/>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1020.54</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="J46" t="n">
+        <v>68.5</v>
+      </c>
+      <c r="K46" t="n">
+        <v>84</v>
+      </c>
+      <c r="L46" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="M46" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="N46" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P46" t="n">
+        <v>63.1</v>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr"/>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>LRCX</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>235.34</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>58.7</v>
+      </c>
+      <c r="J47" t="n">
+        <v>32.8</v>
+      </c>
+      <c r="K47" t="n">
+        <v>97</v>
+      </c>
+      <c r="L47" t="n">
+        <v>6.23</v>
+      </c>
+      <c r="M47" t="n">
+        <v>59.6</v>
+      </c>
+      <c r="N47" t="n">
+        <v>25</v>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P47" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>AMAT</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>384.03</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>56.8</v>
+      </c>
+      <c r="J48" t="n">
+        <v>35.1</v>
+      </c>
+      <c r="K48" t="n">
+        <v>94</v>
+      </c>
+      <c r="L48" t="n">
+        <v>5.65</v>
+      </c>
+      <c r="M48" t="n">
+        <v>56.8</v>
+      </c>
+      <c r="N48" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P48" t="n">
+        <v>40.7</v>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>KLAC</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>157.05</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>56.4</v>
+      </c>
+      <c r="J49" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="K49" t="n">
+        <v>87</v>
+      </c>
+      <c r="L49" t="n">
+        <v>5.44</v>
+      </c>
+      <c r="M49" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="N49" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P49" t="n">
+        <v>42.6</v>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr"/>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>MDB</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>345.56</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Debit Put</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>SQUEEZE</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>56</v>
+      </c>
+      <c r="J50" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="K50" t="n">
+        <v>6</v>
+      </c>
+      <c r="L50" t="n">
+        <v>7.08</v>
+      </c>
+      <c r="M50" t="n">
+        <v>84.40000000000001</v>
+      </c>
+      <c r="N50" t="n">
+        <v>80</v>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P50" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>TTM Squeeze, Divergence, Squeeze Expanding</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>ASML</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1545.61</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>55.9</v>
+      </c>
+      <c r="J51" t="n">
+        <v>37.2</v>
+      </c>
+      <c r="K51" t="n">
+        <v>83</v>
+      </c>
+      <c r="L51" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="M51" t="n">
+        <v>41.7</v>
+      </c>
+      <c r="N51" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P51" t="n">
+        <v>44.7</v>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>200.34</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Credit Put</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="J52" t="n">
+        <v>33.5</v>
+      </c>
+      <c r="K52" t="n">
+        <v>84</v>
+      </c>
+      <c r="L52" t="n">
+        <v>7.46</v>
+      </c>
+      <c r="M52" t="n">
+        <v>90.09999999999999</v>
+      </c>
+      <c r="N52" t="n">
+        <v>61.2</v>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P52" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>MCK</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>993.17</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>44.8</v>
+      </c>
+      <c r="J53" t="n">
+        <v>60.4</v>
+      </c>
+      <c r="K53" t="n">
+        <v>84</v>
+      </c>
+      <c r="L53" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="M53" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="N53" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P53" t="n">
+        <v>69.2</v>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr"/>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>ZTS</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>79.75</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>MEAN_REV</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Credit Call</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>7-21 DTE</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>EXPANSION</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>43.7</v>
+      </c>
+      <c r="J54" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="K54" t="n">
+        <v>92</v>
+      </c>
+      <c r="L54" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="M54" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="N54" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="P54" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>lime</t>
+        </is>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr"/>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>MRK</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>149.74</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Debit Call</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>30-60 DTE</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>40.3</v>
+      </c>
+      <c r="J55" t="n">
+        <v>57.3</v>
+      </c>
+      <c r="K55" t="n">
+        <v>34</v>
+      </c>
+      <c r="L55" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="M55" t="n">
+        <v>30.7</v>
+      </c>
+      <c r="N55" t="n">
+        <v>44</v>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="P55" t="n">
+        <v>65.8</v>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>maroon</t>
+        </is>
+      </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>TTM Squeeze</t>
+        </is>
+      </c>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>ODFL</t>
         </is>
       </c>
-      <c r="B37" t="n">
-        <v>170.05</v>
-      </c>
-      <c r="C37" t="inlineStr">
+      <c r="B56" t="n">
+        <v>173.01</v>
+      </c>
+      <c r="C56" t="inlineStr">
         <is>
           <t>BREAKOUT</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>BEARISH</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E56" t="inlineStr">
         <is>
           <t>SELL</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F56" t="inlineStr">
         <is>
           <t>Debit Put</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="G56" t="inlineStr">
         <is>
           <t>30-60 DTE</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="H56" t="inlineStr">
         <is>
           <t>NEUTRAL</t>
         </is>
       </c>
-      <c r="I37" t="n">
-        <v>34.4</v>
-      </c>
-      <c r="J37" t="n">
-        <v>34.4</v>
-      </c>
-      <c r="K37" t="n">
-        <v>33</v>
-      </c>
-      <c r="L37" t="n">
-        <v>4.44</v>
-      </c>
-      <c r="M37" t="n">
-        <v>34.3</v>
-      </c>
-      <c r="O37" t="inlineStr">
+      <c r="I56" t="n">
+        <v>36.9</v>
+      </c>
+      <c r="J56" t="n">
+        <v>37.4</v>
+      </c>
+      <c r="K56" t="n">
+        <v>35</v>
+      </c>
+      <c r="L56" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="M56" t="n">
+        <v>32.4</v>
+      </c>
+      <c r="N56" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="O56" t="inlineStr">
         <is>
           <t>Bearish</t>
         </is>
       </c>
-      <c r="P37" t="n">
-        <v>37.1</v>
-      </c>
-      <c r="Q37" t="inlineStr">
+      <c r="P56" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="Q56" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="R37" t="inlineStr">
+      <c r="R56" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="S37" t="inlineStr">
+      <c r="S56" t="inlineStr">
         <is>
           <t>red</t>
         </is>
       </c>
-      <c r="T37" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U37" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
-      <c r="V37" t="inlineStr">
-        <is>
-          <t>Yes</t>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U56" t="inlineStr"/>
+      <c r="V56" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>